<commit_message>
Updates made for ICW, AS and MID
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\AZ-Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{690924CF-651C-47AE-9DB5-A81C0F6079F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67EAC93A-2C5A-49A4-9533-EDAD3CE5FD99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="809">
   <si>
     <t>Name</t>
   </si>
@@ -2358,9 +2358,6 @@
     <t>DU_AppCredentials</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>VOE_Exists</t>
   </si>
   <si>
@@ -2464,6 +2461,12 @@
   </si>
   <si>
     <t>Applicant is a Dominium employee. Manual review required.</t>
+  </si>
+  <si>
+    <t>Yardi_States</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -2921,7 +2924,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>772</v>
+        <v>808</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4522,7 +4525,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B42" t="s">
         <v>479</v>
@@ -5792,7 +5795,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z1012"/>
+  <dimension ref="A1:Z1013"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
@@ -5847,325 +5850,332 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>807</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>807</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
         <v>56</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" s="2" t="s">
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>212</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" t="s">
-        <v>562</v>
-      </c>
-      <c r="B12" t="s">
-        <v>562</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B13" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B14" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B15" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>603</v>
+        <v>565</v>
       </c>
       <c r="B16" t="s">
-        <v>603</v>
+        <v>565</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B17" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B18" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="B19" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B20" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>622</v>
+        <v>606</v>
       </c>
       <c r="B21" t="s">
-        <v>622</v>
+        <v>606</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>58</v>
+        <v>622</v>
       </c>
       <c r="B22" t="s">
-        <v>58</v>
+        <v>622</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A24" t="s">
         <v>205</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>205</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A24" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="B24" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>237</v>
+        <v>211</v>
+      </c>
+      <c r="B25" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A27" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>272</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A27" t="s">
-        <v>273</v>
-      </c>
-      <c r="B27" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>330</v>
+        <v>273</v>
       </c>
       <c r="B28" t="s">
-        <v>330</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>489</v>
+        <v>330</v>
       </c>
       <c r="B29" t="s">
-        <v>489</v>
+        <v>330</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" t="s">
+        <v>489</v>
+      </c>
+      <c r="B30" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A31" t="s">
         <v>490</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A31" s="2" t="s">
+    <row r="32" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A32" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>577</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A32" t="s">
+    <row r="33" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A33" t="s">
         <v>579</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B33" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A33" s="2" t="s">
+    <row r="34" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A34" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>578</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A34" t="s">
-        <v>580</v>
-      </c>
-      <c r="B34" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>596</v>
+        <v>580</v>
       </c>
       <c r="B35" t="s">
-        <v>596</v>
+        <v>580</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B36" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>642</v>
+        <v>597</v>
       </c>
       <c r="B37" t="s">
-        <v>642</v>
+        <v>597</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>763</v>
+        <v>642</v>
       </c>
       <c r="B38" t="s">
-        <v>763</v>
+        <v>642</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>679</v>
+        <v>763</v>
       </c>
       <c r="B39" t="s">
-        <v>679</v>
+        <v>763</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>718</v>
+        <v>679</v>
       </c>
       <c r="B40" t="s">
-        <v>718</v>
+        <v>679</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
       <c r="B41" t="s">
-        <v>724</v>
+        <v>718</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
+        <v>724</v>
+      </c>
+      <c r="B42" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A43" t="s">
         <v>770</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>770</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="46" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7135,6 +7145,7 @@
     <row r="1010" ht="14.25" customHeight="1"/>
     <row r="1011" ht="14.25" customHeight="1"/>
     <row r="1012" ht="14.25" customHeight="1"/>
+    <row r="1013" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7224,10 +7235,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
+        <v>788</v>
+      </c>
+      <c r="B10" t="s">
         <v>789</v>
-      </c>
-      <c r="B10" t="s">
-        <v>790</v>
       </c>
       <c r="C10" t="s">
         <v>682</v>
@@ -7273,7 +7284,7 @@
         <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7300,7 +7311,7 @@
         <v>678</v>
       </c>
       <c r="B19" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -7308,7 +7319,7 @@
         <v>690</v>
       </c>
       <c r="B20" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="C20" t="s">
         <v>682</v>
@@ -7330,7 +7341,7 @@
         <v>717</v>
       </c>
       <c r="B22" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="C22" t="s">
         <v>682</v>
@@ -7349,10 +7360,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>801</v>
+      </c>
+      <c r="B24" t="s">
         <v>802</v>
-      </c>
-      <c r="B24" t="s">
-        <v>803</v>
       </c>
       <c r="C24" t="s">
         <v>682</v>
@@ -7363,7 +7374,7 @@
         <v>527</v>
       </c>
       <c r="B25" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -7411,7 +7422,7 @@
         <v>195</v>
       </c>
       <c r="B32" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7419,7 +7430,7 @@
         <v>196</v>
       </c>
       <c r="B33" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -7467,7 +7478,7 @@
         <v>648</v>
       </c>
       <c r="B39" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -7483,10 +7494,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
+        <v>790</v>
+      </c>
+      <c r="B41" t="s">
         <v>791</v>
-      </c>
-      <c r="B41" t="s">
-        <v>792</v>
       </c>
       <c r="C41" t="s">
         <v>682</v>
@@ -7593,10 +7604,10 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
+        <v>778</v>
+      </c>
+      <c r="B55" t="s">
         <v>779</v>
-      </c>
-      <c r="B55" t="s">
-        <v>780</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -7697,7 +7708,7 @@
         <v>201</v>
       </c>
       <c r="B66" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -7705,7 +7716,7 @@
         <v>202</v>
       </c>
       <c r="B67" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="C67" t="s">
         <v>584</v>
@@ -7716,7 +7727,7 @@
         <v>575</v>
       </c>
       <c r="B68" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -7732,7 +7743,7 @@
         <v>551</v>
       </c>
       <c r="B70" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -8126,10 +8137,10 @@
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B118" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="C118" t="s">
         <v>682</v>
@@ -8432,7 +8443,7 @@
         <v>720</v>
       </c>
       <c r="B156" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="C156" t="s">
         <v>682</v>
@@ -8440,10 +8451,10 @@
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B157" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C157" t="s">
         <v>682</v>
@@ -8454,7 +8465,7 @@
         <v>727</v>
       </c>
       <c r="B158" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="C158" t="s">
         <v>682</v>
@@ -8522,10 +8533,10 @@
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
+        <v>775</v>
+      </c>
+      <c r="B166" t="s">
         <v>776</v>
-      </c>
-      <c r="B166" t="s">
-        <v>777</v>
       </c>
       <c r="C166" t="s">
         <v>682</v>
@@ -8632,10 +8643,10 @@
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B179" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="C179" t="s">
         <v>682</v>
@@ -8651,10 +8662,10 @@
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
+        <v>772</v>
+      </c>
+      <c r="B182" t="s">
         <v>773</v>
-      </c>
-      <c r="B182" t="s">
-        <v>774</v>
       </c>
       <c r="C182" t="s">
         <v>682</v>
@@ -9639,10 +9650,10 @@
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
+        <v>792</v>
+      </c>
+      <c r="B302" t="s">
         <v>793</v>
-      </c>
-      <c r="B302" t="s">
-        <v>794</v>
       </c>
       <c r="C302" t="s">
         <v>682</v>

</xml_diff>

<commit_message>
Updates to ICW, AS and MID
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67EAC93A-2C5A-49A4-9533-EDAD3CE5FD99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B2D439-9617-4153-8101-A1B2E1CE38EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
adding ASFA workflow with new prompt naming convention
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B2D439-9617-4153-8101-A1B2E1CE38EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66013D4D-9453-4787-BC81-CCD080ECD2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2466,7 +2466,7 @@
     <t>Yardi_States</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
added the RDC code piece
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66013D4D-9453-4787-BC81-CCD080ECD2A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050BBDAB-F905-4ABC-A1BF-4A0CAADA6BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1018" uniqueCount="809">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="822">
   <si>
     <t>Name</t>
   </si>
@@ -2467,6 +2467,45 @@
   </si>
   <si>
     <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>Household Demographic Reporting Form</t>
+  </si>
+  <si>
+    <t>HDR</t>
+  </si>
+  <si>
+    <t>HDRExists</t>
+  </si>
+  <si>
+    <t>Housing Demographic Reporting Form is a required document, but it is missing from the application.</t>
+  </si>
+  <si>
+    <t>HDR_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Housing Demographic Reporting Form. Needs manual review.</t>
+  </si>
+  <si>
+    <t>RDC_BothHourlyIncomeAndPSDocumented</t>
+  </si>
+  <si>
+    <t>RDC_Missing</t>
+  </si>
+  <si>
+    <t>The ICW includes multiple employments; however, Day Calculator is not available for all of them.</t>
+  </si>
+  <si>
+    <t>Both hourly income and check stub income have been documented on the same Day Calculator. Manual review required.</t>
+  </si>
+  <si>
+    <t>RDC_DominiumEmployee</t>
+  </si>
+  <si>
+    <t>RDC</t>
+  </si>
+  <si>
+    <t>Rounded Day Calculator</t>
   </si>
 </sst>
 </file>
@@ -3135,7 +3174,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="14.25" customHeight="1">
+    <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" t="s">
         <v>378</v>
       </c>
@@ -3143,7 +3182,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="14.25" customHeight="1">
+    <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
         <v>380</v>
       </c>
@@ -3151,7 +3190,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="14.25" customHeight="1">
+    <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
         <v>407</v>
       </c>
@@ -3159,7 +3198,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="14.25" customHeight="1">
+    <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
         <v>405</v>
       </c>
@@ -3167,7 +3206,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="14.25" customHeight="1">
+    <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
         <v>453</v>
       </c>
@@ -3175,7 +3214,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="14.25" customHeight="1">
+    <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
         <v>455</v>
       </c>
@@ -3183,7 +3222,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="14.25" customHeight="1">
+    <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
         <v>403</v>
       </c>
@@ -3191,7 +3230,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="14.25" customHeight="1">
+    <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
         <v>456</v>
       </c>
@@ -3199,7 +3238,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="14.25" customHeight="1">
+    <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
         <v>434</v>
       </c>
@@ -3207,23 +3246,34 @@
         <v>615</v>
       </c>
     </row>
-    <row r="42" spans="1:4" ht="14.25" customHeight="1">
+    <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
         <v>482</v>
       </c>
       <c r="B42" t="s">
         <v>482</v>
       </c>
-      <c r="D42" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="44" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="45" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="46" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="47" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="48" spans="1:4" ht="14.25" customHeight="1"/>
+    </row>
+    <row r="43" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A43" t="s">
+        <v>810</v>
+      </c>
+      <c r="B43" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A44" t="s">
+        <v>820</v>
+      </c>
+      <c r="B44" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="46" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>
     <row r="50" ht="14.25" customHeight="1"/>
     <row r="51" ht="14.25" customHeight="1"/>
@@ -7154,7 +7204,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C329"/>
+  <dimension ref="A1:C336"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -9874,6 +9924,61 @@
         <v>676</v>
       </c>
     </row>
+    <row r="331" spans="1:3">
+      <c r="A331" t="s">
+        <v>811</v>
+      </c>
+      <c r="B331" t="s">
+        <v>812</v>
+      </c>
+      <c r="C331" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3">
+      <c r="A332" t="s">
+        <v>813</v>
+      </c>
+      <c r="B332" t="s">
+        <v>814</v>
+      </c>
+      <c r="C332" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="334" spans="1:3">
+      <c r="A334" t="s">
+        <v>815</v>
+      </c>
+      <c r="B334" t="s">
+        <v>818</v>
+      </c>
+      <c r="C334" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="335" spans="1:3">
+      <c r="A335" t="s">
+        <v>816</v>
+      </c>
+      <c r="B335" t="s">
+        <v>817</v>
+      </c>
+      <c r="C335" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="336" spans="1:3">
+      <c r="A336" t="s">
+        <v>819</v>
+      </c>
+      <c r="B336" t="s">
+        <v>795</v>
+      </c>
+      <c r="C336" t="s">
+        <v>682</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates to config File
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050BBDAB-F905-4ABC-A1BF-4A0CAADA6BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C126E4-4F00-4A69-9116-F055C7916B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="822">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="881">
   <si>
     <t>Name</t>
   </si>
@@ -2202,9 +2202,6 @@
     <t>ICW_NotSupportedIncomeTypes</t>
   </si>
   <si>
-    <t>EDC_BothHourlyIncomeAndPSDocumented</t>
-  </si>
-  <si>
     <t>The {0} process has encountered a System Error.\n\nMachine Name: {1} &lt;br&gt;&lt;br&gt;LAN ID: {2} \n\nException Timestamp: {3} &lt;br&gt;&lt;br&gt;Transaction Reference: {4} &lt;br&gt;&lt;br&gt;Exception Message: {5} &lt;br&gt;&lt;br&gt;Exception Source: {6} &lt;br&gt;&lt;br&gt;Action Required: {7}</t>
   </si>
   <si>
@@ -2223,9 +2220,6 @@
     <t>updated by Harika</t>
   </si>
   <si>
-    <t>EDC_DominiumEmployee</t>
-  </si>
-  <si>
     <t>VRCCDoesNotExist</t>
   </si>
   <si>
@@ -2373,9 +2367,6 @@
     <t>Pay frequency could not be determined from the paystubs to compare to the Exact Day Calculator.</t>
   </si>
   <si>
-    <t>EDC_Missing</t>
-  </si>
-  <si>
     <t>MID_DuplicateSSNs</t>
   </si>
   <si>
@@ -2493,12 +2484,6 @@
     <t>RDC_Missing</t>
   </si>
   <si>
-    <t>The ICW includes multiple employments; however, Day Calculator is not available for all of them.</t>
-  </si>
-  <si>
-    <t>Both hourly income and check stub income have been documented on the same Day Calculator. Manual review required.</t>
-  </si>
-  <si>
     <t>RDC_DominiumEmployee</t>
   </si>
   <si>
@@ -2506,6 +2491,198 @@
   </si>
   <si>
     <t>Rounded Day Calculator</t>
+  </si>
+  <si>
+    <t>CSEI_SupportingDocInIAQ</t>
+  </si>
+  <si>
+    <t>Supporting documents have not been provided for Certification of Self-Employment Income documented on the Income &amp; Asset Questionnaire.</t>
+  </si>
+  <si>
+    <t>CSEI_SupportingDocsExist</t>
+  </si>
+  <si>
+    <t>Supporting documents do not exist for the Certification of Self-Employmet Income.</t>
+  </si>
+  <si>
+    <t>CSEI_MemName</t>
+  </si>
+  <si>
+    <t>Member name is not populated.</t>
+  </si>
+  <si>
+    <t>CSEI_NameOfBusiness</t>
+  </si>
+  <si>
+    <t>Name of Business is not populated.</t>
+  </si>
+  <si>
+    <t>CSEI_BusinessStartDate</t>
+  </si>
+  <si>
+    <t>Business Start Date is not populated.</t>
+  </si>
+  <si>
+    <t>CSEI_TypeOfBusiness</t>
+  </si>
+  <si>
+    <t>Type of Business is not populated.</t>
+  </si>
+  <si>
+    <t>CSEI_Qstn1check</t>
+  </si>
+  <si>
+    <t>Question 1 – Have you filed a Federal Income Tax Return from this business has not been completed appropriately.</t>
+  </si>
+  <si>
+    <t>CSEI_Qstn2check</t>
+  </si>
+  <si>
+    <t>Question 2 – Is your business continuously active throughout the year has not been completed appropriately.</t>
+  </si>
+  <si>
+    <t>CSEI_Qstn3check</t>
+  </si>
+  <si>
+    <t>Question 3 – Does any other member of your household receive a salary or other payments from this business has not been completed appropriately.</t>
+  </si>
+  <si>
+    <t>CSEI_Qstn3IsYes</t>
+  </si>
+  <si>
+    <t>Question 3 – Does any other member of your household receive a salary or other payments from this business has been documented as yes, manual review is required.</t>
+  </si>
+  <si>
+    <t>CSEI_Qstn4Check</t>
+  </si>
+  <si>
+    <t>Question 4 – How much net income was earned from this business over the last 12 months has not been populated.</t>
+  </si>
+  <si>
+    <t>CSEI_Qstn5check</t>
+  </si>
+  <si>
+    <t>Question 5 – How much net income do you anticipate do you anticipate earning from this business over the next 12 months has not been populated.</t>
+  </si>
+  <si>
+    <t>CSEI_Qstn6check</t>
+  </si>
+  <si>
+    <t>Last 12 months income and next 12 months anticipated income does not match but Question 6 documenting applicable reasons was not completed.</t>
+  </si>
+  <si>
+    <t>CSEI_HasSign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certification of Self-Employment Income was not signed. </t>
+  </si>
+  <si>
+    <t>CSEI_HasDate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certification of Self-Employment Income was not dated. </t>
+  </si>
+  <si>
+    <t>CSEI_DateCheckWithMoveIn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date on Certification of Self-Employment Income is not within 120 days of Move-in. </t>
+  </si>
+  <si>
+    <t>CSEI_AmountCheckInICW</t>
+  </si>
+  <si>
+    <t>Amount listed on the Certification of Self-Employment Income and ICW do not match.</t>
+  </si>
+  <si>
+    <t>CSEI_findingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Certification of Self-Employment Income. Needs manual review.</t>
+  </si>
+  <si>
+    <t>PL_ApplicantNameCheck</t>
+  </si>
+  <si>
+    <t>Applicant Name is not populated on the Profit/Loss Statement.</t>
+  </si>
+  <si>
+    <t>PL_BusinessNameCheck</t>
+  </si>
+  <si>
+    <t>Business Name is not populated on the Profit/Loss Statement.</t>
+  </si>
+  <si>
+    <t>PL_TypeofBusinessCheck</t>
+  </si>
+  <si>
+    <t>Type of Business is not populated on the Profit/Loss Statement.</t>
+  </si>
+  <si>
+    <t>PL_BusinessStartDateCheck</t>
+  </si>
+  <si>
+    <t>Business Start Date is not populated on the Profit/Loss Statement.</t>
+  </si>
+  <si>
+    <t>PL_NumberofMonthsCheck</t>
+  </si>
+  <si>
+    <t>Number of Months worked does not match the number of months documents on the Profit/Loss Statement.</t>
+  </si>
+  <si>
+    <t>PL_NetIncomedisplayedCheck</t>
+  </si>
+  <si>
+    <t>Net Income displayed on the Profit/Loss Statement does not match the calculated Net Income.</t>
+  </si>
+  <si>
+    <t>PL_AmountOnProfitLoss</t>
+  </si>
+  <si>
+    <t>Amount listed on the Self-Employment Certification and Profit/Loss Statement do not line up as expected. Needs additional review.</t>
+  </si>
+  <si>
+    <t>PL_ExpensesAreGeneric</t>
+  </si>
+  <si>
+    <t>PL_HasSignature</t>
+  </si>
+  <si>
+    <t>Profit/Loss Statement is not signed.</t>
+  </si>
+  <si>
+    <t>PL_HasDate</t>
+  </si>
+  <si>
+    <t>Profit/Loss Statement is not dated.</t>
+  </si>
+  <si>
+    <t>PL_DateCheckWithMoveIn</t>
+  </si>
+  <si>
+    <t>Date on the Profit/Loss Statement is not withing 120 days of the Move-In date.</t>
+  </si>
+  <si>
+    <t>PL_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Profit/Loss Statement. Manual review required.</t>
+  </si>
+  <si>
+    <t>1040_NameListCheck</t>
+  </si>
+  <si>
+    <t>1040_AmountListCheck</t>
+  </si>
+  <si>
+    <t>Amount listed on the Self-Employment Certification, 1040, and Schedule C do not line up as expected. Needs additional review.</t>
+  </si>
+  <si>
+    <t>1040_HasSignature</t>
+  </si>
+  <si>
+    <t>1040_HasDate</t>
   </si>
 </sst>
 </file>
@@ -2963,7 +3140,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -3256,18 +3433,18 @@
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="B43" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="B44" t="s">
-        <v>821</v>
+        <v>816</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
@@ -4575,7 +4752,7 @@
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="B42" t="s">
         <v>479</v>
@@ -4778,10 +4955,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="B20" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
@@ -4794,10 +4971,10 @@
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B22" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
@@ -5900,10 +6077,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="B3" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -6188,10 +6365,10 @@
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B39" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
@@ -6212,18 +6389,18 @@
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B42" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B43" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7204,7 +7381,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C336"/>
+  <dimension ref="A1:C369"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -7233,7 +7410,7 @@
         <v>714</v>
       </c>
       <c r="B5" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="C5" t="s">
         <v>682</v>
@@ -7241,10 +7418,10 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="B6" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="C6" t="s">
         <v>682</v>
@@ -7252,10 +7429,10 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="B7" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="C7" t="s">
         <v>682</v>
@@ -7263,10 +7440,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="B8" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="C8" t="s">
         <v>682</v>
@@ -7274,10 +7451,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B9" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="C9" t="s">
         <v>682</v>
@@ -7285,10 +7462,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="B10" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C10" t="s">
         <v>682</v>
@@ -7296,10 +7473,10 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="B11" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="C11" t="s">
         <v>682</v>
@@ -7334,7 +7511,7 @@
         <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7361,7 +7538,7 @@
         <v>678</v>
       </c>
       <c r="B19" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -7369,7 +7546,7 @@
         <v>690</v>
       </c>
       <c r="B20" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="C20" t="s">
         <v>682</v>
@@ -7391,7 +7568,7 @@
         <v>717</v>
       </c>
       <c r="B22" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="C22" t="s">
         <v>682</v>
@@ -7402,7 +7579,7 @@
         <v>719</v>
       </c>
       <c r="B23" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="C23" t="s">
         <v>682</v>
@@ -7410,10 +7587,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="B24" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="C24" t="s">
         <v>682</v>
@@ -7424,7 +7601,7 @@
         <v>527</v>
       </c>
       <c r="B25" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -7472,7 +7649,7 @@
         <v>195</v>
       </c>
       <c r="B32" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7480,7 +7657,7 @@
         <v>196</v>
       </c>
       <c r="B33" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -7528,7 +7705,7 @@
         <v>648</v>
       </c>
       <c r="B39" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="40" spans="1:3">
@@ -7544,10 +7721,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="B41" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
       <c r="C41" t="s">
         <v>682</v>
@@ -7654,10 +7831,10 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="B55" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
     </row>
     <row r="56" spans="1:3">
@@ -7758,7 +7935,7 @@
         <v>201</v>
       </c>
       <c r="B66" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -7766,7 +7943,7 @@
         <v>202</v>
       </c>
       <c r="B67" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="C67" t="s">
         <v>584</v>
@@ -7777,7 +7954,7 @@
         <v>575</v>
       </c>
       <c r="B68" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -7793,7 +7970,7 @@
         <v>551</v>
       </c>
       <c r="B70" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -7806,10 +7983,10 @@
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="B72" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C72" t="s">
         <v>682</v>
@@ -7849,10 +8026,10 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="B78" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="C78" t="s">
         <v>682</v>
@@ -7860,10 +8037,10 @@
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B79" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="C79" t="s">
         <v>682</v>
@@ -7871,10 +8048,10 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B80" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="C80" t="s">
         <v>682</v>
@@ -7882,10 +8059,10 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="B81" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="C81" t="s">
         <v>682</v>
@@ -7909,10 +8086,10 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="B85" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="C85" t="s">
         <v>682</v>
@@ -7920,10 +8097,10 @@
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="B86" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="C86" t="s">
         <v>682</v>
@@ -8031,10 +8208,10 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="B98" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="C98" t="s">
         <v>682</v>
@@ -8042,10 +8219,10 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="B99" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C99" t="s">
         <v>682</v>
@@ -8053,10 +8230,10 @@
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="B100" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C100" t="s">
         <v>682</v>
@@ -8187,10 +8364,10 @@
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="B118" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="C118" t="s">
         <v>682</v>
@@ -8309,10 +8486,10 @@
         <v>553</v>
       </c>
       <c r="B133" t="s">
+        <v>724</v>
+      </c>
+      <c r="C133" t="s">
         <v>725</v>
-      </c>
-      <c r="C133" t="s">
-        <v>726</v>
       </c>
     </row>
     <row r="134" spans="1:3">
@@ -8490,10 +8667,10 @@
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>720</v>
+        <v>812</v>
       </c>
       <c r="B156" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="C156" t="s">
         <v>682</v>
@@ -8501,10 +8678,10 @@
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>777</v>
+        <v>813</v>
       </c>
       <c r="B157" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="C157" t="s">
         <v>682</v>
@@ -8512,10 +8689,10 @@
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>727</v>
+        <v>814</v>
       </c>
       <c r="B158" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="C158" t="s">
         <v>682</v>
@@ -8583,10 +8760,10 @@
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="B166" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="C166" t="s">
         <v>682</v>
@@ -8682,10 +8859,10 @@
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="B178" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="C178" t="s">
         <v>682</v>
@@ -8693,10 +8870,10 @@
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="B179" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="C179" t="s">
         <v>682</v>
@@ -8712,10 +8889,10 @@
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B182" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="C182" t="s">
         <v>682</v>
@@ -9266,10 +9443,10 @@
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="B250" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="C250" t="s">
         <v>682</v>
@@ -9565,10 +9742,10 @@
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="B286" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="C286" t="s">
         <v>682</v>
@@ -9576,10 +9753,10 @@
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="B288" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="C288" t="s">
         <v>682</v>
@@ -9700,10 +9877,10 @@
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="B302" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="C302" t="s">
         <v>682</v>
@@ -9856,10 +10033,10 @@
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="B322" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="C322" t="s">
         <v>682</v>
@@ -9926,10 +10103,10 @@
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="B331" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="C331" t="s">
         <v>682</v>
@@ -9937,10 +10114,10 @@
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="B332" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="C332" t="s">
         <v>682</v>
@@ -9948,35 +10125,274 @@
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="B334" t="s">
         <v>818</v>
       </c>
-      <c r="C334" t="s">
-        <v>682</v>
-      </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>816</v>
+        <v>819</v>
       </c>
       <c r="B335" t="s">
-        <v>817</v>
-      </c>
-      <c r="C335" t="s">
-        <v>682</v>
+        <v>820</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
       <c r="B336" t="s">
-        <v>795</v>
-      </c>
-      <c r="C336" t="s">
-        <v>682</v>
+        <v>822</v>
+      </c>
+    </row>
+    <row r="337" spans="1:2">
+      <c r="A337" t="s">
+        <v>823</v>
+      </c>
+      <c r="B337" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="338" spans="1:2">
+      <c r="A338" t="s">
+        <v>825</v>
+      </c>
+      <c r="B338" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="339" spans="1:2">
+      <c r="A339" t="s">
+        <v>827</v>
+      </c>
+      <c r="B339" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2">
+      <c r="A340" t="s">
+        <v>829</v>
+      </c>
+      <c r="B340" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2">
+      <c r="A341" t="s">
+        <v>831</v>
+      </c>
+      <c r="B341" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="342" spans="1:2">
+      <c r="A342" t="s">
+        <v>833</v>
+      </c>
+      <c r="B342" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2">
+      <c r="A343" t="s">
+        <v>835</v>
+      </c>
+      <c r="B343" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2">
+      <c r="A344" t="s">
+        <v>837</v>
+      </c>
+      <c r="B344" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="345" spans="1:2">
+      <c r="A345" t="s">
+        <v>839</v>
+      </c>
+      <c r="B345" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2">
+      <c r="A346" t="s">
+        <v>841</v>
+      </c>
+      <c r="B346" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2">
+      <c r="A347" t="s">
+        <v>843</v>
+      </c>
+      <c r="B347" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="348" spans="1:2">
+      <c r="A348" t="s">
+        <v>845</v>
+      </c>
+      <c r="B348" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2">
+      <c r="A349" t="s">
+        <v>847</v>
+      </c>
+      <c r="B349" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2">
+      <c r="A350" t="s">
+        <v>849</v>
+      </c>
+      <c r="B350" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="351" spans="1:2">
+      <c r="A351" t="s">
+        <v>851</v>
+      </c>
+      <c r="B351" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="353" spans="1:2">
+      <c r="A353" t="s">
+        <v>853</v>
+      </c>
+      <c r="B353" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="354" spans="1:2">
+      <c r="A354" t="s">
+        <v>855</v>
+      </c>
+      <c r="B354" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2">
+      <c r="A355" t="s">
+        <v>857</v>
+      </c>
+      <c r="B355" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="356" spans="1:2">
+      <c r="A356" t="s">
+        <v>859</v>
+      </c>
+      <c r="B356" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2">
+      <c r="A357" t="s">
+        <v>861</v>
+      </c>
+      <c r="B357" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2">
+      <c r="A358" t="s">
+        <v>863</v>
+      </c>
+      <c r="B358" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2">
+      <c r="A359" t="s">
+        <v>865</v>
+      </c>
+      <c r="B359" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="360" spans="1:2">
+      <c r="A360" t="s">
+        <v>867</v>
+      </c>
+      <c r="B360" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="361" spans="1:2">
+      <c r="A361" t="s">
+        <v>868</v>
+      </c>
+      <c r="B361" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2">
+      <c r="A362" t="s">
+        <v>870</v>
+      </c>
+      <c r="B362" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2">
+      <c r="A363" t="s">
+        <v>872</v>
+      </c>
+      <c r="B363" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2">
+      <c r="A364" t="s">
+        <v>874</v>
+      </c>
+      <c r="B364" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2">
+      <c r="A366" t="s">
+        <v>876</v>
+      </c>
+      <c r="B366" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2">
+      <c r="A367" t="s">
+        <v>877</v>
+      </c>
+      <c r="B367" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2">
+      <c r="A368" t="s">
+        <v>879</v>
+      </c>
+      <c r="B368" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2">
+      <c r="A369" t="s">
+        <v>880</v>
+      </c>
+      <c r="B369" t="s">
+        <v>357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes for OL, WN and RDC
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3C126E4-4F00-4A69-9116-F055C7916B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F96CE5-BDF4-4F2F-82F4-CE3ED2C264C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="881">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="870">
   <si>
     <t>Name</t>
   </si>
@@ -909,27 +909,12 @@
     <t>Offer Letter</t>
   </si>
   <si>
-    <t>OL_DateCheck</t>
-  </si>
-  <si>
-    <t>OL_EmployerCheck</t>
-  </si>
-  <si>
     <t>OL_EmployeeCheck</t>
   </si>
   <si>
     <t>OL_PayCycleCheck</t>
   </si>
   <si>
-    <t>Date on the Offer Letter is greater than 120 days in the past.</t>
-  </si>
-  <si>
-    <t>Employer listed on the Offer Letter, Exact Day Calculator, and ICW do not match.</t>
-  </si>
-  <si>
-    <t>Employee Name listed on the Offer Letter, Exact Day Calculator, and ICW do not match.</t>
-  </si>
-  <si>
     <t>VOE_BlankFieldsCheck</t>
   </si>
   <si>
@@ -942,45 +927,27 @@
     <t>PS_PerYearEarningsCheck</t>
   </si>
   <si>
-    <t>OL_PerYearEarningsCheck</t>
-  </si>
-  <si>
     <t>VOE_CommissionsBonusTipsPopulated</t>
   </si>
   <si>
     <t>Commission, bonuses, tips, other amount has been populated. Needs additional review.</t>
   </si>
   <si>
-    <t>OL_HourlyPayRateCheck</t>
-  </si>
-  <si>
     <t>OL_SalariedPayRateCheck</t>
   </si>
   <si>
-    <t>Pay Amount listed on the Offer Letter and Exact Day Calculator do not match.</t>
-  </si>
-  <si>
     <t>OL_WeeklyHoursCheck</t>
   </si>
   <si>
-    <t>Weekly Hours listed on the Offer Letter and Exact Day Calculator do not match.</t>
-  </si>
-  <si>
     <t>OL_NoOfPayPeriodsNot1</t>
   </si>
   <si>
-    <t>Number of pay periods for a salaried employee is not listed as 1 on the Exact Day Calculator.</t>
-  </si>
-  <si>
     <t>WN</t>
   </si>
   <si>
     <t>Work Number</t>
   </si>
   <si>
-    <t>WN_EmployerCheck</t>
-  </si>
-  <si>
     <t>WN_EmployeeCheck</t>
   </si>
   <si>
@@ -990,45 +957,18 @@
     <t>WN_PayCycleCheck</t>
   </si>
   <si>
-    <t>WN_PerYearEarningsCheck</t>
-  </si>
-  <si>
-    <t>Date on the Work Number is greater than 120 days in the past.</t>
-  </si>
-  <si>
-    <t>Employer Name listed on the Work Number, Exact Day Calculator, and ICW do not match.</t>
-  </si>
-  <si>
-    <t>Employee Name listed on the Work Number, Exact Day Calculator, and ICW do not match.</t>
-  </si>
-  <si>
     <t>Work Number status is not listed as active.</t>
   </si>
   <si>
-    <t>WN_TotalMatchSum</t>
-  </si>
-  <si>
-    <t>Total Amount listed on the Work Number does not match the sum of the base, overtime, commission, bonus, and other columns.</t>
-  </si>
-  <si>
     <t>WN_PayPeriodEndingExistsInEDC</t>
   </si>
   <si>
-    <t>Two most recent Period Endings listed on the Work Number and Exact Day Calculator do not match.</t>
-  </si>
-  <si>
-    <t>Two most recent Period Starts listed on the Work Number and Exact Day Calculator do not match.</t>
-  </si>
-  <si>
     <t>WN_PayPeriodStartingExistsInEDC</t>
   </si>
   <si>
     <t>WN_RecentGrossPayMatch</t>
   </si>
   <si>
-    <t>Two most recent Gross Earnings listed on the Work Number and Exact Day Calculator do not match.</t>
-  </si>
-  <si>
     <t>WN_HighestCalValue</t>
   </si>
   <si>
@@ -1527,9 +1467,6 @@
     <t>Saving account value listed does not match that listed on the ICW.</t>
   </si>
   <si>
-    <t>WN_DateCheck</t>
-  </si>
-  <si>
     <t>VS_PayCycleCheck</t>
   </si>
   <si>
@@ -1584,15 +1521,9 @@
     <t>OL_EDCCheck</t>
   </si>
   <si>
-    <t>Exact Day Calculator does not exist for Offer Letter findings</t>
-  </si>
-  <si>
     <t>WN_EDCCheck</t>
   </si>
   <si>
-    <t>Exact Day Calculator does not exist for Work Number findings</t>
-  </si>
-  <si>
     <t>VS_EDCCheck</t>
   </si>
   <si>
@@ -1716,12 +1647,6 @@
     <t>Pay Frequency on the Verification of Employment and Exact Day Calculator do not match.</t>
   </si>
   <si>
-    <t>Pay Frequency listed on the Offer Letter and Exact Day Calculator do not match.</t>
-  </si>
-  <si>
-    <t>Pay Frequency listed on the Work Number and Exact Day Calculator do not match.</t>
-  </si>
-  <si>
     <t>Pay Frequency listed on Verification Services and Exact Day Calculator do not match.</t>
   </si>
   <si>
@@ -2683,6 +2608,48 @@
   </si>
   <si>
     <t>1040_HasDate</t>
+  </si>
+  <si>
+    <t>Day Calculator does not exist for Work Number findings</t>
+  </si>
+  <si>
+    <t>Employee Name listed on the Work Number, Day Calculator, and ICW do not match.</t>
+  </si>
+  <si>
+    <t>Pay Frequency listed on the Work Number and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>Two most recent Period Starts listed on the Work Number and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>Two most recent Period Endings listed on the Work Number and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>Two most recent Gross Earnings listed on the Work Number and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>Highest Calculated Income on the Day Calculator does not match Verified Income on the ICW.</t>
+  </si>
+  <si>
+    <t>Multiple employment documents provided for same employment. Can't determine which employment document to use to validate Day Calculator. Manual review required.</t>
+  </si>
+  <si>
+    <t>Day Calculator does not exist for Offer Letter findings</t>
+  </si>
+  <si>
+    <t>Employee Name listed on the Offer Letter, Day Calculator, and ICW do not match.</t>
+  </si>
+  <si>
+    <t>Pay Frequency listed on the Offer Letter and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>Weekly Hours listed on the Offer Letter and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>Number of pay periods for a salaried employee is not listed as 1 on the Day Calculator.</t>
+  </si>
+  <si>
+    <t>Pay Amount listed on the Offer Letter and Day Calculator do not match.</t>
   </si>
 </sst>
 </file>
@@ -3140,7 +3107,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>805</v>
+        <v>780</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -3173,7 +3140,7 @@
         <v>214</v>
       </c>
       <c r="B12" t="s">
-        <v>458</v>
+        <v>438</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -3186,10 +3153,10 @@
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>697</v>
+        <v>672</v>
       </c>
       <c r="B14" t="s">
-        <v>698</v>
+        <v>673</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
@@ -3197,7 +3164,7 @@
         <v>216</v>
       </c>
       <c r="B15" t="s">
-        <v>611</v>
+        <v>586</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
@@ -3205,7 +3172,7 @@
         <v>217</v>
       </c>
       <c r="B16" t="s">
-        <v>463</v>
+        <v>443</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
@@ -3213,7 +3180,7 @@
         <v>218</v>
       </c>
       <c r="B17" t="s">
-        <v>460</v>
+        <v>440</v>
       </c>
       <c r="C17" t="s">
         <v>233</v>
@@ -3235,7 +3202,7 @@
         <v>220</v>
       </c>
       <c r="B19" t="s">
-        <v>608</v>
+        <v>583</v>
       </c>
       <c r="C19" t="s">
         <v>235</v>
@@ -3246,7 +3213,7 @@
         <v>221</v>
       </c>
       <c r="B20" t="s">
-        <v>461</v>
+        <v>441</v>
       </c>
       <c r="C20" t="s">
         <v>236</v>
@@ -3257,7 +3224,7 @@
         <v>222</v>
       </c>
       <c r="B21" t="s">
-        <v>612</v>
+        <v>587</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
@@ -3265,7 +3232,7 @@
         <v>223</v>
       </c>
       <c r="B22" t="s">
-        <v>475</v>
+        <v>455</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
@@ -3273,7 +3240,7 @@
         <v>224</v>
       </c>
       <c r="B23" t="s">
-        <v>613</v>
+        <v>588</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
@@ -3281,12 +3248,12 @@
         <v>225</v>
       </c>
       <c r="B24" t="s">
-        <v>488</v>
+        <v>468</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>452</v>
+        <v>432</v>
       </c>
       <c r="B25" t="s">
         <v>234</v>
@@ -3297,7 +3264,7 @@
         <v>238</v>
       </c>
       <c r="B26" t="s">
-        <v>464</v>
+        <v>444</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
@@ -3321,26 +3288,26 @@
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="B29" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>331</v>
+        <v>311</v>
       </c>
       <c r="B30" t="s">
-        <v>332</v>
+        <v>312</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>376</v>
+        <v>356</v>
       </c>
       <c r="B31" t="s">
-        <v>614</v>
+        <v>589</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
@@ -3353,98 +3320,98 @@
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>378</v>
+        <v>358</v>
       </c>
       <c r="B33" t="s">
-        <v>379</v>
+        <v>359</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="B34" t="s">
-        <v>465</v>
+        <v>445</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>407</v>
+        <v>387</v>
       </c>
       <c r="B35" t="s">
-        <v>602</v>
+        <v>577</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>405</v>
+        <v>385</v>
       </c>
       <c r="B36" t="s">
-        <v>406</v>
+        <v>386</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>453</v>
+        <v>433</v>
       </c>
       <c r="B37" t="s">
-        <v>454</v>
+        <v>434</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>455</v>
+        <v>435</v>
       </c>
       <c r="B38" t="s">
-        <v>467</v>
+        <v>447</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>403</v>
+        <v>383</v>
       </c>
       <c r="B39" t="s">
-        <v>404</v>
+        <v>384</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>456</v>
+        <v>436</v>
       </c>
       <c r="B40" t="s">
-        <v>457</v>
+        <v>437</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>434</v>
+        <v>414</v>
       </c>
       <c r="B41" t="s">
-        <v>615</v>
+        <v>590</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>482</v>
+        <v>462</v>
       </c>
       <c r="B42" t="s">
-        <v>482</v>
+        <v>462</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="B43" t="s">
-        <v>806</v>
+        <v>781</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>815</v>
+        <v>790</v>
       </c>
       <c r="B44" t="s">
-        <v>816</v>
+        <v>791</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
@@ -4424,10 +4391,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>468</v>
+        <v>448</v>
       </c>
       <c r="B1" t="s">
-        <v>469</v>
+        <v>449</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -4435,15 +4402,15 @@
         <v>231</v>
       </c>
       <c r="B2" t="s">
-        <v>470</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>458</v>
+        <v>438</v>
       </c>
       <c r="B3" t="s">
-        <v>470</v>
+        <v>450</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -4451,15 +4418,15 @@
         <v>232</v>
       </c>
       <c r="B4" t="s">
-        <v>471</v>
+        <v>451</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>459</v>
+        <v>439</v>
       </c>
       <c r="B5" t="s">
-        <v>472</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -4467,15 +4434,15 @@
         <v>230</v>
       </c>
       <c r="B6" t="s">
-        <v>473</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>460</v>
+        <v>440</v>
       </c>
       <c r="B7" t="s">
-        <v>473</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -4483,15 +4450,15 @@
         <v>226</v>
       </c>
       <c r="B8" t="s">
-        <v>471</v>
+        <v>451</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>461</v>
+        <v>441</v>
       </c>
       <c r="B9" t="s">
-        <v>471</v>
+        <v>451</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -4499,15 +4466,15 @@
         <v>229</v>
       </c>
       <c r="B10" t="s">
-        <v>474</v>
+        <v>454</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>475</v>
+        <v>455</v>
       </c>
       <c r="B11" t="s">
-        <v>476</v>
+        <v>456</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -4523,47 +4490,47 @@
         <v>227</v>
       </c>
       <c r="B13" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>462</v>
+        <v>442</v>
       </c>
       <c r="B14" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>463</v>
+        <v>443</v>
       </c>
       <c r="B15" t="s">
-        <v>476</v>
+        <v>456</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>478</v>
+        <v>458</v>
       </c>
       <c r="B16" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>480</v>
+        <v>460</v>
       </c>
       <c r="B17" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18" t="s">
-        <v>481</v>
+        <v>461</v>
       </c>
       <c r="B18" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="19" spans="1:2">
@@ -4571,7 +4538,7 @@
         <v>236</v>
       </c>
       <c r="B19" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -4579,23 +4546,23 @@
         <v>233</v>
       </c>
       <c r="B20" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" t="s">
-        <v>482</v>
+        <v>462</v>
       </c>
       <c r="B21" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22" t="s">
-        <v>483</v>
+        <v>463</v>
       </c>
       <c r="B22" t="s">
-        <v>484</v>
+        <v>464</v>
       </c>
     </row>
     <row r="23" spans="1:2">
@@ -4603,7 +4570,7 @@
         <v>234</v>
       </c>
       <c r="B23" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -4611,23 +4578,23 @@
         <v>235</v>
       </c>
       <c r="B24" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
       <c r="B25" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26" t="s">
-        <v>464</v>
+        <v>444</v>
       </c>
       <c r="B26" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="27" spans="1:2">
@@ -4635,31 +4602,31 @@
         <v>288</v>
       </c>
       <c r="B27" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="B28" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29" t="s">
-        <v>332</v>
+        <v>312</v>
       </c>
       <c r="B29" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30" t="s">
-        <v>377</v>
+        <v>357</v>
       </c>
       <c r="B30" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="31" spans="1:2">
@@ -4667,95 +4634,95 @@
         <v>1040</v>
       </c>
       <c r="B31" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32" t="s">
-        <v>379</v>
+        <v>359</v>
       </c>
       <c r="B32" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33" t="s">
-        <v>381</v>
+        <v>361</v>
       </c>
       <c r="B33" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34" t="s">
-        <v>466</v>
+        <v>446</v>
       </c>
       <c r="B34" t="s">
-        <v>485</v>
+        <v>465</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" t="s">
-        <v>406</v>
+        <v>386</v>
       </c>
       <c r="B35" t="s">
-        <v>485</v>
+        <v>465</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36" t="s">
-        <v>404</v>
+        <v>384</v>
       </c>
       <c r="B36" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37" t="s">
+        <v>437</v>
+      </c>
+      <c r="B37" t="s">
         <v>457</v>
-      </c>
-      <c r="B37" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" t="s">
-        <v>454</v>
+        <v>434</v>
       </c>
       <c r="B38" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39" t="s">
-        <v>486</v>
+        <v>466</v>
       </c>
       <c r="B39" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40" t="s">
-        <v>487</v>
+        <v>467</v>
       </c>
       <c r="B40" t="s">
-        <v>477</v>
+        <v>457</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41" t="s">
-        <v>482</v>
+        <v>462</v>
       </c>
       <c r="B41" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42" t="s">
-        <v>784</v>
+        <v>759</v>
       </c>
       <c r="B42" t="s">
-        <v>479</v>
+        <v>459</v>
       </c>
     </row>
   </sheetData>
@@ -4955,10 +4922,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>769</v>
+        <v>744</v>
       </c>
       <c r="B20" t="s">
-        <v>769</v>
+        <v>744</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
@@ -4966,23 +4933,23 @@
         <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>498</v>
+        <v>477</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>721</v>
+        <v>696</v>
       </c>
       <c r="B22" t="s">
-        <v>720</v>
+        <v>695</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>598</v>
+        <v>573</v>
       </c>
       <c r="B23" t="s">
-        <v>598</v>
+        <v>573</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
@@ -6077,10 +6044,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>804</v>
+        <v>779</v>
       </c>
       <c r="B3" t="s">
-        <v>804</v>
+        <v>779</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -6157,82 +6124,82 @@
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>562</v>
+        <v>537</v>
       </c>
       <c r="B13" t="s">
-        <v>562</v>
+        <v>537</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>563</v>
+        <v>538</v>
       </c>
       <c r="B14" t="s">
-        <v>563</v>
+        <v>538</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>564</v>
+        <v>539</v>
       </c>
       <c r="B15" t="s">
-        <v>564</v>
+        <v>539</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>565</v>
+        <v>540</v>
       </c>
       <c r="B16" t="s">
-        <v>565</v>
+        <v>540</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>603</v>
+        <v>578</v>
       </c>
       <c r="B17" t="s">
-        <v>603</v>
+        <v>578</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>605</v>
+        <v>580</v>
       </c>
       <c r="B18" t="s">
-        <v>605</v>
+        <v>580</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>607</v>
+        <v>582</v>
       </c>
       <c r="B19" t="s">
-        <v>607</v>
+        <v>582</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>604</v>
+        <v>579</v>
       </c>
       <c r="B20" t="s">
-        <v>604</v>
+        <v>579</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>606</v>
+        <v>581</v>
       </c>
       <c r="B21" t="s">
-        <v>606</v>
+        <v>581</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>622</v>
+        <v>597</v>
       </c>
       <c r="B22" t="s">
-        <v>622</v>
+        <v>597</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
@@ -6285,122 +6252,122 @@
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>330</v>
+        <v>310</v>
       </c>
       <c r="B29" t="s">
-        <v>330</v>
+        <v>310</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>489</v>
+        <v>469</v>
       </c>
       <c r="B30" t="s">
-        <v>489</v>
+        <v>469</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>490</v>
+        <v>470</v>
       </c>
       <c r="B31" t="s">
-        <v>490</v>
+        <v>470</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>577</v>
+        <v>552</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>577</v>
+        <v>552</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>579</v>
+        <v>554</v>
       </c>
       <c r="B33" t="s">
-        <v>579</v>
+        <v>554</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>578</v>
+        <v>553</v>
       </c>
       <c r="B34" t="s">
-        <v>578</v>
+        <v>553</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>580</v>
+        <v>555</v>
       </c>
       <c r="B35" t="s">
-        <v>580</v>
+        <v>555</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>596</v>
+        <v>571</v>
       </c>
       <c r="B36" t="s">
-        <v>596</v>
+        <v>571</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>597</v>
+        <v>572</v>
       </c>
       <c r="B37" t="s">
-        <v>597</v>
+        <v>572</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>642</v>
+        <v>617</v>
       </c>
       <c r="B38" t="s">
-        <v>642</v>
+        <v>617</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>761</v>
+        <v>736</v>
       </c>
       <c r="B39" t="s">
-        <v>761</v>
+        <v>736</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>679</v>
+        <v>654</v>
       </c>
       <c r="B40" t="s">
-        <v>679</v>
+        <v>654</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>718</v>
+        <v>693</v>
       </c>
       <c r="B41" t="s">
-        <v>718</v>
+        <v>693</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>723</v>
+        <v>698</v>
       </c>
       <c r="B42" t="s">
-        <v>723</v>
+        <v>698</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>768</v>
+        <v>743</v>
       </c>
       <c r="B43" t="s">
-        <v>768</v>
+        <v>743</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7381,7 +7348,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C369"/>
+  <dimension ref="A1:C361"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -7407,79 +7374,79 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>714</v>
+        <v>689</v>
       </c>
       <c r="B5" t="s">
-        <v>752</v>
+        <v>727</v>
       </c>
       <c r="C5" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>746</v>
+        <v>721</v>
       </c>
       <c r="B6" t="s">
-        <v>753</v>
+        <v>728</v>
       </c>
       <c r="C6" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>747</v>
+        <v>722</v>
       </c>
       <c r="B7" t="s">
-        <v>754</v>
+        <v>729</v>
       </c>
       <c r="C7" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>748</v>
+        <v>723</v>
       </c>
       <c r="B8" t="s">
-        <v>756</v>
+        <v>731</v>
       </c>
       <c r="C8" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>757</v>
+        <v>732</v>
       </c>
       <c r="B9" t="s">
-        <v>755</v>
+        <v>730</v>
       </c>
       <c r="C9" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>785</v>
+        <v>760</v>
       </c>
       <c r="B10" t="s">
-        <v>786</v>
+        <v>761</v>
       </c>
       <c r="C10" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>749</v>
+        <v>724</v>
       </c>
       <c r="B11" t="s">
-        <v>750</v>
+        <v>725</v>
       </c>
       <c r="C11" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -7487,7 +7454,7 @@
         <v>179</v>
       </c>
       <c r="B13" t="s">
-        <v>492</v>
+        <v>472</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -7511,7 +7478,7 @@
         <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>801</v>
+        <v>776</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7522,86 +7489,86 @@
         <v>204</v>
       </c>
       <c r="C17" t="s">
-        <v>651</v>
+        <v>626</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>545</v>
+        <v>522</v>
       </c>
       <c r="B18" t="s">
-        <v>546</v>
+        <v>523</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>678</v>
+        <v>653</v>
       </c>
       <c r="B19" t="s">
-        <v>791</v>
+        <v>766</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>690</v>
+        <v>665</v>
       </c>
       <c r="B20" t="s">
-        <v>802</v>
+        <v>777</v>
       </c>
       <c r="C20" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>704</v>
+        <v>679</v>
       </c>
       <c r="B21" t="s">
-        <v>705</v>
+        <v>680</v>
       </c>
       <c r="C21" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>717</v>
+        <v>692</v>
       </c>
       <c r="B22" t="s">
-        <v>803</v>
+        <v>778</v>
       </c>
       <c r="C22" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>719</v>
+        <v>694</v>
       </c>
       <c r="B23" t="s">
-        <v>722</v>
+        <v>697</v>
       </c>
       <c r="C23" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>798</v>
+        <v>773</v>
       </c>
       <c r="B24" t="s">
-        <v>799</v>
+        <v>774</v>
       </c>
       <c r="C24" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>527</v>
+        <v>504</v>
       </c>
       <c r="B25" t="s">
-        <v>800</v>
+        <v>775</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -7622,10 +7589,10 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>554</v>
+        <v>531</v>
       </c>
       <c r="B29" t="s">
-        <v>555</v>
+        <v>532</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -7649,7 +7616,7 @@
         <v>195</v>
       </c>
       <c r="B32" t="s">
-        <v>781</v>
+        <v>756</v>
       </c>
     </row>
     <row r="33" spans="1:3">
@@ -7657,7 +7624,7 @@
         <v>196</v>
       </c>
       <c r="B33" t="s">
-        <v>782</v>
+        <v>757</v>
       </c>
     </row>
     <row r="34" spans="1:3">
@@ -7694,48 +7661,48 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>624</v>
+        <v>599</v>
       </c>
       <c r="B38" t="s">
-        <v>625</v>
+        <v>600</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>648</v>
+        <v>623</v>
       </c>
       <c r="B39" t="s">
-        <v>793</v>
+        <v>768</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>706</v>
+        <v>681</v>
       </c>
       <c r="B40" t="s">
-        <v>707</v>
+        <v>682</v>
       </c>
       <c r="C40" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>787</v>
+        <v>762</v>
       </c>
       <c r="B41" t="s">
-        <v>788</v>
+        <v>763</v>
       </c>
       <c r="C41" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>542</v>
+        <v>519</v>
       </c>
       <c r="B42" t="s">
-        <v>659</v>
+        <v>634</v>
       </c>
     </row>
     <row r="44" spans="1:3">
@@ -7802,7 +7769,7 @@
         <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="52" spans="1:3">
@@ -7815,37 +7782,37 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>626</v>
+        <v>601</v>
       </c>
       <c r="B53" t="s">
-        <v>627</v>
+        <v>602</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>541</v>
+        <v>518</v>
       </c>
       <c r="B54" t="s">
-        <v>660</v>
+        <v>635</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>775</v>
+        <v>750</v>
       </c>
       <c r="B55" t="s">
-        <v>776</v>
+        <v>751</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>683</v>
+        <v>658</v>
       </c>
       <c r="B56" t="s">
-        <v>684</v>
+        <v>659</v>
       </c>
       <c r="C56" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="58" spans="1:3">
@@ -7853,7 +7820,7 @@
         <v>183</v>
       </c>
       <c r="B58" t="s">
-        <v>587</v>
+        <v>562</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -7864,7 +7831,7 @@
         <v>107</v>
       </c>
       <c r="C59" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -7875,7 +7842,7 @@
         <v>117</v>
       </c>
       <c r="C60" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="61" spans="1:3">
@@ -7886,7 +7853,7 @@
         <v>119</v>
       </c>
       <c r="C61" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="62" spans="1:3">
@@ -7897,7 +7864,7 @@
         <v>108</v>
       </c>
       <c r="C62" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="63" spans="1:3">
@@ -7908,7 +7875,7 @@
         <v>109</v>
       </c>
       <c r="C63" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="64" spans="1:3">
@@ -7919,7 +7886,7 @@
         <v>110</v>
       </c>
       <c r="C64" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="65" spans="1:3">
@@ -7935,7 +7902,7 @@
         <v>201</v>
       </c>
       <c r="B66" t="s">
-        <v>777</v>
+        <v>752</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -7943,53 +7910,53 @@
         <v>202</v>
       </c>
       <c r="B67" t="s">
-        <v>778</v>
+        <v>753</v>
       </c>
       <c r="C67" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>575</v>
+        <v>550</v>
       </c>
       <c r="B68" t="s">
-        <v>779</v>
+        <v>754</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>543</v>
+        <v>520</v>
       </c>
       <c r="B69" t="s">
-        <v>544</v>
+        <v>521</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>551</v>
+        <v>528</v>
       </c>
       <c r="B70" t="s">
-        <v>780</v>
+        <v>755</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>540</v>
+        <v>517</v>
       </c>
       <c r="B71" t="s">
-        <v>661</v>
+        <v>636</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>734</v>
+        <v>709</v>
       </c>
       <c r="B72" t="s">
-        <v>733</v>
+        <v>708</v>
       </c>
       <c r="C72" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="74" spans="1:3">
@@ -8005,7 +7972,7 @@
         <v>121</v>
       </c>
       <c r="B75" t="s">
-        <v>588</v>
+        <v>563</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -8018,62 +7985,62 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>628</v>
+        <v>603</v>
       </c>
       <c r="B77" t="s">
-        <v>629</v>
+        <v>604</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>744</v>
+        <v>719</v>
       </c>
       <c r="B78" t="s">
-        <v>745</v>
+        <v>720</v>
       </c>
       <c r="C78" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>764</v>
+        <v>739</v>
       </c>
       <c r="B79" t="s">
-        <v>765</v>
+        <v>740</v>
       </c>
       <c r="C79" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>763</v>
+        <v>738</v>
       </c>
       <c r="B80" t="s">
-        <v>766</v>
+        <v>741</v>
       </c>
       <c r="C80" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>762</v>
+        <v>737</v>
       </c>
       <c r="B81" t="s">
-        <v>767</v>
+        <v>742</v>
       </c>
       <c r="C81" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>539</v>
+        <v>516</v>
       </c>
       <c r="B82" t="s">
-        <v>662</v>
+        <v>637</v>
       </c>
     </row>
     <row r="84" spans="1:3">
@@ -8086,24 +8053,24 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>743</v>
+        <v>718</v>
       </c>
       <c r="B85" t="s">
-        <v>758</v>
+        <v>733</v>
       </c>
       <c r="C85" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>741</v>
+        <v>716</v>
       </c>
       <c r="B86" t="s">
-        <v>742</v>
+        <v>717</v>
       </c>
       <c r="C86" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -8127,7 +8094,7 @@
         <v>137</v>
       </c>
       <c r="B89" t="s">
-        <v>589</v>
+        <v>564</v>
       </c>
     </row>
     <row r="90" spans="1:3">
@@ -8135,7 +8102,7 @@
         <v>138</v>
       </c>
       <c r="B90" t="s">
-        <v>590</v>
+        <v>565</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -8143,7 +8110,7 @@
         <v>139</v>
       </c>
       <c r="B91" t="s">
-        <v>591</v>
+        <v>566</v>
       </c>
     </row>
     <row r="92" spans="1:3">
@@ -8151,7 +8118,7 @@
         <v>140</v>
       </c>
       <c r="B92" t="s">
-        <v>592</v>
+        <v>567</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -8159,10 +8126,10 @@
         <v>141</v>
       </c>
       <c r="B93" t="s">
-        <v>491</v>
+        <v>471</v>
       </c>
       <c r="C93" t="s">
-        <v>677</v>
+        <v>652</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -8170,10 +8137,10 @@
         <v>142</v>
       </c>
       <c r="B94" t="s">
-        <v>493</v>
+        <v>473</v>
       </c>
       <c r="C94" t="s">
-        <v>552</v>
+        <v>529</v>
       </c>
     </row>
     <row r="95" spans="1:3">
@@ -8181,70 +8148,70 @@
         <v>143</v>
       </c>
       <c r="B95" t="s">
-        <v>494</v>
+        <v>474</v>
       </c>
       <c r="C95" t="s">
-        <v>552</v>
+        <v>529</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>630</v>
+        <v>605</v>
       </c>
       <c r="B96" t="s">
-        <v>631</v>
+        <v>606</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>708</v>
+        <v>683</v>
       </c>
       <c r="B97" t="s">
-        <v>709</v>
+        <v>684</v>
       </c>
       <c r="C97" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>735</v>
+        <v>710</v>
       </c>
       <c r="B98" t="s">
-        <v>736</v>
+        <v>711</v>
       </c>
       <c r="C98" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>738</v>
+        <v>713</v>
       </c>
       <c r="B99" t="s">
-        <v>737</v>
+        <v>712</v>
       </c>
       <c r="C99" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>740</v>
+        <v>715</v>
       </c>
       <c r="B100" t="s">
-        <v>739</v>
+        <v>714</v>
       </c>
       <c r="C100" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>538</v>
+        <v>515</v>
       </c>
       <c r="B101" t="s">
-        <v>663</v>
+        <v>638</v>
       </c>
     </row>
     <row r="103" spans="1:3">
@@ -8276,18 +8243,18 @@
         <v>144</v>
       </c>
       <c r="B106" t="s">
-        <v>576</v>
+        <v>551</v>
       </c>
       <c r="C106" t="s">
-        <v>681</v>
+        <v>656</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>680</v>
+        <v>655</v>
       </c>
       <c r="B107" t="s">
-        <v>576</v>
+        <v>551</v>
       </c>
     </row>
     <row r="108" spans="1:3">
@@ -8303,7 +8270,7 @@
         <v>130</v>
       </c>
       <c r="B109" t="s">
-        <v>593</v>
+        <v>568</v>
       </c>
     </row>
     <row r="110" spans="1:3">
@@ -8316,18 +8283,18 @@
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>632</v>
+        <v>607</v>
       </c>
       <c r="B111" t="s">
-        <v>633</v>
+        <v>608</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>537</v>
+        <v>514</v>
       </c>
       <c r="B112" t="s">
-        <v>664</v>
+        <v>639</v>
       </c>
     </row>
     <row r="114" spans="1:3">
@@ -8364,13 +8331,13 @@
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>797</v>
+        <v>772</v>
       </c>
       <c r="B118" t="s">
-        <v>796</v>
+        <v>771</v>
       </c>
       <c r="C118" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="119" spans="1:3">
@@ -8391,62 +8358,62 @@
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>623</v>
+        <v>598</v>
       </c>
       <c r="B121" t="s">
-        <v>685</v>
+        <v>660</v>
       </c>
       <c r="C121" t="s">
-        <v>689</v>
+        <v>664</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>634</v>
+        <v>609</v>
       </c>
       <c r="B122" t="s">
-        <v>635</v>
+        <v>610</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>536</v>
+        <v>513</v>
       </c>
       <c r="B123" t="s">
-        <v>665</v>
+        <v>640</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>710</v>
+        <v>685</v>
       </c>
       <c r="B124" t="s">
-        <v>711</v>
+        <v>686</v>
       </c>
       <c r="C124" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>699</v>
+        <v>674</v>
       </c>
       <c r="B126" t="s">
-        <v>700</v>
+        <v>675</v>
       </c>
       <c r="C126" t="s">
-        <v>701</v>
+        <v>676</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>702</v>
+        <v>677</v>
       </c>
       <c r="B127" t="s">
-        <v>703</v>
+        <v>678</v>
       </c>
       <c r="C127" t="s">
-        <v>701</v>
+        <v>676</v>
       </c>
     </row>
     <row r="129" spans="1:3">
@@ -8478,34 +8445,34 @@
         <v>161</v>
       </c>
       <c r="B132" t="s">
-        <v>594</v>
+        <v>569</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>553</v>
+        <v>530</v>
       </c>
       <c r="B133" t="s">
-        <v>724</v>
+        <v>699</v>
       </c>
       <c r="C133" t="s">
-        <v>725</v>
+        <v>700</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>640</v>
+        <v>615</v>
       </c>
       <c r="B134" t="s">
-        <v>641</v>
+        <v>616</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>535</v>
+        <v>512</v>
       </c>
       <c r="B135" t="s">
-        <v>666</v>
+        <v>641</v>
       </c>
     </row>
     <row r="137" spans="1:3">
@@ -8534,29 +8501,29 @@
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>636</v>
+        <v>611</v>
       </c>
       <c r="B140" t="s">
-        <v>637</v>
+        <v>612</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>534</v>
+        <v>511</v>
       </c>
       <c r="B141" t="s">
-        <v>667</v>
+        <v>642</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>712</v>
+        <v>687</v>
       </c>
       <c r="B142" t="s">
-        <v>713</v>
+        <v>688</v>
       </c>
       <c r="C142" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="144" spans="1:3">
@@ -8575,7 +8542,7 @@
         <v>171</v>
       </c>
       <c r="C145" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="146" spans="1:3">
@@ -8586,7 +8553,7 @@
         <v>172</v>
       </c>
       <c r="C146" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="147" spans="1:3">
@@ -8597,7 +8564,7 @@
         <v>173</v>
       </c>
       <c r="C147" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="148" spans="1:3">
@@ -8624,108 +8591,108 @@
         <v>176</v>
       </c>
       <c r="C150" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>638</v>
+        <v>613</v>
       </c>
       <c r="B151" t="s">
-        <v>639</v>
+        <v>614</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>523</v>
+        <v>500</v>
       </c>
       <c r="B152" t="s">
-        <v>668</v>
+        <v>643</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>645</v>
+        <v>620</v>
       </c>
       <c r="B154" t="s">
-        <v>646</v>
+        <v>621</v>
       </c>
       <c r="C154" t="s">
-        <v>647</v>
+        <v>622</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>715</v>
+        <v>690</v>
       </c>
       <c r="B155" t="s">
-        <v>716</v>
+        <v>691</v>
       </c>
       <c r="C155" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>812</v>
+        <v>787</v>
       </c>
       <c r="B156" t="s">
-        <v>794</v>
+        <v>769</v>
       </c>
       <c r="C156" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>813</v>
+        <v>788</v>
       </c>
       <c r="B157" t="s">
-        <v>783</v>
+        <v>758</v>
       </c>
       <c r="C157" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>814</v>
+        <v>789</v>
       </c>
       <c r="B158" t="s">
-        <v>792</v>
+        <v>767</v>
       </c>
       <c r="C158" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>509</v>
+        <v>488</v>
       </c>
       <c r="B160" t="s">
-        <v>510</v>
+        <v>489</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>653</v>
+        <v>628</v>
       </c>
       <c r="B161" t="s">
-        <v>657</v>
+        <v>632</v>
       </c>
       <c r="C161" t="s">
-        <v>655</v>
+        <v>630</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>654</v>
+        <v>629</v>
       </c>
       <c r="B162" t="s">
-        <v>656</v>
+        <v>631</v>
       </c>
       <c r="C162" t="s">
-        <v>655</v>
+        <v>630</v>
       </c>
     </row>
     <row r="163" spans="1:3">
@@ -8736,7 +8703,7 @@
         <v>240</v>
       </c>
       <c r="C163" t="s">
-        <v>584</v>
+        <v>559</v>
       </c>
     </row>
     <row r="164" spans="1:3">
@@ -8752,21 +8719,21 @@
         <v>255</v>
       </c>
       <c r="B165" t="s">
-        <v>556</v>
+        <v>533</v>
       </c>
       <c r="C165" t="s">
-        <v>643</v>
+        <v>618</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>773</v>
+        <v>748</v>
       </c>
       <c r="B166" t="s">
-        <v>774</v>
+        <v>749</v>
       </c>
       <c r="C166" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -8779,10 +8746,10 @@
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>499</v>
+        <v>478</v>
       </c>
       <c r="B168" t="s">
-        <v>508</v>
+        <v>487</v>
       </c>
     </row>
     <row r="169" spans="1:3">
@@ -8827,7 +8794,7 @@
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="B174" t="s">
         <v>245</v>
@@ -8835,75 +8802,75 @@
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>346</v>
+        <v>326</v>
       </c>
       <c r="B175" t="s">
-        <v>347</v>
+        <v>327</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>649</v>
+        <v>624</v>
       </c>
       <c r="B176" t="s">
-        <v>650</v>
+        <v>625</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>691</v>
+        <v>666</v>
       </c>
       <c r="B177" t="s">
-        <v>692</v>
+        <v>667</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>759</v>
+        <v>734</v>
       </c>
       <c r="B178" t="s">
-        <v>760</v>
+        <v>735</v>
       </c>
       <c r="C178" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>772</v>
+        <v>747</v>
       </c>
       <c r="B179" t="s">
-        <v>795</v>
+        <v>770</v>
       </c>
       <c r="C179" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>522</v>
+        <v>499</v>
       </c>
       <c r="B180" t="s">
-        <v>669</v>
+        <v>644</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>770</v>
+        <v>745</v>
       </c>
       <c r="B182" t="s">
-        <v>771</v>
+        <v>746</v>
       </c>
       <c r="C182" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>511</v>
+        <v>490</v>
       </c>
       <c r="B183" t="s">
-        <v>512</v>
+        <v>491</v>
       </c>
     </row>
     <row r="184" spans="1:3">
@@ -8914,7 +8881,7 @@
         <v>259</v>
       </c>
       <c r="C184" t="s">
-        <v>652</v>
+        <v>627</v>
       </c>
     </row>
     <row r="185" spans="1:3" ht="13.5" customHeight="1">
@@ -8922,10 +8889,10 @@
         <v>258</v>
       </c>
       <c r="B185" t="s">
-        <v>557</v>
+        <v>534</v>
       </c>
       <c r="C185" t="s">
-        <v>686</v>
+        <v>661</v>
       </c>
     </row>
     <row r="186" spans="1:3">
@@ -8960,15 +8927,15 @@
         <v>265</v>
       </c>
       <c r="C189" t="s">
-        <v>652</v>
+        <v>627</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>500</v>
+        <v>479</v>
       </c>
       <c r="B190" t="s">
-        <v>566</v>
+        <v>541</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -9011,7 +8978,7 @@
         <v>282</v>
       </c>
       <c r="C195" t="s">
-        <v>652</v>
+        <v>627</v>
       </c>
     </row>
     <row r="196" spans="1:3">
@@ -9019,7 +8986,7 @@
         <v>277</v>
       </c>
       <c r="B196" t="s">
-        <v>599</v>
+        <v>574</v>
       </c>
     </row>
     <row r="197" spans="1:3">
@@ -9030,7 +8997,7 @@
         <v>281</v>
       </c>
       <c r="C197" t="s">
-        <v>652</v>
+        <v>627</v>
       </c>
     </row>
     <row r="198" spans="1:3">
@@ -9043,15 +9010,15 @@
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B199" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="B200" t="s">
         <v>245</v>
@@ -9059,801 +9026,781 @@
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="B201" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>693</v>
+        <v>668</v>
       </c>
       <c r="B202" t="s">
-        <v>692</v>
+        <v>667</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>533</v>
+        <v>510</v>
       </c>
       <c r="B203" t="s">
-        <v>670</v>
+        <v>645</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>687</v>
+        <v>662</v>
       </c>
       <c r="B204" t="s">
-        <v>688</v>
+        <v>663</v>
       </c>
       <c r="C204" t="s">
-        <v>682</v>
+        <v>657</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>513</v>
+        <v>492</v>
       </c>
       <c r="B206" t="s">
-        <v>514</v>
+        <v>864</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>289</v>
+        <v>480</v>
       </c>
       <c r="B207" t="s">
-        <v>293</v>
-      </c>
-      <c r="C207" t="s">
-        <v>584</v>
+        <v>542</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>501</v>
+        <v>289</v>
       </c>
       <c r="B208" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="209" spans="1:3">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2">
       <c r="A209" t="s">
         <v>290</v>
       </c>
       <c r="B209" t="s">
-        <v>294</v>
-      </c>
-      <c r="C209" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="210" spans="1:3">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2">
       <c r="A210" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B210" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="211" spans="1:3">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2">
       <c r="A211" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B211" t="s">
-        <v>558</v>
-      </c>
-    </row>
-    <row r="212" spans="1:3">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2">
       <c r="A212" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B212" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="213" spans="1:3">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2">
       <c r="A213" t="s">
+        <v>669</v>
+      </c>
+      <c r="B213" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2">
+      <c r="A214" t="s">
+        <v>509</v>
+      </c>
+      <c r="B214" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2">
+      <c r="A216" t="s">
+        <v>493</v>
+      </c>
+      <c r="B216" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2">
+      <c r="A217" t="s">
+        <v>481</v>
+      </c>
+      <c r="B217" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2">
+      <c r="A218" t="s">
+        <v>302</v>
+      </c>
+      <c r="B218" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2">
+      <c r="A219" t="s">
+        <v>303</v>
+      </c>
+      <c r="B219" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2">
+      <c r="A220" t="s">
+        <v>304</v>
+      </c>
+      <c r="B220" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2">
+      <c r="A221" t="s">
         <v>306</v>
       </c>
-      <c r="B213" t="s">
+      <c r="B221" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2">
+      <c r="A222" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="214" spans="1:3">
-      <c r="A214" t="s">
-        <v>303</v>
-      </c>
-      <c r="B214" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="215" spans="1:3">
-      <c r="A215" t="s">
-        <v>304</v>
-      </c>
-      <c r="B215" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="216" spans="1:3">
-      <c r="A216" t="s">
+      <c r="B222" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2">
+      <c r="A223" t="s">
         <v>308</v>
       </c>
-      <c r="B216" t="s">
+      <c r="B223" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2">
+      <c r="A224" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="217" spans="1:3">
-      <c r="A217" t="s">
-        <v>694</v>
-      </c>
-      <c r="B217" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="218" spans="1:3">
-      <c r="A218" t="s">
-        <v>532</v>
-      </c>
-      <c r="B218" t="s">
-        <v>671</v>
-      </c>
-    </row>
-    <row r="220" spans="1:3">
-      <c r="A220" t="s">
-        <v>515</v>
-      </c>
-      <c r="B220" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="221" spans="1:3">
-      <c r="A221" t="s">
-        <v>495</v>
-      </c>
-      <c r="B221" t="s">
-        <v>317</v>
-      </c>
-      <c r="C221" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="222" spans="1:3">
-      <c r="A222" t="s">
-        <v>502</v>
-      </c>
-      <c r="B222" t="s">
-        <v>568</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3">
-      <c r="A223" t="s">
-        <v>312</v>
-      </c>
-      <c r="B223" t="s">
-        <v>318</v>
-      </c>
-      <c r="C223" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="224" spans="1:3">
-      <c r="A224" t="s">
-        <v>313</v>
-      </c>
       <c r="B224" t="s">
-        <v>319</v>
+        <v>862</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>314</v>
+        <v>670</v>
       </c>
       <c r="B225" t="s">
-        <v>320</v>
+        <v>863</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>315</v>
+        <v>508</v>
       </c>
       <c r="B226" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="227" spans="1:3">
-      <c r="A227" t="s">
-        <v>316</v>
-      </c>
-      <c r="B227" t="s">
-        <v>245</v>
+        <v>647</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>321</v>
+        <v>494</v>
       </c>
       <c r="B228" t="s">
-        <v>322</v>
-      </c>
-      <c r="C228" t="s">
-        <v>584</v>
+        <v>495</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>323</v>
+        <v>476</v>
       </c>
       <c r="B229" t="s">
-        <v>324</v>
+        <v>315</v>
+      </c>
+      <c r="C229" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>326</v>
+        <v>482</v>
       </c>
       <c r="B230" t="s">
-        <v>325</v>
+        <v>544</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>327</v>
+        <v>313</v>
       </c>
       <c r="B231" t="s">
-        <v>328</v>
+        <v>316</v>
+      </c>
+      <c r="C231" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="B232" t="s">
-        <v>253</v>
+        <v>317</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>695</v>
+        <v>475</v>
       </c>
       <c r="B233" t="s">
-        <v>692</v>
+        <v>535</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>531</v>
+        <v>321</v>
       </c>
       <c r="B234" t="s">
-        <v>672</v>
+        <v>245</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3">
+      <c r="A235" t="s">
+        <v>322</v>
+      </c>
+      <c r="B235" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>517</v>
+        <v>323</v>
       </c>
       <c r="B236" t="s">
-        <v>518</v>
+        <v>319</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>497</v>
+        <v>324</v>
       </c>
       <c r="B237" t="s">
-        <v>335</v>
-      </c>
-      <c r="C237" t="s">
-        <v>584</v>
+        <v>320</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>503</v>
+        <v>325</v>
       </c>
       <c r="B238" t="s">
-        <v>569</v>
+        <v>253</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>333</v>
+        <v>671</v>
       </c>
       <c r="B239" t="s">
-        <v>336</v>
-      </c>
-      <c r="C239" t="s">
-        <v>584</v>
+        <v>667</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>334</v>
+        <v>507</v>
       </c>
       <c r="B240" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="241" spans="1:3">
-      <c r="A241" t="s">
-        <v>496</v>
-      </c>
-      <c r="B241" t="s">
-        <v>560</v>
+        <v>648</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>341</v>
+        <v>705</v>
       </c>
       <c r="B242" t="s">
-        <v>245</v>
+        <v>706</v>
+      </c>
+      <c r="C242" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>342</v>
+        <v>524</v>
       </c>
       <c r="B243" t="s">
-        <v>338</v>
+        <v>527</v>
+      </c>
+      <c r="C243" t="s">
+        <v>557</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>343</v>
+        <v>525</v>
       </c>
       <c r="B244" t="s">
-        <v>339</v>
+        <v>526</v>
+      </c>
+      <c r="C244" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>344</v>
+        <v>556</v>
       </c>
       <c r="B245" t="s">
-        <v>340</v>
+        <v>570</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B246" t="s">
-        <v>253</v>
+        <v>328</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>696</v>
+        <v>343</v>
       </c>
       <c r="B247" t="s">
-        <v>692</v>
+        <v>329</v>
+      </c>
+      <c r="C247" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>530</v>
+        <v>483</v>
       </c>
       <c r="B248" t="s">
-        <v>673</v>
+        <v>545</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3">
+      <c r="A249" t="s">
+        <v>344</v>
+      </c>
+      <c r="B249" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>730</v>
+        <v>345</v>
       </c>
       <c r="B250" t="s">
-        <v>731</v>
-      </c>
-      <c r="C250" t="s">
-        <v>682</v>
+        <v>331</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>547</v>
+        <v>346</v>
       </c>
       <c r="B251" t="s">
-        <v>550</v>
-      </c>
-      <c r="C251" t="s">
-        <v>582</v>
+        <v>332</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>548</v>
+        <v>347</v>
       </c>
       <c r="B252" t="s">
-        <v>549</v>
+        <v>333</v>
       </c>
       <c r="C252" t="s">
-        <v>583</v>
+        <v>559</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>581</v>
+        <v>348</v>
       </c>
       <c r="B253" t="s">
-        <v>595</v>
+        <v>334</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>362</v>
+        <v>349</v>
       </c>
       <c r="B254" t="s">
-        <v>348</v>
+        <v>335</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>363</v>
+        <v>350</v>
       </c>
       <c r="B255" t="s">
-        <v>349</v>
-      </c>
-      <c r="C255" t="s">
-        <v>584</v>
+        <v>336</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>504</v>
+        <v>351</v>
       </c>
       <c r="B256" t="s">
-        <v>570</v>
+        <v>337</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>364</v>
+        <v>352</v>
       </c>
       <c r="B257" t="s">
-        <v>350</v>
+        <v>338</v>
+      </c>
+      <c r="C257" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>365</v>
+        <v>353</v>
       </c>
       <c r="B258" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>366</v>
+        <v>354</v>
       </c>
       <c r="B259" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="B260" t="s">
-        <v>353</v>
-      </c>
-      <c r="C260" t="s">
-        <v>584</v>
+        <v>341</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>368</v>
+        <v>506</v>
       </c>
       <c r="B261" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="262" spans="1:3">
-      <c r="A262" t="s">
-        <v>369</v>
-      </c>
-      <c r="B262" t="s">
-        <v>355</v>
+        <v>633</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>370</v>
+        <v>575</v>
       </c>
       <c r="B263" t="s">
-        <v>356</v>
+        <v>576</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="B264" t="s">
-        <v>357</v>
+        <v>380</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="B265" t="s">
-        <v>358</v>
-      </c>
-      <c r="C265" t="s">
-        <v>584</v>
+        <v>377</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="B266" t="s">
-        <v>359</v>
+        <v>378</v>
+      </c>
+      <c r="C266" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>374</v>
+        <v>484</v>
       </c>
       <c r="B267" t="s">
-        <v>360</v>
+        <v>546</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="B268" t="s">
-        <v>361</v>
+        <v>379</v>
+      </c>
+      <c r="C268" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>529</v>
+        <v>365</v>
       </c>
       <c r="B269" t="s">
-        <v>658</v>
+        <v>371</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3">
+      <c r="A270" t="s">
+        <v>382</v>
+      </c>
+      <c r="B270" t="s">
+        <v>372</v>
+      </c>
+      <c r="C270" t="s">
+        <v>536</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>600</v>
+        <v>366</v>
       </c>
       <c r="B271" t="s">
-        <v>601</v>
+        <v>373</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>382</v>
+        <v>368</v>
       </c>
       <c r="B272" t="s">
-        <v>400</v>
+        <v>374</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>383</v>
+        <v>367</v>
       </c>
       <c r="B273" t="s">
-        <v>397</v>
+        <v>375</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="B274" t="s">
-        <v>398</v>
-      </c>
-      <c r="C274" t="s">
-        <v>584</v>
+        <v>376</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>505</v>
+        <v>370</v>
       </c>
       <c r="B275" t="s">
-        <v>571</v>
+        <v>373</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>401</v>
+        <v>505</v>
       </c>
       <c r="B276" t="s">
-        <v>399</v>
-      </c>
-      <c r="C276" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="277" spans="1:3">
-      <c r="A277" t="s">
-        <v>385</v>
-      </c>
-      <c r="B277" t="s">
-        <v>391</v>
+        <v>649</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>402</v>
+        <v>707</v>
       </c>
       <c r="B278" t="s">
-        <v>392</v>
+        <v>726</v>
       </c>
       <c r="C278" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="279" spans="1:3">
-      <c r="A279" t="s">
-        <v>386</v>
-      </c>
-      <c r="B279" t="s">
-        <v>393</v>
+        <v>657</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>388</v>
+        <v>703</v>
       </c>
       <c r="B280" t="s">
-        <v>394</v>
+        <v>704</v>
+      </c>
+      <c r="C280" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>387</v>
+        <v>496</v>
       </c>
       <c r="B281" t="s">
-        <v>395</v>
+        <v>497</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B282" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B283" t="s">
-        <v>393</v>
+        <v>400</v>
+      </c>
+      <c r="C283" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>528</v>
+        <v>547</v>
       </c>
       <c r="B284" t="s">
-        <v>674</v>
+        <v>548</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3">
+      <c r="A285" t="s">
+        <v>390</v>
+      </c>
+      <c r="B285" t="s">
+        <v>401</v>
+      </c>
+      <c r="C285" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>732</v>
+        <v>391</v>
       </c>
       <c r="B286" t="s">
-        <v>751</v>
+        <v>402</v>
       </c>
       <c r="C286" t="s">
-        <v>682</v>
+        <v>559</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3">
+      <c r="A287" t="s">
+        <v>392</v>
+      </c>
+      <c r="B287" t="s">
+        <v>560</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>728</v>
+        <v>393</v>
       </c>
       <c r="B288" t="s">
-        <v>729</v>
-      </c>
-      <c r="C288" t="s">
-        <v>682</v>
+        <v>403</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>519</v>
+        <v>394</v>
       </c>
       <c r="B289" t="s">
-        <v>520</v>
+        <v>404</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>408</v>
+        <v>395</v>
       </c>
       <c r="B290" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>409</v>
+        <v>396</v>
       </c>
       <c r="B291" t="s">
-        <v>420</v>
-      </c>
-      <c r="C291" t="s">
-        <v>584</v>
+        <v>406</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>572</v>
+        <v>397</v>
       </c>
       <c r="B292" t="s">
-        <v>573</v>
+        <v>407</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>410</v>
+        <v>398</v>
       </c>
       <c r="B293" t="s">
-        <v>421</v>
-      </c>
-      <c r="C293" t="s">
-        <v>584</v>
+        <v>408</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>411</v>
+        <v>764</v>
       </c>
       <c r="B294" t="s">
-        <v>422</v>
+        <v>765</v>
       </c>
       <c r="C294" t="s">
-        <v>584</v>
+        <v>657</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>412</v>
+        <v>503</v>
       </c>
       <c r="B295" t="s">
-        <v>585</v>
+        <v>650</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>413</v>
+        <v>584</v>
       </c>
       <c r="B296" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="297" spans="1:3">
-      <c r="A297" t="s">
-        <v>414</v>
-      </c>
-      <c r="B297" t="s">
-        <v>424</v>
+        <v>585</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>415</v>
+        <v>498</v>
       </c>
       <c r="B298" t="s">
-        <v>425</v>
+        <v>497</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B299" t="s">
         <v>426</v>
@@ -9861,538 +9808,479 @@
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="B300" t="s">
         <v>427</v>
       </c>
+      <c r="C300" t="s">
+        <v>559</v>
+      </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>418</v>
+        <v>485</v>
       </c>
       <c r="B301" t="s">
-        <v>428</v>
+        <v>549</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>789</v>
+        <v>417</v>
       </c>
       <c r="B302" t="s">
-        <v>790</v>
+        <v>428</v>
       </c>
       <c r="C302" t="s">
-        <v>682</v>
+        <v>559</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>526</v>
+        <v>418</v>
       </c>
       <c r="B303" t="s">
-        <v>675</v>
+        <v>429</v>
+      </c>
+      <c r="C303" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>609</v>
+        <v>419</v>
       </c>
       <c r="B304" t="s">
-        <v>610</v>
+        <v>561</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3">
+      <c r="A305" t="s">
+        <v>420</v>
+      </c>
+      <c r="B305" t="s">
+        <v>403</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>521</v>
+        <v>421</v>
       </c>
       <c r="B306" t="s">
-        <v>520</v>
+        <v>404</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>435</v>
+        <v>422</v>
       </c>
       <c r="B307" t="s">
-        <v>446</v>
+        <v>430</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>436</v>
+        <v>423</v>
       </c>
       <c r="B308" t="s">
-        <v>447</v>
-      </c>
-      <c r="C308" t="s">
-        <v>584</v>
+        <v>431</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>506</v>
+        <v>424</v>
       </c>
       <c r="B309" t="s">
-        <v>574</v>
+        <v>407</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>437</v>
+        <v>425</v>
       </c>
       <c r="B310" t="s">
-        <v>448</v>
-      </c>
-      <c r="C310" t="s">
-        <v>584</v>
+        <v>408</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>438</v>
+        <v>502</v>
       </c>
       <c r="B311" t="s">
-        <v>449</v>
-      </c>
-      <c r="C311" t="s">
-        <v>584</v>
+        <v>650</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>439</v>
+        <v>591</v>
       </c>
       <c r="B312" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="313" spans="1:3">
-      <c r="A313" t="s">
-        <v>440</v>
-      </c>
-      <c r="B313" t="s">
-        <v>423</v>
+        <v>585</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>441</v>
+        <v>701</v>
       </c>
       <c r="B314" t="s">
-        <v>424</v>
+        <v>702</v>
+      </c>
+      <c r="C314" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>442</v>
+        <v>409</v>
       </c>
       <c r="B315" t="s">
-        <v>450</v>
+        <v>592</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>443</v>
+        <v>410</v>
       </c>
       <c r="B316" t="s">
-        <v>451</v>
+        <v>593</v>
+      </c>
+      <c r="C316" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>444</v>
+        <v>486</v>
       </c>
       <c r="B317" t="s">
-        <v>427</v>
+        <v>594</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>445</v>
+        <v>411</v>
       </c>
       <c r="B318" t="s">
-        <v>428</v>
+        <v>619</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>525</v>
+        <v>412</v>
       </c>
       <c r="B319" t="s">
-        <v>675</v>
+        <v>595</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>616</v>
+        <v>413</v>
       </c>
       <c r="B320" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="322" spans="1:3">
-      <c r="A322" t="s">
-        <v>726</v>
-      </c>
-      <c r="B322" t="s">
-        <v>727</v>
-      </c>
-      <c r="C322" t="s">
-        <v>682</v>
+        <v>596</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3">
+      <c r="A321" t="s">
+        <v>501</v>
+      </c>
+      <c r="B321" t="s">
+        <v>651</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>429</v>
+        <v>783</v>
       </c>
       <c r="B323" t="s">
-        <v>617</v>
+        <v>784</v>
+      </c>
+      <c r="C323" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>430</v>
+        <v>785</v>
       </c>
       <c r="B324" t="s">
-        <v>618</v>
+        <v>786</v>
       </c>
       <c r="C324" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="325" spans="1:3">
-      <c r="A325" t="s">
-        <v>507</v>
-      </c>
-      <c r="B325" t="s">
-        <v>619</v>
+        <v>657</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
-        <v>431</v>
+        <v>792</v>
       </c>
       <c r="B326" t="s">
-        <v>644</v>
+        <v>793</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
-        <v>432</v>
+        <v>794</v>
       </c>
       <c r="B327" t="s">
-        <v>620</v>
+        <v>795</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>433</v>
+        <v>796</v>
       </c>
       <c r="B328" t="s">
-        <v>621</v>
+        <v>797</v>
       </c>
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>524</v>
+        <v>798</v>
       </c>
       <c r="B329" t="s">
-        <v>676</v>
+        <v>799</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3">
+      <c r="A330" t="s">
+        <v>800</v>
+      </c>
+      <c r="B330" t="s">
+        <v>801</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>808</v>
+        <v>802</v>
       </c>
       <c r="B331" t="s">
-        <v>809</v>
-      </c>
-      <c r="C331" t="s">
-        <v>682</v>
+        <v>803</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>810</v>
+        <v>804</v>
       </c>
       <c r="B332" t="s">
-        <v>811</v>
-      </c>
-      <c r="C332" t="s">
-        <v>682</v>
+        <v>805</v>
+      </c>
+    </row>
+    <row r="333" spans="1:3">
+      <c r="A333" t="s">
+        <v>806</v>
+      </c>
+      <c r="B333" t="s">
+        <v>807</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>817</v>
+        <v>808</v>
       </c>
       <c r="B334" t="s">
-        <v>818</v>
+        <v>809</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>819</v>
+        <v>810</v>
       </c>
       <c r="B335" t="s">
-        <v>820</v>
+        <v>811</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
-        <v>821</v>
+        <v>812</v>
       </c>
       <c r="B336" t="s">
-        <v>822</v>
+        <v>813</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="A337" t="s">
-        <v>823</v>
+        <v>814</v>
       </c>
       <c r="B337" t="s">
-        <v>824</v>
+        <v>815</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="A338" t="s">
-        <v>825</v>
+        <v>816</v>
       </c>
       <c r="B338" t="s">
-        <v>826</v>
+        <v>817</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="A339" t="s">
-        <v>827</v>
+        <v>818</v>
       </c>
       <c r="B339" t="s">
-        <v>828</v>
+        <v>819</v>
       </c>
     </row>
     <row r="340" spans="1:2">
       <c r="A340" t="s">
-        <v>829</v>
+        <v>820</v>
       </c>
       <c r="B340" t="s">
-        <v>830</v>
+        <v>821</v>
       </c>
     </row>
     <row r="341" spans="1:2">
       <c r="A341" t="s">
-        <v>831</v>
+        <v>822</v>
       </c>
       <c r="B341" t="s">
-        <v>832</v>
+        <v>823</v>
       </c>
     </row>
     <row r="342" spans="1:2">
       <c r="A342" t="s">
-        <v>833</v>
+        <v>824</v>
       </c>
       <c r="B342" t="s">
-        <v>834</v>
+        <v>825</v>
       </c>
     </row>
     <row r="343" spans="1:2">
       <c r="A343" t="s">
-        <v>835</v>
+        <v>826</v>
       </c>
       <c r="B343" t="s">
-        <v>836</v>
-      </c>
-    </row>
-    <row r="344" spans="1:2">
-      <c r="A344" t="s">
-        <v>837</v>
-      </c>
-      <c r="B344" t="s">
-        <v>838</v>
+        <v>827</v>
       </c>
     </row>
     <row r="345" spans="1:2">
       <c r="A345" t="s">
-        <v>839</v>
+        <v>828</v>
       </c>
       <c r="B345" t="s">
-        <v>840</v>
+        <v>829</v>
       </c>
     </row>
     <row r="346" spans="1:2">
       <c r="A346" t="s">
-        <v>841</v>
+        <v>830</v>
       </c>
       <c r="B346" t="s">
-        <v>842</v>
+        <v>831</v>
       </c>
     </row>
     <row r="347" spans="1:2">
       <c r="A347" t="s">
-        <v>843</v>
+        <v>832</v>
       </c>
       <c r="B347" t="s">
-        <v>844</v>
+        <v>833</v>
       </c>
     </row>
     <row r="348" spans="1:2">
       <c r="A348" t="s">
-        <v>845</v>
+        <v>834</v>
       </c>
       <c r="B348" t="s">
-        <v>846</v>
+        <v>835</v>
       </c>
     </row>
     <row r="349" spans="1:2">
       <c r="A349" t="s">
-        <v>847</v>
+        <v>836</v>
       </c>
       <c r="B349" t="s">
-        <v>848</v>
+        <v>837</v>
       </c>
     </row>
     <row r="350" spans="1:2">
       <c r="A350" t="s">
-        <v>849</v>
+        <v>838</v>
       </c>
       <c r="B350" t="s">
-        <v>850</v>
+        <v>839</v>
       </c>
     </row>
     <row r="351" spans="1:2">
       <c r="A351" t="s">
-        <v>851</v>
+        <v>840</v>
       </c>
       <c r="B351" t="s">
-        <v>852</v>
+        <v>841</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2">
+      <c r="A352" t="s">
+        <v>842</v>
+      </c>
+      <c r="B352" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>853</v>
+        <v>843</v>
       </c>
       <c r="B353" t="s">
-        <v>854</v>
+        <v>844</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>855</v>
+        <v>845</v>
       </c>
       <c r="B354" t="s">
-        <v>856</v>
+        <v>846</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>857</v>
+        <v>847</v>
       </c>
       <c r="B355" t="s">
-        <v>858</v>
+        <v>848</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>859</v>
+        <v>849</v>
       </c>
       <c r="B356" t="s">
-        <v>860</v>
-      </c>
-    </row>
-    <row r="357" spans="1:2">
-      <c r="A357" t="s">
-        <v>861</v>
-      </c>
-      <c r="B357" t="s">
-        <v>862</v>
+        <v>850</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>863</v>
+        <v>851</v>
       </c>
       <c r="B358" t="s">
-        <v>864</v>
+        <v>334</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>865</v>
+        <v>852</v>
       </c>
       <c r="B359" t="s">
-        <v>866</v>
+        <v>853</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>867</v>
+        <v>854</v>
       </c>
       <c r="B360" t="s">
-        <v>361</v>
+        <v>336</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>868</v>
+        <v>855</v>
       </c>
       <c r="B361" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="362" spans="1:2">
-      <c r="A362" t="s">
-        <v>870</v>
-      </c>
-      <c r="B362" t="s">
-        <v>871</v>
-      </c>
-    </row>
-    <row r="363" spans="1:2">
-      <c r="A363" t="s">
-        <v>872</v>
-      </c>
-      <c r="B363" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="364" spans="1:2">
-      <c r="A364" t="s">
-        <v>874</v>
-      </c>
-      <c r="B364" t="s">
-        <v>875</v>
-      </c>
-    </row>
-    <row r="366" spans="1:2">
-      <c r="A366" t="s">
-        <v>876</v>
-      </c>
-      <c r="B366" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="367" spans="1:2">
-      <c r="A367" t="s">
-        <v>877</v>
-      </c>
-      <c r="B367" t="s">
-        <v>878</v>
-      </c>
-    </row>
-    <row r="368" spans="1:2">
-      <c r="A368" t="s">
-        <v>879</v>
-      </c>
-      <c r="B368" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="369" spans="1:2">
-      <c r="A369" t="s">
-        <v>880</v>
-      </c>
-      <c r="B369" t="s">
-        <v>357</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to ATRC, HAB, Paystubs, RDC
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F96CE5-BDF4-4F2F-82F4-CE3ED2C264C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C42FE32C-D10D-495C-8D2B-6BF49DBFE173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="870">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="895">
   <si>
     <t>Name</t>
   </si>
@@ -2382,9 +2382,6 @@
     <t>Yardi_States</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Household Demographic Reporting Form</t>
   </si>
   <si>
@@ -2650,6 +2647,84 @@
   </si>
   <si>
     <t>Pay Amount listed on the Offer Letter and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>ARC_ConfirmDate</t>
+  </si>
+  <si>
+    <t>ARC_CheckDateWithMoveIn</t>
+  </si>
+  <si>
+    <t>ARC_ConfirmSign</t>
+  </si>
+  <si>
+    <t>Not all adults have signed the document.</t>
+  </si>
+  <si>
+    <t>Not all adults have dated the document.</t>
+  </si>
+  <si>
+    <t>Dates are not within 120 days of move in.</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Application/Tenant Release and Consent. Needs manual review.</t>
+  </si>
+  <si>
+    <t>ARC_FindingError</t>
+  </si>
+  <si>
+    <t>Not all adults names are listed on the “I/We” line.</t>
+  </si>
+  <si>
+    <t>ARC_NamesCheck</t>
+  </si>
+  <si>
+    <t>ARCExists</t>
+  </si>
+  <si>
+    <t>Application/Tenant Release and Consent is missing from the application.</t>
+  </si>
+  <si>
+    <t>ARC</t>
+  </si>
+  <si>
+    <t>Applicant Tenant Release and Consent</t>
+  </si>
+  <si>
+    <t>HABExists</t>
+  </si>
+  <si>
+    <t>HAB_ConfirmSign</t>
+  </si>
+  <si>
+    <t>HAB_ConfirmDate</t>
+  </si>
+  <si>
+    <t>HAB_CheckDateWithMoveIn</t>
+  </si>
+  <si>
+    <t>HAB_FindingError</t>
+  </si>
+  <si>
+    <t>Household Asset Breakdown is missing from the application.</t>
+  </si>
+  <si>
+    <t>Asset type, member name, or asset value does not match Income &amp; Asset Questionnaire for all assets.</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Household Asset Breakdown. Needs manual review.</t>
+  </si>
+  <si>
+    <t>HAB_NameAndAssetsinIAQ</t>
+  </si>
+  <si>
+    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>HAB</t>
+  </si>
+  <si>
+    <t>Household Asset Breakdown</t>
   </si>
 </sst>
 </file>
@@ -3107,7 +3182,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>780</v>
+        <v>892</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -3400,22 +3475,36 @@
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B43" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
+        <v>789</v>
+      </c>
+      <c r="B44" t="s">
         <v>790</v>
       </c>
-      <c r="B44" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="46" spans="1:2" ht="14.25" customHeight="1"/>
+    </row>
+    <row r="45" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A45" t="s">
+        <v>881</v>
+      </c>
+      <c r="B45" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A46" t="s">
+        <v>893</v>
+      </c>
+      <c r="B46" t="s">
+        <v>894</v>
+      </c>
+    </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>
@@ -7348,7 +7437,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C361"/>
+  <dimension ref="A1:C375"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8634,7 +8723,7 @@
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="B156" t="s">
         <v>769</v>
@@ -8645,7 +8734,7 @@
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B157" t="s">
         <v>758</v>
@@ -8656,7 +8745,7 @@
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="B158" t="s">
         <v>767</v>
@@ -9064,7 +9153,7 @@
         <v>492</v>
       </c>
       <c r="B206" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="207" spans="1:3">
@@ -9080,7 +9169,7 @@
         <v>289</v>
       </c>
       <c r="B208" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
     </row>
     <row r="209" spans="1:2">
@@ -9088,7 +9177,7 @@
         <v>290</v>
       </c>
       <c r="B209" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="210" spans="1:2">
@@ -9096,7 +9185,7 @@
         <v>298</v>
       </c>
       <c r="B210" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
     </row>
     <row r="211" spans="1:2">
@@ -9104,7 +9193,7 @@
         <v>297</v>
       </c>
       <c r="B211" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="212" spans="1:2">
@@ -9112,7 +9201,7 @@
         <v>299</v>
       </c>
       <c r="B212" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
     </row>
     <row r="213" spans="1:2">
@@ -9120,7 +9209,7 @@
         <v>669</v>
       </c>
       <c r="B213" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="214" spans="1:2">
@@ -9136,7 +9225,7 @@
         <v>493</v>
       </c>
       <c r="B216" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
     </row>
     <row r="217" spans="1:2">
@@ -9152,7 +9241,7 @@
         <v>302</v>
       </c>
       <c r="B218" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="219" spans="1:2">
@@ -9168,7 +9257,7 @@
         <v>304</v>
       </c>
       <c r="B220" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="221" spans="1:2">
@@ -9176,7 +9265,7 @@
         <v>306</v>
       </c>
       <c r="B221" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
     </row>
     <row r="222" spans="1:2">
@@ -9184,7 +9273,7 @@
         <v>307</v>
       </c>
       <c r="B222" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
     </row>
     <row r="223" spans="1:2">
@@ -9192,7 +9281,7 @@
         <v>308</v>
       </c>
       <c r="B223" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
     </row>
     <row r="224" spans="1:2">
@@ -9200,7 +9289,7 @@
         <v>309</v>
       </c>
       <c r="B224" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
     </row>
     <row r="225" spans="1:3">
@@ -9208,7 +9297,7 @@
         <v>670</v>
       </c>
       <c r="B225" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
     </row>
     <row r="226" spans="1:3">
@@ -9991,10 +10080,10 @@
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
+        <v>782</v>
+      </c>
+      <c r="B323" t="s">
         <v>783</v>
-      </c>
-      <c r="B323" t="s">
-        <v>784</v>
       </c>
       <c r="C323" t="s">
         <v>657</v>
@@ -10002,10 +10091,10 @@
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
+        <v>784</v>
+      </c>
+      <c r="B324" t="s">
         <v>785</v>
-      </c>
-      <c r="B324" t="s">
-        <v>786</v>
       </c>
       <c r="C324" t="s">
         <v>657</v>
@@ -10013,207 +10102,207 @@
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
+        <v>791</v>
+      </c>
+      <c r="B326" t="s">
         <v>792</v>
-      </c>
-      <c r="B326" t="s">
-        <v>793</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
+        <v>793</v>
+      </c>
+      <c r="B327" t="s">
         <v>794</v>
-      </c>
-      <c r="B327" t="s">
-        <v>795</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
+        <v>795</v>
+      </c>
+      <c r="B328" t="s">
         <v>796</v>
-      </c>
-      <c r="B328" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
+        <v>797</v>
+      </c>
+      <c r="B329" t="s">
         <v>798</v>
-      </c>
-      <c r="B329" t="s">
-        <v>799</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
+        <v>799</v>
+      </c>
+      <c r="B330" t="s">
         <v>800</v>
-      </c>
-      <c r="B330" t="s">
-        <v>801</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
+        <v>801</v>
+      </c>
+      <c r="B331" t="s">
         <v>802</v>
-      </c>
-      <c r="B331" t="s">
-        <v>803</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
+        <v>803</v>
+      </c>
+      <c r="B332" t="s">
         <v>804</v>
-      </c>
-      <c r="B332" t="s">
-        <v>805</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
+        <v>805</v>
+      </c>
+      <c r="B333" t="s">
         <v>806</v>
-      </c>
-      <c r="B333" t="s">
-        <v>807</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
+        <v>807</v>
+      </c>
+      <c r="B334" t="s">
         <v>808</v>
-      </c>
-      <c r="B334" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
+        <v>809</v>
+      </c>
+      <c r="B335" t="s">
         <v>810</v>
-      </c>
-      <c r="B335" t="s">
-        <v>811</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
+        <v>811</v>
+      </c>
+      <c r="B336" t="s">
         <v>812</v>
-      </c>
-      <c r="B336" t="s">
-        <v>813</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="A337" t="s">
+        <v>813</v>
+      </c>
+      <c r="B337" t="s">
         <v>814</v>
-      </c>
-      <c r="B337" t="s">
-        <v>815</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="A338" t="s">
+        <v>815</v>
+      </c>
+      <c r="B338" t="s">
         <v>816</v>
-      </c>
-      <c r="B338" t="s">
-        <v>817</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="A339" t="s">
+        <v>817</v>
+      </c>
+      <c r="B339" t="s">
         <v>818</v>
-      </c>
-      <c r="B339" t="s">
-        <v>819</v>
       </c>
     </row>
     <row r="340" spans="1:2">
       <c r="A340" t="s">
+        <v>819</v>
+      </c>
+      <c r="B340" t="s">
         <v>820</v>
-      </c>
-      <c r="B340" t="s">
-        <v>821</v>
       </c>
     </row>
     <row r="341" spans="1:2">
       <c r="A341" t="s">
+        <v>821</v>
+      </c>
+      <c r="B341" t="s">
         <v>822</v>
-      </c>
-      <c r="B341" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="342" spans="1:2">
       <c r="A342" t="s">
+        <v>823</v>
+      </c>
+      <c r="B342" t="s">
         <v>824</v>
-      </c>
-      <c r="B342" t="s">
-        <v>825</v>
       </c>
     </row>
     <row r="343" spans="1:2">
       <c r="A343" t="s">
+        <v>825</v>
+      </c>
+      <c r="B343" t="s">
         <v>826</v>
-      </c>
-      <c r="B343" t="s">
-        <v>827</v>
       </c>
     </row>
     <row r="345" spans="1:2">
       <c r="A345" t="s">
+        <v>827</v>
+      </c>
+      <c r="B345" t="s">
         <v>828</v>
-      </c>
-      <c r="B345" t="s">
-        <v>829</v>
       </c>
     </row>
     <row r="346" spans="1:2">
       <c r="A346" t="s">
+        <v>829</v>
+      </c>
+      <c r="B346" t="s">
         <v>830</v>
-      </c>
-      <c r="B346" t="s">
-        <v>831</v>
       </c>
     </row>
     <row r="347" spans="1:2">
       <c r="A347" t="s">
+        <v>831</v>
+      </c>
+      <c r="B347" t="s">
         <v>832</v>
-      </c>
-      <c r="B347" t="s">
-        <v>833</v>
       </c>
     </row>
     <row r="348" spans="1:2">
       <c r="A348" t="s">
+        <v>833</v>
+      </c>
+      <c r="B348" t="s">
         <v>834</v>
-      </c>
-      <c r="B348" t="s">
-        <v>835</v>
       </c>
     </row>
     <row r="349" spans="1:2">
       <c r="A349" t="s">
+        <v>835</v>
+      </c>
+      <c r="B349" t="s">
         <v>836</v>
-      </c>
-      <c r="B349" t="s">
-        <v>837</v>
       </c>
     </row>
     <row r="350" spans="1:2">
       <c r="A350" t="s">
+        <v>837</v>
+      </c>
+      <c r="B350" t="s">
         <v>838</v>
-      </c>
-      <c r="B350" t="s">
-        <v>839</v>
       </c>
     </row>
     <row r="351" spans="1:2">
       <c r="A351" t="s">
+        <v>839</v>
+      </c>
+      <c r="B351" t="s">
         <v>840</v>
-      </c>
-      <c r="B351" t="s">
-        <v>841</v>
       </c>
     </row>
     <row r="352" spans="1:2">
       <c r="A352" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="B352" t="s">
         <v>341</v>
@@ -10221,39 +10310,39 @@
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
+        <v>842</v>
+      </c>
+      <c r="B353" t="s">
         <v>843</v>
-      </c>
-      <c r="B353" t="s">
-        <v>844</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
+        <v>844</v>
+      </c>
+      <c r="B354" t="s">
         <v>845</v>
-      </c>
-      <c r="B354" t="s">
-        <v>846</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
+        <v>846</v>
+      </c>
+      <c r="B355" t="s">
         <v>847</v>
-      </c>
-      <c r="B355" t="s">
-        <v>848</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
+        <v>848</v>
+      </c>
+      <c r="B356" t="s">
         <v>849</v>
-      </c>
-      <c r="B356" t="s">
-        <v>850</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B358" t="s">
         <v>334</v>
@@ -10261,15 +10350,15 @@
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
+        <v>851</v>
+      </c>
+      <c r="B359" t="s">
         <v>852</v>
-      </c>
-      <c r="B359" t="s">
-        <v>853</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B360" t="s">
         <v>336</v>
@@ -10277,10 +10366,106 @@
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="B361" t="s">
         <v>337</v>
+      </c>
+    </row>
+    <row r="363" spans="1:2">
+      <c r="A363" t="s">
+        <v>879</v>
+      </c>
+      <c r="B363" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="364" spans="1:2">
+      <c r="A364" t="s">
+        <v>878</v>
+      </c>
+      <c r="B364" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="365" spans="1:2">
+      <c r="A365" t="s">
+        <v>871</v>
+      </c>
+      <c r="B365" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="366" spans="1:2">
+      <c r="A366" t="s">
+        <v>869</v>
+      </c>
+      <c r="B366" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2">
+      <c r="A367" t="s">
+        <v>870</v>
+      </c>
+      <c r="B367" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="368" spans="1:2">
+      <c r="A368" t="s">
+        <v>876</v>
+      </c>
+      <c r="B368" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="370" spans="1:2">
+      <c r="A370" t="s">
+        <v>883</v>
+      </c>
+      <c r="B370" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="371" spans="1:2">
+      <c r="A371" t="s">
+        <v>891</v>
+      </c>
+      <c r="B371" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="372" spans="1:2">
+      <c r="A372" t="s">
+        <v>884</v>
+      </c>
+      <c r="B372" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2">
+      <c r="A373" t="s">
+        <v>885</v>
+      </c>
+      <c r="B373" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2">
+      <c r="A374" t="s">
+        <v>886</v>
+      </c>
+      <c r="B374" t="s">
+        <v>874</v>
+      </c>
+    </row>
+    <row r="375" spans="1:2">
+      <c r="A375" t="s">
+        <v>887</v>
+      </c>
+      <c r="B375" t="s">
+        <v>890</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
started working on EV
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C42FE32C-D10D-495C-8D2B-6BF49DBFE173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30BD9E1-2C15-4501-91F7-BFCA012F2A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1102" uniqueCount="895">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1140" uniqueCount="924">
   <si>
     <t>Name</t>
   </si>
@@ -2725,6 +2725,93 @@
   </si>
   <si>
     <t>Household Asset Breakdown</t>
+  </si>
+  <si>
+    <t>EV</t>
+  </si>
+  <si>
+    <t>Employment Verification</t>
+  </si>
+  <si>
+    <t>EVExists</t>
+  </si>
+  <si>
+    <t>Employment Verification is missing from the application.</t>
+  </si>
+  <si>
+    <t>EV_CheckRDC</t>
+  </si>
+  <si>
+    <t>Day Calculator does not exist for Verification of employment findings.</t>
+  </si>
+  <si>
+    <t>EV_EmailReceiptAndClarification</t>
+  </si>
+  <si>
+    <t>Employee Name across the Verification of Employment, Day Calculator, and ICW do not match.</t>
+  </si>
+  <si>
+    <t>EV_EmployeeName</t>
+  </si>
+  <si>
+    <t>Date on the Verification of Employment is not within 120 days of Move-In date.</t>
+  </si>
+  <si>
+    <t>Amount listed on Verification of Employment and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>The calculated Gross Wage Per Year based on the Verification of Employment does not match the Regular Rate Total Per Year on the Day Calculator.</t>
+  </si>
+  <si>
+    <t>Overtime Rate listed on Verification of Employment and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>Shift Differential Rate listed on Verification of Employment and Day Calculator do not match.</t>
+  </si>
+  <si>
+    <t>Total listed on the Day Calculator does not match the Verified Income on the ICW.</t>
+  </si>
+  <si>
+    <t>EV_PresentlyEmployedNo</t>
+  </si>
+  <si>
+    <t>EV_PresentlyEmployedYes</t>
+  </si>
+  <si>
+    <t>EV_CheckDateWithMoveIn</t>
+  </si>
+  <si>
+    <t>EV_FindingError</t>
+  </si>
+  <si>
+    <t>EV_AnticipatedIncrease</t>
+  </si>
+  <si>
+    <t>EV_AmountListed</t>
+  </si>
+  <si>
+    <t>EV_HasSignature</t>
+  </si>
+  <si>
+    <t>EV_GrossWageCheck</t>
+  </si>
+  <si>
+    <t>EV_OvertimeRateCheck</t>
+  </si>
+  <si>
+    <t>EV_ShiftDifferentialRateCheck</t>
+  </si>
+  <si>
+    <t>EV_TotalListedCheck</t>
+  </si>
+  <si>
+    <t>EV_NotAllFieldsDocumented</t>
+  </si>
+  <si>
+    <t>EV_CommissionCheck</t>
+  </si>
+  <si>
+    <t>EV_MultipleEmploymentCheck</t>
   </si>
 </sst>
 </file>
@@ -3505,7 +3592,14 @@
         <v>894</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="47" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A47" t="s">
+        <v>895</v>
+      </c>
+      <c r="B47" t="s">
+        <v>896</v>
+      </c>
+    </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>
     <row r="50" ht="14.25" customHeight="1"/>
@@ -7437,7 +7531,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C375"/>
+  <dimension ref="A1:C394"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -10468,6 +10562,150 @@
         <v>890</v>
       </c>
     </row>
+    <row r="377" spans="1:2">
+      <c r="A377" t="s">
+        <v>897</v>
+      </c>
+      <c r="B377" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="378" spans="1:2">
+      <c r="A378" t="s">
+        <v>899</v>
+      </c>
+      <c r="B378" t="s">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="379" spans="1:2">
+      <c r="A379" t="s">
+        <v>901</v>
+      </c>
+      <c r="B379" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="380" spans="1:2">
+      <c r="A380" t="s">
+        <v>903</v>
+      </c>
+      <c r="B380" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2">
+      <c r="A381" t="s">
+        <v>910</v>
+      </c>
+      <c r="B381" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="382" spans="1:2">
+      <c r="A382" t="s">
+        <v>911</v>
+      </c>
+      <c r="B382" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="383" spans="1:2">
+      <c r="A383" t="s">
+        <v>912</v>
+      </c>
+      <c r="B383" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="384" spans="1:2">
+      <c r="A384" t="s">
+        <v>915</v>
+      </c>
+      <c r="B384" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2">
+      <c r="A385" t="s">
+        <v>916</v>
+      </c>
+      <c r="B385" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2">
+      <c r="A386" t="s">
+        <v>917</v>
+      </c>
+      <c r="B386" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="387" spans="1:2">
+      <c r="A387" t="s">
+        <v>918</v>
+      </c>
+      <c r="B387" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="388" spans="1:2">
+      <c r="A388" t="s">
+        <v>919</v>
+      </c>
+      <c r="B388" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="389" spans="1:2">
+      <c r="A389" t="s">
+        <v>920</v>
+      </c>
+      <c r="B389" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="390" spans="1:2">
+      <c r="A390" t="s">
+        <v>921</v>
+      </c>
+      <c r="B390" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2">
+      <c r="A391" t="s">
+        <v>922</v>
+      </c>
+      <c r="B391" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="392" spans="1:2">
+      <c r="A392" t="s">
+        <v>923</v>
+      </c>
+      <c r="B392" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="393" spans="1:2">
+      <c r="A393" t="s">
+        <v>914</v>
+      </c>
+      <c r="B393" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="394" spans="1:2">
+      <c r="A394" t="s">
+        <v>913</v>
+      </c>
+      <c r="B394" t="s">
+        <v>645</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates to HAB, testing for CSEI and Profit Loss and Child Support Payment History
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30BD9E1-2C15-4501-91F7-BFCA012F2A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD799AB-8424-41B0-AAB8-464AD4FC3533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1140" uniqueCount="924">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="926">
   <si>
     <t>Name</t>
   </si>
@@ -2812,6 +2812,12 @@
   </si>
   <si>
     <t>EV_MultipleEmploymentCheck</t>
+  </si>
+  <si>
+    <t>CSEI</t>
+  </si>
+  <si>
+    <t>Certification of Self Employment Income</t>
   </si>
 </sst>
 </file>
@@ -3600,7 +3606,14 @@
         <v>896</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="48" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A48" t="s">
+        <v>924</v>
+      </c>
+      <c r="B48" t="s">
+        <v>925</v>
+      </c>
+    </row>
     <row r="49" ht="14.25" customHeight="1"/>
     <row r="50" ht="14.25" customHeight="1"/>
     <row r="51" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Updates to SS and SSI, COLA Letter, COLA Calc
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD799AB-8424-41B0-AAB8-464AD4FC3533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FC7981-2869-4CFA-9F7E-29973942FA94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="450" yWindow="435" windowWidth="21510" windowHeight="11160" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="926">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="928">
   <si>
     <t>Name</t>
   </si>
@@ -2364,9 +2364,6 @@
     <t>ICW_ZeroAnnualIncome</t>
   </si>
   <si>
-    <t>The Anuual Incime is listd as zero. Manual review required.</t>
-  </si>
-  <si>
     <t>Unable to validate findings for Income Calculation Worksheet. Needs manual review.</t>
   </si>
   <si>
@@ -2818,6 +2815,15 @@
   </si>
   <si>
     <t>Certification of Self Employment Income</t>
+  </si>
+  <si>
+    <t>ICW_Section811</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This application is a Section 811 unit, manual review is required. </t>
+  </si>
+  <si>
+    <t>The Anuual Income is listd as zero. Manual review required.</t>
   </si>
 </sst>
 </file>
@@ -3275,7 +3281,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -3568,50 +3574,50 @@
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="B43" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
+        <v>788</v>
+      </c>
+      <c r="B44" t="s">
         <v>789</v>
-      </c>
-      <c r="B44" t="s">
-        <v>790</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
+        <v>880</v>
+      </c>
+      <c r="B45" t="s">
         <v>881</v>
-      </c>
-      <c r="B45" t="s">
-        <v>882</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
+        <v>892</v>
+      </c>
+      <c r="B46" t="s">
         <v>893</v>
-      </c>
-      <c r="B46" t="s">
-        <v>894</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
+        <v>894</v>
+      </c>
+      <c r="B47" t="s">
         <v>895</v>
-      </c>
-      <c r="B47" t="s">
-        <v>896</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
+        <v>923</v>
+      </c>
+      <c r="B48" t="s">
         <v>924</v>
-      </c>
-      <c r="B48" t="s">
-        <v>925</v>
       </c>
     </row>
     <row r="49" ht="14.25" customHeight="1"/>
@@ -6240,10 +6246,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="B3" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -7544,7 +7550,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C394"/>
+  <dimension ref="A1:C395"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -7674,7 +7680,7 @@
         <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -7709,7 +7715,7 @@
         <v>665</v>
       </c>
       <c r="B20" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C20" t="s">
         <v>657</v>
@@ -7731,7 +7737,7 @@
         <v>692</v>
       </c>
       <c r="B22" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C22" t="s">
         <v>657</v>
@@ -7753,7 +7759,7 @@
         <v>773</v>
       </c>
       <c r="B24" t="s">
-        <v>774</v>
+        <v>927</v>
       </c>
       <c r="C24" t="s">
         <v>657</v>
@@ -7761,133 +7767,130 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>925</v>
+      </c>
+      <c r="B25" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
         <v>504</v>
       </c>
-      <c r="B25" t="s">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>180</v>
-      </c>
-      <c r="B27" t="s">
-        <v>181</v>
+      <c r="B26" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>180</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>181</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>531</v>
+        <v>78</v>
       </c>
       <c r="B29" t="s">
-        <v>532</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>531</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>532</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>195</v>
+        <v>81</v>
       </c>
       <c r="B32" t="s">
-        <v>756</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B33" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>196</v>
       </c>
       <c r="B34" t="s">
-        <v>84</v>
+        <v>757</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B35" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B37" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>599</v>
+        <v>88</v>
       </c>
       <c r="B38" t="s">
-        <v>600</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>623</v>
+        <v>599</v>
       </c>
       <c r="B39" t="s">
-        <v>768</v>
+        <v>600</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>681</v>
+        <v>623</v>
       </c>
       <c r="B40" t="s">
-        <v>682</v>
-      </c>
-      <c r="C40" t="s">
-        <v>657</v>
+        <v>768</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>762</v>
+        <v>681</v>
       </c>
       <c r="B41" t="s">
-        <v>763</v>
+        <v>682</v>
       </c>
       <c r="C41" t="s">
         <v>657</v>
@@ -7895,147 +7898,147 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
+        <v>762</v>
+      </c>
+      <c r="B42" t="s">
+        <v>763</v>
+      </c>
+      <c r="C42" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
         <v>519</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>634</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>182</v>
-      </c>
-      <c r="B44" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>90</v>
+        <v>182</v>
       </c>
       <c r="B45" t="s">
-        <v>91</v>
+        <v>184</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B46" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="B47" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B48" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B49" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B50" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B51" t="s">
-        <v>98</v>
-      </c>
-      <c r="C51" t="s">
-        <v>559</v>
+        <v>97</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B52" t="s">
-        <v>99</v>
+        <v>98</v>
+      </c>
+      <c r="C52" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>601</v>
+        <v>105</v>
       </c>
       <c r="B53" t="s">
-        <v>602</v>
+        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>518</v>
+        <v>601</v>
       </c>
       <c r="B54" t="s">
-        <v>635</v>
+        <v>602</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>750</v>
+        <v>518</v>
       </c>
       <c r="B55" t="s">
-        <v>751</v>
+        <v>635</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
+        <v>750</v>
+      </c>
+      <c r="B56" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
         <v>658</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B57" t="s">
         <v>659</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C57" t="s">
         <v>657</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
-      <c r="A58" t="s">
-        <v>183</v>
-      </c>
-      <c r="B58" t="s">
-        <v>562</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>106</v>
+        <v>183</v>
       </c>
       <c r="B59" t="s">
-        <v>107</v>
-      </c>
-      <c r="C59" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B60" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C60" t="s">
         <v>559</v>
@@ -8043,10 +8046,10 @@
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B61" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C61" t="s">
         <v>559</v>
@@ -8054,10 +8057,10 @@
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B62" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="C62" t="s">
         <v>559</v>
@@ -8065,10 +8068,10 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B63" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C63" t="s">
         <v>559</v>
@@ -8076,10 +8079,10 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B64" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C64" t="s">
         <v>559</v>
@@ -8087,123 +8090,123 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B65" t="s">
-        <v>111</v>
+        <v>110</v>
+      </c>
+      <c r="C65" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>201</v>
+        <v>115</v>
       </c>
       <c r="B66" t="s">
-        <v>752</v>
+        <v>111</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B67" t="s">
-        <v>753</v>
-      </c>
-      <c r="C67" t="s">
-        <v>559</v>
+        <v>752</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>550</v>
+        <v>202</v>
       </c>
       <c r="B68" t="s">
-        <v>754</v>
+        <v>753</v>
+      </c>
+      <c r="C68" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="B69" t="s">
-        <v>521</v>
+        <v>754</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="B70" t="s">
-        <v>755</v>
+        <v>521</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="B71" t="s">
-        <v>636</v>
+        <v>755</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
+        <v>517</v>
+      </c>
+      <c r="B72" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3">
+      <c r="A73" t="s">
         <v>709</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B73" t="s">
         <v>708</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C73" t="s">
         <v>657</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3">
-      <c r="A74" t="s">
-        <v>157</v>
-      </c>
-      <c r="B74" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>121</v>
+        <v>157</v>
       </c>
       <c r="B75" t="s">
-        <v>563</v>
+        <v>120</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B76" t="s">
-        <v>122</v>
+        <v>563</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>603</v>
+        <v>123</v>
       </c>
       <c r="B77" t="s">
-        <v>604</v>
+        <v>122</v>
       </c>
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>719</v>
+        <v>603</v>
       </c>
       <c r="B78" t="s">
-        <v>720</v>
-      </c>
-      <c r="C78" t="s">
-        <v>657</v>
+        <v>604</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>739</v>
+        <v>719</v>
       </c>
       <c r="B79" t="s">
-        <v>740</v>
+        <v>720</v>
       </c>
       <c r="C79" t="s">
         <v>657</v>
@@ -8211,10 +8214,10 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B80" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="C80" t="s">
         <v>657</v>
@@ -8222,10 +8225,10 @@
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B81" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="C81" t="s">
         <v>657</v>
@@ -8233,37 +8236,37 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
+        <v>737</v>
+      </c>
+      <c r="B82" t="s">
+        <v>742</v>
+      </c>
+      <c r="C82" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3">
+      <c r="A83" t="s">
         <v>516</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B83" t="s">
         <v>637</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3">
-      <c r="A84" t="s">
-        <v>185</v>
-      </c>
-      <c r="B84" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>718</v>
+        <v>185</v>
       </c>
       <c r="B85" t="s">
-        <v>733</v>
-      </c>
-      <c r="C85" t="s">
-        <v>657</v>
+        <v>186</v>
       </c>
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B86" t="s">
-        <v>717</v>
+        <v>733</v>
       </c>
       <c r="C86" t="s">
         <v>657</v>
@@ -8271,80 +8274,80 @@
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>124</v>
+        <v>716</v>
       </c>
       <c r="B87" t="s">
-        <v>126</v>
+        <v>717</v>
+      </c>
+      <c r="C87" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B88" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="B89" t="s">
-        <v>564</v>
+        <v>127</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B90" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B91" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B92" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B93" t="s">
-        <v>471</v>
-      </c>
-      <c r="C93" t="s">
-        <v>652</v>
+        <v>567</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B94" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="C94" t="s">
-        <v>529</v>
+        <v>652</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B95" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C95" t="s">
         <v>529</v>
@@ -8352,29 +8355,29 @@
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>605</v>
+        <v>143</v>
       </c>
       <c r="B96" t="s">
-        <v>606</v>
+        <v>474</v>
+      </c>
+      <c r="C96" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>683</v>
+        <v>605</v>
       </c>
       <c r="B97" t="s">
-        <v>684</v>
-      </c>
-      <c r="C97" t="s">
-        <v>657</v>
+        <v>606</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>710</v>
+        <v>683</v>
       </c>
       <c r="B98" t="s">
-        <v>711</v>
+        <v>684</v>
       </c>
       <c r="C98" t="s">
         <v>657</v>
@@ -8382,10 +8385,10 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="B99" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C99" t="s">
         <v>657</v>
@@ -8393,10 +8396,10 @@
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="B100" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="C100" t="s">
         <v>657</v>
@@ -8404,349 +8407,349 @@
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
+        <v>715</v>
+      </c>
+      <c r="B101" t="s">
+        <v>714</v>
+      </c>
+      <c r="C101" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3">
+      <c r="A102" t="s">
         <v>515</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B102" t="s">
         <v>638</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3">
-      <c r="A103" t="s">
-        <v>146</v>
-      </c>
-      <c r="B103" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B104" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B105" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B106" t="s">
-        <v>551</v>
-      </c>
-      <c r="C106" t="s">
-        <v>656</v>
+        <v>151</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>655</v>
+        <v>144</v>
       </c>
       <c r="B107" t="s">
         <v>551</v>
       </c>
+      <c r="C107" t="s">
+        <v>656</v>
+      </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>145</v>
+        <v>655</v>
       </c>
       <c r="B108" t="s">
-        <v>128</v>
+        <v>551</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="B109" t="s">
-        <v>568</v>
+        <v>128</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B110" t="s">
-        <v>129</v>
+        <v>568</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>607</v>
+        <v>131</v>
       </c>
       <c r="B111" t="s">
-        <v>608</v>
+        <v>129</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
+        <v>607</v>
+      </c>
+      <c r="B112" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" t="s">
         <v>514</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B113" t="s">
         <v>639</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3">
-      <c r="A114" t="s">
-        <v>187</v>
-      </c>
-      <c r="B114" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>132</v>
+        <v>187</v>
       </c>
       <c r="B115" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B116" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B117" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>772</v>
+        <v>133</v>
       </c>
       <c r="B118" t="s">
-        <v>771</v>
-      </c>
-      <c r="C118" t="s">
-        <v>657</v>
+        <v>154</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>135</v>
+        <v>772</v>
       </c>
       <c r="B119" t="s">
-        <v>155</v>
+        <v>771</v>
+      </c>
+      <c r="C119" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B120" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>598</v>
+        <v>136</v>
       </c>
       <c r="B121" t="s">
-        <v>660</v>
-      </c>
-      <c r="C121" t="s">
-        <v>664</v>
+        <v>156</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>609</v>
+        <v>598</v>
       </c>
       <c r="B122" t="s">
-        <v>610</v>
+        <v>660</v>
+      </c>
+      <c r="C122" t="s">
+        <v>664</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>513</v>
+        <v>609</v>
       </c>
       <c r="B123" t="s">
-        <v>640</v>
+        <v>610</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
+        <v>513</v>
+      </c>
+      <c r="B124" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3">
+      <c r="A125" t="s">
         <v>685</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B125" t="s">
         <v>686</v>
       </c>
-      <c r="C124" t="s">
+      <c r="C125" t="s">
         <v>657</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3">
-      <c r="A126" t="s">
-        <v>674</v>
-      </c>
-      <c r="B126" t="s">
-        <v>675</v>
-      </c>
-      <c r="C126" t="s">
-        <v>676</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="B127" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="C127" t="s">
         <v>676</v>
       </c>
     </row>
-    <row r="129" spans="1:3">
-      <c r="A129" t="s">
-        <v>158</v>
-      </c>
-      <c r="B129" t="s">
-        <v>162</v>
+    <row r="128" spans="1:3">
+      <c r="A128" t="s">
+        <v>677</v>
+      </c>
+      <c r="B128" t="s">
+        <v>678</v>
+      </c>
+      <c r="C128" t="s">
+        <v>676</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B130" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B131" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B132" t="s">
-        <v>569</v>
+        <v>164</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>530</v>
+        <v>161</v>
       </c>
       <c r="B133" t="s">
-        <v>699</v>
-      </c>
-      <c r="C133" t="s">
-        <v>700</v>
+        <v>569</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>615</v>
+        <v>530</v>
       </c>
       <c r="B134" t="s">
-        <v>616</v>
+        <v>699</v>
+      </c>
+      <c r="C134" t="s">
+        <v>700</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
+        <v>615</v>
+      </c>
+      <c r="B135" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3">
+      <c r="A136" t="s">
         <v>512</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B136" t="s">
         <v>641</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3">
-      <c r="A137" t="s">
-        <v>191</v>
-      </c>
-      <c r="B137" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>165</v>
+        <v>191</v>
       </c>
       <c r="B138" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B139" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>611</v>
+        <v>166</v>
       </c>
       <c r="B140" t="s">
-        <v>612</v>
+        <v>168</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>511</v>
+        <v>611</v>
       </c>
       <c r="B141" t="s">
-        <v>642</v>
+        <v>612</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
+        <v>511</v>
+      </c>
+      <c r="B142" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3">
+      <c r="A143" t="s">
         <v>687</v>
       </c>
-      <c r="B142" t="s">
+      <c r="B143" t="s">
         <v>688</v>
       </c>
-      <c r="C142" t="s">
+      <c r="C143" t="s">
         <v>657</v>
-      </c>
-    </row>
-    <row r="144" spans="1:3">
-      <c r="A144" t="s">
-        <v>189</v>
-      </c>
-      <c r="B144" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="B145" t="s">
-        <v>171</v>
-      </c>
-      <c r="C145" t="s">
-        <v>559</v>
+        <v>190</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B146" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C146" t="s">
         <v>559</v>
@@ -8754,10 +8757,10 @@
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B147" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C147" t="s">
         <v>559</v>
@@ -8765,75 +8768,75 @@
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="B148" t="s">
-        <v>199</v>
+        <v>173</v>
+      </c>
+      <c r="C148" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B149" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>175</v>
+        <v>197</v>
       </c>
       <c r="B150" t="s">
-        <v>176</v>
-      </c>
-      <c r="C150" t="s">
-        <v>559</v>
+        <v>198</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>613</v>
+        <v>175</v>
       </c>
       <c r="B151" t="s">
-        <v>614</v>
+        <v>176</v>
+      </c>
+      <c r="C151" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
+        <v>613</v>
+      </c>
+      <c r="B152" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3">
+      <c r="A153" t="s">
         <v>500</v>
       </c>
-      <c r="B152" t="s">
+      <c r="B153" t="s">
         <v>643</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3">
-      <c r="A154" t="s">
-        <v>620</v>
-      </c>
-      <c r="B154" t="s">
-        <v>621</v>
-      </c>
-      <c r="C154" t="s">
-        <v>622</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>690</v>
+        <v>620</v>
       </c>
       <c r="B155" t="s">
-        <v>691</v>
+        <v>621</v>
       </c>
       <c r="C155" t="s">
-        <v>657</v>
+        <v>622</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>786</v>
+        <v>690</v>
       </c>
       <c r="B156" t="s">
-        <v>769</v>
+        <v>691</v>
       </c>
       <c r="C156" t="s">
         <v>657</v>
@@ -8841,10 +8844,10 @@
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="B157" t="s">
-        <v>758</v>
+        <v>769</v>
       </c>
       <c r="C157" t="s">
         <v>657</v>
@@ -8852,40 +8855,40 @@
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="B158" t="s">
-        <v>767</v>
+        <v>758</v>
       </c>
       <c r="C158" t="s">
         <v>657</v>
       </c>
     </row>
-    <row r="160" spans="1:3">
-      <c r="A160" t="s">
-        <v>488</v>
-      </c>
-      <c r="B160" t="s">
-        <v>489</v>
+    <row r="159" spans="1:3">
+      <c r="A159" t="s">
+        <v>787</v>
+      </c>
+      <c r="B159" t="s">
+        <v>767</v>
+      </c>
+      <c r="C159" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>628</v>
+        <v>488</v>
       </c>
       <c r="B161" t="s">
-        <v>632</v>
-      </c>
-      <c r="C161" t="s">
-        <v>630</v>
+        <v>489</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B162" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="C162" t="s">
         <v>630</v>
@@ -8893,150 +8896,150 @@
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>239</v>
+        <v>629</v>
       </c>
       <c r="B163" t="s">
-        <v>240</v>
+        <v>631</v>
       </c>
       <c r="C163" t="s">
-        <v>559</v>
+        <v>630</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B164" t="s">
-        <v>242</v>
+        <v>240</v>
+      </c>
+      <c r="C164" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="B165" t="s">
-        <v>533</v>
-      </c>
-      <c r="C165" t="s">
-        <v>618</v>
+        <v>242</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>748</v>
+        <v>255</v>
       </c>
       <c r="B166" t="s">
-        <v>749</v>
+        <v>533</v>
       </c>
       <c r="C166" t="s">
-        <v>657</v>
+        <v>618</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>244</v>
+        <v>748</v>
       </c>
       <c r="B167" t="s">
-        <v>243</v>
+        <v>749</v>
+      </c>
+      <c r="C167" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>478</v>
+        <v>244</v>
       </c>
       <c r="B168" t="s">
-        <v>487</v>
+        <v>243</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>246</v>
+        <v>478</v>
       </c>
       <c r="B169" t="s">
-        <v>245</v>
+        <v>487</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B170" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B171" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="B172" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B173" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>294</v>
+        <v>254</v>
       </c>
       <c r="B174" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>326</v>
+        <v>294</v>
       </c>
       <c r="B175" t="s">
-        <v>327</v>
+        <v>245</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>624</v>
+        <v>326</v>
       </c>
       <c r="B176" t="s">
-        <v>625</v>
+        <v>327</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>666</v>
+        <v>624</v>
       </c>
       <c r="B177" t="s">
-        <v>667</v>
+        <v>625</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>734</v>
+        <v>666</v>
       </c>
       <c r="B178" t="s">
-        <v>735</v>
-      </c>
-      <c r="C178" t="s">
-        <v>657</v>
+        <v>667</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>747</v>
+        <v>734</v>
       </c>
       <c r="B179" t="s">
-        <v>770</v>
+        <v>735</v>
       </c>
       <c r="C179" t="s">
         <v>657</v>
@@ -9044,268 +9047,271 @@
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
+        <v>747</v>
+      </c>
+      <c r="B180" t="s">
+        <v>770</v>
+      </c>
+      <c r="C180" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3">
+      <c r="A181" t="s">
         <v>499</v>
       </c>
-      <c r="B180" t="s">
+      <c r="B181" t="s">
         <v>644</v>
-      </c>
-    </row>
-    <row r="182" spans="1:3">
-      <c r="A182" t="s">
-        <v>745</v>
-      </c>
-      <c r="B182" t="s">
-        <v>746</v>
-      </c>
-      <c r="C182" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>490</v>
+        <v>745</v>
       </c>
       <c r="B183" t="s">
-        <v>491</v>
+        <v>746</v>
+      </c>
+      <c r="C183" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
+        <v>490</v>
+      </c>
+      <c r="B184" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3">
+      <c r="A185" t="s">
         <v>256</v>
       </c>
-      <c r="B184" t="s">
+      <c r="B185" t="s">
         <v>259</v>
       </c>
-      <c r="C184" t="s">
+      <c r="C185" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="185" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A185" t="s">
+    <row r="186" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A186" t="s">
         <v>258</v>
       </c>
-      <c r="B185" t="s">
+      <c r="B186" t="s">
         <v>534</v>
       </c>
-      <c r="C185" t="s">
+      <c r="C186" t="s">
         <v>661</v>
-      </c>
-    </row>
-    <row r="186" spans="1:3">
-      <c r="A186" t="s">
-        <v>257</v>
-      </c>
-      <c r="B186" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B187" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B188" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B189" t="s">
-        <v>265</v>
-      </c>
-      <c r="C189" t="s">
-        <v>627</v>
+        <v>264</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>479</v>
+        <v>266</v>
       </c>
       <c r="B190" t="s">
-        <v>541</v>
+        <v>265</v>
+      </c>
+      <c r="C190" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>267</v>
+        <v>479</v>
       </c>
       <c r="B191" t="s">
-        <v>268</v>
+        <v>541</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B192" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B193" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B194" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B195" t="s">
-        <v>282</v>
-      </c>
-      <c r="C195" t="s">
-        <v>627</v>
+        <v>283</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B196" t="s">
-        <v>574</v>
+        <v>282</v>
+      </c>
+      <c r="C196" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B197" t="s">
-        <v>281</v>
-      </c>
-      <c r="C197" t="s">
-        <v>627</v>
+        <v>574</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B198" t="s">
-        <v>280</v>
+        <v>281</v>
+      </c>
+      <c r="C198" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
       <c r="B199" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B200" t="s">
-        <v>245</v>
+        <v>292</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B201" t="s">
-        <v>296</v>
+        <v>245</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>668</v>
+        <v>295</v>
       </c>
       <c r="B202" t="s">
-        <v>667</v>
+        <v>296</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>510</v>
+        <v>668</v>
       </c>
       <c r="B203" t="s">
-        <v>645</v>
+        <v>667</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
+        <v>510</v>
+      </c>
+      <c r="B204" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3">
+      <c r="A205" t="s">
         <v>662</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B205" t="s">
         <v>663</v>
       </c>
-      <c r="C204" t="s">
+      <c r="C205" t="s">
         <v>657</v>
-      </c>
-    </row>
-    <row r="206" spans="1:3">
-      <c r="A206" t="s">
-        <v>492</v>
-      </c>
-      <c r="B206" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>480</v>
+        <v>492</v>
       </c>
       <c r="B207" t="s">
-        <v>542</v>
+        <v>862</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>289</v>
+        <v>480</v>
       </c>
       <c r="B208" t="s">
-        <v>864</v>
+        <v>542</v>
       </c>
     </row>
     <row r="209" spans="1:2">
       <c r="A209" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B209" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
     </row>
     <row r="210" spans="1:2">
       <c r="A210" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="B210" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="211" spans="1:2">
       <c r="A211" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B211" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
     </row>
     <row r="212" spans="1:2">
       <c r="A212" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B212" t="s">
         <v>867</v>
@@ -9313,71 +9319,71 @@
     </row>
     <row r="213" spans="1:2">
       <c r="A213" t="s">
-        <v>669</v>
+        <v>299</v>
       </c>
       <c r="B213" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
     </row>
     <row r="214" spans="1:2">
       <c r="A214" t="s">
+        <v>669</v>
+      </c>
+      <c r="B214" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2">
+      <c r="A215" t="s">
         <v>509</v>
       </c>
-      <c r="B214" t="s">
+      <c r="B215" t="s">
         <v>646</v>
-      </c>
-    </row>
-    <row r="216" spans="1:2">
-      <c r="A216" t="s">
-        <v>493</v>
-      </c>
-      <c r="B216" t="s">
-        <v>855</v>
       </c>
     </row>
     <row r="217" spans="1:2">
       <c r="A217" t="s">
-        <v>481</v>
+        <v>493</v>
       </c>
       <c r="B217" t="s">
-        <v>543</v>
+        <v>854</v>
       </c>
     </row>
     <row r="218" spans="1:2">
       <c r="A218" t="s">
-        <v>302</v>
+        <v>481</v>
       </c>
       <c r="B218" t="s">
-        <v>856</v>
+        <v>543</v>
       </c>
     </row>
     <row r="219" spans="1:2">
       <c r="A219" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B219" t="s">
-        <v>305</v>
+        <v>855</v>
       </c>
     </row>
     <row r="220" spans="1:2">
       <c r="A220" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B220" t="s">
-        <v>857</v>
+        <v>305</v>
       </c>
     </row>
     <row r="221" spans="1:2">
       <c r="A221" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B221" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
     </row>
     <row r="222" spans="1:2">
       <c r="A222" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B222" t="s">
         <v>858</v>
@@ -9385,519 +9391,516 @@
     </row>
     <row r="223" spans="1:2">
       <c r="A223" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B223" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
     </row>
     <row r="224" spans="1:2">
       <c r="A224" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B224" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>670</v>
+        <v>309</v>
       </c>
       <c r="B225" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
+        <v>670</v>
+      </c>
+      <c r="B226" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3">
+      <c r="A227" t="s">
         <v>508</v>
       </c>
-      <c r="B226" t="s">
+      <c r="B227" t="s">
         <v>647</v>
-      </c>
-    </row>
-    <row r="228" spans="1:3">
-      <c r="A228" t="s">
-        <v>494</v>
-      </c>
-      <c r="B228" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>476</v>
+        <v>494</v>
       </c>
       <c r="B229" t="s">
-        <v>315</v>
-      </c>
-      <c r="C229" t="s">
-        <v>559</v>
+        <v>495</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="B230" t="s">
-        <v>544</v>
+        <v>315</v>
+      </c>
+      <c r="C230" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>313</v>
+        <v>482</v>
       </c>
       <c r="B231" t="s">
-        <v>316</v>
-      </c>
-      <c r="C231" t="s">
-        <v>559</v>
+        <v>544</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B232" t="s">
-        <v>317</v>
+        <v>316</v>
+      </c>
+      <c r="C232" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>475</v>
+        <v>314</v>
       </c>
       <c r="B233" t="s">
-        <v>535</v>
+        <v>317</v>
       </c>
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>321</v>
+        <v>475</v>
       </c>
       <c r="B234" t="s">
-        <v>245</v>
+        <v>535</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B235" t="s">
-        <v>318</v>
+        <v>245</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B236" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B237" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B238" t="s">
-        <v>253</v>
+        <v>320</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>671</v>
+        <v>325</v>
       </c>
       <c r="B239" t="s">
-        <v>667</v>
+        <v>253</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
+        <v>671</v>
+      </c>
+      <c r="B240" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3">
+      <c r="A241" t="s">
         <v>507</v>
       </c>
-      <c r="B240" t="s">
+      <c r="B241" t="s">
         <v>648</v>
-      </c>
-    </row>
-    <row r="242" spans="1:3">
-      <c r="A242" t="s">
-        <v>705</v>
-      </c>
-      <c r="B242" t="s">
-        <v>706</v>
-      </c>
-      <c r="C242" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>524</v>
+        <v>705</v>
       </c>
       <c r="B243" t="s">
-        <v>527</v>
+        <v>706</v>
       </c>
       <c r="C243" t="s">
-        <v>557</v>
+        <v>657</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B244" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="C244" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>556</v>
+        <v>525</v>
       </c>
       <c r="B245" t="s">
-        <v>570</v>
+        <v>526</v>
+      </c>
+      <c r="C245" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>342</v>
+        <v>556</v>
       </c>
       <c r="B246" t="s">
-        <v>328</v>
+        <v>570</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B247" t="s">
-        <v>329</v>
-      </c>
-      <c r="C247" t="s">
-        <v>559</v>
+        <v>328</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>483</v>
+        <v>343</v>
       </c>
       <c r="B248" t="s">
-        <v>545</v>
+        <v>329</v>
+      </c>
+      <c r="C248" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>344</v>
+        <v>483</v>
       </c>
       <c r="B249" t="s">
-        <v>330</v>
+        <v>545</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B250" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B251" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B252" t="s">
-        <v>333</v>
-      </c>
-      <c r="C252" t="s">
-        <v>559</v>
+        <v>332</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B253" t="s">
-        <v>334</v>
+        <v>333</v>
+      </c>
+      <c r="C253" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B254" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B255" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B256" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="B257" t="s">
-        <v>338</v>
-      </c>
-      <c r="C257" t="s">
-        <v>559</v>
+        <v>337</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B258" t="s">
-        <v>339</v>
+        <v>338</v>
+      </c>
+      <c r="C258" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B259" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B260" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
+        <v>355</v>
+      </c>
+      <c r="B261" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3">
+      <c r="A262" t="s">
         <v>506</v>
       </c>
-      <c r="B261" t="s">
+      <c r="B262" t="s">
         <v>633</v>
-      </c>
-    </row>
-    <row r="263" spans="1:3">
-      <c r="A263" t="s">
-        <v>575</v>
-      </c>
-      <c r="B263" t="s">
-        <v>576</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>362</v>
+        <v>575</v>
       </c>
       <c r="B264" t="s">
-        <v>380</v>
+        <v>576</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B265" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B266" t="s">
-        <v>378</v>
-      </c>
-      <c r="C266" t="s">
-        <v>559</v>
+        <v>377</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>484</v>
+        <v>364</v>
       </c>
       <c r="B267" t="s">
-        <v>546</v>
+        <v>378</v>
+      </c>
+      <c r="C267" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>381</v>
+        <v>484</v>
       </c>
       <c r="B268" t="s">
-        <v>379</v>
-      </c>
-      <c r="C268" t="s">
-        <v>559</v>
+        <v>546</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="B269" t="s">
-        <v>371</v>
+        <v>379</v>
+      </c>
+      <c r="C269" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>382</v>
+        <v>365</v>
       </c>
       <c r="B270" t="s">
-        <v>372</v>
-      </c>
-      <c r="C270" t="s">
-        <v>536</v>
+        <v>371</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>366</v>
+        <v>382</v>
       </c>
       <c r="B271" t="s">
-        <v>373</v>
+        <v>372</v>
+      </c>
+      <c r="C271" t="s">
+        <v>536</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B272" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B273" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="B274" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B275" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
+        <v>370</v>
+      </c>
+      <c r="B276" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3">
+      <c r="A277" t="s">
         <v>505</v>
       </c>
-      <c r="B276" t="s">
+      <c r="B277" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="278" spans="1:3">
-      <c r="A278" t="s">
+    <row r="279" spans="1:3">
+      <c r="A279" t="s">
         <v>707</v>
       </c>
-      <c r="B278" t="s">
+      <c r="B279" t="s">
         <v>726</v>
       </c>
-      <c r="C278" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="280" spans="1:3">
-      <c r="A280" t="s">
-        <v>703</v>
-      </c>
-      <c r="B280" t="s">
-        <v>704</v>
-      </c>
-      <c r="C280" t="s">
+      <c r="C279" t="s">
         <v>657</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>496</v>
+        <v>703</v>
       </c>
       <c r="B281" t="s">
-        <v>497</v>
+        <v>704</v>
+      </c>
+      <c r="C281" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>388</v>
+        <v>496</v>
       </c>
       <c r="B282" t="s">
-        <v>399</v>
+        <v>497</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B283" t="s">
-        <v>400</v>
-      </c>
-      <c r="C283" t="s">
-        <v>559</v>
+        <v>399</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>547</v>
+        <v>389</v>
       </c>
       <c r="B284" t="s">
-        <v>548</v>
+        <v>400</v>
+      </c>
+      <c r="C284" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>390</v>
+        <v>547</v>
       </c>
       <c r="B285" t="s">
-        <v>401</v>
-      </c>
-      <c r="C285" t="s">
-        <v>559</v>
+        <v>548</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B286" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C286" t="s">
         <v>559</v>
@@ -9905,139 +9908,139 @@
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B287" t="s">
-        <v>560</v>
+        <v>402</v>
+      </c>
+      <c r="C287" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B288" t="s">
-        <v>403</v>
+        <v>560</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B289" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B290" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B291" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B292" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B293" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>764</v>
+        <v>398</v>
       </c>
       <c r="B294" t="s">
-        <v>765</v>
-      </c>
-      <c r="C294" t="s">
-        <v>657</v>
+        <v>408</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>503</v>
+        <v>764</v>
       </c>
       <c r="B295" t="s">
-        <v>650</v>
+        <v>765</v>
+      </c>
+      <c r="C295" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
+        <v>503</v>
+      </c>
+      <c r="B296" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3">
+      <c r="A297" t="s">
         <v>584</v>
       </c>
-      <c r="B296" t="s">
+      <c r="B297" t="s">
         <v>585</v>
-      </c>
-    </row>
-    <row r="298" spans="1:3">
-      <c r="A298" t="s">
-        <v>498</v>
-      </c>
-      <c r="B298" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>415</v>
+        <v>498</v>
       </c>
       <c r="B299" t="s">
-        <v>426</v>
+        <v>497</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B300" t="s">
-        <v>427</v>
-      </c>
-      <c r="C300" t="s">
-        <v>559</v>
+        <v>426</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>485</v>
+        <v>416</v>
       </c>
       <c r="B301" t="s">
-        <v>549</v>
+        <v>427</v>
+      </c>
+      <c r="C301" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="302" spans="1:3">
       <c r="A302" t="s">
-        <v>417</v>
+        <v>485</v>
       </c>
       <c r="B302" t="s">
-        <v>428</v>
-      </c>
-      <c r="C302" t="s">
-        <v>559</v>
+        <v>549</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B303" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C303" t="s">
         <v>559</v>
@@ -10045,446 +10048,449 @@
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="B304" t="s">
-        <v>561</v>
+        <v>429</v>
+      </c>
+      <c r="C304" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="B305" t="s">
-        <v>403</v>
+        <v>561</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="B306" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B307" t="s">
-        <v>430</v>
+        <v>404</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B308" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B309" t="s">
-        <v>407</v>
+        <v>431</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B310" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>502</v>
+        <v>425</v>
       </c>
       <c r="B311" t="s">
-        <v>650</v>
+        <v>408</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
+        <v>502</v>
+      </c>
+      <c r="B312" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3">
+      <c r="A313" t="s">
         <v>591</v>
       </c>
-      <c r="B312" t="s">
+      <c r="B313" t="s">
         <v>585</v>
-      </c>
-    </row>
-    <row r="314" spans="1:3">
-      <c r="A314" t="s">
-        <v>701</v>
-      </c>
-      <c r="B314" t="s">
-        <v>702</v>
-      </c>
-      <c r="C314" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>409</v>
+        <v>701</v>
       </c>
       <c r="B315" t="s">
-        <v>592</v>
+        <v>702</v>
+      </c>
+      <c r="C315" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B316" t="s">
-        <v>593</v>
-      </c>
-      <c r="C316" t="s">
-        <v>559</v>
+        <v>592</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>486</v>
+        <v>410</v>
       </c>
       <c r="B317" t="s">
-        <v>594</v>
+        <v>593</v>
+      </c>
+      <c r="C317" t="s">
+        <v>559</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>411</v>
+        <v>486</v>
       </c>
       <c r="B318" t="s">
-        <v>619</v>
+        <v>594</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="B319" t="s">
-        <v>595</v>
+        <v>619</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B320" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
+        <v>413</v>
+      </c>
+      <c r="B321" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3">
+      <c r="A322" t="s">
         <v>501</v>
       </c>
-      <c r="B321" t="s">
+      <c r="B322" t="s">
         <v>651</v>
-      </c>
-    </row>
-    <row r="323" spans="1:3">
-      <c r="A323" t="s">
-        <v>782</v>
-      </c>
-      <c r="B323" t="s">
-        <v>783</v>
-      </c>
-      <c r="C323" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="B324" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
       <c r="C324" t="s">
         <v>657</v>
       </c>
     </row>
-    <row r="326" spans="1:3">
-      <c r="A326" t="s">
-        <v>791</v>
-      </c>
-      <c r="B326" t="s">
-        <v>792</v>
+    <row r="325" spans="1:3">
+      <c r="A325" t="s">
+        <v>783</v>
+      </c>
+      <c r="B325" t="s">
+        <v>784</v>
+      </c>
+      <c r="C325" t="s">
+        <v>657</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="B327" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
       <c r="B328" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="B329" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="B330" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
       <c r="B331" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
       <c r="B332" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
       <c r="B333" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
       <c r="B334" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="B335" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="B336" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="A337" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
       <c r="B337" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="A338" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
       <c r="B338" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="A339" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
       <c r="B339" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
     </row>
     <row r="340" spans="1:2">
       <c r="A340" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="B340" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
     </row>
     <row r="341" spans="1:2">
       <c r="A341" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="B341" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
     </row>
     <row r="342" spans="1:2">
       <c r="A342" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="B342" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
     </row>
     <row r="343" spans="1:2">
       <c r="A343" t="s">
+        <v>822</v>
+      </c>
+      <c r="B343" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="344" spans="1:2">
+      <c r="A344" t="s">
+        <v>824</v>
+      </c>
+      <c r="B344" t="s">
         <v>825</v>
-      </c>
-      <c r="B343" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="345" spans="1:2">
-      <c r="A345" t="s">
-        <v>827</v>
-      </c>
-      <c r="B345" t="s">
-        <v>828</v>
       </c>
     </row>
     <row r="346" spans="1:2">
       <c r="A346" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
       <c r="B346" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
     </row>
     <row r="347" spans="1:2">
       <c r="A347" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="B347" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
     </row>
     <row r="348" spans="1:2">
       <c r="A348" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="B348" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
     </row>
     <row r="349" spans="1:2">
       <c r="A349" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="B349" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
     </row>
     <row r="350" spans="1:2">
       <c r="A350" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="B350" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
     </row>
     <row r="351" spans="1:2">
       <c r="A351" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="B351" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
     </row>
     <row r="352" spans="1:2">
       <c r="A352" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="B352" t="s">
-        <v>341</v>
+        <v>839</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="B353" t="s">
-        <v>843</v>
+        <v>341</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="B354" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
       <c r="B355" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
+        <v>845</v>
+      </c>
+      <c r="B356" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="357" spans="1:2">
+      <c r="A357" t="s">
+        <v>847</v>
+      </c>
+      <c r="B357" t="s">
         <v>848</v>
-      </c>
-      <c r="B356" t="s">
-        <v>849</v>
-      </c>
-    </row>
-    <row r="358" spans="1:2">
-      <c r="A358" t="s">
-        <v>850</v>
-      </c>
-      <c r="B358" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
       <c r="B359" t="s">
-        <v>852</v>
+        <v>334</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="B360" t="s">
-        <v>336</v>
+        <v>851</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="B361" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2">
+      <c r="A362" t="s">
+        <v>853</v>
+      </c>
+      <c r="B362" t="s">
         <v>337</v>
-      </c>
-    </row>
-    <row r="363" spans="1:2">
-      <c r="A363" t="s">
-        <v>879</v>
-      </c>
-      <c r="B363" t="s">
-        <v>880</v>
       </c>
     </row>
     <row r="364" spans="1:2">
@@ -10492,223 +10498,223 @@
         <v>878</v>
       </c>
       <c r="B364" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="B365" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B366" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="B367" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>876</v>
+        <v>869</v>
       </c>
       <c r="B368" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="369" spans="1:2">
+      <c r="A369" t="s">
         <v>875</v>
       </c>
-    </row>
-    <row r="370" spans="1:2">
-      <c r="A370" t="s">
-        <v>883</v>
-      </c>
-      <c r="B370" t="s">
-        <v>888</v>
+      <c r="B369" t="s">
+        <v>874</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>891</v>
+        <v>882</v>
       </c>
       <c r="B371" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>884</v>
+        <v>890</v>
       </c>
       <c r="B372" t="s">
-        <v>872</v>
+        <v>888</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="B373" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
     </row>
     <row r="374" spans="1:2">
       <c r="A374" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="B374" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="B375" t="s">
-        <v>890</v>
-      </c>
-    </row>
-    <row r="377" spans="1:2">
-      <c r="A377" t="s">
-        <v>897</v>
-      </c>
-      <c r="B377" t="s">
-        <v>898</v>
+        <v>873</v>
+      </c>
+    </row>
+    <row r="376" spans="1:2">
+      <c r="A376" t="s">
+        <v>886</v>
+      </c>
+      <c r="B376" t="s">
+        <v>889</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="B378" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="B379" t="s">
-        <v>746</v>
+        <v>899</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>903</v>
+        <v>900</v>
       </c>
       <c r="B380" t="s">
-        <v>902</v>
+        <v>746</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>910</v>
+        <v>902</v>
       </c>
       <c r="B381" t="s">
-        <v>261</v>
+        <v>901</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="B382" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="B383" t="s">
-        <v>904</v>
+        <v>264</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="B384" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="B385" t="s">
-        <v>270</v>
+        <v>904</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="B386" t="s">
-        <v>906</v>
+        <v>270</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="B387" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="B388" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
       <c r="B389" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="B390" t="s">
-        <v>292</v>
+        <v>908</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="B391" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="B392" t="s">
-        <v>862</v>
+        <v>296</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>914</v>
+        <v>922</v>
       </c>
       <c r="B393" t="s">
-        <v>663</v>
+        <v>861</v>
       </c>
     </row>
     <row r="394" spans="1:2">
@@ -10716,6 +10722,14 @@
         <v>913</v>
       </c>
       <c r="B394" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="395" spans="1:2">
+      <c r="A395" t="s">
+        <v>912</v>
+      </c>
+      <c r="B395" t="s">
         <v>645</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updates to ASC, Paystubs testing, VSI
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56197263-7E09-4346-BEA5-EB43DFA1FDEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F76C44-90AE-4DD6-A743-85F407FE2AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1152" uniqueCount="928">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="932">
   <si>
     <t>Name</t>
   </si>
@@ -2824,6 +2824,18 @@
   </si>
   <si>
     <t>Asset Self-Certification has not been dated by all adults.</t>
+  </si>
+  <si>
+    <t>Total Cash Value of Real Property does not match the sum of the Asset Type of Real Estate/Real Property on the Household Asset Breakdown.</t>
+  </si>
+  <si>
+    <t>ASC_GA_AssetValueMatchWithHAB</t>
+  </si>
+  <si>
+    <t>Cash Value of an asset source does not match the sum of the same asset sources on the Household Asset Breakdown for Section 1 – Non-Necessary Personal Property.</t>
+  </si>
+  <si>
+    <t>ASC_GA_RealPrptyValue</t>
   </si>
 </sst>
 </file>
@@ -7550,7 +7562,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C399"/>
+  <dimension ref="A1:C401"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -8448,354 +8460,348 @@
         <v>925</v>
       </c>
     </row>
+    <row r="106" spans="1:3">
+      <c r="A106" t="s">
+        <v>929</v>
+      </c>
+      <c r="B106" t="s">
+        <v>930</v>
+      </c>
+    </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>146</v>
+        <v>931</v>
       </c>
       <c r="B107" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3">
-      <c r="A108" t="s">
-        <v>147</v>
-      </c>
-      <c r="B108" t="s">
-        <v>150</v>
+        <v>928</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B109" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B110" t="s">
-        <v>525</v>
-      </c>
-      <c r="C110" t="s">
-        <v>628</v>
+        <v>150</v>
       </c>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>627</v>
+        <v>148</v>
       </c>
       <c r="B111" t="s">
-        <v>525</v>
+        <v>151</v>
       </c>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B112" t="s">
-        <v>128</v>
+        <v>525</v>
+      </c>
+      <c r="C112" t="s">
+        <v>628</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>130</v>
+        <v>627</v>
       </c>
       <c r="B113" t="s">
-        <v>542</v>
+        <v>525</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="B114" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>580</v>
+        <v>130</v>
       </c>
       <c r="B115" t="s">
-        <v>581</v>
+        <v>542</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>491</v>
+        <v>131</v>
       </c>
       <c r="B116" t="s">
-        <v>611</v>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3">
+      <c r="A117" t="s">
+        <v>580</v>
+      </c>
+      <c r="B117" t="s">
+        <v>581</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>187</v>
+        <v>491</v>
       </c>
       <c r="B118" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3">
-      <c r="A119" t="s">
-        <v>132</v>
-      </c>
-      <c r="B119" t="s">
-        <v>152</v>
+        <v>611</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>134</v>
+        <v>187</v>
       </c>
       <c r="B120" t="s">
-        <v>153</v>
+        <v>188</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B121" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>740</v>
+        <v>134</v>
       </c>
       <c r="B122" t="s">
-        <v>739</v>
-      </c>
-      <c r="C122" t="s">
-        <v>629</v>
+        <v>153</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B123" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>136</v>
+        <v>740</v>
       </c>
       <c r="B124" t="s">
-        <v>156</v>
+        <v>739</v>
+      </c>
+      <c r="C124" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>571</v>
+        <v>135</v>
       </c>
       <c r="B125" t="s">
-        <v>632</v>
-      </c>
-      <c r="C125" t="s">
-        <v>636</v>
+        <v>155</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>582</v>
+        <v>136</v>
       </c>
       <c r="B126" t="s">
-        <v>583</v>
+        <v>156</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>490</v>
+        <v>571</v>
       </c>
       <c r="B127" t="s">
-        <v>612</v>
+        <v>632</v>
+      </c>
+      <c r="C127" t="s">
+        <v>636</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>656</v>
+        <v>582</v>
       </c>
       <c r="B128" t="s">
-        <v>657</v>
-      </c>
-      <c r="C128" t="s">
-        <v>629</v>
+        <v>583</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3">
+      <c r="A129" t="s">
+        <v>490</v>
+      </c>
+      <c r="B129" t="s">
+        <v>612</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
+        <v>656</v>
+      </c>
+      <c r="B130" t="s">
+        <v>657</v>
+      </c>
+      <c r="C130" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3">
+      <c r="A132" t="s">
         <v>645</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B132" t="s">
         <v>646</v>
       </c>
-      <c r="C130" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3">
-      <c r="A131" t="s">
-        <v>648</v>
-      </c>
-      <c r="B131" t="s">
-        <v>649</v>
-      </c>
-      <c r="C131" t="s">
+      <c r="C132" t="s">
         <v>647</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>158</v>
+        <v>648</v>
       </c>
       <c r="B133" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3">
-      <c r="A134" t="s">
-        <v>159</v>
-      </c>
-      <c r="B134" t="s">
-        <v>163</v>
+        <v>649</v>
+      </c>
+      <c r="C133" t="s">
+        <v>647</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B135" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B136" t="s">
-        <v>543</v>
+        <v>163</v>
       </c>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>507</v>
+        <v>160</v>
       </c>
       <c r="B137" t="s">
-        <v>670</v>
-      </c>
-      <c r="C137" t="s">
-        <v>671</v>
+        <v>164</v>
       </c>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>588</v>
+        <v>161</v>
       </c>
       <c r="B138" t="s">
-        <v>589</v>
+        <v>543</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>489</v>
+        <v>507</v>
       </c>
       <c r="B139" t="s">
-        <v>613</v>
+        <v>670</v>
+      </c>
+      <c r="C139" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3">
+      <c r="A140" t="s">
+        <v>588</v>
+      </c>
+      <c r="B140" t="s">
+        <v>589</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>489</v>
       </c>
       <c r="B141" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3">
-      <c r="A142" t="s">
-        <v>165</v>
-      </c>
-      <c r="B142" t="s">
-        <v>167</v>
+        <v>613</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="B143" t="s">
-        <v>168</v>
+        <v>192</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>584</v>
+        <v>165</v>
       </c>
       <c r="B144" t="s">
-        <v>585</v>
+        <v>167</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>488</v>
+        <v>166</v>
       </c>
       <c r="B145" t="s">
-        <v>614</v>
+        <v>168</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>658</v>
+        <v>584</v>
       </c>
       <c r="B146" t="s">
-        <v>659</v>
-      </c>
-      <c r="C146" t="s">
-        <v>629</v>
+        <v>585</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3">
+      <c r="A147" t="s">
+        <v>488</v>
+      </c>
+      <c r="B147" t="s">
+        <v>614</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>189</v>
+        <v>658</v>
       </c>
       <c r="B148" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3">
-      <c r="A149" t="s">
-        <v>174</v>
-      </c>
-      <c r="B149" t="s">
-        <v>171</v>
-      </c>
-      <c r="C149" t="s">
-        <v>533</v>
+        <v>659</v>
+      </c>
+      <c r="C148" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
       <c r="B150" t="s">
-        <v>172</v>
-      </c>
-      <c r="C150" t="s">
-        <v>533</v>
+        <v>190</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B151" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C151" t="s">
         <v>533</v>
@@ -8803,86 +8809,86 @@
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>200</v>
+        <v>169</v>
       </c>
       <c r="B152" t="s">
-        <v>199</v>
+        <v>172</v>
+      </c>
+      <c r="C152" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>197</v>
+        <v>170</v>
       </c>
       <c r="B153" t="s">
-        <v>198</v>
+        <v>173</v>
+      </c>
+      <c r="C153" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="B154" t="s">
-        <v>176</v>
-      </c>
-      <c r="C154" t="s">
-        <v>533</v>
+        <v>199</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>586</v>
+        <v>197</v>
       </c>
       <c r="B155" t="s">
-        <v>587</v>
+        <v>198</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>477</v>
+        <v>175</v>
       </c>
       <c r="B156" t="s">
-        <v>615</v>
+        <v>176</v>
+      </c>
+      <c r="C156" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3">
+      <c r="A157" t="s">
+        <v>586</v>
+      </c>
+      <c r="B157" t="s">
+        <v>587</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>593</v>
+        <v>477</v>
       </c>
       <c r="B158" t="s">
-        <v>898</v>
-      </c>
-      <c r="C158" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3">
-      <c r="A159" t="s">
-        <v>661</v>
-      </c>
-      <c r="B159" t="s">
-        <v>662</v>
-      </c>
-      <c r="C159" t="s">
-        <v>629</v>
+        <v>615</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>753</v>
+        <v>593</v>
       </c>
       <c r="B160" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="C160" t="s">
-        <v>629</v>
+        <v>594</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>754</v>
+        <v>661</v>
       </c>
       <c r="B161" t="s">
-        <v>900</v>
+        <v>662</v>
       </c>
       <c r="C161" t="s">
         <v>629</v>
@@ -8890,353 +8896,356 @@
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="B162" t="s">
-        <v>736</v>
+        <v>899</v>
       </c>
       <c r="C162" t="s">
         <v>629</v>
       </c>
     </row>
+    <row r="163" spans="1:3">
+      <c r="A163" t="s">
+        <v>754</v>
+      </c>
+      <c r="B163" t="s">
+        <v>900</v>
+      </c>
+      <c r="C163" t="s">
+        <v>629</v>
+      </c>
+    </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>468</v>
+        <v>755</v>
       </c>
       <c r="B164" t="s">
-        <v>901</v>
-      </c>
-    </row>
-    <row r="165" spans="1:3">
-      <c r="A165" t="s">
-        <v>600</v>
-      </c>
-      <c r="B165" t="s">
-        <v>604</v>
-      </c>
-      <c r="C165" t="s">
-        <v>602</v>
+        <v>736</v>
+      </c>
+      <c r="C164" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>601</v>
+        <v>468</v>
       </c>
       <c r="B166" t="s">
-        <v>603</v>
-      </c>
-      <c r="C166" t="s">
-        <v>602</v>
+        <v>901</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>239</v>
+        <v>600</v>
       </c>
       <c r="B167" t="s">
-        <v>902</v>
+        <v>604</v>
       </c>
       <c r="C167" t="s">
-        <v>533</v>
+        <v>602</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>240</v>
+        <v>601</v>
       </c>
       <c r="B168" t="s">
-        <v>903</v>
+        <v>603</v>
+      </c>
+      <c r="C168" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="B169" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="C169" t="s">
-        <v>591</v>
+        <v>533</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>719</v>
+        <v>240</v>
       </c>
       <c r="B170" t="s">
-        <v>905</v>
-      </c>
-      <c r="C170" t="s">
-        <v>629</v>
+        <v>903</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="B171" t="s">
-        <v>241</v>
+        <v>904</v>
+      </c>
+      <c r="C171" t="s">
+        <v>591</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>458</v>
+        <v>719</v>
       </c>
       <c r="B172" t="s">
-        <v>467</v>
+        <v>905</v>
+      </c>
+      <c r="C172" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B173" t="s">
-        <v>906</v>
+        <v>241</v>
       </c>
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>244</v>
+        <v>458</v>
       </c>
       <c r="B174" t="s">
-        <v>907</v>
+        <v>467</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B175" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B176" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B177" t="s">
-        <v>828</v>
+        <v>908</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>279</v>
+        <v>246</v>
       </c>
       <c r="B178" t="s">
-        <v>906</v>
+        <v>909</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>306</v>
+        <v>247</v>
       </c>
       <c r="B179" t="s">
-        <v>307</v>
+        <v>828</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>596</v>
+        <v>279</v>
       </c>
       <c r="B180" t="s">
-        <v>597</v>
+        <v>906</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>638</v>
+        <v>306</v>
       </c>
       <c r="B181" t="s">
-        <v>829</v>
+        <v>307</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>705</v>
+        <v>596</v>
       </c>
       <c r="B182" t="s">
-        <v>706</v>
-      </c>
-      <c r="C182" t="s">
-        <v>629</v>
+        <v>597</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>718</v>
+        <v>638</v>
       </c>
       <c r="B183" t="s">
-        <v>738</v>
-      </c>
-      <c r="C183" t="s">
-        <v>629</v>
+        <v>829</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>920</v>
+        <v>705</v>
       </c>
       <c r="B184" t="s">
-        <v>921</v>
+        <v>706</v>
+      </c>
+      <c r="C184" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>476</v>
+        <v>718</v>
       </c>
       <c r="B185" t="s">
-        <v>616</v>
+        <v>738</v>
+      </c>
+      <c r="C185" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3">
+      <c r="A186" t="s">
+        <v>920</v>
+      </c>
+      <c r="B186" t="s">
+        <v>921</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>716</v>
+        <v>476</v>
       </c>
       <c r="B187" t="s">
-        <v>717</v>
-      </c>
-      <c r="C187" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="188" spans="1:3">
-      <c r="A188" t="s">
-        <v>469</v>
-      </c>
-      <c r="B188" t="s">
-        <v>910</v>
+        <v>616</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>249</v>
+        <v>716</v>
       </c>
       <c r="B189" t="s">
-        <v>911</v>
+        <v>717</v>
       </c>
       <c r="C189" t="s">
-        <v>599</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3" ht="13.5" customHeight="1">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>251</v>
+        <v>469</v>
       </c>
       <c r="B190" t="s">
-        <v>912</v>
-      </c>
-      <c r="C190" t="s">
-        <v>633</v>
+        <v>910</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B191" t="s">
-        <v>869</v>
-      </c>
-    </row>
-    <row r="192" spans="1:3">
+        <v>911</v>
+      </c>
+      <c r="C191" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" ht="13.5" customHeight="1">
       <c r="A192" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B192" t="s">
-        <v>252</v>
+        <v>912</v>
+      </c>
+      <c r="C192" t="s">
+        <v>633</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B193" t="s">
-        <v>255</v>
+        <v>869</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B194" t="s">
-        <v>256</v>
-      </c>
-      <c r="C194" t="s">
-        <v>599</v>
+        <v>252</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>459</v>
+        <v>254</v>
       </c>
       <c r="B195" t="s">
-        <v>515</v>
+        <v>255</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B196" t="s">
-        <v>872</v>
+        <v>256</v>
+      </c>
+      <c r="C196" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>259</v>
+        <v>459</v>
       </c>
       <c r="B197" t="s">
-        <v>260</v>
+        <v>515</v>
       </c>
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="B198" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B199" t="s">
-        <v>874</v>
+        <v>260</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B200" t="s">
-        <v>913</v>
-      </c>
-      <c r="C200" t="s">
-        <v>599</v>
+        <v>873</v>
       </c>
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B201" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B202" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="C202" t="s">
         <v>599</v>
@@ -9244,256 +9253,256 @@
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B203" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="B204" t="s">
-        <v>277</v>
+        <v>914</v>
+      </c>
+      <c r="C204" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="B205" t="s">
-        <v>906</v>
+        <v>876</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="B206" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>639</v>
+        <v>278</v>
       </c>
       <c r="B207" t="s">
-        <v>829</v>
+        <v>906</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>487</v>
+        <v>280</v>
       </c>
       <c r="B208" t="s">
-        <v>617</v>
+        <v>281</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="B209" t="s">
-        <v>635</v>
-      </c>
-      <c r="C209" t="s">
-        <v>629</v>
+        <v>829</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3">
+      <c r="A210" t="s">
+        <v>487</v>
+      </c>
+      <c r="B210" t="s">
+        <v>617</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>470</v>
+        <v>634</v>
       </c>
       <c r="B211" t="s">
-        <v>830</v>
-      </c>
-    </row>
-    <row r="212" spans="1:3">
-      <c r="A212" t="s">
-        <v>460</v>
-      </c>
-      <c r="B212" t="s">
-        <v>516</v>
+        <v>635</v>
+      </c>
+      <c r="C211" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>274</v>
+        <v>470</v>
       </c>
       <c r="B213" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>275</v>
+        <v>460</v>
       </c>
       <c r="B214" t="s">
-        <v>832</v>
+        <v>516</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="B215" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="B216" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B217" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>640</v>
+        <v>282</v>
       </c>
       <c r="B218" t="s">
-        <v>829</v>
+        <v>835</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>486</v>
+        <v>284</v>
       </c>
       <c r="B219" t="s">
-        <v>618</v>
+        <v>834</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3">
+      <c r="A220" t="s">
+        <v>640</v>
+      </c>
+      <c r="B220" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>471</v>
+        <v>486</v>
       </c>
       <c r="B221" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="222" spans="1:3">
-      <c r="A222" t="s">
-        <v>461</v>
-      </c>
-      <c r="B222" t="s">
-        <v>517</v>
+        <v>618</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>287</v>
+        <v>471</v>
       </c>
       <c r="B223" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>288</v>
+        <v>461</v>
       </c>
       <c r="B224" t="s">
-        <v>290</v>
+        <v>517</v>
       </c>
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B225" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B226" t="s">
-        <v>826</v>
+        <v>290</v>
       </c>
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B227" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B228" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B229" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>641</v>
+        <v>293</v>
       </c>
       <c r="B230" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>485</v>
+        <v>294</v>
       </c>
       <c r="B231" t="s">
-        <v>619</v>
+        <v>828</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3">
+      <c r="A232" t="s">
+        <v>641</v>
+      </c>
+      <c r="B232" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>472</v>
+        <v>485</v>
       </c>
       <c r="B233" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="234" spans="1:3">
-      <c r="A234" t="s">
-        <v>456</v>
-      </c>
-      <c r="B234" t="s">
-        <v>300</v>
-      </c>
-      <c r="C234" t="s">
-        <v>533</v>
+        <v>619</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>462</v>
+        <v>472</v>
       </c>
       <c r="B235" t="s">
-        <v>518</v>
+        <v>915</v>
       </c>
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>298</v>
+        <v>456</v>
       </c>
       <c r="B236" t="s">
-        <v>916</v>
+        <v>300</v>
       </c>
       <c r="C236" t="s">
         <v>533</v>
@@ -9501,303 +9510,303 @@
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>299</v>
+        <v>462</v>
       </c>
       <c r="B237" t="s">
-        <v>896</v>
+        <v>518</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>455</v>
+        <v>298</v>
       </c>
       <c r="B238" t="s">
-        <v>897</v>
+        <v>916</v>
+      </c>
+      <c r="C238" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B239" t="s">
-        <v>906</v>
+        <v>896</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>302</v>
+        <v>455</v>
       </c>
       <c r="B240" t="s">
-        <v>917</v>
+        <v>897</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B241" t="s">
-        <v>918</v>
+        <v>906</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B242" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B243" t="s">
-        <v>828</v>
+        <v>918</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>642</v>
+        <v>304</v>
       </c>
       <c r="B244" t="s">
-        <v>829</v>
+        <v>919</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>484</v>
+        <v>305</v>
       </c>
       <c r="B245" t="s">
-        <v>620</v>
+        <v>828</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3">
+      <c r="A246" t="s">
+        <v>642</v>
+      </c>
+      <c r="B246" t="s">
+        <v>829</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>676</v>
+        <v>484</v>
       </c>
       <c r="B247" t="s">
-        <v>677</v>
-      </c>
-      <c r="C247" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="248" spans="1:3">
-      <c r="A248" t="s">
-        <v>501</v>
-      </c>
-      <c r="B248" t="s">
-        <v>504</v>
-      </c>
-      <c r="C248" t="s">
-        <v>531</v>
+        <v>620</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>502</v>
+        <v>676</v>
       </c>
       <c r="B249" t="s">
-        <v>503</v>
+        <v>677</v>
       </c>
       <c r="C249" t="s">
-        <v>532</v>
+        <v>629</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>530</v>
+        <v>501</v>
       </c>
       <c r="B250" t="s">
-        <v>544</v>
+        <v>504</v>
+      </c>
+      <c r="C250" t="s">
+        <v>531</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>322</v>
+        <v>502</v>
       </c>
       <c r="B251" t="s">
-        <v>308</v>
+        <v>503</v>
+      </c>
+      <c r="C251" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>323</v>
+        <v>530</v>
       </c>
       <c r="B252" t="s">
-        <v>309</v>
-      </c>
-      <c r="C252" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>463</v>
+        <v>322</v>
       </c>
       <c r="B253" t="s">
-        <v>519</v>
+        <v>308</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B254" t="s">
-        <v>310</v>
+        <v>309</v>
+      </c>
+      <c r="C254" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>325</v>
+        <v>463</v>
       </c>
       <c r="B255" t="s">
-        <v>311</v>
+        <v>519</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B256" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B257" t="s">
-        <v>313</v>
-      </c>
-      <c r="C257" t="s">
-        <v>533</v>
+        <v>311</v>
       </c>
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B258" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="B259" t="s">
-        <v>315</v>
+        <v>313</v>
+      </c>
+      <c r="C259" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B260" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="B261" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B262" t="s">
-        <v>318</v>
-      </c>
-      <c r="C262" t="s">
-        <v>533</v>
+        <v>316</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B263" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="B264" t="s">
-        <v>320</v>
+        <v>318</v>
+      </c>
+      <c r="C264" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B265" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>483</v>
+        <v>334</v>
       </c>
       <c r="B266" t="s">
-        <v>605</v>
+        <v>320</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3">
+      <c r="A267" t="s">
+        <v>335</v>
+      </c>
+      <c r="B267" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>548</v>
+        <v>483</v>
       </c>
       <c r="B268" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="269" spans="1:3">
-      <c r="A269" t="s">
-        <v>342</v>
-      </c>
-      <c r="B269" t="s">
-        <v>360</v>
+        <v>605</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>343</v>
+        <v>548</v>
       </c>
       <c r="B270" t="s">
-        <v>357</v>
+        <v>549</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B271" t="s">
-        <v>358</v>
-      </c>
-      <c r="C271" t="s">
-        <v>533</v>
+        <v>360</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>464</v>
+        <v>343</v>
       </c>
       <c r="B272" t="s">
-        <v>520</v>
+        <v>357</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>361</v>
+        <v>344</v>
       </c>
       <c r="B273" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C273" t="s">
         <v>533</v>
@@ -9805,134 +9814,134 @@
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>345</v>
+        <v>464</v>
       </c>
       <c r="B274" t="s">
-        <v>351</v>
+        <v>520</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B275" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="C275" t="s">
-        <v>510</v>
+        <v>533</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B276" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>348</v>
+        <v>362</v>
       </c>
       <c r="B277" t="s">
-        <v>354</v>
+        <v>352</v>
+      </c>
+      <c r="C277" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B278" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B279" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B280" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>482</v>
+        <v>349</v>
       </c>
       <c r="B281" t="s">
-        <v>621</v>
+        <v>356</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3">
+      <c r="A282" t="s">
+        <v>350</v>
+      </c>
+      <c r="B282" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>678</v>
+        <v>482</v>
       </c>
       <c r="B283" t="s">
-        <v>697</v>
-      </c>
-      <c r="C283" t="s">
-        <v>629</v>
+        <v>621</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="B285" t="s">
-        <v>675</v>
+        <v>697</v>
       </c>
       <c r="C285" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="286" spans="1:3">
-      <c r="A286" t="s">
-        <v>473</v>
-      </c>
-      <c r="B286" t="s">
-        <v>474</v>
-      </c>
-    </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>368</v>
+        <v>674</v>
       </c>
       <c r="B287" t="s">
-        <v>379</v>
+        <v>675</v>
+      </c>
+      <c r="C287" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>369</v>
+        <v>473</v>
       </c>
       <c r="B288" t="s">
-        <v>380</v>
-      </c>
-      <c r="C288" t="s">
-        <v>533</v>
+        <v>474</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>521</v>
+        <v>368</v>
       </c>
       <c r="B289" t="s">
-        <v>522</v>
+        <v>379</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B290" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C290" t="s">
         <v>533</v>
@@ -9940,139 +9949,139 @@
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>371</v>
+        <v>521</v>
       </c>
       <c r="B291" t="s">
-        <v>382</v>
-      </c>
-      <c r="C291" t="s">
-        <v>533</v>
+        <v>522</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B292" t="s">
-        <v>534</v>
+        <v>381</v>
+      </c>
+      <c r="C292" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="B293" t="s">
-        <v>383</v>
+        <v>382</v>
+      </c>
+      <c r="C293" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="B294" t="s">
-        <v>384</v>
+        <v>534</v>
       </c>
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B295" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B296" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="297" spans="1:3">
       <c r="A297" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B297" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="298" spans="1:3">
       <c r="A298" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="B298" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>733</v>
+        <v>377</v>
       </c>
       <c r="B299" t="s">
-        <v>734</v>
-      </c>
-      <c r="C299" t="s">
-        <v>629</v>
+        <v>387</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>480</v>
+        <v>378</v>
       </c>
       <c r="B300" t="s">
-        <v>622</v>
+        <v>388</v>
       </c>
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>557</v>
+        <v>733</v>
       </c>
       <c r="B301" t="s">
-        <v>558</v>
+        <v>734</v>
+      </c>
+      <c r="C301" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3">
+      <c r="A302" t="s">
+        <v>480</v>
+      </c>
+      <c r="B302" t="s">
+        <v>622</v>
       </c>
     </row>
     <row r="303" spans="1:3">
       <c r="A303" t="s">
-        <v>475</v>
+        <v>557</v>
       </c>
       <c r="B303" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="304" spans="1:3">
-      <c r="A304" t="s">
-        <v>395</v>
-      </c>
-      <c r="B304" t="s">
-        <v>406</v>
+        <v>558</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>396</v>
+        <v>475</v>
       </c>
       <c r="B305" t="s">
-        <v>407</v>
-      </c>
-      <c r="C305" t="s">
-        <v>533</v>
+        <v>474</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>465</v>
+        <v>395</v>
       </c>
       <c r="B306" t="s">
-        <v>523</v>
+        <v>406</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B307" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C307" t="s">
         <v>533</v>
@@ -10080,688 +10089,707 @@
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>398</v>
+        <v>465</v>
       </c>
       <c r="B308" t="s">
-        <v>409</v>
-      </c>
-      <c r="C308" t="s">
-        <v>533</v>
+        <v>523</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B309" t="s">
-        <v>535</v>
+        <v>408</v>
+      </c>
+      <c r="C309" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="B310" t="s">
-        <v>383</v>
+        <v>409</v>
+      </c>
+      <c r="C310" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="B311" t="s">
-        <v>384</v>
+        <v>535</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="B312" t="s">
-        <v>410</v>
+        <v>383</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="B313" t="s">
-        <v>411</v>
+        <v>384</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B314" t="s">
-        <v>387</v>
+        <v>410</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="B315" t="s">
-        <v>388</v>
+        <v>411</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>479</v>
+        <v>404</v>
       </c>
       <c r="B316" t="s">
-        <v>622</v>
+        <v>387</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>564</v>
+        <v>405</v>
       </c>
       <c r="B317" t="s">
-        <v>558</v>
+        <v>388</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3">
+      <c r="A318" t="s">
+        <v>479</v>
+      </c>
+      <c r="B318" t="s">
+        <v>622</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>672</v>
+        <v>564</v>
       </c>
       <c r="B319" t="s">
-        <v>673</v>
-      </c>
-      <c r="C319" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="320" spans="1:3">
-      <c r="A320" t="s">
-        <v>389</v>
-      </c>
-      <c r="B320" t="s">
-        <v>565</v>
+        <v>558</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
-        <v>390</v>
+        <v>672</v>
       </c>
       <c r="B321" t="s">
-        <v>566</v>
+        <v>673</v>
       </c>
       <c r="C321" t="s">
-        <v>533</v>
+        <v>629</v>
       </c>
     </row>
     <row r="322" spans="1:3">
       <c r="A322" t="s">
-        <v>466</v>
+        <v>389</v>
       </c>
       <c r="B322" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="323" spans="1:3">
       <c r="A323" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="B323" t="s">
-        <v>592</v>
+        <v>566</v>
+      </c>
+      <c r="C323" t="s">
+        <v>533</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>392</v>
+        <v>466</v>
       </c>
       <c r="B324" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="B325" t="s">
-        <v>569</v>
+        <v>592</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
-        <v>478</v>
+        <v>392</v>
       </c>
       <c r="B326" t="s">
-        <v>623</v>
+        <v>568</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3">
+      <c r="A327" t="s">
+        <v>393</v>
+      </c>
+      <c r="B327" t="s">
+        <v>569</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
+        <v>478</v>
+      </c>
+      <c r="B328" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3">
+      <c r="A330" t="s">
         <v>749</v>
       </c>
-      <c r="B328" t="s">
+      <c r="B330" t="s">
         <v>750</v>
       </c>
-      <c r="C328" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="329" spans="1:3">
-      <c r="A329" t="s">
-        <v>751</v>
-      </c>
-      <c r="B329" t="s">
-        <v>752</v>
-      </c>
-      <c r="C329" t="s">
+      <c r="C330" t="s">
         <v>629</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>758</v>
+        <v>751</v>
       </c>
       <c r="B331" t="s">
-        <v>759</v>
-      </c>
-    </row>
-    <row r="332" spans="1:3">
-      <c r="A332" t="s">
-        <v>760</v>
-      </c>
-      <c r="B332" t="s">
-        <v>761</v>
+        <v>752</v>
+      </c>
+      <c r="C331" t="s">
+        <v>629</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>762</v>
+        <v>758</v>
       </c>
       <c r="B333" t="s">
-        <v>763</v>
+        <v>759</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>764</v>
+        <v>760</v>
       </c>
       <c r="B334" t="s">
-        <v>765</v>
+        <v>761</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="B335" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="B336" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="A337" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="B337" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="A338" t="s">
-        <v>772</v>
+        <v>768</v>
       </c>
       <c r="B338" t="s">
-        <v>773</v>
+        <v>769</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="A339" t="s">
-        <v>774</v>
+        <v>770</v>
       </c>
       <c r="B339" t="s">
-        <v>775</v>
+        <v>771</v>
       </c>
     </row>
     <row r="340" spans="1:2">
       <c r="A340" t="s">
-        <v>776</v>
+        <v>772</v>
       </c>
       <c r="B340" t="s">
-        <v>777</v>
+        <v>773</v>
       </c>
     </row>
     <row r="341" spans="1:2">
       <c r="A341" t="s">
-        <v>778</v>
+        <v>774</v>
       </c>
       <c r="B341" t="s">
-        <v>779</v>
+        <v>775</v>
       </c>
     </row>
     <row r="342" spans="1:2">
       <c r="A342" t="s">
-        <v>780</v>
+        <v>776</v>
       </c>
       <c r="B342" t="s">
-        <v>781</v>
+        <v>777</v>
       </c>
     </row>
     <row r="343" spans="1:2">
       <c r="A343" t="s">
-        <v>782</v>
+        <v>778</v>
       </c>
       <c r="B343" t="s">
-        <v>783</v>
+        <v>779</v>
       </c>
     </row>
     <row r="344" spans="1:2">
       <c r="A344" t="s">
-        <v>784</v>
+        <v>780</v>
       </c>
       <c r="B344" t="s">
-        <v>785</v>
+        <v>781</v>
       </c>
     </row>
     <row r="345" spans="1:2">
       <c r="A345" t="s">
-        <v>786</v>
+        <v>782</v>
       </c>
       <c r="B345" t="s">
-        <v>787</v>
+        <v>783</v>
       </c>
     </row>
     <row r="346" spans="1:2">
       <c r="A346" t="s">
-        <v>788</v>
+        <v>784</v>
       </c>
       <c r="B346" t="s">
-        <v>789</v>
+        <v>785</v>
       </c>
     </row>
     <row r="347" spans="1:2">
       <c r="A347" t="s">
-        <v>790</v>
+        <v>786</v>
       </c>
       <c r="B347" t="s">
-        <v>791</v>
+        <v>787</v>
       </c>
     </row>
     <row r="348" spans="1:2">
       <c r="A348" t="s">
-        <v>792</v>
+        <v>788</v>
       </c>
       <c r="B348" t="s">
-        <v>793</v>
+        <v>789</v>
+      </c>
+    </row>
+    <row r="349" spans="1:2">
+      <c r="A349" t="s">
+        <v>790</v>
+      </c>
+      <c r="B349" t="s">
+        <v>791</v>
       </c>
     </row>
     <row r="350" spans="1:2">
       <c r="A350" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="B350" t="s">
-        <v>795</v>
-      </c>
-    </row>
-    <row r="351" spans="1:2">
-      <c r="A351" t="s">
-        <v>796</v>
-      </c>
-      <c r="B351" t="s">
-        <v>797</v>
+        <v>793</v>
       </c>
     </row>
     <row r="352" spans="1:2">
       <c r="A352" t="s">
-        <v>798</v>
+        <v>794</v>
       </c>
       <c r="B352" t="s">
-        <v>799</v>
+        <v>795</v>
       </c>
     </row>
     <row r="353" spans="1:2">
       <c r="A353" t="s">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="B353" t="s">
-        <v>801</v>
+        <v>797</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>802</v>
+        <v>798</v>
       </c>
       <c r="B354" t="s">
-        <v>803</v>
+        <v>799</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>804</v>
+        <v>800</v>
       </c>
       <c r="B355" t="s">
-        <v>805</v>
+        <v>801</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>806</v>
+        <v>802</v>
       </c>
       <c r="B356" t="s">
-        <v>807</v>
+        <v>803</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
-        <v>808</v>
+        <v>804</v>
       </c>
       <c r="B357" t="s">
-        <v>321</v>
+        <v>805</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
       <c r="B358" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
       <c r="B359" t="s">
-        <v>812</v>
+        <v>321</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>813</v>
+        <v>809</v>
       </c>
       <c r="B360" t="s">
-        <v>814</v>
+        <v>810</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>815</v>
+        <v>811</v>
       </c>
       <c r="B361" t="s">
-        <v>816</v>
+        <v>812</v>
+      </c>
+    </row>
+    <row r="362" spans="1:2">
+      <c r="A362" t="s">
+        <v>813</v>
+      </c>
+      <c r="B362" t="s">
+        <v>814</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="B363" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="364" spans="1:2">
-      <c r="A364" t="s">
-        <v>818</v>
-      </c>
-      <c r="B364" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
       <c r="B365" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="B366" t="s">
-        <v>317</v>
+        <v>819</v>
+      </c>
+    </row>
+    <row r="367" spans="1:2">
+      <c r="A367" t="s">
+        <v>820</v>
+      </c>
+      <c r="B367" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>846</v>
+        <v>821</v>
       </c>
       <c r="B368" t="s">
-        <v>847</v>
-      </c>
-    </row>
-    <row r="369" spans="1:2">
-      <c r="A369" t="s">
-        <v>845</v>
-      </c>
-      <c r="B369" t="s">
-        <v>844</v>
+        <v>317</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>838</v>
+        <v>846</v>
       </c>
       <c r="B370" t="s">
-        <v>839</v>
+        <v>847</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>836</v>
+        <v>845</v>
       </c>
       <c r="B371" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="B372" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
     </row>
     <row r="373" spans="1:2">
       <c r="A373" t="s">
-        <v>843</v>
+        <v>836</v>
       </c>
       <c r="B373" t="s">
-        <v>842</v>
+        <v>840</v>
+      </c>
+    </row>
+    <row r="374" spans="1:2">
+      <c r="A374" t="s">
+        <v>837</v>
+      </c>
+      <c r="B374" t="s">
+        <v>841</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>850</v>
+        <v>843</v>
       </c>
       <c r="B375" t="s">
-        <v>855</v>
-      </c>
-    </row>
-    <row r="376" spans="1:2">
-      <c r="A376" t="s">
-        <v>858</v>
-      </c>
-      <c r="B376" t="s">
-        <v>856</v>
+        <v>842</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="B377" t="s">
-        <v>839</v>
+        <v>855</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="B378" t="s">
-        <v>840</v>
+        <v>856</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="B379" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="B380" t="s">
-        <v>857</v>
+        <v>840</v>
+      </c>
+    </row>
+    <row r="381" spans="1:2">
+      <c r="A381" t="s">
+        <v>853</v>
+      </c>
+      <c r="B381" t="s">
+        <v>841</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>864</v>
+        <v>854</v>
       </c>
       <c r="B382" t="s">
-        <v>865</v>
-      </c>
-    </row>
-    <row r="383" spans="1:2">
-      <c r="A383" t="s">
-        <v>866</v>
-      </c>
-      <c r="B383" t="s">
-        <v>867</v>
+        <v>857</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>868</v>
+        <v>864</v>
       </c>
       <c r="B384" t="s">
-        <v>717</v>
+        <v>865</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
-        <v>870</v>
+        <v>866</v>
       </c>
       <c r="B385" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>877</v>
+        <v>868</v>
       </c>
       <c r="B386" t="s">
-        <v>252</v>
+        <v>717</v>
       </c>
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>878</v>
+        <v>870</v>
       </c>
       <c r="B387" t="s">
-        <v>255</v>
+        <v>869</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="B388" t="s">
-        <v>871</v>
+        <v>252</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>882</v>
+        <v>878</v>
       </c>
       <c r="B389" t="s">
-        <v>872</v>
+        <v>255</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>883</v>
+        <v>879</v>
       </c>
       <c r="B390" t="s">
-        <v>260</v>
+        <v>871</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="B391" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="B392" t="s">
-        <v>874</v>
+        <v>260</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="B393" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="B394" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="B395" t="s">
-        <v>277</v>
+        <v>875</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="B396" t="s">
-        <v>281</v>
+        <v>876</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="B397" t="s">
-        <v>829</v>
+        <v>277</v>
       </c>
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>881</v>
+        <v>889</v>
       </c>
       <c r="B398" t="s">
-        <v>635</v>
+        <v>281</v>
       </c>
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
+        <v>890</v>
+      </c>
+      <c r="B399" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="400" spans="1:2">
+      <c r="A400" t="s">
+        <v>881</v>
+      </c>
+      <c r="B400" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="401" spans="1:2">
+      <c r="A401" t="s">
         <v>880</v>
       </c>
-      <c r="B399" t="s">
+      <c r="B401" t="s">
         <v>617</v>
       </c>
     </row>

</xml_diff>

<commit_message>
CSS workflow added and EV tested
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F76C44-90AE-4DD6-A743-85F407FE2AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86ADE0F1-BE37-448B-995B-A2DB5F7A767E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1158" uniqueCount="934">
   <si>
     <t>Name</t>
   </si>
@@ -2619,9 +2619,6 @@
     <t>HAB_NameAndAssetsinIAQ</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>HAB</t>
   </si>
   <si>
@@ -2836,6 +2833,15 @@
   </si>
   <si>
     <t>ASC_GA_RealPrptyValue</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>CSS</t>
+  </si>
+  <si>
+    <t>Certification of Student Status</t>
   </si>
 </sst>
 </file>
@@ -3293,7 +3299,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>859</v>
+        <v>931</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -3610,44 +3616,51 @@
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
+        <v>859</v>
+      </c>
+      <c r="B46" t="s">
         <v>860</v>
-      </c>
-      <c r="B46" t="s">
-        <v>861</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
+        <v>861</v>
+      </c>
+      <c r="B47" t="s">
         <v>862</v>
-      </c>
-      <c r="B47" t="s">
-        <v>863</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
+        <v>890</v>
+      </c>
+      <c r="B48" t="s">
         <v>891</v>
       </c>
-      <c r="B48" t="s">
-        <v>892</v>
-      </c>
-    </row>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
+    </row>
+    <row r="49" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A49" t="s">
+        <v>932</v>
+      </c>
+      <c r="B49" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="57" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="63" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>
@@ -7771,7 +7784,7 @@
         <v>741</v>
       </c>
       <c r="B24" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="C24" t="s">
         <v>629</v>
@@ -7779,10 +7792,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>892</v>
+      </c>
+      <c r="B25" t="s">
         <v>893</v>
-      </c>
-      <c r="B25" t="s">
-        <v>894</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -8397,10 +8410,10 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
+        <v>925</v>
+      </c>
+      <c r="B99" t="s">
         <v>926</v>
-      </c>
-      <c r="B99" t="s">
-        <v>927</v>
       </c>
     </row>
     <row r="100" spans="1:3">
@@ -8446,34 +8459,34 @@
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
+        <v>921</v>
+      </c>
+      <c r="B104" t="s">
         <v>922</v>
-      </c>
-      <c r="B104" t="s">
-        <v>923</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
+        <v>923</v>
+      </c>
+      <c r="B105" t="s">
         <v>924</v>
-      </c>
-      <c r="B105" t="s">
-        <v>925</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
+        <v>928</v>
+      </c>
+      <c r="B106" t="s">
         <v>929</v>
-      </c>
-      <c r="B106" t="s">
-        <v>930</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B107" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -8877,7 +8890,7 @@
         <v>593</v>
       </c>
       <c r="B160" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C160" t="s">
         <v>594</v>
@@ -8899,7 +8912,7 @@
         <v>753</v>
       </c>
       <c r="B162" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="C162" t="s">
         <v>629</v>
@@ -8910,7 +8923,7 @@
         <v>754</v>
       </c>
       <c r="B163" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C163" t="s">
         <v>629</v>
@@ -8932,7 +8945,7 @@
         <v>468</v>
       </c>
       <c r="B166" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -8962,7 +8975,7 @@
         <v>239</v>
       </c>
       <c r="B169" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C169" t="s">
         <v>533</v>
@@ -8973,7 +8986,7 @@
         <v>240</v>
       </c>
       <c r="B170" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -8981,7 +8994,7 @@
         <v>248</v>
       </c>
       <c r="B171" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C171" t="s">
         <v>591</v>
@@ -8992,7 +9005,7 @@
         <v>719</v>
       </c>
       <c r="B172" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="C172" t="s">
         <v>629</v>
@@ -9019,7 +9032,7 @@
         <v>243</v>
       </c>
       <c r="B175" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -9027,7 +9040,7 @@
         <v>244</v>
       </c>
       <c r="B176" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -9035,7 +9048,7 @@
         <v>245</v>
       </c>
       <c r="B177" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -9043,7 +9056,7 @@
         <v>246</v>
       </c>
       <c r="B178" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
     </row>
     <row r="179" spans="1:3">
@@ -9059,7 +9072,7 @@
         <v>279</v>
       </c>
       <c r="B180" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -9110,10 +9123,10 @@
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
+        <v>919</v>
+      </c>
+      <c r="B186" t="s">
         <v>920</v>
-      </c>
-      <c r="B186" t="s">
-        <v>921</v>
       </c>
     </row>
     <row r="187" spans="1:3">
@@ -9140,7 +9153,7 @@
         <v>469</v>
       </c>
       <c r="B190" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -9148,7 +9161,7 @@
         <v>249</v>
       </c>
       <c r="B191" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="C191" t="s">
         <v>599</v>
@@ -9159,7 +9172,7 @@
         <v>251</v>
       </c>
       <c r="B192" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="C192" t="s">
         <v>633</v>
@@ -9170,7 +9183,7 @@
         <v>250</v>
       </c>
       <c r="B193" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -9213,7 +9226,7 @@
         <v>258</v>
       </c>
       <c r="B198" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="199" spans="1:3">
@@ -9229,7 +9242,7 @@
         <v>264</v>
       </c>
       <c r="B200" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="201" spans="1:3">
@@ -9237,7 +9250,7 @@
         <v>265</v>
       </c>
       <c r="B201" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="202" spans="1:3">
@@ -9245,7 +9258,7 @@
         <v>266</v>
       </c>
       <c r="B202" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="C202" t="s">
         <v>599</v>
@@ -9256,7 +9269,7 @@
         <v>267</v>
       </c>
       <c r="B203" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -9264,7 +9277,7 @@
         <v>268</v>
       </c>
       <c r="B204" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="C204" t="s">
         <v>599</v>
@@ -9275,7 +9288,7 @@
         <v>269</v>
       </c>
       <c r="B205" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="206" spans="1:3">
@@ -9291,7 +9304,7 @@
         <v>278</v>
       </c>
       <c r="B207" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="208" spans="1:3">
@@ -9494,7 +9507,7 @@
         <v>472</v>
       </c>
       <c r="B235" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
     </row>
     <row r="236" spans="1:3">
@@ -9521,7 +9534,7 @@
         <v>298</v>
       </c>
       <c r="B238" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="C238" t="s">
         <v>533</v>
@@ -9532,7 +9545,7 @@
         <v>299</v>
       </c>
       <c r="B239" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
     </row>
     <row r="240" spans="1:3">
@@ -9540,7 +9553,7 @@
         <v>455</v>
       </c>
       <c r="B240" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
     </row>
     <row r="241" spans="1:3">
@@ -9548,7 +9561,7 @@
         <v>301</v>
       </c>
       <c r="B241" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
     </row>
     <row r="242" spans="1:3">
@@ -9556,7 +9569,7 @@
         <v>302</v>
       </c>
       <c r="B242" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
     </row>
     <row r="243" spans="1:3">
@@ -9564,7 +9577,7 @@
         <v>303</v>
       </c>
       <c r="B243" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
     </row>
     <row r="244" spans="1:3">
@@ -9572,7 +9585,7 @@
         <v>304</v>
       </c>
       <c r="B244" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
     </row>
     <row r="245" spans="1:3">
@@ -10651,23 +10664,23 @@
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
+        <v>863</v>
+      </c>
+      <c r="B384" t="s">
         <v>864</v>
-      </c>
-      <c r="B384" t="s">
-        <v>865</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
+        <v>865</v>
+      </c>
+      <c r="B385" t="s">
         <v>866</v>
-      </c>
-      <c r="B385" t="s">
-        <v>867</v>
       </c>
     </row>
     <row r="386" spans="1:2">
       <c r="A386" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="B386" t="s">
         <v>717</v>
@@ -10675,15 +10688,15 @@
     </row>
     <row r="387" spans="1:2">
       <c r="A387" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="B387" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="B388" t="s">
         <v>252</v>
@@ -10691,7 +10704,7 @@
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="B389" t="s">
         <v>255</v>
@@ -10699,23 +10712,23 @@
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="B390" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
     </row>
     <row r="391" spans="1:2">
       <c r="A391" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="B391" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
     </row>
     <row r="392" spans="1:2">
       <c r="A392" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="B392" t="s">
         <v>260</v>
@@ -10723,39 +10736,39 @@
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="B393" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="B394" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="B395" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B396" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="B397" t="s">
         <v>277</v>
@@ -10763,7 +10776,7 @@
     </row>
     <row r="398" spans="1:2">
       <c r="A398" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="B398" t="s">
         <v>281</v>
@@ -10771,7 +10784,7 @@
     </row>
     <row r="399" spans="1:2">
       <c r="A399" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="B399" t="s">
         <v>829</v>
@@ -10779,7 +10792,7 @@
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="B400" t="s">
         <v>635</v>
@@ -10787,7 +10800,7 @@
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="B401" t="s">
         <v>617</v>

</xml_diff>

<commit_message>
updates to remove all DU workflows from performer, Code updates to RCV, IAQ
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86ADE0F1-BE37-448B-995B-A2DB5F7A767E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7522168-46FC-4AF1-AA2C-E4613CE95A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1158" uniqueCount="934">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="998">
   <si>
     <t>Name</t>
   </si>
@@ -2842,6 +2842,198 @@
   </si>
   <si>
     <t>Certification of Student Status</t>
+  </si>
+  <si>
+    <t>CSSExists</t>
+  </si>
+  <si>
+    <t>Certification of Student Status is missing from the application.</t>
+  </si>
+  <si>
+    <t>CSS_MoveInEffectiveDate</t>
+  </si>
+  <si>
+    <t>Move In Date and Effective Date do not match.</t>
+  </si>
+  <si>
+    <t>CSS_PropertyName</t>
+  </si>
+  <si>
+    <t>Property name is not populated on the Certification of Student Status.</t>
+  </si>
+  <si>
+    <t>CSS_GAID</t>
+  </si>
+  <si>
+    <t>GA ID is not populated on the Certification of Student Status.</t>
+  </si>
+  <si>
+    <t>CSS_HeadOfHousehold</t>
+  </si>
+  <si>
+    <t>Head of Household is not populated on the Certification of Student Status.</t>
+  </si>
+  <si>
+    <t>CSS_UnitNumber</t>
+  </si>
+  <si>
+    <t>Unit Number is not populated on the Certification of Student Status.</t>
+  </si>
+  <si>
+    <t>CSS_MoveInDate</t>
+  </si>
+  <si>
+    <t>Move In Date is not populated on the Certification of Student Status.</t>
+  </si>
+  <si>
+    <t>CSS_EffectiveDate</t>
+  </si>
+  <si>
+    <t>Effective Date is not populated on the Certification of Student Status.</t>
+  </si>
+  <si>
+    <t>CSS_Section1</t>
+  </si>
+  <si>
+    <t>Section One – Household Members and Status does not contain all household members.</t>
+  </si>
+  <si>
+    <t>CSS_ICWDOB</t>
+  </si>
+  <si>
+    <t>Date of Birth listed does not match the ICW for all household members.</t>
+  </si>
+  <si>
+    <t>CSS_ICWAge</t>
+  </si>
+  <si>
+    <t>Age listed does not match the ICW for all household members.</t>
+  </si>
+  <si>
+    <t>CSS_ICWStudentStatus</t>
+  </si>
+  <si>
+    <t>Student Status listed does not match the ICW for all household members.</t>
+  </si>
+  <si>
+    <t>CSS_PartTimeStudents</t>
+  </si>
+  <si>
+    <t>All household members are listed as Part-Time Students, but the Verified Checkbox has not been checked yes for all household members.</t>
+  </si>
+  <si>
+    <t>CSS_Graduate</t>
+  </si>
+  <si>
+    <t>Did anyone graduate during the calendar year question has not been answered appropriately.</t>
+  </si>
+  <si>
+    <t>CSS_FullTimeStudents</t>
+  </si>
+  <si>
+    <t>Are all residents of the household full-time students has not been answered appropriately.</t>
+  </si>
+  <si>
+    <t>CSS_HouseholdInitial</t>
+  </si>
+  <si>
+    <t>Documented that no household members are part of the original qualifying household. Manual review required.</t>
+  </si>
+  <si>
+    <t>CSS_FirstLineCheck</t>
+  </si>
+  <si>
+    <t>Not all adults have initialed the first line of Section Three – Signatures and Acknowledgements.</t>
+  </si>
+  <si>
+    <t>CSS_NotSigned</t>
+  </si>
+  <si>
+    <t>Not all adults have signed the Certification of Student Status.</t>
+  </si>
+  <si>
+    <t>CSS_NotDated</t>
+  </si>
+  <si>
+    <t>Not all adults have dated the Certification of Student Status.</t>
+  </si>
+  <si>
+    <t>CSS_CheckDateWithMoveIn</t>
+  </si>
+  <si>
+    <t>Dates on the Certification of Student Status are not within 120 days of the Move-In date.</t>
+  </si>
+  <si>
+    <t>CSS_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for the Certification of Student Status. Needs manual review.</t>
+  </si>
+  <si>
+    <t>RCV_SupportingDocInIAQ</t>
+  </si>
+  <si>
+    <t>Supporting documents have not been provided for Regular Contributions Verification documented on the Income &amp; Asset Questionnaire.</t>
+  </si>
+  <si>
+    <t>RCV_RecipientNameCheck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name listed on the Regular Contributions Verification and ICW do not match. </t>
+  </si>
+  <si>
+    <t>RCV_CheckDateWithMoveIn</t>
+  </si>
+  <si>
+    <t>Date listed on the Regular Contributions Verification is not within 120 days of Move-In date.</t>
+  </si>
+  <si>
+    <t>RCV_ContributorAmountCheck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contributor and Amount listed on the Regular Contributions Verification and ICW do not match. </t>
+  </si>
+  <si>
+    <t>RCV_RecipientSignCheck</t>
+  </si>
+  <si>
+    <t>Verification of Regular Contributions Verification has not been signed by recipient.</t>
+  </si>
+  <si>
+    <t>RCV_RecipientDateCheck</t>
+  </si>
+  <si>
+    <t>Verification of Regular Contributions Verification has not been dated appropriately by recipient.</t>
+  </si>
+  <si>
+    <t>RCV_ContributorSignCheck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verification of Regular Contributions Verification has not been signed by contributor. </t>
+  </si>
+  <si>
+    <t>RCV_ContributorDateCheck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regular Contributions Verification has not been dated appropriately by contributor. </t>
+  </si>
+  <si>
+    <t>RCV_FrequencyCheck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frequency of payments checkbox on the Regular Contributions Verification has not been documented appropriately. </t>
+  </si>
+  <si>
+    <t>RCV_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Regular Contributions Verification. Needs manual review.</t>
+  </si>
+  <si>
+    <t>RCV</t>
+  </si>
+  <si>
+    <t>Regular Contributions Verification</t>
   </si>
 </sst>
 </file>
@@ -2907,7 +3099,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -3646,7 +3849,14 @@
         <v>933</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="50" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A50" t="s">
+        <v>996</v>
+      </c>
+      <c r="B50" t="s">
+        <v>997</v>
+      </c>
+    </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
@@ -7575,7 +7785,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C401"/>
+  <dimension ref="A1:C434"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -10806,7 +11016,258 @@
         <v>617</v>
       </c>
     </row>
+    <row r="403" spans="1:2">
+      <c r="A403" t="s">
+        <v>934</v>
+      </c>
+      <c r="B403" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="404" spans="1:2">
+      <c r="A404" t="s">
+        <v>936</v>
+      </c>
+      <c r="B404" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2">
+      <c r="A405" t="s">
+        <v>938</v>
+      </c>
+      <c r="B405" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="406" spans="1:2">
+      <c r="A406" t="s">
+        <v>940</v>
+      </c>
+      <c r="B406" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="407" spans="1:2">
+      <c r="A407" t="s">
+        <v>942</v>
+      </c>
+      <c r="B407" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="408" spans="1:2">
+      <c r="A408" t="s">
+        <v>944</v>
+      </c>
+      <c r="B408" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="409" spans="1:2">
+      <c r="A409" t="s">
+        <v>946</v>
+      </c>
+      <c r="B409" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="410" spans="1:2">
+      <c r="A410" t="s">
+        <v>948</v>
+      </c>
+      <c r="B410" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="411" spans="1:2">
+      <c r="A411" t="s">
+        <v>950</v>
+      </c>
+      <c r="B411" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="412" spans="1:2">
+      <c r="A412" t="s">
+        <v>952</v>
+      </c>
+      <c r="B412" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="413" spans="1:2">
+      <c r="A413" t="s">
+        <v>954</v>
+      </c>
+      <c r="B413" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="414" spans="1:2">
+      <c r="A414" t="s">
+        <v>956</v>
+      </c>
+      <c r="B414" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="415" spans="1:2">
+      <c r="A415" t="s">
+        <v>958</v>
+      </c>
+      <c r="B415" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="416" spans="1:2">
+      <c r="A416" t="s">
+        <v>960</v>
+      </c>
+      <c r="B416" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="417" spans="1:2">
+      <c r="A417" t="s">
+        <v>962</v>
+      </c>
+      <c r="B417" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="418" spans="1:2">
+      <c r="A418" t="s">
+        <v>964</v>
+      </c>
+      <c r="B418" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="419" spans="1:2">
+      <c r="A419" t="s">
+        <v>966</v>
+      </c>
+      <c r="B419" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="420" spans="1:2">
+      <c r="A420" t="s">
+        <v>968</v>
+      </c>
+      <c r="B420" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="421" spans="1:2">
+      <c r="A421" t="s">
+        <v>970</v>
+      </c>
+      <c r="B421" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="422" spans="1:2">
+      <c r="A422" t="s">
+        <v>972</v>
+      </c>
+      <c r="B422" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="423" spans="1:2">
+      <c r="A423" t="s">
+        <v>974</v>
+      </c>
+      <c r="B423" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="425" spans="1:2">
+      <c r="A425" t="s">
+        <v>976</v>
+      </c>
+      <c r="B425" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="426" spans="1:2">
+      <c r="A426" t="s">
+        <v>978</v>
+      </c>
+      <c r="B426" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="427" spans="1:2">
+      <c r="A427" t="s">
+        <v>980</v>
+      </c>
+      <c r="B427" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="428" spans="1:2">
+      <c r="A428" t="s">
+        <v>982</v>
+      </c>
+      <c r="B428" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="429" spans="1:2">
+      <c r="A429" t="s">
+        <v>984</v>
+      </c>
+      <c r="B429" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="430" spans="1:2">
+      <c r="A430" t="s">
+        <v>986</v>
+      </c>
+      <c r="B430" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="431" spans="1:2">
+      <c r="A431" t="s">
+        <v>988</v>
+      </c>
+      <c r="B431" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="432" spans="1:2">
+      <c r="A432" t="s">
+        <v>990</v>
+      </c>
+      <c r="B432" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="433" spans="1:2">
+      <c r="A433" t="s">
+        <v>992</v>
+      </c>
+      <c r="B433" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="434" spans="1:2">
+      <c r="A434" t="s">
+        <v>994</v>
+      </c>
+      <c r="B434" t="s">
+        <v>995</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="A425:A434">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update to libraries and any dependency issues
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7522168-46FC-4AF1-AA2C-E4613CE95A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A809A62-166D-4351-B6DF-DEF4F806EA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -2835,9 +2835,6 @@
     <t>ASC_GA_RealPrptyValue</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>CSS</t>
   </si>
   <si>
@@ -3034,6 +3031,9 @@
   </si>
   <si>
     <t>Regular Contributions Verification</t>
+  </si>
+  <si>
+    <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3502,7 +3502,7 @@
         <v>206</v>
       </c>
       <c r="B7" t="s">
-        <v>931</v>
+        <v>997</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -3843,18 +3843,18 @@
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" t="s">
+        <v>931</v>
+      </c>
+      <c r="B49" t="s">
         <v>932</v>
-      </c>
-      <c r="B49" t="s">
-        <v>933</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" t="s">
+        <v>995</v>
+      </c>
+      <c r="B50" t="s">
         <v>996</v>
-      </c>
-      <c r="B50" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
@@ -11018,250 +11018,250 @@
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
+        <v>933</v>
+      </c>
+      <c r="B403" t="s">
         <v>934</v>
-      </c>
-      <c r="B403" t="s">
-        <v>935</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
+        <v>935</v>
+      </c>
+      <c r="B404" t="s">
         <v>936</v>
-      </c>
-      <c r="B404" t="s">
-        <v>937</v>
       </c>
     </row>
     <row r="405" spans="1:2">
       <c r="A405" t="s">
+        <v>937</v>
+      </c>
+      <c r="B405" t="s">
         <v>938</v>
-      </c>
-      <c r="B405" t="s">
-        <v>939</v>
       </c>
     </row>
     <row r="406" spans="1:2">
       <c r="A406" t="s">
+        <v>939</v>
+      </c>
+      <c r="B406" t="s">
         <v>940</v>
-      </c>
-      <c r="B406" t="s">
-        <v>941</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
+        <v>941</v>
+      </c>
+      <c r="B407" t="s">
         <v>942</v>
-      </c>
-      <c r="B407" t="s">
-        <v>943</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
+        <v>943</v>
+      </c>
+      <c r="B408" t="s">
         <v>944</v>
-      </c>
-      <c r="B408" t="s">
-        <v>945</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
+        <v>945</v>
+      </c>
+      <c r="B409" t="s">
         <v>946</v>
-      </c>
-      <c r="B409" t="s">
-        <v>947</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
+        <v>947</v>
+      </c>
+      <c r="B410" t="s">
         <v>948</v>
-      </c>
-      <c r="B410" t="s">
-        <v>949</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
+        <v>949</v>
+      </c>
+      <c r="B411" t="s">
         <v>950</v>
-      </c>
-      <c r="B411" t="s">
-        <v>951</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
+        <v>951</v>
+      </c>
+      <c r="B412" t="s">
         <v>952</v>
-      </c>
-      <c r="B412" t="s">
-        <v>953</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
+        <v>953</v>
+      </c>
+      <c r="B413" t="s">
         <v>954</v>
-      </c>
-      <c r="B413" t="s">
-        <v>955</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
+        <v>955</v>
+      </c>
+      <c r="B414" t="s">
         <v>956</v>
-      </c>
-      <c r="B414" t="s">
-        <v>957</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
+        <v>957</v>
+      </c>
+      <c r="B415" t="s">
         <v>958</v>
-      </c>
-      <c r="B415" t="s">
-        <v>959</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
+        <v>959</v>
+      </c>
+      <c r="B416" t="s">
         <v>960</v>
-      </c>
-      <c r="B416" t="s">
-        <v>961</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
+        <v>961</v>
+      </c>
+      <c r="B417" t="s">
         <v>962</v>
-      </c>
-      <c r="B417" t="s">
-        <v>963</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
+        <v>963</v>
+      </c>
+      <c r="B418" t="s">
         <v>964</v>
-      </c>
-      <c r="B418" t="s">
-        <v>965</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
+        <v>965</v>
+      </c>
+      <c r="B419" t="s">
         <v>966</v>
-      </c>
-      <c r="B419" t="s">
-        <v>967</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
+        <v>967</v>
+      </c>
+      <c r="B420" t="s">
         <v>968</v>
-      </c>
-      <c r="B420" t="s">
-        <v>969</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
+        <v>969</v>
+      </c>
+      <c r="B421" t="s">
         <v>970</v>
-      </c>
-      <c r="B421" t="s">
-        <v>971</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
+        <v>971</v>
+      </c>
+      <c r="B422" t="s">
         <v>972</v>
-      </c>
-      <c r="B422" t="s">
-        <v>973</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
+        <v>973</v>
+      </c>
+      <c r="B423" t="s">
         <v>974</v>
-      </c>
-      <c r="B423" t="s">
-        <v>975</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
+        <v>975</v>
+      </c>
+      <c r="B425" t="s">
         <v>976</v>
-      </c>
-      <c r="B425" t="s">
-        <v>977</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
+        <v>977</v>
+      </c>
+      <c r="B426" t="s">
         <v>978</v>
-      </c>
-      <c r="B426" t="s">
-        <v>979</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
+        <v>979</v>
+      </c>
+      <c r="B427" t="s">
         <v>980</v>
-      </c>
-      <c r="B427" t="s">
-        <v>981</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
+        <v>981</v>
+      </c>
+      <c r="B428" t="s">
         <v>982</v>
-      </c>
-      <c r="B428" t="s">
-        <v>983</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
+        <v>983</v>
+      </c>
+      <c r="B429" t="s">
         <v>984</v>
-      </c>
-      <c r="B429" t="s">
-        <v>985</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
+        <v>985</v>
+      </c>
+      <c r="B430" t="s">
         <v>986</v>
-      </c>
-      <c r="B430" t="s">
-        <v>987</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
+        <v>987</v>
+      </c>
+      <c r="B431" t="s">
         <v>988</v>
-      </c>
-      <c r="B431" t="s">
-        <v>989</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
+        <v>989</v>
+      </c>
+      <c r="B432" t="s">
         <v>990</v>
-      </c>
-      <c r="B432" t="s">
-        <v>991</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
+        <v>991</v>
+      </c>
+      <c r="B433" t="s">
         <v>992</v>
-      </c>
-      <c r="B433" t="s">
-        <v>993</v>
       </c>
     </row>
     <row r="434" spans="1:2">
       <c r="A434" t="s">
+        <v>993</v>
+      </c>
+      <c r="B434" t="s">
         <v>994</v>
-      </c>
-      <c r="B434" t="s">
-        <v>995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to AS in library, and also Yardi Libraries to resolve I am Back prompt
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A809A62-166D-4351-B6DF-DEF4F806EA11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBC45A6-C6CB-4DFE-A437-8B62E2842455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1222" uniqueCount="998">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="1001">
   <si>
     <t>Name</t>
   </si>
@@ -3034,6 +3034,15 @@
   </si>
   <si>
     <t>C:\Users\Harika.Malyala\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>ShortTimeDelay</t>
+  </si>
+  <si>
+    <t>MediumTimeDelay</t>
+  </si>
+  <si>
+    <t>LongTimeDelay</t>
   </si>
 </sst>
 </file>
@@ -6807,9 +6816,30 @@
         <v>714</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="45" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="46" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="44" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A44" t="s">
+        <v>998</v>
+      </c>
+      <c r="B44" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A45" t="s">
+        <v>999</v>
+      </c>
+      <c r="B45" t="s">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A46" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B46" t="s">
+        <v>1000</v>
+      </c>
+    </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Updates to Parallel processing to handle erroor in parallel process
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBC45A6-C6CB-4DFE-A437-8B62E2842455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB92BE8-E7F2-42B2-8EDA-3DE7CF9C585D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1228" uniqueCount="1001">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1230" uniqueCount="1002">
   <si>
     <t>Name</t>
   </si>
@@ -3043,6 +3043,9 @@
   </si>
   <si>
     <t>LongTimeDelay</t>
+  </si>
+  <si>
+    <t>DU_TimeOut</t>
   </si>
 </sst>
 </file>
@@ -6840,7 +6843,14 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="47" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A47" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1001</v>
+      </c>
+    </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>
     <row r="50" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Upadtes for ICW, CSS, HAB Business checks
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CB92BE8-E7F2-42B2-8EDA-3DE7CF9C585D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFABEDC6-390A-4207-A6EB-851F5D30249E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1230" uniqueCount="1002">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1307" uniqueCount="1077">
   <si>
     <t>Name</t>
   </si>
@@ -3046,6 +3046,231 @@
   </si>
   <si>
     <t>DU_TimeOut</t>
+  </si>
+  <si>
+    <t>BSExists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank Statements are present in the application, manual review required. </t>
+  </si>
+  <si>
+    <t>BS_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Bank Statements. Needs manual review.</t>
+  </si>
+  <si>
+    <t>LESExists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leave and Earnings Statement is present in the application, manual review required. </t>
+  </si>
+  <si>
+    <t>LES_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Leave and Earnings Statement. Needs manual review.</t>
+  </si>
+  <si>
+    <t>VABL_CheckDateMoveIn</t>
+  </si>
+  <si>
+    <t>Date on the Veterans Affairs Benefit Letter is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>VABL_ICWCheck</t>
+  </si>
+  <si>
+    <t>Gross Benefit Amount listed on the Veterans Affairs Benefit Letter does not match the $/Period on the ICW. </t>
+  </si>
+  <si>
+    <t>VABL_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Veterans Affairs Benefits Letter. Manual review required.</t>
+  </si>
+  <si>
+    <t>RCFExists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Release and Consent for is missing from the application. </t>
+  </si>
+  <si>
+    <t>RCF_ApplicantName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All adults have not been listed on the Applicant/Resident Name line of the Release and Consent Form. </t>
+  </si>
+  <si>
+    <t>RCF_WeLine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All adults have not been listed on the I/We line of the Release and Consent Form. </t>
+  </si>
+  <si>
+    <t>RCF_Signed</t>
+  </si>
+  <si>
+    <t>Not all adults have signed the Release and Consent Form.  </t>
+  </si>
+  <si>
+    <t>RCF_Dated</t>
+  </si>
+  <si>
+    <t>Not all adults have dated the Release and Consent Form.  </t>
+  </si>
+  <si>
+    <t>RCF_DateCheckMoveIn</t>
+  </si>
+  <si>
+    <t>Date on the Release and Consent Form is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>RCF_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Release and Consent Form. Needs manual review. </t>
+  </si>
+  <si>
+    <t>TRRG_HeadOfHousehold</t>
+  </si>
+  <si>
+    <t>Household name listed on the Tenant Rights and Resource Guide (TRRG) does not match the Head of Household listed on the ICW. </t>
+  </si>
+  <si>
+    <t>TRRG_UnitNumber</t>
+  </si>
+  <si>
+    <t>Unit Number listed on the Tenant Rights and Resource Guide (TRRG) does not match the Unit Number listed on the Application Summary. </t>
+  </si>
+  <si>
+    <t>TRRG_Signed</t>
+  </si>
+  <si>
+    <t>All adults have not signed the Tenant Rights and Resource Guide (TRRG). </t>
+  </si>
+  <si>
+    <t>TRRG_Dated</t>
+  </si>
+  <si>
+    <t>All adults have not dated the Tenant Rights and Resource Guide (TRRG). </t>
+  </si>
+  <si>
+    <t>TRRG_CheckDateMoveIn</t>
+  </si>
+  <si>
+    <t>Date on the Tenant Rights and Resource Guide (TRRG) is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>TRRG_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for the Tenant Rights and Resource Guide (TRRG). Manual review required. </t>
+  </si>
+  <si>
+    <t>TSAHCExists</t>
+  </si>
+  <si>
+    <t>TSAHC document is missing from the application, and it is a required document for this property. </t>
+  </si>
+  <si>
+    <t>TSAHC_PropertyName</t>
+  </si>
+  <si>
+    <t>Property name listed on the TSAHC does not match the property listed on the Application Summary. </t>
+  </si>
+  <si>
+    <t>TSAHC_Signed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The TSAHC has not been signed. </t>
+  </si>
+  <si>
+    <t>TSAHC_Dated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The TSAHC has not been dated. </t>
+  </si>
+  <si>
+    <t>TSAHC_CheckDateMoveIn</t>
+  </si>
+  <si>
+    <t>The date on the TSAHC is not within 120 days of the move-in date. </t>
+  </si>
+  <si>
+    <t>TSAHC_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for the TSAHC. Manual review required. </t>
+  </si>
+  <si>
+    <t>VSAExists</t>
+  </si>
+  <si>
+    <t>Verification Services (Assets) is missing from the application and this property requires asset verification. Manual review required.</t>
+  </si>
+  <si>
+    <t>VSA_AssetAccount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asset Account Type listed on Verification Services does not match the ICW. </t>
+  </si>
+  <si>
+    <t>VSA_ICWInstitutionName</t>
+  </si>
+  <si>
+    <t>Asset Institution Name listed on Verification Services does not match the ICW. </t>
+  </si>
+  <si>
+    <t>VSA_ICWCurrentBalance</t>
+  </si>
+  <si>
+    <t>Asset Current Balance listed on Verification Services does not match the ICW. </t>
+  </si>
+  <si>
+    <t>VSA_FindingError</t>
+  </si>
+  <si>
+    <t>Unable to validate findings for Verification Services. Needs manual review. </t>
+  </si>
+  <si>
+    <t>BS</t>
+  </si>
+  <si>
+    <t>Bank Statements</t>
+  </si>
+  <si>
+    <t>LES</t>
+  </si>
+  <si>
+    <t>Leave and Earnings Statement</t>
+  </si>
+  <si>
+    <t>VABL</t>
+  </si>
+  <si>
+    <t>Veterans Benefits Letter</t>
+  </si>
+  <si>
+    <t>RCF</t>
+  </si>
+  <si>
+    <t>Release and Consent Form</t>
+  </si>
+  <si>
+    <t>TRRG</t>
+  </si>
+  <si>
+    <t>A Tenant Rights and Resource Guide (TRRG)</t>
+  </si>
+  <si>
+    <t>TSAHC</t>
+  </si>
+  <si>
+    <t>VSA</t>
+  </si>
+  <si>
+    <t>Verification Services (Assets)</t>
   </si>
 </sst>
 </file>
@@ -3111,7 +3336,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3853,7 +4088,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="49" spans="1:2" ht="14.25" customHeight="1">
+    <row r="49" spans="1:3" ht="14.25" customHeight="1">
       <c r="A49" t="s">
         <v>931</v>
       </c>
@@ -3861,7 +4096,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="14.25" customHeight="1">
+    <row r="50" spans="1:3" ht="14.25" customHeight="1">
       <c r="A50" t="s">
         <v>995</v>
       </c>
@@ -3869,20 +4104,72 @@
         <v>996</v>
       </c>
     </row>
-    <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="62" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="63" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="51" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A51" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B51" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A52" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A53" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A54" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A55" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A56" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A57" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B57" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="61" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="63" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="64" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>
@@ -7825,7 +8112,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C434"/>
+  <dimension ref="A1:C472"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -11304,8 +11591,259 @@
         <v>994</v>
       </c>
     </row>
+    <row r="436" spans="1:2">
+      <c r="A436" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B436" t="s">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="437" spans="1:2">
+      <c r="A437" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B437" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="439" spans="1:2">
+      <c r="A439" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B439" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="440" spans="1:2">
+      <c r="A440" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B440" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="442" spans="1:2">
+      <c r="A442" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B442" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="443" spans="1:2">
+      <c r="A443" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B443" t="s">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="444" spans="1:2">
+      <c r="A444" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B444" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="446" spans="1:2">
+      <c r="A446" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B446" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="447" spans="1:2">
+      <c r="A447" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B447" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="448" spans="1:2">
+      <c r="A448" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B448" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="449" spans="1:2">
+      <c r="A449" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B449" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="450" spans="1:2">
+      <c r="A450" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B450" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="451" spans="1:2">
+      <c r="A451" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B451" t="s">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="452" spans="1:2">
+      <c r="A452" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B452" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="454" spans="1:2">
+      <c r="A454" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B454" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="455" spans="1:2">
+      <c r="A455" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B455" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2">
+      <c r="A456" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B456" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2">
+      <c r="A457" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B457" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2">
+      <c r="A458" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B458" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2">
+      <c r="A459" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B459" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2">
+      <c r="A461" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B461" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2">
+      <c r="A462" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B462" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="463" spans="1:2">
+      <c r="A463" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B463" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="464" spans="1:2">
+      <c r="A464" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B464" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="465" spans="1:2">
+      <c r="A465" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B465" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2">
+      <c r="A466" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B466" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2">
+      <c r="A468" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B468" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="469" spans="1:2">
+      <c r="A469" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B469" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2">
+      <c r="A470" t="s">
+        <v>1058</v>
+      </c>
+      <c r="B470" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="471" spans="1:2">
+      <c r="A471" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B471" t="s">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="472" spans="1:2">
+      <c r="A472" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B472" t="s">
+        <v>1063</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A425:A434">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A442:A443 A439:A440 A436:A437">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated library for ICW
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFABEDC6-390A-4207-A6EB-851F5D30249E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3496164A-B55F-4F2A-B1BC-AA50A5293085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="10620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added the logic to VSA flow to be checked only for some of the properties
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0196D4-446A-4545-9EEA-9640A7B67A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CD990D-C65E-4DF2-BEB1-C0B3F692DC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17760" uniqueCount="1151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17762" uniqueCount="1152">
   <si>
     <t>Name</t>
   </si>
@@ -3459,9 +3459,6 @@
     <t>Unable to validate findings for Child Support Calcs. Needs manual review.</t>
   </si>
   <si>
-    <t>C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Regular Contributions Verification has not been signed by recipient.</t>
   </si>
   <si>
@@ -3493,6 +3490,12 @@
   </si>
   <si>
     <t>LLM_Classification_RetryCount</t>
+  </si>
+  <si>
+    <t>TX_VSACheck</t>
+  </si>
+  <si>
+    <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
   </si>
 </sst>
 </file>
@@ -3971,7 +3974,7 @@
         <v>204</v>
       </c>
       <c r="B7" t="s">
-        <v>1139</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4382,15 +4385,15 @@
         <v>1064</v>
       </c>
       <c r="B57" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1">
       <c r="A58" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="B58" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1"/>
@@ -7161,10 +7164,10 @@
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="B22" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
@@ -7375,22 +7378,29 @@
         <v>990</v>
       </c>
     </row>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
+    <row r="49" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A49" t="s">
+        <v>1150</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="57" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="60" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="63" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>
@@ -8558,7 +8568,7 @@
         <v>737</v>
       </c>
       <c r="B24" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="C24" t="s">
         <v>626</v>
@@ -58870,7 +58880,7 @@
     </row>
     <row r="166" spans="1:3">
       <c r="A166" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="B166" t="s">
         <v>898</v>
@@ -59027,7 +59037,7 @@
         <v>594</v>
       </c>
       <c r="B184" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="185" spans="1:3">
@@ -60056,7 +60066,7 @@
         <v>730</v>
       </c>
       <c r="B309" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="C309" t="s">
         <v>626</v>
@@ -61080,7 +61090,7 @@
         <v>976</v>
       </c>
       <c r="B445" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="446" spans="1:2">
@@ -61088,7 +61098,7 @@
         <v>977</v>
       </c>
       <c r="B446" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
     </row>
     <row r="447" spans="1:2">
@@ -61096,7 +61106,7 @@
         <v>978</v>
       </c>
       <c r="B447" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="448" spans="1:2">

</xml_diff>

<commit_message>
updated library version and the logic for TSAHC check
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CD990D-C65E-4DF2-BEB1-C0B3F692DC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FA63EB0-5E97-4629-A5A7-2EA2A9153198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17762" uniqueCount="1152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17764" uniqueCount="1153">
   <si>
     <t>Name</t>
   </si>
@@ -3496,6 +3496,9 @@
   </si>
   <si>
     <t>C:\Users\raluca.ilinca.azureai-jump2\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>TX_TSAHCCheck</t>
   </si>
 </sst>
 </file>
@@ -7386,7 +7389,14 @@
         <v>1150</v>
       </c>
     </row>
-    <row r="50" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="50" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A50" t="s">
+        <v>1152</v>
+      </c>
+      <c r="B50" t="s">
+        <v>1152</v>
+      </c>
+    </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="53" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
updated the library version
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harika.malyala\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD297167-7867-4948-9745-E1B72A22FEE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{491FDE0F-4300-4BA0-B63D-7BBFAFB7DB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -3504,9 +3504,6 @@
     <t>CZI_PartAYes</t>
   </si>
   <si>
-    <t>One adult answered "Yes" to a question in section A.</t>
-  </si>
-  <si>
     <t>VSI</t>
   </si>
   <si>
@@ -3526,6 +3523,9 @@
   </si>
   <si>
     <t>General</t>
+  </si>
+  <si>
+    <t>Anticipated income in the next 12 months has been documented as yes for at least one question in Part A of the Certification of Zero Income. Manual review required.</t>
   </si>
 </sst>
 </file>
@@ -4034,10 +4034,10 @@
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B12" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -4428,10 +4428,10 @@
     </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1">
       <c r="A59" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B59" t="s">
         <v>1155</v>
-      </c>
-      <c r="B59" t="s">
-        <v>1156</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="14.25" customHeight="1">
@@ -8438,10 +8438,10 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B5" t="s">
         <v>1159</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1160</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -58738,7 +58738,7 @@
         <v>1153</v>
       </c>
       <c r="B143" t="s">
-        <v>1154</v>
+        <v>1161</v>
       </c>
       <c r="C143" t="s">
         <v>626</v>
@@ -60146,10 +60146,10 @@
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
+        <v>1156</v>
+      </c>
+      <c r="B313" t="s">
         <v>1157</v>
-      </c>
-      <c r="B313" t="s">
-        <v>1158</v>
       </c>
     </row>
     <row r="314" spans="1:3">

</xml_diff>

<commit_message>
updated rcv check in config
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88450D25-9E98-471D-9679-B728E5FFA1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91F530C-6A03-413B-AD59-2701A5A3B39B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="22710" windowHeight="10695" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28920" windowHeight="13860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17777" uniqueCount="1166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17779" uniqueCount="1168">
   <si>
     <t>Name</t>
   </si>
@@ -3522,9 +3522,6 @@
     <t>There are more Schedule Cs than CSEI</t>
   </si>
   <si>
-    <t>C:\Users\harika.malyala\Documents\AZApplicationReview\Prompts\</t>
-  </si>
-  <si>
     <t>Application Incomplete</t>
   </si>
   <si>
@@ -3538,6 +3535,15 @@
   </si>
   <si>
     <t>Newly added by Bagi for Arizona</t>
+  </si>
+  <si>
+    <t>C:\Users\harmandeep.singh\Documents\AZApplicationReview\Prompts\</t>
+  </si>
+  <si>
+    <t>RCV_EmailReceiptAndClarification</t>
+  </si>
+  <si>
+    <t>Regular Contributions Verification email receipt requires manual review.</t>
   </si>
 </sst>
 </file>
@@ -4016,7 +4022,7 @@
         <v>204</v>
       </c>
       <c r="B7" t="s">
-        <v>1160</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -4049,7 +4055,7 @@
         <v>1147</v>
       </c>
       <c r="B12" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
@@ -8424,7 +8430,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:XFD508"/>
+  <dimension ref="A1:XFD509"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -60352,7 +60358,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="338" spans="1:3" customFormat="1">
+    <row r="338" spans="1:3">
       <c r="A338" t="s">
         <v>391</v>
       </c>
@@ -60360,18 +60366,18 @@
         <v>567</v>
       </c>
     </row>
-    <row r="339" spans="1:3" customFormat="1">
+    <row r="339" spans="1:3">
       <c r="A339" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B339" t="s">
         <v>1163</v>
       </c>
-      <c r="B339" t="s">
+      <c r="C339" t="s">
         <v>1164</v>
       </c>
-      <c r="C339" t="s">
-        <v>1165</v>
-      </c>
-    </row>
-    <row r="340" spans="1:3" customFormat="1">
+    </row>
+    <row r="340" spans="1:3">
       <c r="A340" t="s">
         <v>476</v>
       </c>
@@ -60379,7 +60385,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="342" spans="1:3" customFormat="1">
+    <row r="342" spans="1:3">
       <c r="A342" t="s">
         <v>740</v>
       </c>
@@ -60390,7 +60396,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="343" spans="1:3" customFormat="1">
+    <row r="343" spans="1:3">
       <c r="A343" t="s">
         <v>742</v>
       </c>
@@ -60401,7 +60407,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="345" spans="1:3" customFormat="1">
+    <row r="345" spans="1:3">
       <c r="A345" t="s">
         <v>749</v>
       </c>
@@ -60409,7 +60415,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="346" spans="1:3" customFormat="1">
+    <row r="346" spans="1:3">
       <c r="A346" t="s">
         <v>751</v>
       </c>
@@ -60417,7 +60423,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="347" spans="1:3" customFormat="1">
+    <row r="347" spans="1:3">
       <c r="A347" t="s">
         <v>753</v>
       </c>
@@ -60425,7 +60431,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="348" spans="1:3" customFormat="1">
+    <row r="348" spans="1:3">
       <c r="A348" t="s">
         <v>755</v>
       </c>
@@ -60433,7 +60439,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="349" spans="1:3" customFormat="1">
+    <row r="349" spans="1:3">
       <c r="A349" t="s">
         <v>757</v>
       </c>
@@ -60441,7 +60447,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="350" spans="1:3" customFormat="1">
+    <row r="350" spans="1:3">
       <c r="A350" t="s">
         <v>759</v>
       </c>
@@ -60449,7 +60455,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="351" spans="1:3" customFormat="1">
+    <row r="351" spans="1:3">
       <c r="A351" t="s">
         <v>761</v>
       </c>
@@ -60457,7 +60463,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="352" spans="1:3" customFormat="1">
+    <row r="352" spans="1:3">
       <c r="A352" t="s">
         <v>763</v>
       </c>
@@ -60465,7 +60471,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="353" spans="1:2" customFormat="1">
+    <row r="353" spans="1:2">
       <c r="A353" t="s">
         <v>765</v>
       </c>
@@ -60473,7 +60479,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="354" spans="1:2" customFormat="1">
+    <row r="354" spans="1:2">
       <c r="A354" t="s">
         <v>767</v>
       </c>
@@ -60481,7 +60487,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="355" spans="1:2" customFormat="1">
+    <row r="355" spans="1:2">
       <c r="A355" t="s">
         <v>769</v>
       </c>
@@ -60489,7 +60495,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="356" spans="1:2" customFormat="1">
+    <row r="356" spans="1:2">
       <c r="A356" t="s">
         <v>771</v>
       </c>
@@ -60497,7 +60503,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="357" spans="1:2" customFormat="1">
+    <row r="357" spans="1:2">
       <c r="A357" t="s">
         <v>773</v>
       </c>
@@ -60505,7 +60511,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="358" spans="1:2" customFormat="1">
+    <row r="358" spans="1:2">
       <c r="A358" t="s">
         <v>775</v>
       </c>
@@ -60513,7 +60519,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="359" spans="1:2" customFormat="1">
+    <row r="359" spans="1:2">
       <c r="A359" t="s">
         <v>777</v>
       </c>
@@ -60521,7 +60527,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="360" spans="1:2" customFormat="1">
+    <row r="360" spans="1:2">
       <c r="A360" t="s">
         <v>779</v>
       </c>
@@ -60529,7 +60535,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="361" spans="1:2" customFormat="1">
+    <row r="361" spans="1:2">
       <c r="A361" t="s">
         <v>1158</v>
       </c>
@@ -60537,7 +60543,7 @@
         <v>1159</v>
       </c>
     </row>
-    <row r="362" spans="1:2" customFormat="1">
+    <row r="362" spans="1:2">
       <c r="A362" t="s">
         <v>781</v>
       </c>
@@ -60545,15 +60551,15 @@
         <v>782</v>
       </c>
     </row>
-    <row r="363" spans="1:2" customFormat="1">
+    <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B363" t="s">
         <v>783</v>
       </c>
     </row>
-    <row r="365" spans="1:2" customFormat="1">
+    <row r="365" spans="1:2">
       <c r="A365" t="s">
         <v>784</v>
       </c>
@@ -60561,7 +60567,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="366" spans="1:2" customFormat="1">
+    <row r="366" spans="1:2">
       <c r="A366" t="s">
         <v>786</v>
       </c>
@@ -60569,7 +60575,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="367" spans="1:2" customFormat="1">
+    <row r="367" spans="1:2">
       <c r="A367" t="s">
         <v>788</v>
       </c>
@@ -60577,7 +60583,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="368" spans="1:2" customFormat="1">
+    <row r="368" spans="1:2">
       <c r="A368" t="s">
         <v>790</v>
       </c>
@@ -60585,7 +60591,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="369" spans="1:2" customFormat="1">
+    <row r="369" spans="1:2">
       <c r="A369" t="s">
         <v>792</v>
       </c>
@@ -60593,7 +60599,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="370" spans="1:2" customFormat="1">
+    <row r="370" spans="1:2">
       <c r="A370" t="s">
         <v>794</v>
       </c>
@@ -60601,7 +60607,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="371" spans="1:2" customFormat="1">
+    <row r="371" spans="1:2">
       <c r="A371" t="s">
         <v>796</v>
       </c>
@@ -60609,7 +60615,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="372" spans="1:2" customFormat="1">
+    <row r="372" spans="1:2">
       <c r="A372" t="s">
         <v>798</v>
       </c>
@@ -60617,7 +60623,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="373" spans="1:2" customFormat="1">
+    <row r="373" spans="1:2">
       <c r="A373" t="s">
         <v>799</v>
       </c>
@@ -60625,7 +60631,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="374" spans="1:2" customFormat="1">
+    <row r="374" spans="1:2">
       <c r="A374" t="s">
         <v>801</v>
       </c>
@@ -60633,7 +60639,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="375" spans="1:2" customFormat="1">
+    <row r="375" spans="1:2">
       <c r="A375" t="s">
         <v>803</v>
       </c>
@@ -60641,7 +60647,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="376" spans="1:2" customFormat="1">
+    <row r="376" spans="1:2">
       <c r="A376" t="s">
         <v>805</v>
       </c>
@@ -60649,7 +60655,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="378" spans="1:2" customFormat="1">
+    <row r="378" spans="1:2">
       <c r="A378" t="s">
         <v>807</v>
       </c>
@@ -60657,7 +60663,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="379" spans="1:2" customFormat="1">
+    <row r="379" spans="1:2">
       <c r="A379" t="s">
         <v>808</v>
       </c>
@@ -60665,7 +60671,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="380" spans="1:2" customFormat="1">
+    <row r="380" spans="1:2">
       <c r="A380" t="s">
         <v>810</v>
       </c>
@@ -60673,7 +60679,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="381" spans="1:2" customFormat="1">
+    <row r="381" spans="1:2">
       <c r="A381" t="s">
         <v>811</v>
       </c>
@@ -60681,7 +60687,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="383" spans="1:2" customFormat="1">
+    <row r="383" spans="1:2">
       <c r="A383" t="s">
         <v>834</v>
       </c>
@@ -60689,7 +60695,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="384" spans="1:2" customFormat="1">
+    <row r="384" spans="1:2">
       <c r="A384" t="s">
         <v>833</v>
       </c>
@@ -60697,7 +60703,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="385" spans="1:2" customFormat="1">
+    <row r="385" spans="1:2">
       <c r="A385" t="s">
         <v>826</v>
       </c>
@@ -60705,7 +60711,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="386" spans="1:2" customFormat="1">
+    <row r="386" spans="1:2">
       <c r="A386" t="s">
         <v>824</v>
       </c>
@@ -60713,7 +60719,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="387" spans="1:2" customFormat="1">
+    <row r="387" spans="1:2">
       <c r="A387" t="s">
         <v>825</v>
       </c>
@@ -60721,7 +60727,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="388" spans="1:2" customFormat="1">
+    <row r="388" spans="1:2">
       <c r="A388" t="s">
         <v>831</v>
       </c>
@@ -60729,7 +60735,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="390" spans="1:2" customFormat="1">
+    <row r="390" spans="1:2">
       <c r="A390" t="s">
         <v>838</v>
       </c>
@@ -60737,7 +60743,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="391" spans="1:2" customFormat="1">
+    <row r="391" spans="1:2">
       <c r="A391" t="s">
         <v>846</v>
       </c>
@@ -60745,7 +60751,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="392" spans="1:2" customFormat="1">
+    <row r="392" spans="1:2">
       <c r="A392" t="s">
         <v>839</v>
       </c>
@@ -60753,7 +60759,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="393" spans="1:2" customFormat="1">
+    <row r="393" spans="1:2">
       <c r="A393" t="s">
         <v>840</v>
       </c>
@@ -60761,7 +60767,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="394" spans="1:2" customFormat="1">
+    <row r="394" spans="1:2">
       <c r="A394" t="s">
         <v>841</v>
       </c>
@@ -60769,7 +60775,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="395" spans="1:2" customFormat="1">
+    <row r="395" spans="1:2">
       <c r="A395" t="s">
         <v>842</v>
       </c>
@@ -60777,7 +60783,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="397" spans="1:2" customFormat="1">
+    <row r="397" spans="1:2">
       <c r="A397" t="s">
         <v>851</v>
       </c>
@@ -60785,7 +60791,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="398" spans="1:2" customFormat="1">
+    <row r="398" spans="1:2">
       <c r="A398" t="s">
         <v>853</v>
       </c>
@@ -60793,7 +60799,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="399" spans="1:2" customFormat="1">
+    <row r="399" spans="1:2">
       <c r="A399" t="s">
         <v>854</v>
       </c>
@@ -60801,7 +60807,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="400" spans="1:2" customFormat="1">
+    <row r="400" spans="1:2">
       <c r="A400" t="s">
         <v>856</v>
       </c>
@@ -60809,7 +60815,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="401" spans="1:2" customFormat="1">
+    <row r="401" spans="1:2">
       <c r="A401" t="s">
         <v>862</v>
       </c>
@@ -60817,7 +60823,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="402" spans="1:2" customFormat="1">
+    <row r="402" spans="1:2">
       <c r="A402" t="s">
         <v>863</v>
       </c>
@@ -60825,7 +60831,7 @@
         <v>1059</v>
       </c>
     </row>
-    <row r="403" spans="1:2" customFormat="1">
+    <row r="403" spans="1:2">
       <c r="A403" t="s">
         <v>864</v>
       </c>
@@ -60833,7 +60839,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="404" spans="1:2" customFormat="1">
+    <row r="404" spans="1:2">
       <c r="A404" t="s">
         <v>867</v>
       </c>
@@ -60841,7 +60847,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="405" spans="1:2" customFormat="1">
+    <row r="405" spans="1:2">
       <c r="A405" t="s">
         <v>868</v>
       </c>
@@ -60849,7 +60855,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="406" spans="1:2" customFormat="1">
+    <row r="406" spans="1:2">
       <c r="A406" t="s">
         <v>869</v>
       </c>
@@ -60857,7 +60863,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="407" spans="1:2" customFormat="1">
+    <row r="407" spans="1:2">
       <c r="A407" t="s">
         <v>870</v>
       </c>
@@ -60865,7 +60871,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="408" spans="1:2" customFormat="1">
+    <row r="408" spans="1:2">
       <c r="A408" t="s">
         <v>871</v>
       </c>
@@ -60873,7 +60879,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="409" spans="1:2" customFormat="1">
+    <row r="409" spans="1:2">
       <c r="A409" t="s">
         <v>872</v>
       </c>
@@ -60881,7 +60887,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="410" spans="1:2" customFormat="1">
+    <row r="410" spans="1:2">
       <c r="A410" t="s">
         <v>873</v>
       </c>
@@ -60889,7 +60895,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="411" spans="1:2" customFormat="1">
+    <row r="411" spans="1:2">
       <c r="A411" t="s">
         <v>874</v>
       </c>
@@ -60897,7 +60903,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="412" spans="1:2" customFormat="1">
+    <row r="412" spans="1:2">
       <c r="A412" t="s">
         <v>875</v>
       </c>
@@ -60905,7 +60911,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="413" spans="1:2" customFormat="1">
+    <row r="413" spans="1:2">
       <c r="A413" t="s">
         <v>866</v>
       </c>
@@ -60913,7 +60919,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="414" spans="1:2" customFormat="1">
+    <row r="414" spans="1:2">
       <c r="A414" t="s">
         <v>865</v>
       </c>
@@ -60921,7 +60927,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="415" spans="1:2" customFormat="1">
+    <row r="415" spans="1:2">
       <c r="A415" t="s">
         <v>1068</v>
       </c>
@@ -60929,7 +60935,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="416" spans="1:2" customFormat="1">
+    <row r="416" spans="1:2">
       <c r="A416" t="s">
         <v>1070</v>
       </c>
@@ -60937,7 +60943,7 @@
         <v>1071</v>
       </c>
     </row>
-    <row r="417" spans="1:2" customFormat="1">
+    <row r="417" spans="1:2">
       <c r="A417" t="s">
         <v>1072</v>
       </c>
@@ -60945,7 +60951,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="418" spans="1:2" customFormat="1">
+    <row r="418" spans="1:2">
       <c r="A418" t="s">
         <v>1074</v>
       </c>
@@ -60953,7 +60959,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="419" spans="1:2" customFormat="1">
+    <row r="419" spans="1:2">
       <c r="A419" t="s">
         <v>1076</v>
       </c>
@@ -60961,7 +60967,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="420" spans="1:2" customFormat="1">
+    <row r="420" spans="1:2">
       <c r="A420" t="s">
         <v>1078</v>
       </c>
@@ -60969,7 +60975,7 @@
         <v>1079</v>
       </c>
     </row>
-    <row r="421" spans="1:2" customFormat="1">
+    <row r="421" spans="1:2">
       <c r="A421" t="s">
         <v>1080</v>
       </c>
@@ -60977,7 +60983,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="422" spans="1:2" customFormat="1">
+    <row r="422" spans="1:2">
       <c r="A422" t="s">
         <v>1082</v>
       </c>
@@ -60985,7 +60991,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="424" spans="1:2" customFormat="1">
+    <row r="424" spans="1:2">
       <c r="A424" t="s">
         <v>915</v>
       </c>
@@ -60993,7 +60999,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="425" spans="1:2" customFormat="1">
+    <row r="425" spans="1:2">
       <c r="A425" t="s">
         <v>917</v>
       </c>
@@ -61001,7 +61007,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="426" spans="1:2" customFormat="1">
+    <row r="426" spans="1:2">
       <c r="A426" t="s">
         <v>919</v>
       </c>
@@ -61009,7 +61015,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="427" spans="1:2" customFormat="1">
+    <row r="427" spans="1:2">
       <c r="A427" t="s">
         <v>921</v>
       </c>
@@ -61017,7 +61023,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="428" spans="1:2" customFormat="1">
+    <row r="428" spans="1:2">
       <c r="A428" t="s">
         <v>923</v>
       </c>
@@ -61025,7 +61031,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="429" spans="1:2" customFormat="1">
+    <row r="429" spans="1:2">
       <c r="A429" t="s">
         <v>925</v>
       </c>
@@ -61033,7 +61039,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="430" spans="1:2" customFormat="1">
+    <row r="430" spans="1:2">
       <c r="A430" t="s">
         <v>927</v>
       </c>
@@ -61041,7 +61047,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="431" spans="1:2" customFormat="1">
+    <row r="431" spans="1:2">
       <c r="A431" t="s">
         <v>929</v>
       </c>
@@ -61049,7 +61055,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="432" spans="1:2" customFormat="1">
+    <row r="432" spans="1:2">
       <c r="A432" t="s">
         <v>931</v>
       </c>
@@ -61057,7 +61063,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="433" spans="1:2" customFormat="1">
+    <row r="433" spans="1:2">
       <c r="A433" t="s">
         <v>933</v>
       </c>
@@ -61065,7 +61071,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="434" spans="1:2" customFormat="1">
+    <row r="434" spans="1:2">
       <c r="A434" t="s">
         <v>935</v>
       </c>
@@ -61073,7 +61079,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="435" spans="1:2" customFormat="1">
+    <row r="435" spans="1:2">
       <c r="A435" t="s">
         <v>937</v>
       </c>
@@ -61081,7 +61087,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="436" spans="1:2" customFormat="1">
+    <row r="436" spans="1:2">
       <c r="A436" t="s">
         <v>939</v>
       </c>
@@ -61089,7 +61095,7 @@
         <v>940</v>
       </c>
     </row>
-    <row r="437" spans="1:2" customFormat="1">
+    <row r="437" spans="1:2">
       <c r="A437" t="s">
         <v>941</v>
       </c>
@@ -61097,7 +61103,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="438" spans="1:2" customFormat="1">
+    <row r="438" spans="1:2">
       <c r="A438" t="s">
         <v>943</v>
       </c>
@@ -61105,7 +61111,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="439" spans="1:2" customFormat="1">
+    <row r="439" spans="1:2">
       <c r="A439" t="s">
         <v>945</v>
       </c>
@@ -61113,7 +61119,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="440" spans="1:2" customFormat="1">
+    <row r="440" spans="1:2">
       <c r="A440" t="s">
         <v>947</v>
       </c>
@@ -61121,7 +61127,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="441" spans="1:2" customFormat="1">
+    <row r="441" spans="1:2">
       <c r="A441" t="s">
         <v>949</v>
       </c>
@@ -61129,7 +61135,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="442" spans="1:2" customFormat="1">
+    <row r="442" spans="1:2">
       <c r="A442" t="s">
         <v>951</v>
       </c>
@@ -61137,7 +61143,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="443" spans="1:2" customFormat="1">
+    <row r="443" spans="1:2">
       <c r="A443" t="s">
         <v>953</v>
       </c>
@@ -61145,7 +61151,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="444" spans="1:2" customFormat="1">
+    <row r="444" spans="1:2">
       <c r="A444" t="s">
         <v>955</v>
       </c>
@@ -61153,452 +61159,460 @@
         <v>956</v>
       </c>
     </row>
+    <row r="445" spans="1:2" customFormat="1"/>
     <row r="446" spans="1:2" customFormat="1">
       <c r="A446" t="s">
-        <v>957</v>
+        <v>1166</v>
       </c>
       <c r="B446" t="s">
-        <v>958</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="447" spans="1:2" customFormat="1">
       <c r="A447" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="B447" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
     </row>
     <row r="448" spans="1:2" customFormat="1">
       <c r="A448" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="B448" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
     </row>
     <row r="449" spans="1:2" customFormat="1">
       <c r="A449" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="B449" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
     </row>
     <row r="450" spans="1:2" customFormat="1">
       <c r="A450" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="B450" t="s">
-        <v>1127</v>
+        <v>964</v>
       </c>
     </row>
     <row r="451" spans="1:2" customFormat="1">
       <c r="A451" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B451" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="452" spans="1:2" customFormat="1">
       <c r="A452" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B452" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="453" spans="1:2" customFormat="1">
       <c r="A453" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
       <c r="B453" t="s">
-        <v>969</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="454" spans="1:2" customFormat="1">
       <c r="A454" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="B454" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
     </row>
     <row r="455" spans="1:2" customFormat="1">
       <c r="A455" t="s">
+        <v>970</v>
+      </c>
+      <c r="B455" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="456" spans="1:2" customFormat="1">
+      <c r="A456" t="s">
         <v>972</v>
       </c>
-      <c r="B455" t="s">
+      <c r="B456" t="s">
         <v>973</v>
-      </c>
-    </row>
-    <row r="457" spans="1:2" customFormat="1">
-      <c r="A457" t="s">
-        <v>980</v>
-      </c>
-      <c r="B457" t="s">
-        <v>981</v>
       </c>
     </row>
     <row r="458" spans="1:2" customFormat="1">
       <c r="A458" t="s">
+        <v>980</v>
+      </c>
+      <c r="B458" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="459" spans="1:2" customFormat="1">
+      <c r="A459" t="s">
         <v>982</v>
       </c>
-      <c r="B458" t="s">
+      <c r="B459" t="s">
         <v>983</v>
-      </c>
-    </row>
-    <row r="460" spans="1:2" customFormat="1">
-      <c r="A460" t="s">
-        <v>984</v>
-      </c>
-      <c r="B460" t="s">
-        <v>985</v>
       </c>
     </row>
     <row r="461" spans="1:2" customFormat="1">
       <c r="A461" t="s">
+        <v>984</v>
+      </c>
+      <c r="B461" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="462" spans="1:2" customFormat="1">
+      <c r="A462" t="s">
         <v>986</v>
       </c>
-      <c r="B461" t="s">
+      <c r="B462" t="s">
         <v>987</v>
-      </c>
-    </row>
-    <row r="463" spans="1:2" customFormat="1">
-      <c r="A463" t="s">
-        <v>988</v>
-      </c>
-      <c r="B463" t="s">
-        <v>989</v>
       </c>
     </row>
     <row r="464" spans="1:2" customFormat="1">
       <c r="A464" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="B464" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
     </row>
     <row r="465" spans="1:2" customFormat="1">
       <c r="A465" t="s">
+        <v>990</v>
+      </c>
+      <c r="B465" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="466" spans="1:2" customFormat="1">
+      <c r="A466" t="s">
         <v>992</v>
       </c>
-      <c r="B465" t="s">
+      <c r="B466" t="s">
         <v>993</v>
-      </c>
-    </row>
-    <row r="467" spans="1:2" customFormat="1">
-      <c r="A467" t="s">
-        <v>994</v>
-      </c>
-      <c r="B467" t="s">
-        <v>995</v>
       </c>
     </row>
     <row r="468" spans="1:2" customFormat="1">
       <c r="A468" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="B468" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
     </row>
     <row r="469" spans="1:2" customFormat="1">
       <c r="A469" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
       <c r="B469" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
     </row>
     <row r="470" spans="1:2" customFormat="1">
       <c r="A470" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
       <c r="B470" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
     </row>
     <row r="471" spans="1:2" customFormat="1">
       <c r="A471" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
       <c r="B471" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="472" spans="1:2" customFormat="1">
       <c r="A472" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="B472" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="473" spans="1:2" customFormat="1">
       <c r="A473" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B473" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="474" spans="1:2" customFormat="1">
+      <c r="A474" t="s">
         <v>1006</v>
       </c>
-      <c r="B473" t="s">
+      <c r="B474" t="s">
         <v>1007</v>
-      </c>
-    </row>
-    <row r="475" spans="1:2" customFormat="1">
-      <c r="A475" t="s">
-        <v>1008</v>
-      </c>
-      <c r="B475" t="s">
-        <v>1009</v>
       </c>
     </row>
     <row r="476" spans="1:2" customFormat="1">
       <c r="A476" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="B476" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="477" spans="1:2" customFormat="1">
       <c r="A477" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="B477" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="478" spans="1:2" customFormat="1">
       <c r="A478" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="B478" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="479" spans="1:2" customFormat="1">
       <c r="A479" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="B479" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="480" spans="1:2" customFormat="1">
       <c r="A480" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B480" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="481" spans="1:2" customFormat="1">
+      <c r="A481" t="s">
         <v>1018</v>
       </c>
-      <c r="B480" t="s">
+      <c r="B481" t="s">
         <v>1019</v>
-      </c>
-    </row>
-    <row r="481" spans="1:2" customFormat="1"/>
-    <row r="482" spans="1:2" customFormat="1">
-      <c r="A482" t="s">
-        <v>1020</v>
-      </c>
-      <c r="B482" t="s">
-        <v>1021</v>
       </c>
     </row>
     <row r="483" spans="1:2" customFormat="1">
       <c r="A483" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
       <c r="B483" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="484" spans="1:2" customFormat="1">
       <c r="A484" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="B484" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="485" spans="1:2" customFormat="1">
       <c r="A485" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="B485" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="486" spans="1:2" customFormat="1">
       <c r="A486" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="B486" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="487" spans="1:2" customFormat="1">
       <c r="A487" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B487" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="488" spans="1:2" customFormat="1">
+      <c r="A488" t="s">
         <v>1030</v>
       </c>
-      <c r="B487" t="s">
+      <c r="B488" t="s">
         <v>1031</v>
-      </c>
-    </row>
-    <row r="489" spans="1:2" customFormat="1">
-      <c r="A489" t="s">
-        <v>1032</v>
-      </c>
-      <c r="B489" t="s">
-        <v>1033</v>
       </c>
     </row>
     <row r="490" spans="1:2" customFormat="1">
       <c r="A490" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="B490" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="491" spans="1:2" customFormat="1">
       <c r="A491" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="B491" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="492" spans="1:2" customFormat="1">
       <c r="A492" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B492" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="493" spans="1:2" customFormat="1">
       <c r="A493" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B493" t="s">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="494" spans="1:2" customFormat="1">
+      <c r="A494" t="s">
         <v>1040</v>
       </c>
-      <c r="B493" t="s">
+      <c r="B494" t="s">
         <v>1041</v>
-      </c>
-    </row>
-    <row r="495" spans="1:2" customFormat="1">
-      <c r="A495" t="s">
-        <v>1084</v>
-      </c>
-      <c r="B495" t="s">
-        <v>1085</v>
       </c>
     </row>
     <row r="496" spans="1:2" customFormat="1">
       <c r="A496" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="B496" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="497" spans="1:2" customFormat="1">
       <c r="A497" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="B497" t="s">
-        <v>1089</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="498" spans="1:2" customFormat="1">
       <c r="A498" t="s">
-        <v>1090</v>
+        <v>1088</v>
       </c>
       <c r="B498" t="s">
-        <v>1091</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="499" spans="1:2" customFormat="1">
       <c r="A499" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="B499" t="s">
-        <v>1093</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="500" spans="1:2" customFormat="1">
       <c r="A500" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="B500" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="501" spans="1:2" customFormat="1">
       <c r="A501" t="s">
-        <v>1096</v>
+        <v>1094</v>
       </c>
       <c r="B501" t="s">
-        <v>1097</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="502" spans="1:2" customFormat="1">
       <c r="A502" t="s">
-        <v>1098</v>
+        <v>1096</v>
       </c>
       <c r="B502" t="s">
-        <v>1099</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="503" spans="1:2" customFormat="1">
       <c r="A503" t="s">
-        <v>1100</v>
+        <v>1098</v>
       </c>
       <c r="B503" t="s">
-        <v>1101</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="504" spans="1:2" customFormat="1">
       <c r="A504" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
       <c r="B504" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="505" spans="1:2" customFormat="1">
       <c r="A505" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="B505" t="s">
-        <v>1105</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="506" spans="1:2" customFormat="1">
       <c r="A506" t="s">
-        <v>1106</v>
+        <v>1104</v>
       </c>
       <c r="B506" t="s">
-        <v>1107</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="507" spans="1:2" customFormat="1">
       <c r="A507" t="s">
-        <v>1108</v>
+        <v>1106</v>
       </c>
       <c r="B507" t="s">
-        <v>1109</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="508" spans="1:2" customFormat="1">
       <c r="A508" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B508" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="509" spans="1:2" customFormat="1">
+      <c r="A509" t="s">
         <v>1110</v>
       </c>
-      <c r="B508" t="s">
+      <c r="B509" t="s">
         <v>1111</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A446:A455">
+  <conditionalFormatting sqref="A447:A456">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A463:A464 A460:A461 A457:A458">
+  <conditionalFormatting sqref="A464:A465 A461:A462 A458:A459">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add edc in config
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5281E73C-F4DD-46B6-A1BB-26FDD8F43FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55063BCC-8208-4D71-9060-48F3F79EAC62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="11010" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17781" uniqueCount="1170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17784" uniqueCount="1172">
   <si>
     <t>Name</t>
   </si>
@@ -3550,6 +3550,12 @@
   </si>
   <si>
     <t xml:space="preserve">Applicant Name across the Employment Verification, Day Calculator, and ICW do not match. </t>
+  </si>
+  <si>
+    <t>EDC_HighestCalValue</t>
+  </si>
+  <si>
+    <t>Newly added by Harmandeep</t>
   </si>
 </sst>
 </file>
@@ -8436,7 +8442,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:XFD510"/>
+  <dimension ref="A1:XFD511"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -58919,2713 +58925,2728 @@
         <v>1143</v>
       </c>
     </row>
-    <row r="164" spans="1:3">
+    <row r="163" spans="1:3" customFormat="1"/>
+    <row r="164" spans="1:3" customFormat="1">
       <c r="A164" t="s">
+        <v>1170</v>
+      </c>
+      <c r="B164" t="s">
+        <v>792</v>
+      </c>
+      <c r="C164" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" customFormat="1">
+      <c r="A165" t="s">
         <v>591</v>
       </c>
-      <c r="B164" t="s">
+      <c r="B165" t="s">
         <v>855</v>
       </c>
-      <c r="C164" t="s">
+      <c r="C165" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="165" spans="1:3">
-      <c r="A165" t="s">
+    <row r="166" spans="1:3" customFormat="1">
+      <c r="A166" t="s">
         <v>633</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B166" t="s">
         <v>634</v>
-      </c>
-      <c r="C165" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="166" spans="1:3">
-      <c r="A166" t="s">
-        <v>721</v>
-      </c>
-      <c r="B166" t="s">
-        <v>856</v>
       </c>
       <c r="C166" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="167" spans="1:3">
+    <row r="167" spans="1:3" customFormat="1">
       <c r="A167" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B167" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="C167" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="168" spans="1:3">
+    <row r="168" spans="1:3" customFormat="1">
       <c r="A168" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B168" t="s">
-        <v>706</v>
+        <v>857</v>
       </c>
       <c r="C168" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="169" spans="1:3">
+    <row r="169" spans="1:3" customFormat="1">
       <c r="A169" t="s">
-        <v>1096</v>
+        <v>723</v>
       </c>
       <c r="B169" t="s">
-        <v>862</v>
+        <v>706</v>
       </c>
       <c r="C169" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="171" spans="1:3">
-      <c r="A171" t="s">
+    <row r="170" spans="1:3" customFormat="1">
+      <c r="A170" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B170" t="s">
+        <v>862</v>
+      </c>
+      <c r="C170" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" customFormat="1">
+      <c r="A172" t="s">
         <v>466</v>
       </c>
-      <c r="B171" t="s">
+      <c r="B172" t="s">
         <v>1113</v>
       </c>
     </row>
-    <row r="172" spans="1:3">
-      <c r="A172" t="s">
+    <row r="173" spans="1:3" customFormat="1">
+      <c r="A173" t="s">
         <v>1110</v>
       </c>
-      <c r="B172" t="s">
+      <c r="B173" t="s">
         <v>1111</v>
       </c>
-      <c r="C172" t="s">
+      <c r="C173" t="s">
         <v>1112</v>
       </c>
     </row>
-    <row r="173" spans="1:3">
-      <c r="A173" t="s">
+    <row r="174" spans="1:3" customFormat="1">
+      <c r="A174" t="s">
         <v>237</v>
       </c>
-      <c r="B173" t="s">
+      <c r="B174" t="s">
         <v>858</v>
       </c>
-      <c r="C173" t="s">
+      <c r="C174" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="174" spans="1:3">
-      <c r="A174" t="s">
+    <row r="175" spans="1:3" customFormat="1">
+      <c r="A175" t="s">
         <v>238</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B175" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="175" spans="1:3">
-      <c r="A175" t="s">
+    <row r="176" spans="1:3" customFormat="1">
+      <c r="A176" t="s">
         <v>246</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B176" t="s">
         <v>860</v>
       </c>
-      <c r="C175" t="s">
+      <c r="C176" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="176" spans="1:3">
-      <c r="A176" t="s">
+    <row r="177" spans="1:3" customFormat="1">
+      <c r="A177" t="s">
         <v>690</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B177" t="s">
         <v>861</v>
       </c>
-      <c r="C176" t="s">
+      <c r="C177" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="177" spans="1:3">
-      <c r="A177" t="s">
+    <row r="178" spans="1:3" customFormat="1">
+      <c r="A178" t="s">
         <v>240</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B178" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="178" spans="1:3">
-      <c r="A178" t="s">
+    <row r="179" spans="1:3" customFormat="1">
+      <c r="A179" t="s">
         <v>456</v>
       </c>
-      <c r="B178" t="s">
+      <c r="B179" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="179" spans="1:3">
-      <c r="A179" t="s">
+    <row r="180" spans="1:3" customFormat="1">
+      <c r="A180" t="s">
         <v>241</v>
       </c>
-      <c r="B179" t="s">
+      <c r="B180" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="180" spans="1:3">
-      <c r="A180" t="s">
+    <row r="181" spans="1:3" customFormat="1">
+      <c r="A181" t="s">
         <v>242</v>
       </c>
-      <c r="B180" t="s">
+      <c r="B181" t="s">
         <v>863</v>
       </c>
     </row>
-    <row r="181" spans="1:3">
-      <c r="A181" t="s">
+    <row r="182" spans="1:3" customFormat="1">
+      <c r="A182" t="s">
         <v>243</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B182" t="s">
         <v>864</v>
       </c>
     </row>
-    <row r="182" spans="1:3">
-      <c r="A182" t="s">
+    <row r="183" spans="1:3" customFormat="1">
+      <c r="A183" t="s">
         <v>244</v>
       </c>
-      <c r="B182" t="s">
+      <c r="B183" t="s">
         <v>865</v>
       </c>
     </row>
-    <row r="183" spans="1:3">
-      <c r="A183" t="s">
+    <row r="184" spans="1:3" customFormat="1">
+      <c r="A184" t="s">
         <v>245</v>
       </c>
-      <c r="B183" t="s">
+      <c r="B184" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="184" spans="1:3">
-      <c r="A184" t="s">
+    <row r="185" spans="1:3" customFormat="1">
+      <c r="A185" t="s">
         <v>277</v>
       </c>
-      <c r="B184" t="s">
+      <c r="B185" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="185" spans="1:3">
-      <c r="A185" t="s">
+    <row r="186" spans="1:3" customFormat="1">
+      <c r="A186" t="s">
         <v>304</v>
       </c>
-      <c r="B185" t="s">
+      <c r="B186" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="186" spans="1:3">
-      <c r="A186" t="s">
+    <row r="187" spans="1:3" customFormat="1">
+      <c r="A187" t="s">
         <v>594</v>
       </c>
-      <c r="B186" t="s">
+      <c r="B187" t="s">
         <v>1094</v>
       </c>
     </row>
-    <row r="187" spans="1:3">
-      <c r="A187" t="s">
+    <row r="188" spans="1:3" customFormat="1">
+      <c r="A188" t="s">
         <v>611</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B188" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="188" spans="1:3">
-      <c r="A188" t="s">
+    <row r="189" spans="1:3" customFormat="1">
+      <c r="A189" t="s">
         <v>676</v>
       </c>
-      <c r="B188" t="s">
+      <c r="B189" t="s">
         <v>677</v>
-      </c>
-      <c r="C188" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3">
-      <c r="A189" t="s">
-        <v>689</v>
-      </c>
-      <c r="B189" t="s">
-        <v>708</v>
       </c>
       <c r="C189" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="190" spans="1:3">
+    <row r="190" spans="1:3" customFormat="1">
       <c r="A190" t="s">
+        <v>689</v>
+      </c>
+      <c r="B190" t="s">
+        <v>708</v>
+      </c>
+      <c r="C190" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" customFormat="1">
+      <c r="A191" t="s">
         <v>874</v>
       </c>
-      <c r="B190" t="s">
+      <c r="B191" t="s">
         <v>875</v>
       </c>
     </row>
-    <row r="191" spans="1:3">
-      <c r="A191" t="s">
+    <row r="192" spans="1:3" customFormat="1">
+      <c r="A192" t="s">
         <v>474</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B192" t="s">
         <v>1144</v>
       </c>
     </row>
-    <row r="193" spans="1:3">
-      <c r="A193" t="s">
+    <row r="193" spans="1:3" customFormat="1"/>
+    <row r="194" spans="1:3" customFormat="1">
+      <c r="A194" t="s">
         <v>687</v>
       </c>
-      <c r="B193" t="s">
+      <c r="B194" t="s">
         <v>688</v>
       </c>
-      <c r="C193" t="s">
+      <c r="C194" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="194" spans="1:3">
-      <c r="A194" t="s">
+    <row r="195" spans="1:3" customFormat="1">
+      <c r="A195" t="s">
         <v>467</v>
       </c>
-      <c r="B194" t="s">
+      <c r="B195" t="s">
         <v>1118</v>
       </c>
     </row>
-    <row r="195" spans="1:3">
-      <c r="A195" t="s">
+    <row r="196" spans="1:3" customFormat="1">
+      <c r="A196" t="s">
         <v>247</v>
       </c>
-      <c r="B195" t="s">
+      <c r="B196" t="s">
         <v>866</v>
       </c>
-      <c r="C195" t="s">
+      <c r="C196" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="196" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A196" t="s">
+    <row r="197" spans="1:3" customFormat="1" ht="13.5" customHeight="1">
+      <c r="A197" t="s">
         <v>249</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B197" t="s">
         <v>867</v>
       </c>
-      <c r="C196" t="s">
+      <c r="C197" t="s">
         <v>606</v>
       </c>
     </row>
-    <row r="197" spans="1:3">
-      <c r="A197" t="s">
+    <row r="198" spans="1:3" customFormat="1">
+      <c r="A198" t="s">
         <v>248</v>
       </c>
-      <c r="B197" t="s">
+      <c r="B198" t="s">
         <v>828</v>
       </c>
     </row>
-    <row r="198" spans="1:3">
-      <c r="A198" t="s">
+    <row r="199" spans="1:3" customFormat="1">
+      <c r="A199" t="s">
         <v>251</v>
       </c>
-      <c r="B198" t="s">
+      <c r="B199" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="199" spans="1:3">
-      <c r="A199" t="s">
+    <row r="200" spans="1:3" customFormat="1">
+      <c r="A200" t="s">
         <v>252</v>
       </c>
-      <c r="B199" t="s">
+      <c r="B200" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="200" spans="1:3">
-      <c r="A200" t="s">
+    <row r="201" spans="1:3" customFormat="1">
+      <c r="A201" t="s">
         <v>255</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B201" t="s">
         <v>254</v>
       </c>
-      <c r="C200" t="s">
+      <c r="C201" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="201" spans="1:3">
-      <c r="A201" t="s">
+    <row r="202" spans="1:3" customFormat="1">
+      <c r="A202" t="s">
         <v>457</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B202" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="202" spans="1:3">
-      <c r="A202" t="s">
+    <row r="203" spans="1:3" customFormat="1">
+      <c r="A203" t="s">
         <v>256</v>
       </c>
-      <c r="B202" t="s">
+      <c r="B203" t="s">
         <v>830</v>
       </c>
     </row>
-    <row r="203" spans="1:3">
-      <c r="A203" t="s">
+    <row r="204" spans="1:3" customFormat="1">
+      <c r="A204" t="s">
         <v>257</v>
       </c>
-      <c r="B203" t="s">
+      <c r="B204" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="204" spans="1:3">
-      <c r="A204" t="s">
+    <row r="205" spans="1:3" customFormat="1">
+      <c r="A205" t="s">
         <v>262</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B205" t="s">
         <v>831</v>
       </c>
     </row>
-    <row r="205" spans="1:3">
-      <c r="A205" t="s">
+    <row r="206" spans="1:3" customFormat="1">
+      <c r="A206" t="s">
         <v>263</v>
       </c>
-      <c r="B205" t="s">
+      <c r="B206" t="s">
         <v>832</v>
       </c>
     </row>
-    <row r="206" spans="1:3">
-      <c r="A206" t="s">
+    <row r="207" spans="1:3" customFormat="1">
+      <c r="A207" t="s">
         <v>264</v>
       </c>
-      <c r="B206" t="s">
+      <c r="B207" t="s">
         <v>868</v>
       </c>
-      <c r="C206" t="s">
+      <c r="C207" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="207" spans="1:3">
-      <c r="A207" t="s">
+    <row r="208" spans="1:3" customFormat="1">
+      <c r="A208" t="s">
         <v>265</v>
       </c>
-      <c r="B207" t="s">
+      <c r="B208" t="s">
         <v>833</v>
       </c>
     </row>
-    <row r="208" spans="1:3">
-      <c r="A208" t="s">
+    <row r="209" spans="1:3" customFormat="1">
+      <c r="A209" t="s">
         <v>266</v>
       </c>
-      <c r="B208" t="s">
+      <c r="B209" t="s">
         <v>869</v>
       </c>
-      <c r="C208" t="s">
+      <c r="C209" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="209" spans="1:3">
-      <c r="A209" t="s">
+    <row r="210" spans="1:3" customFormat="1">
+      <c r="A210" t="s">
         <v>267</v>
       </c>
-      <c r="B209" t="s">
+      <c r="B210" t="s">
         <v>834</v>
       </c>
     </row>
-    <row r="210" spans="1:3">
-      <c r="A210" t="s">
+    <row r="211" spans="1:3" customFormat="1">
+      <c r="A211" t="s">
         <v>274</v>
       </c>
-      <c r="B210" t="s">
+      <c r="B211" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="211" spans="1:3">
-      <c r="A211" t="s">
+    <row r="212" spans="1:3" customFormat="1">
+      <c r="A212" t="s">
         <v>276</v>
       </c>
-      <c r="B211" t="s">
+      <c r="B212" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="212" spans="1:3">
-      <c r="A212" t="s">
+    <row r="213" spans="1:3" customFormat="1">
+      <c r="A213" t="s">
         <v>278</v>
       </c>
-      <c r="B212" t="s">
+      <c r="B213" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="213" spans="1:3">
-      <c r="A213" t="s">
+    <row r="214" spans="1:3" customFormat="1">
+      <c r="A214" t="s">
         <v>612</v>
       </c>
-      <c r="B213" t="s">
+      <c r="B214" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="214" spans="1:3">
-      <c r="A214" t="s">
+    <row r="215" spans="1:3" customFormat="1">
+      <c r="A215" t="s">
         <v>485</v>
       </c>
-      <c r="B214" t="s">
+      <c r="B215" t="s">
         <v>1145</v>
       </c>
     </row>
-    <row r="215" spans="1:3">
-      <c r="A215" t="s">
+    <row r="216" spans="1:3" customFormat="1">
+      <c r="A216" t="s">
         <v>607</v>
       </c>
-      <c r="B215" t="s">
+      <c r="B216" t="s">
         <v>608</v>
       </c>
-      <c r="C215" t="s">
+      <c r="C216" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="217" spans="1:3">
-      <c r="A217" t="s">
+    <row r="218" spans="1:3" customFormat="1">
+      <c r="A218" t="s">
         <v>468</v>
       </c>
-      <c r="B217" t="s">
+      <c r="B218" t="s">
         <v>1117</v>
       </c>
     </row>
-    <row r="218" spans="1:3">
-      <c r="A218" t="s">
+    <row r="219" spans="1:3" customFormat="1">
+      <c r="A219" t="s">
         <v>458</v>
       </c>
-      <c r="B218" t="s">
+      <c r="B219" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="219" spans="1:3">
-      <c r="A219" t="s">
+    <row r="220" spans="1:3" customFormat="1">
+      <c r="A220" t="s">
         <v>272</v>
       </c>
-      <c r="B219" t="s">
+      <c r="B220" t="s">
         <v>794</v>
       </c>
     </row>
-    <row r="220" spans="1:3">
-      <c r="A220" t="s">
+    <row r="221" spans="1:3" customFormat="1">
+      <c r="A221" t="s">
         <v>273</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B221" t="s">
         <v>795</v>
       </c>
     </row>
-    <row r="221" spans="1:3">
-      <c r="A221" t="s">
+    <row r="222" spans="1:3" customFormat="1">
+      <c r="A222" t="s">
         <v>281</v>
       </c>
-      <c r="B221" t="s">
+      <c r="B222" t="s">
         <v>796</v>
       </c>
     </row>
-    <row r="222" spans="1:3">
-      <c r="A222" t="s">
+    <row r="223" spans="1:3" customFormat="1">
+      <c r="A223" t="s">
         <v>280</v>
       </c>
-      <c r="B222" t="s">
+      <c r="B223" t="s">
         <v>798</v>
       </c>
     </row>
-    <row r="223" spans="1:3">
-      <c r="A223" t="s">
+    <row r="224" spans="1:3" customFormat="1">
+      <c r="A224" t="s">
         <v>282</v>
       </c>
-      <c r="B223" t="s">
+      <c r="B224" t="s">
         <v>797</v>
       </c>
     </row>
-    <row r="224" spans="1:3">
-      <c r="A224" t="s">
+    <row r="225" spans="1:2" customFormat="1">
+      <c r="A225" t="s">
         <v>613</v>
       </c>
-      <c r="B224" t="s">
+      <c r="B225" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="225" spans="1:3">
-      <c r="A225" t="s">
+    <row r="226" spans="1:2" customFormat="1">
+      <c r="A226" t="s">
         <v>484</v>
       </c>
-      <c r="B225" t="s">
+      <c r="B226" t="s">
         <v>1146</v>
       </c>
     </row>
-    <row r="227" spans="1:3">
-      <c r="A227" t="s">
+    <row r="228" spans="1:2" customFormat="1">
+      <c r="A228" t="s">
         <v>469</v>
       </c>
-      <c r="B227" t="s">
+      <c r="B228" t="s">
         <v>1114</v>
       </c>
     </row>
-    <row r="228" spans="1:3">
-      <c r="A228" t="s">
+    <row r="229" spans="1:2" customFormat="1">
+      <c r="A229" t="s">
         <v>459</v>
       </c>
-      <c r="B228" t="s">
+      <c r="B229" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="229" spans="1:3">
-      <c r="A229" t="s">
+    <row r="230" spans="1:2" customFormat="1">
+      <c r="A230" t="s">
         <v>285</v>
       </c>
-      <c r="B229" t="s">
+      <c r="B230" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="230" spans="1:3">
-      <c r="A230" t="s">
+    <row r="231" spans="1:2" customFormat="1">
+      <c r="A231" t="s">
         <v>286</v>
       </c>
-      <c r="B230" t="s">
+      <c r="B231" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="231" spans="1:3">
-      <c r="A231" t="s">
+    <row r="232" spans="1:2" customFormat="1">
+      <c r="A232" t="s">
         <v>287</v>
       </c>
-      <c r="B231" t="s">
+      <c r="B232" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="232" spans="1:3">
-      <c r="A232" t="s">
+    <row r="233" spans="1:2" customFormat="1">
+      <c r="A233" t="s">
         <v>289</v>
       </c>
-      <c r="B232" t="s">
+      <c r="B233" t="s">
         <v>790</v>
       </c>
     </row>
-    <row r="233" spans="1:3">
-      <c r="A233" t="s">
+    <row r="234" spans="1:2" customFormat="1">
+      <c r="A234" t="s">
         <v>290</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B234" t="s">
         <v>789</v>
       </c>
     </row>
-    <row r="234" spans="1:3">
-      <c r="A234" t="s">
+    <row r="235" spans="1:2" customFormat="1">
+      <c r="A235" t="s">
         <v>291</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B235" t="s">
         <v>791</v>
       </c>
     </row>
-    <row r="235" spans="1:3">
-      <c r="A235" t="s">
+    <row r="236" spans="1:2" customFormat="1">
+      <c r="A236" t="s">
         <v>292</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B236" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="236" spans="1:3">
-      <c r="A236" t="s">
+    <row r="237" spans="1:2" customFormat="1">
+      <c r="A237" t="s">
         <v>614</v>
       </c>
-      <c r="B236" t="s">
+      <c r="B237" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="237" spans="1:3">
-      <c r="A237" t="s">
+    <row r="238" spans="1:2" customFormat="1">
+      <c r="A238" t="s">
         <v>483</v>
       </c>
-      <c r="B237" t="s">
+      <c r="B238" t="s">
         <v>1147</v>
       </c>
     </row>
-    <row r="239" spans="1:3">
-      <c r="A239" t="s">
+    <row r="240" spans="1:2" customFormat="1">
+      <c r="A240" t="s">
         <v>470</v>
       </c>
-      <c r="B239" t="s">
+      <c r="B240" t="s">
         <v>1115</v>
       </c>
     </row>
-    <row r="240" spans="1:3">
-      <c r="A240" t="s">
+    <row r="241" spans="1:3" customFormat="1">
+      <c r="A241" t="s">
         <v>454</v>
       </c>
-      <c r="B240" t="s">
+      <c r="B241" t="s">
         <v>298</v>
       </c>
-      <c r="C240" t="s">
+      <c r="C241" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="241" spans="1:3">
-      <c r="A241" t="s">
+    <row r="242" spans="1:3" customFormat="1">
+      <c r="A242" t="s">
         <v>460</v>
       </c>
-      <c r="B241" t="s">
+      <c r="B242" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="242" spans="1:3">
-      <c r="A242" t="s">
+    <row r="243" spans="1:3" customFormat="1">
+      <c r="A243" t="s">
         <v>296</v>
       </c>
-      <c r="B242" t="s">
+      <c r="B243" t="s">
         <v>870</v>
       </c>
-      <c r="C242" t="s">
+      <c r="C243" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="243" spans="1:3">
-      <c r="A243" t="s">
+    <row r="244" spans="1:3" customFormat="1">
+      <c r="A244" t="s">
         <v>297</v>
       </c>
-      <c r="B243" t="s">
+      <c r="B244" t="s">
         <v>853</v>
       </c>
     </row>
-    <row r="244" spans="1:3">
-      <c r="A244" t="s">
+    <row r="245" spans="1:3" customFormat="1">
+      <c r="A245" t="s">
         <v>453</v>
       </c>
-      <c r="B244" t="s">
+      <c r="B245" t="s">
         <v>854</v>
       </c>
     </row>
-    <row r="245" spans="1:3">
-      <c r="A245" t="s">
+    <row r="246" spans="1:3" customFormat="1">
+      <c r="A246" t="s">
         <v>299</v>
       </c>
-      <c r="B245" t="s">
+      <c r="B246" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="246" spans="1:3">
-      <c r="A246" t="s">
+    <row r="247" spans="1:3" customFormat="1">
+      <c r="A247" t="s">
         <v>300</v>
       </c>
-      <c r="B246" t="s">
+      <c r="B247" t="s">
         <v>871</v>
       </c>
     </row>
-    <row r="247" spans="1:3">
-      <c r="A247" t="s">
+    <row r="248" spans="1:3" customFormat="1">
+      <c r="A248" t="s">
         <v>301</v>
       </c>
-      <c r="B247" t="s">
+      <c r="B248" t="s">
         <v>872</v>
       </c>
     </row>
-    <row r="248" spans="1:3">
-      <c r="A248" t="s">
+    <row r="249" spans="1:3" customFormat="1">
+      <c r="A249" t="s">
         <v>302</v>
       </c>
-      <c r="B248" t="s">
+      <c r="B249" t="s">
         <v>873</v>
       </c>
     </row>
-    <row r="249" spans="1:3">
-      <c r="A249" t="s">
+    <row r="250" spans="1:3" customFormat="1">
+      <c r="A250" t="s">
         <v>303</v>
       </c>
-      <c r="B249" t="s">
+      <c r="B250" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="250" spans="1:3">
-      <c r="A250" t="s">
+    <row r="251" spans="1:3" customFormat="1">
+      <c r="A251" t="s">
         <v>615</v>
       </c>
-      <c r="B250" t="s">
+      <c r="B251" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="251" spans="1:3">
-      <c r="A251" t="s">
+    <row r="252" spans="1:3" customFormat="1">
+      <c r="A252" t="s">
         <v>482</v>
       </c>
-      <c r="B251" t="s">
+      <c r="B252" t="s">
         <v>1148</v>
       </c>
     </row>
-    <row r="253" spans="1:3">
-      <c r="A253" t="s">
+    <row r="254" spans="1:3" customFormat="1">
+      <c r="A254" t="s">
         <v>648</v>
       </c>
-      <c r="B253" t="s">
+      <c r="B254" t="s">
         <v>649</v>
       </c>
-      <c r="C253" t="s">
+      <c r="C254" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="254" spans="1:3">
-      <c r="A254" t="s">
+    <row r="255" spans="1:3" customFormat="1">
+      <c r="A255" t="s">
         <v>499</v>
       </c>
-      <c r="B254" t="s">
+      <c r="B255" t="s">
         <v>502</v>
       </c>
-      <c r="C254" t="s">
+      <c r="C255" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="255" spans="1:3">
-      <c r="A255" t="s">
+    <row r="256" spans="1:3" customFormat="1">
+      <c r="A256" t="s">
         <v>500</v>
       </c>
-      <c r="B255" t="s">
+      <c r="B256" t="s">
         <v>501</v>
       </c>
-      <c r="C255" t="s">
+      <c r="C256" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="256" spans="1:3">
-      <c r="A256" t="s">
+    <row r="257" spans="1:3" customFormat="1">
+      <c r="A257" t="s">
         <v>528</v>
       </c>
-      <c r="B256" t="s">
+      <c r="B257" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="257" spans="1:3">
-      <c r="A257" t="s">
+    <row r="258" spans="1:3" customFormat="1">
+      <c r="A258" t="s">
         <v>320</v>
       </c>
-      <c r="B257" t="s">
+      <c r="B258" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="258" spans="1:3">
-      <c r="A258" t="s">
+    <row r="259" spans="1:3" customFormat="1">
+      <c r="A259" t="s">
         <v>321</v>
       </c>
-      <c r="B258" t="s">
+      <c r="B259" t="s">
         <v>307</v>
       </c>
-      <c r="C258" t="s">
+      <c r="C259" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="259" spans="1:3">
-      <c r="A259" t="s">
+    <row r="260" spans="1:3" customFormat="1">
+      <c r="A260" t="s">
         <v>461</v>
       </c>
-      <c r="B259" t="s">
+      <c r="B260" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="260" spans="1:3">
-      <c r="A260" t="s">
+    <row r="261" spans="1:3" customFormat="1">
+      <c r="A261" t="s">
         <v>322</v>
       </c>
-      <c r="B260" t="s">
+      <c r="B261" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="261" spans="1:3">
-      <c r="A261" t="s">
+    <row r="262" spans="1:3" customFormat="1">
+      <c r="A262" t="s">
         <v>323</v>
       </c>
-      <c r="B261" t="s">
+      <c r="B262" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="262" spans="1:3">
-      <c r="A262" t="s">
+    <row r="263" spans="1:3" customFormat="1">
+      <c r="A263" t="s">
         <v>324</v>
       </c>
-      <c r="B262" t="s">
+      <c r="B263" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="263" spans="1:3">
-      <c r="A263" t="s">
+    <row r="264" spans="1:3" customFormat="1">
+      <c r="A264" t="s">
         <v>325</v>
       </c>
-      <c r="B263" t="s">
+      <c r="B264" t="s">
         <v>311</v>
       </c>
-      <c r="C263" t="s">
+      <c r="C264" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="264" spans="1:3">
-      <c r="A264" t="s">
+    <row r="265" spans="1:3" customFormat="1">
+      <c r="A265" t="s">
         <v>326</v>
       </c>
-      <c r="B264" t="s">
+      <c r="B265" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="265" spans="1:3">
-      <c r="A265" t="s">
+    <row r="266" spans="1:3" customFormat="1">
+      <c r="A266" t="s">
         <v>327</v>
       </c>
-      <c r="B265" t="s">
+      <c r="B266" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="266" spans="1:3">
-      <c r="A266" t="s">
+    <row r="267" spans="1:3" customFormat="1">
+      <c r="A267" t="s">
         <v>328</v>
       </c>
-      <c r="B266" t="s">
+      <c r="B267" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="267" spans="1:3">
-      <c r="A267" t="s">
+    <row r="268" spans="1:3" customFormat="1">
+      <c r="A268" t="s">
         <v>329</v>
       </c>
-      <c r="B267" t="s">
+      <c r="B268" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="268" spans="1:3">
-      <c r="A268" t="s">
+    <row r="269" spans="1:3" customFormat="1">
+      <c r="A269" t="s">
         <v>330</v>
       </c>
-      <c r="B268" t="s">
+      <c r="B269" t="s">
         <v>316</v>
       </c>
-      <c r="C268" t="s">
+      <c r="C269" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="269" spans="1:3">
-      <c r="A269" t="s">
+    <row r="270" spans="1:3" customFormat="1">
+      <c r="A270" t="s">
         <v>331</v>
       </c>
-      <c r="B269" t="s">
+      <c r="B270" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="270" spans="1:3">
-      <c r="A270" t="s">
+    <row r="271" spans="1:3" customFormat="1">
+      <c r="A271" t="s">
         <v>332</v>
       </c>
-      <c r="B270" t="s">
+      <c r="B271" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="271" spans="1:3">
-      <c r="A271" t="s">
+    <row r="272" spans="1:3" customFormat="1">
+      <c r="A272" t="s">
         <v>333</v>
       </c>
-      <c r="B271" t="s">
+      <c r="B272" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="272" spans="1:3">
-      <c r="A272" t="s">
+    <row r="273" spans="1:3" customFormat="1">
+      <c r="A273" t="s">
         <v>481</v>
       </c>
-      <c r="B272" t="s">
+      <c r="B273" t="s">
         <v>1149</v>
       </c>
     </row>
-    <row r="274" spans="1:3">
-      <c r="A274" t="s">
+    <row r="275" spans="1:3" customFormat="1">
+      <c r="A275" t="s">
         <v>546</v>
       </c>
-      <c r="B274" t="s">
+      <c r="B275" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="275" spans="1:3">
-      <c r="A275" t="s">
+    <row r="276" spans="1:3" customFormat="1">
+      <c r="A276" t="s">
         <v>340</v>
       </c>
-      <c r="B275" t="s">
+      <c r="B276" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="276" spans="1:3">
-      <c r="A276" t="s">
+    <row r="277" spans="1:3" customFormat="1">
+      <c r="A277" t="s">
         <v>341</v>
       </c>
-      <c r="B276" t="s">
+      <c r="B277" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="277" spans="1:3">
-      <c r="A277" t="s">
+    <row r="278" spans="1:3" customFormat="1">
+      <c r="A278" t="s">
         <v>342</v>
       </c>
-      <c r="B277" t="s">
+      <c r="B278" t="s">
         <v>356</v>
       </c>
-      <c r="C277" t="s">
+      <c r="C278" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="278" spans="1:3">
-      <c r="A278" t="s">
+    <row r="279" spans="1:3" customFormat="1">
+      <c r="A279" t="s">
         <v>462</v>
       </c>
-      <c r="B278" t="s">
+      <c r="B279" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="279" spans="1:3">
-      <c r="A279" t="s">
+    <row r="280" spans="1:3" customFormat="1">
+      <c r="A280" t="s">
         <v>359</v>
       </c>
-      <c r="B279" t="s">
+      <c r="B280" t="s">
         <v>357</v>
       </c>
-      <c r="C279" t="s">
+      <c r="C280" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="280" spans="1:3">
-      <c r="A280" t="s">
+    <row r="281" spans="1:3" customFormat="1">
+      <c r="A281" t="s">
         <v>343</v>
       </c>
-      <c r="B280" t="s">
+      <c r="B281" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="281" spans="1:3">
-      <c r="A281" t="s">
+    <row r="282" spans="1:3" customFormat="1">
+      <c r="A282" t="s">
         <v>360</v>
       </c>
-      <c r="B281" t="s">
+      <c r="B282" t="s">
         <v>350</v>
       </c>
-      <c r="C281" t="s">
+      <c r="C282" t="s">
         <v>508</v>
       </c>
     </row>
-    <row r="282" spans="1:3">
-      <c r="A282" t="s">
+    <row r="283" spans="1:3" customFormat="1">
+      <c r="A283" t="s">
         <v>344</v>
       </c>
-      <c r="B282" t="s">
+      <c r="B283" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="283" spans="1:3">
-      <c r="A283" t="s">
+    <row r="284" spans="1:3" customFormat="1">
+      <c r="A284" t="s">
         <v>346</v>
       </c>
-      <c r="B283" t="s">
+      <c r="B284" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="284" spans="1:3">
-      <c r="A284" t="s">
+    <row r="285" spans="1:3" customFormat="1">
+      <c r="A285" t="s">
         <v>345</v>
       </c>
-      <c r="B284" t="s">
+      <c r="B285" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="285" spans="1:3">
-      <c r="A285" t="s">
+    <row r="286" spans="1:3" customFormat="1">
+      <c r="A286" t="s">
         <v>347</v>
       </c>
-      <c r="B285" t="s">
+      <c r="B286" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="286" spans="1:3">
-      <c r="A286" t="s">
+    <row r="287" spans="1:3" customFormat="1">
+      <c r="A287" t="s">
         <v>348</v>
       </c>
-      <c r="B286" t="s">
+      <c r="B287" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="287" spans="1:3">
-      <c r="A287" t="s">
+    <row r="288" spans="1:3" customFormat="1">
+      <c r="A288" t="s">
         <v>1076</v>
       </c>
-      <c r="B287" t="s">
+      <c r="B288" t="s">
         <v>1077</v>
-      </c>
-      <c r="C287" t="s">
-        <v>1078</v>
-      </c>
-    </row>
-    <row r="288" spans="1:3">
-      <c r="A288" t="s">
-        <v>1079</v>
-      </c>
-      <c r="B288" t="s">
-        <v>1080</v>
       </c>
       <c r="C288" t="s">
         <v>1078</v>
       </c>
     </row>
-    <row r="289" spans="1:3">
+    <row r="289" spans="1:3" customFormat="1">
       <c r="A289" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="B289" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="C289" t="s">
         <v>1078</v>
       </c>
     </row>
-    <row r="290" spans="1:3">
+    <row r="290" spans="1:3" customFormat="1">
       <c r="A290" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B290" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C290" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3" customFormat="1">
+      <c r="A291" t="s">
         <v>480</v>
       </c>
-      <c r="B290" t="s">
+      <c r="B291" t="s">
         <v>1150</v>
       </c>
     </row>
-    <row r="292" spans="1:3">
-      <c r="A292" t="s">
+    <row r="293" spans="1:3" customFormat="1">
+      <c r="A293" t="s">
         <v>650</v>
       </c>
-      <c r="B292" t="s">
+      <c r="B293" t="s">
         <v>668</v>
       </c>
-      <c r="C292" t="s">
+      <c r="C293" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="293" spans="1:3">
-      <c r="A293" t="s">
+    <row r="294" spans="1:3" customFormat="1">
+      <c r="A294" t="s">
         <v>1083</v>
       </c>
-      <c r="B293" t="s">
+      <c r="B294" t="s">
         <v>1084</v>
-      </c>
-      <c r="C293" t="s">
-        <v>1078</v>
-      </c>
-    </row>
-    <row r="294" spans="1:3">
-      <c r="A294" t="s">
-        <v>1085</v>
-      </c>
-      <c r="B294" t="s">
-        <v>1086</v>
       </c>
       <c r="C294" t="s">
         <v>1078</v>
       </c>
     </row>
-    <row r="295" spans="1:3">
+    <row r="295" spans="1:3" customFormat="1">
       <c r="A295" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="B295" t="s">
-        <v>1151</v>
+        <v>1086</v>
       </c>
       <c r="C295" t="s">
         <v>1078</v>
       </c>
     </row>
-    <row r="297" spans="1:3">
-      <c r="A297" t="s">
+    <row r="296" spans="1:3" customFormat="1">
+      <c r="A296" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B296" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C296" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" customFormat="1">
+      <c r="A298" t="s">
         <v>646</v>
       </c>
-      <c r="B297" t="s">
+      <c r="B298" t="s">
         <v>647</v>
       </c>
-      <c r="C297" t="s">
+      <c r="C298" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="298" spans="1:3">
-      <c r="A298" t="s">
+    <row r="299" spans="1:3" customFormat="1">
+      <c r="A299" t="s">
         <v>471</v>
       </c>
-      <c r="B298" t="s">
+      <c r="B299" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="299" spans="1:3">
-      <c r="A299" t="s">
+    <row r="300" spans="1:3" customFormat="1">
+      <c r="A300" t="s">
         <v>366</v>
       </c>
-      <c r="B299" t="s">
+      <c r="B300" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="300" spans="1:3">
-      <c r="A300" t="s">
+    <row r="301" spans="1:3" customFormat="1">
+      <c r="A301" t="s">
         <v>367</v>
       </c>
-      <c r="B300" t="s">
+      <c r="B301" t="s">
         <v>378</v>
       </c>
-      <c r="C300" t="s">
+      <c r="C301" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="301" spans="1:3">
-      <c r="A301" t="s">
+    <row r="302" spans="1:3" customFormat="1">
+      <c r="A302" t="s">
         <v>519</v>
       </c>
-      <c r="B301" t="s">
+      <c r="B302" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="302" spans="1:3">
-      <c r="A302" t="s">
+    <row r="303" spans="1:3" customFormat="1">
+      <c r="A303" t="s">
         <v>368</v>
       </c>
-      <c r="B302" t="s">
+      <c r="B303" t="s">
         <v>379</v>
-      </c>
-      <c r="C302" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="303" spans="1:3">
-      <c r="A303" t="s">
-        <v>369</v>
-      </c>
-      <c r="B303" t="s">
-        <v>380</v>
       </c>
       <c r="C303" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="304" spans="1:3">
+    <row r="304" spans="1:3" customFormat="1">
       <c r="A304" t="s">
+        <v>369</v>
+      </c>
+      <c r="B304" t="s">
+        <v>380</v>
+      </c>
+      <c r="C304" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" customFormat="1">
+      <c r="A305" t="s">
         <v>370</v>
       </c>
-      <c r="B304" t="s">
+      <c r="B305" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="305" spans="1:3">
-      <c r="A305" t="s">
+    <row r="306" spans="1:3" customFormat="1">
+      <c r="A306" t="s">
         <v>371</v>
       </c>
-      <c r="B305" t="s">
+      <c r="B306" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="306" spans="1:3">
-      <c r="A306" t="s">
+    <row r="307" spans="1:3" customFormat="1">
+      <c r="A307" t="s">
         <v>372</v>
       </c>
-      <c r="B306" t="s">
+      <c r="B307" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="307" spans="1:3">
-      <c r="A307" t="s">
+    <row r="308" spans="1:3" customFormat="1">
+      <c r="A308" t="s">
         <v>373</v>
       </c>
-      <c r="B307" t="s">
+      <c r="B308" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="308" spans="1:3">
-      <c r="A308" t="s">
+    <row r="309" spans="1:3" customFormat="1">
+      <c r="A309" t="s">
         <v>374</v>
       </c>
-      <c r="B308" t="s">
+      <c r="B309" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="309" spans="1:3">
-      <c r="A309" t="s">
+    <row r="310" spans="1:3" customFormat="1">
+      <c r="A310" t="s">
         <v>375</v>
       </c>
-      <c r="B309" t="s">
+      <c r="B310" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="310" spans="1:3">
-      <c r="A310" t="s">
+    <row r="311" spans="1:3" customFormat="1">
+      <c r="A311" t="s">
         <v>376</v>
       </c>
-      <c r="B310" t="s">
+      <c r="B311" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="311" spans="1:3">
-      <c r="A311" t="s">
+    <row r="312" spans="1:3" customFormat="1">
+      <c r="A312" t="s">
         <v>704</v>
       </c>
-      <c r="B311" t="s">
+      <c r="B312" t="s">
         <v>1091</v>
       </c>
-      <c r="C311" t="s">
+      <c r="C312" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="312" spans="1:3">
-      <c r="A312" t="s">
+    <row r="313" spans="1:3" customFormat="1">
+      <c r="A313" t="s">
         <v>1104</v>
       </c>
-      <c r="B312" t="s">
+      <c r="B313" t="s">
         <v>1105</v>
       </c>
     </row>
-    <row r="313" spans="1:3">
-      <c r="A313" t="s">
+    <row r="314" spans="1:3" customFormat="1">
+      <c r="A314" t="s">
         <v>478</v>
       </c>
-      <c r="B313" t="s">
+      <c r="B314" t="s">
         <v>1152</v>
       </c>
     </row>
-    <row r="314" spans="1:3">
-      <c r="A314" t="s">
+    <row r="315" spans="1:3" customFormat="1">
+      <c r="A315" t="s">
         <v>555</v>
       </c>
-      <c r="B314" t="s">
+      <c r="B315" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="316" spans="1:3">
-      <c r="A316" t="s">
+    <row r="317" spans="1:3" customFormat="1">
+      <c r="A317" t="s">
         <v>473</v>
       </c>
-      <c r="B316" t="s">
+      <c r="B317" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="317" spans="1:3">
-      <c r="A317" t="s">
+    <row r="318" spans="1:3" customFormat="1">
+      <c r="A318" t="s">
         <v>393</v>
       </c>
-      <c r="B317" t="s">
+      <c r="B318" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="318" spans="1:3">
-      <c r="A318" t="s">
+    <row r="319" spans="1:3" customFormat="1">
+      <c r="A319" t="s">
         <v>394</v>
       </c>
-      <c r="B318" t="s">
+      <c r="B319" t="s">
         <v>405</v>
       </c>
-      <c r="C318" t="s">
+      <c r="C319" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="319" spans="1:3">
-      <c r="A319" t="s">
+    <row r="320" spans="1:3" customFormat="1">
+      <c r="A320" t="s">
         <v>463</v>
       </c>
-      <c r="B319" t="s">
+      <c r="B320" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="320" spans="1:3">
-      <c r="A320" t="s">
+    <row r="321" spans="1:3" customFormat="1">
+      <c r="A321" t="s">
         <v>395</v>
       </c>
-      <c r="B320" t="s">
+      <c r="B321" t="s">
         <v>406</v>
-      </c>
-      <c r="C320" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="321" spans="1:3">
-      <c r="A321" t="s">
-        <v>396</v>
-      </c>
-      <c r="B321" t="s">
-        <v>407</v>
       </c>
       <c r="C321" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="322" spans="1:3">
+    <row r="322" spans="1:3" customFormat="1">
       <c r="A322" t="s">
+        <v>396</v>
+      </c>
+      <c r="B322" t="s">
+        <v>407</v>
+      </c>
+      <c r="C322" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" customFormat="1">
+      <c r="A323" t="s">
         <v>397</v>
       </c>
-      <c r="B322" t="s">
+      <c r="B323" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="323" spans="1:3">
-      <c r="A323" t="s">
+    <row r="324" spans="1:3" customFormat="1">
+      <c r="A324" t="s">
         <v>398</v>
       </c>
-      <c r="B323" t="s">
+      <c r="B324" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="324" spans="1:3">
-      <c r="A324" t="s">
+    <row r="325" spans="1:3" customFormat="1">
+      <c r="A325" t="s">
         <v>399</v>
       </c>
-      <c r="B324" t="s">
+      <c r="B325" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="325" spans="1:3">
-      <c r="A325" t="s">
+    <row r="326" spans="1:3" customFormat="1">
+      <c r="A326" t="s">
         <v>400</v>
       </c>
-      <c r="B325" t="s">
+      <c r="B326" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="326" spans="1:3">
-      <c r="A326" t="s">
+    <row r="327" spans="1:3" customFormat="1">
+      <c r="A327" t="s">
         <v>401</v>
       </c>
-      <c r="B326" t="s">
+      <c r="B327" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="327" spans="1:3">
-      <c r="A327" t="s">
+    <row r="328" spans="1:3" customFormat="1">
+      <c r="A328" t="s">
         <v>402</v>
       </c>
-      <c r="B327" t="s">
+      <c r="B328" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="328" spans="1:3">
-      <c r="A328" t="s">
+    <row r="329" spans="1:3" customFormat="1">
+      <c r="A329" t="s">
         <v>403</v>
       </c>
-      <c r="B328" t="s">
+      <c r="B329" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="329" spans="1:3">
-      <c r="A329" t="s">
+    <row r="330" spans="1:3" customFormat="1">
+      <c r="A330" t="s">
         <v>477</v>
       </c>
-      <c r="B329" t="s">
+      <c r="B330" t="s">
         <v>1152</v>
       </c>
     </row>
-    <row r="330" spans="1:3">
-      <c r="A330" t="s">
+    <row r="331" spans="1:3" customFormat="1">
+      <c r="A331" t="s">
         <v>562</v>
       </c>
-      <c r="B330" t="s">
+      <c r="B331" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="332" spans="1:3">
-      <c r="A332" t="s">
+    <row r="333" spans="1:3" customFormat="1">
+      <c r="A333" t="s">
         <v>644</v>
       </c>
-      <c r="B332" t="s">
+      <c r="B333" t="s">
         <v>645</v>
       </c>
-      <c r="C332" t="s">
+      <c r="C333" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="333" spans="1:3">
-      <c r="A333" t="s">
+    <row r="334" spans="1:3" customFormat="1">
+      <c r="A334" t="s">
         <v>387</v>
       </c>
-      <c r="B333" t="s">
+      <c r="B334" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="334" spans="1:3">
-      <c r="A334" t="s">
+    <row r="335" spans="1:3" customFormat="1">
+      <c r="A335" t="s">
         <v>388</v>
       </c>
-      <c r="B334" t="s">
+      <c r="B335" t="s">
         <v>564</v>
       </c>
-      <c r="C334" t="s">
+      <c r="C335" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="335" spans="1:3">
-      <c r="A335" t="s">
+    <row r="336" spans="1:3" customFormat="1">
+      <c r="A336" t="s">
         <v>464</v>
       </c>
-      <c r="B335" t="s">
+      <c r="B336" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="336" spans="1:3">
-      <c r="A336" t="s">
+    <row r="337" spans="1:3" customFormat="1">
+      <c r="A337" t="s">
         <v>389</v>
       </c>
-      <c r="B336" t="s">
+      <c r="B337" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="337" spans="1:3">
-      <c r="A337" t="s">
+    <row r="338" spans="1:3" customFormat="1">
+      <c r="A338" t="s">
         <v>390</v>
       </c>
-      <c r="B337" t="s">
+      <c r="B338" t="s">
         <v>566</v>
       </c>
     </row>
-    <row r="338" spans="1:3">
-      <c r="A338" t="s">
+    <row r="339" spans="1:3" customFormat="1">
+      <c r="A339" t="s">
         <v>391</v>
       </c>
-      <c r="B338" t="s">
+      <c r="B339" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="339" spans="1:3">
-      <c r="A339" t="s">
+    <row r="340" spans="1:3" customFormat="1">
+      <c r="A340" t="s">
         <v>1123</v>
       </c>
-      <c r="B339" t="s">
+      <c r="B340" t="s">
         <v>1124</v>
       </c>
-      <c r="C339" t="s">
+      <c r="C340" t="s">
         <v>1125</v>
       </c>
     </row>
-    <row r="340" spans="1:3">
-      <c r="A340" t="s">
+    <row r="341" spans="1:3" customFormat="1">
+      <c r="A341" t="s">
         <v>476</v>
       </c>
-      <c r="B340" t="s">
+      <c r="B341" t="s">
         <v>1153</v>
       </c>
     </row>
-    <row r="342" spans="1:3">
-      <c r="A342" t="s">
+    <row r="343" spans="1:3" customFormat="1">
+      <c r="A343" t="s">
         <v>718</v>
       </c>
-      <c r="B342" t="s">
+      <c r="B343" t="s">
         <v>719</v>
-      </c>
-      <c r="C342" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="343" spans="1:3">
-      <c r="A343" t="s">
-        <v>720</v>
-      </c>
-      <c r="B343" t="s">
-        <v>1154</v>
       </c>
       <c r="C343" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="345" spans="1:3">
-      <c r="A345" t="s">
+    <row r="344" spans="1:3" customFormat="1">
+      <c r="A344" t="s">
+        <v>720</v>
+      </c>
+      <c r="B344" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C344" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" customFormat="1">
+      <c r="A346" t="s">
         <v>726</v>
       </c>
-      <c r="B345" t="s">
+      <c r="B346" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="346" spans="1:3">
-      <c r="A346" t="s">
+    <row r="347" spans="1:3" customFormat="1">
+      <c r="A347" t="s">
         <v>728</v>
       </c>
-      <c r="B346" t="s">
+      <c r="B347" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="347" spans="1:3">
-      <c r="A347" t="s">
+    <row r="348" spans="1:3" customFormat="1">
+      <c r="A348" t="s">
         <v>730</v>
       </c>
-      <c r="B347" t="s">
+      <c r="B348" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="348" spans="1:3">
-      <c r="A348" t="s">
+    <row r="349" spans="1:3" customFormat="1">
+      <c r="A349" t="s">
         <v>732</v>
       </c>
-      <c r="B348" t="s">
+      <c r="B349" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="349" spans="1:3">
-      <c r="A349" t="s">
+    <row r="350" spans="1:3" customFormat="1">
+      <c r="A350" t="s">
         <v>734</v>
       </c>
-      <c r="B349" t="s">
+      <c r="B350" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="350" spans="1:3">
-      <c r="A350" t="s">
+    <row r="351" spans="1:3" customFormat="1">
+      <c r="A351" t="s">
         <v>736</v>
       </c>
-      <c r="B350" t="s">
+      <c r="B351" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="351" spans="1:3">
-      <c r="A351" t="s">
+    <row r="352" spans="1:3" customFormat="1">
+      <c r="A352" t="s">
         <v>738</v>
       </c>
-      <c r="B351" t="s">
+      <c r="B352" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="352" spans="1:3">
-      <c r="A352" t="s">
+    <row r="353" spans="1:2" customFormat="1">
+      <c r="A353" t="s">
         <v>740</v>
       </c>
-      <c r="B352" t="s">
+      <c r="B353" t="s">
         <v>741</v>
       </c>
     </row>
-    <row r="353" spans="1:2">
-      <c r="A353" t="s">
+    <row r="354" spans="1:2" customFormat="1">
+      <c r="A354" t="s">
         <v>742</v>
       </c>
-      <c r="B353" t="s">
+      <c r="B354" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="354" spans="1:2">
-      <c r="A354" t="s">
+    <row r="355" spans="1:2" customFormat="1">
+      <c r="A355" t="s">
         <v>744</v>
       </c>
-      <c r="B354" t="s">
+      <c r="B355" t="s">
         <v>745</v>
       </c>
     </row>
-    <row r="355" spans="1:2">
-      <c r="A355" t="s">
+    <row r="356" spans="1:2" customFormat="1">
+      <c r="A356" t="s">
         <v>746</v>
       </c>
-      <c r="B355" t="s">
+      <c r="B356" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="356" spans="1:2">
-      <c r="A356" t="s">
+    <row r="357" spans="1:2" customFormat="1">
+      <c r="A357" t="s">
         <v>748</v>
       </c>
-      <c r="B356" t="s">
+      <c r="B357" t="s">
         <v>749</v>
       </c>
     </row>
-    <row r="357" spans="1:2">
-      <c r="A357" t="s">
+    <row r="358" spans="1:2" customFormat="1">
+      <c r="A358" t="s">
         <v>750</v>
       </c>
-      <c r="B357" t="s">
+      <c r="B358" t="s">
         <v>751</v>
       </c>
     </row>
-    <row r="358" spans="1:2">
-      <c r="A358" t="s">
+    <row r="359" spans="1:2" customFormat="1">
+      <c r="A359" t="s">
         <v>752</v>
       </c>
-      <c r="B358" t="s">
+      <c r="B359" t="s">
         <v>753</v>
       </c>
     </row>
-    <row r="359" spans="1:2">
-      <c r="A359" t="s">
+    <row r="360" spans="1:2" customFormat="1">
+      <c r="A360" t="s">
         <v>754</v>
       </c>
-      <c r="B359" t="s">
+      <c r="B360" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="360" spans="1:2">
-      <c r="A360" t="s">
+    <row r="361" spans="1:2" customFormat="1">
+      <c r="A361" t="s">
         <v>756</v>
       </c>
-      <c r="B360" t="s">
+      <c r="B361" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="361" spans="1:2">
-      <c r="A361" t="s">
+    <row r="362" spans="1:2" customFormat="1">
+      <c r="A362" t="s">
         <v>1119</v>
       </c>
-      <c r="B361" t="s">
+      <c r="B362" t="s">
         <v>1120</v>
       </c>
     </row>
-    <row r="362" spans="1:2">
-      <c r="A362" t="s">
+    <row r="363" spans="1:2" customFormat="1">
+      <c r="A363" t="s">
         <v>758</v>
       </c>
-      <c r="B362" t="s">
+      <c r="B363" t="s">
         <v>759</v>
       </c>
     </row>
-    <row r="363" spans="1:2">
-      <c r="A363" t="s">
+    <row r="364" spans="1:2" customFormat="1">
+      <c r="A364" t="s">
         <v>1122</v>
       </c>
-      <c r="B363" t="s">
+      <c r="B364" t="s">
         <v>1155</v>
       </c>
     </row>
-    <row r="365" spans="1:2">
-      <c r="A365" t="s">
+    <row r="366" spans="1:2" customFormat="1">
+      <c r="A366" t="s">
         <v>760</v>
       </c>
-      <c r="B365" t="s">
+      <c r="B366" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="366" spans="1:2">
-      <c r="A366" t="s">
+    <row r="367" spans="1:2" customFormat="1">
+      <c r="A367" t="s">
         <v>762</v>
       </c>
-      <c r="B366" t="s">
+      <c r="B367" t="s">
         <v>763</v>
       </c>
     </row>
-    <row r="367" spans="1:2">
-      <c r="A367" t="s">
+    <row r="368" spans="1:2" customFormat="1">
+      <c r="A368" t="s">
         <v>764</v>
       </c>
-      <c r="B367" t="s">
+      <c r="B368" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="368" spans="1:2">
-      <c r="A368" t="s">
+    <row r="369" spans="1:2" customFormat="1">
+      <c r="A369" t="s">
         <v>766</v>
       </c>
-      <c r="B368" t="s">
+      <c r="B369" t="s">
         <v>767</v>
       </c>
     </row>
-    <row r="369" spans="1:2">
-      <c r="A369" t="s">
+    <row r="370" spans="1:2" customFormat="1">
+      <c r="A370" t="s">
         <v>768</v>
       </c>
-      <c r="B369" t="s">
+      <c r="B370" t="s">
         <v>769</v>
       </c>
     </row>
-    <row r="370" spans="1:2">
-      <c r="A370" t="s">
+    <row r="371" spans="1:2" customFormat="1">
+      <c r="A371" t="s">
         <v>770</v>
       </c>
-      <c r="B370" t="s">
+      <c r="B371" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="371" spans="1:2">
-      <c r="A371" t="s">
+    <row r="372" spans="1:2" customFormat="1">
+      <c r="A372" t="s">
         <v>772</v>
       </c>
-      <c r="B371" t="s">
+      <c r="B372" t="s">
         <v>773</v>
       </c>
     </row>
-    <row r="372" spans="1:2">
-      <c r="A372" t="s">
+    <row r="373" spans="1:2" customFormat="1">
+      <c r="A373" t="s">
         <v>774</v>
       </c>
-      <c r="B372" t="s">
+      <c r="B373" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="373" spans="1:2">
-      <c r="A373" t="s">
+    <row r="374" spans="1:2" customFormat="1">
+      <c r="A374" t="s">
         <v>775</v>
       </c>
-      <c r="B373" t="s">
+      <c r="B374" t="s">
         <v>776</v>
       </c>
     </row>
-    <row r="374" spans="1:2">
-      <c r="A374" t="s">
+    <row r="375" spans="1:2" customFormat="1">
+      <c r="A375" t="s">
         <v>777</v>
       </c>
-      <c r="B374" t="s">
+      <c r="B375" t="s">
         <v>778</v>
       </c>
     </row>
-    <row r="375" spans="1:2">
-      <c r="A375" t="s">
+    <row r="376" spans="1:2" customFormat="1">
+      <c r="A376" t="s">
         <v>779</v>
       </c>
-      <c r="B375" t="s">
+      <c r="B376" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="376" spans="1:2">
-      <c r="A376" t="s">
+    <row r="377" spans="1:2" customFormat="1">
+      <c r="A377" t="s">
         <v>781</v>
       </c>
-      <c r="B376" t="s">
+      <c r="B377" t="s">
         <v>1156</v>
       </c>
     </row>
-    <row r="378" spans="1:2">
-      <c r="A378" t="s">
+    <row r="379" spans="1:2" customFormat="1">
+      <c r="A379" t="s">
         <v>782</v>
       </c>
-      <c r="B378" t="s">
+      <c r="B379" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="379" spans="1:2">
-      <c r="A379" t="s">
+    <row r="380" spans="1:2" customFormat="1">
+      <c r="A380" t="s">
         <v>783</v>
       </c>
-      <c r="B379" t="s">
+      <c r="B380" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="380" spans="1:2">
-      <c r="A380" t="s">
+    <row r="381" spans="1:2" customFormat="1">
+      <c r="A381" t="s">
         <v>785</v>
       </c>
-      <c r="B380" t="s">
+      <c r="B381" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="381" spans="1:2">
-      <c r="A381" t="s">
+    <row r="382" spans="1:2" customFormat="1">
+      <c r="A382" t="s">
         <v>786</v>
       </c>
-      <c r="B381" t="s">
+      <c r="B382" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="383" spans="1:2">
-      <c r="A383" t="s">
+    <row r="384" spans="1:2" customFormat="1">
+      <c r="A384" t="s">
         <v>808</v>
       </c>
-      <c r="B383" t="s">
+      <c r="B384" t="s">
         <v>809</v>
       </c>
     </row>
-    <row r="384" spans="1:2">
-      <c r="A384" t="s">
+    <row r="385" spans="1:2" customFormat="1">
+      <c r="A385" t="s">
         <v>807</v>
       </c>
-      <c r="B384" t="s">
+      <c r="B385" t="s">
         <v>806</v>
       </c>
     </row>
-    <row r="385" spans="1:2">
-      <c r="A385" t="s">
+    <row r="386" spans="1:2" customFormat="1">
+      <c r="A386" t="s">
         <v>801</v>
       </c>
-      <c r="B385" t="s">
+      <c r="B386" t="s">
         <v>802</v>
       </c>
     </row>
-    <row r="386" spans="1:2">
-      <c r="A386" t="s">
+    <row r="387" spans="1:2" customFormat="1">
+      <c r="A387" t="s">
         <v>799</v>
       </c>
-      <c r="B386" t="s">
+      <c r="B387" t="s">
         <v>803</v>
       </c>
     </row>
-    <row r="387" spans="1:2">
-      <c r="A387" t="s">
+    <row r="388" spans="1:2" customFormat="1">
+      <c r="A388" t="s">
         <v>800</v>
       </c>
-      <c r="B387" t="s">
+      <c r="B388" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="388" spans="1:2">
-      <c r="A388" t="s">
+    <row r="389" spans="1:2" customFormat="1">
+      <c r="A389" t="s">
         <v>805</v>
       </c>
-      <c r="B388" t="s">
+      <c r="B389" t="s">
         <v>1157</v>
       </c>
     </row>
-    <row r="390" spans="1:2">
-      <c r="A390" t="s">
+    <row r="391" spans="1:2" customFormat="1">
+      <c r="A391" t="s">
         <v>812</v>
       </c>
-      <c r="B390" t="s">
+      <c r="B391" t="s">
         <v>817</v>
       </c>
     </row>
-    <row r="391" spans="1:2">
-      <c r="A391" t="s">
+    <row r="392" spans="1:2" customFormat="1">
+      <c r="A392" t="s">
         <v>819</v>
       </c>
-      <c r="B391" t="s">
+      <c r="B392" t="s">
         <v>818</v>
       </c>
     </row>
-    <row r="392" spans="1:2">
-      <c r="A392" t="s">
+    <row r="393" spans="1:2" customFormat="1">
+      <c r="A393" t="s">
         <v>813</v>
       </c>
-      <c r="B392" t="s">
+      <c r="B393" t="s">
         <v>802</v>
       </c>
     </row>
-    <row r="393" spans="1:2">
-      <c r="A393" t="s">
+    <row r="394" spans="1:2" customFormat="1">
+      <c r="A394" t="s">
         <v>814</v>
       </c>
-      <c r="B393" t="s">
+      <c r="B394" t="s">
         <v>803</v>
       </c>
     </row>
-    <row r="394" spans="1:2">
-      <c r="A394" t="s">
+    <row r="395" spans="1:2" customFormat="1">
+      <c r="A395" t="s">
         <v>815</v>
       </c>
-      <c r="B394" t="s">
+      <c r="B395" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="395" spans="1:2">
-      <c r="A395" t="s">
+    <row r="396" spans="1:2" customFormat="1">
+      <c r="A396" t="s">
         <v>816</v>
       </c>
-      <c r="B395" t="s">
+      <c r="B396" t="s">
         <v>1158</v>
       </c>
     </row>
-    <row r="397" spans="1:2">
-      <c r="A397" t="s">
+    <row r="398" spans="1:2" customFormat="1">
+      <c r="A398" t="s">
         <v>824</v>
       </c>
-      <c r="B397" t="s">
+      <c r="B398" t="s">
         <v>825</v>
       </c>
     </row>
-    <row r="398" spans="1:2">
-      <c r="A398" t="s">
+    <row r="399" spans="1:2" customFormat="1">
+      <c r="A399" t="s">
         <v>826</v>
       </c>
-      <c r="B398" t="s">
+      <c r="B399" t="s">
         <v>1116</v>
       </c>
     </row>
-    <row r="399" spans="1:2">
-      <c r="A399" t="s">
+    <row r="400" spans="1:2" customFormat="1">
+      <c r="A400" t="s">
         <v>827</v>
       </c>
-      <c r="B399" t="s">
+      <c r="B400" t="s">
         <v>1020</v>
       </c>
     </row>
-    <row r="400" spans="1:2">
-      <c r="A400" t="s">
+    <row r="401" spans="1:2" customFormat="1">
+      <c r="A401" t="s">
         <v>829</v>
       </c>
-      <c r="B400" t="s">
+      <c r="B401" t="s">
         <v>1021</v>
       </c>
     </row>
-    <row r="401" spans="1:2">
-      <c r="A401" t="s">
+    <row r="402" spans="1:2" customFormat="1">
+      <c r="A402" t="s">
         <v>835</v>
       </c>
-      <c r="B401" t="s">
+      <c r="B402" t="s">
         <v>1022</v>
       </c>
     </row>
-    <row r="402" spans="1:2">
-      <c r="A402" t="s">
+    <row r="403" spans="1:2" customFormat="1">
+      <c r="A403" t="s">
         <v>836</v>
       </c>
-      <c r="B402" t="s">
+      <c r="B403" t="s">
         <v>1023</v>
       </c>
     </row>
-    <row r="403" spans="1:2">
-      <c r="A403" t="s">
+    <row r="404" spans="1:2" customFormat="1">
+      <c r="A404" t="s">
         <v>837</v>
       </c>
-      <c r="B403" t="s">
+      <c r="B404" t="s">
         <v>1024</v>
       </c>
     </row>
-    <row r="404" spans="1:2">
-      <c r="A404" t="s">
+    <row r="405" spans="1:2" customFormat="1">
+      <c r="A405" t="s">
         <v>840</v>
       </c>
-      <c r="B404" t="s">
+      <c r="B405" t="s">
         <v>1025</v>
       </c>
     </row>
-    <row r="405" spans="1:2">
-      <c r="A405" t="s">
+    <row r="406" spans="1:2" customFormat="1">
+      <c r="A406" t="s">
         <v>841</v>
       </c>
-      <c r="B405" t="s">
+      <c r="B406" t="s">
         <v>1026</v>
       </c>
     </row>
-    <row r="406" spans="1:2">
-      <c r="A406" t="s">
+    <row r="407" spans="1:2" customFormat="1">
+      <c r="A407" t="s">
         <v>842</v>
       </c>
-      <c r="B406" t="s">
+      <c r="B407" t="s">
         <v>1027</v>
       </c>
     </row>
-    <row r="407" spans="1:2">
-      <c r="A407" t="s">
+    <row r="408" spans="1:2" customFormat="1">
+      <c r="A408" t="s">
         <v>843</v>
       </c>
-      <c r="B407" t="s">
+      <c r="B408" t="s">
         <v>1028</v>
       </c>
     </row>
-    <row r="408" spans="1:2">
-      <c r="A408" t="s">
+    <row r="409" spans="1:2" customFormat="1">
+      <c r="A409" t="s">
         <v>844</v>
       </c>
-      <c r="B408" t="s">
+      <c r="B409" t="s">
         <v>1029</v>
       </c>
     </row>
-    <row r="409" spans="1:2">
-      <c r="A409" t="s">
+    <row r="410" spans="1:2" customFormat="1">
+      <c r="A410" t="s">
         <v>845</v>
       </c>
-      <c r="B409" t="s">
+      <c r="B410" t="s">
         <v>834</v>
       </c>
     </row>
-    <row r="410" spans="1:2">
-      <c r="A410" t="s">
+    <row r="411" spans="1:2" customFormat="1">
+      <c r="A411" t="s">
         <v>846</v>
       </c>
-      <c r="B410" t="s">
+      <c r="B411" t="s">
         <v>1030</v>
       </c>
     </row>
-    <row r="411" spans="1:2">
-      <c r="A411" t="s">
+    <row r="412" spans="1:2" customFormat="1">
+      <c r="A412" t="s">
         <v>847</v>
       </c>
-      <c r="B411" t="s">
+      <c r="B412" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="412" spans="1:2">
-      <c r="A412" t="s">
+    <row r="413" spans="1:2" customFormat="1">
+      <c r="A413" t="s">
         <v>848</v>
       </c>
-      <c r="B412" t="s">
+      <c r="B413" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="413" spans="1:2">
-      <c r="A413" t="s">
+    <row r="414" spans="1:2" customFormat="1">
+      <c r="A414" t="s">
         <v>839</v>
       </c>
-      <c r="B413" t="s">
+      <c r="B414" t="s">
         <v>608</v>
       </c>
     </row>
-    <row r="414" spans="1:2">
-      <c r="A414" t="s">
+    <row r="415" spans="1:2" customFormat="1">
+      <c r="A415" t="s">
         <v>838</v>
       </c>
-      <c r="B414" t="s">
+      <c r="B415" t="s">
         <v>1159</v>
       </c>
     </row>
-    <row r="415" spans="1:2">
-      <c r="A415" t="s">
+    <row r="416" spans="1:2" customFormat="1">
+      <c r="A416" t="s">
         <v>1031</v>
       </c>
-      <c r="B415" t="s">
+      <c r="B416" t="s">
         <v>1032</v>
       </c>
     </row>
-    <row r="416" spans="1:2">
-      <c r="A416" t="s">
+    <row r="417" spans="1:2" customFormat="1">
+      <c r="A417" t="s">
         <v>1033</v>
       </c>
-      <c r="B416" t="s">
+      <c r="B417" t="s">
         <v>1034</v>
       </c>
     </row>
-    <row r="417" spans="1:2">
-      <c r="A417" t="s">
+    <row r="418" spans="1:2" customFormat="1">
+      <c r="A418" t="s">
         <v>1035</v>
       </c>
-      <c r="B417" t="s">
+      <c r="B418" t="s">
         <v>1036</v>
       </c>
     </row>
-    <row r="418" spans="1:2">
-      <c r="A418" t="s">
+    <row r="419" spans="1:2" customFormat="1">
+      <c r="A419" t="s">
         <v>1037</v>
       </c>
-      <c r="B418" t="s">
+      <c r="B419" t="s">
         <v>1038</v>
       </c>
     </row>
-    <row r="419" spans="1:2">
-      <c r="A419" t="s">
+    <row r="420" spans="1:2" customFormat="1">
+      <c r="A420" t="s">
         <v>1039</v>
       </c>
-      <c r="B419" t="s">
+      <c r="B420" t="s">
         <v>1040</v>
       </c>
     </row>
-    <row r="420" spans="1:2">
-      <c r="A420" t="s">
+    <row r="421" spans="1:2" customFormat="1">
+      <c r="A421" t="s">
         <v>1041</v>
       </c>
-      <c r="B420" t="s">
+      <c r="B421" t="s">
         <v>1042</v>
-      </c>
-    </row>
-    <row r="421" spans="1:2">
-      <c r="A421" t="s">
-        <v>1043</v>
-      </c>
-      <c r="B421" t="s">
-        <v>1044</v>
       </c>
     </row>
     <row r="422" spans="1:2" customFormat="1">
       <c r="A422" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="B422" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="423" spans="1:2" customFormat="1">
       <c r="A423" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B423" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="424" spans="1:2" customFormat="1">
+      <c r="A424" t="s">
         <v>1168</v>
       </c>
-      <c r="B423" t="s">
+      <c r="B424" t="s">
         <v>1169</v>
-      </c>
-    </row>
-    <row r="425" spans="1:2" customFormat="1">
-      <c r="A425" t="s">
-        <v>888</v>
-      </c>
-      <c r="B425" t="s">
-        <v>889</v>
       </c>
     </row>
     <row r="426" spans="1:2" customFormat="1">
       <c r="A426" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="B426" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
     </row>
     <row r="427" spans="1:2" customFormat="1">
       <c r="A427" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="B427" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
     </row>
     <row r="428" spans="1:2" customFormat="1">
       <c r="A428" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="B428" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
     </row>
     <row r="429" spans="1:2" customFormat="1">
       <c r="A429" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="B429" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
     </row>
     <row r="430" spans="1:2" customFormat="1">
       <c r="A430" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="B430" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
     </row>
     <row r="431" spans="1:2" customFormat="1">
       <c r="A431" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="B431" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
     </row>
     <row r="432" spans="1:2" customFormat="1">
       <c r="A432" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="B432" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
     </row>
     <row r="433" spans="1:2" customFormat="1">
       <c r="A433" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="B433" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
     </row>
     <row r="434" spans="1:2" customFormat="1">
       <c r="A434" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="B434" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
     </row>
     <row r="435" spans="1:2" customFormat="1">
       <c r="A435" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="B435" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
     </row>
     <row r="436" spans="1:2" customFormat="1">
       <c r="A436" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="B436" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
     </row>
     <row r="437" spans="1:2" customFormat="1">
       <c r="A437" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="B437" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
     </row>
     <row r="438" spans="1:2" customFormat="1">
       <c r="A438" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
       <c r="B438" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
     </row>
     <row r="439" spans="1:2" customFormat="1">
       <c r="A439" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="B439" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
     </row>
     <row r="440" spans="1:2" customFormat="1">
       <c r="A440" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="B440" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
     </row>
     <row r="441" spans="1:2" customFormat="1">
       <c r="A441" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
       <c r="B441" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
     </row>
     <row r="442" spans="1:2" customFormat="1">
       <c r="A442" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="B442" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
     </row>
     <row r="443" spans="1:2" customFormat="1">
       <c r="A443" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="B443" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
     </row>
     <row r="444" spans="1:2" customFormat="1">
       <c r="A444" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="B444" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
     </row>
     <row r="445" spans="1:2" customFormat="1">
       <c r="A445" t="s">
+        <v>926</v>
+      </c>
+      <c r="B445" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="446" spans="1:2" customFormat="1">
+      <c r="A446" t="s">
         <v>928</v>
       </c>
-      <c r="B445" t="s">
+      <c r="B446" t="s">
         <v>1160</v>
-      </c>
-    </row>
-    <row r="447" spans="1:2" customFormat="1">
-      <c r="A447" t="s">
-        <v>1127</v>
-      </c>
-      <c r="B447" t="s">
-        <v>1128</v>
       </c>
     </row>
     <row r="448" spans="1:2" customFormat="1">
       <c r="A448" t="s">
-        <v>929</v>
+        <v>1127</v>
       </c>
       <c r="B448" t="s">
-        <v>930</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="449" spans="1:2" customFormat="1">
       <c r="A449" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="B449" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
     </row>
     <row r="450" spans="1:2" customFormat="1">
       <c r="A450" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="B450" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
     </row>
     <row r="451" spans="1:2" customFormat="1">
       <c r="A451" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="B451" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
     </row>
     <row r="452" spans="1:2" customFormat="1">
       <c r="A452" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="B452" t="s">
-        <v>1088</v>
+        <v>936</v>
       </c>
     </row>
     <row r="453" spans="1:2" customFormat="1">
       <c r="A453" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="B453" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="454" spans="1:2" customFormat="1">
       <c r="A454" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="B454" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="455" spans="1:2" customFormat="1">
       <c r="A455" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="B455" t="s">
-        <v>941</v>
+        <v>1090</v>
       </c>
     </row>
     <row r="456" spans="1:2" customFormat="1">
       <c r="A456" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="B456" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
     </row>
     <row r="457" spans="1:2" customFormat="1">
       <c r="A457" t="s">
+        <v>942</v>
+      </c>
+      <c r="B457" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="458" spans="1:2" customFormat="1">
+      <c r="A458" t="s">
         <v>944</v>
       </c>
-      <c r="B457" t="s">
+      <c r="B458" t="s">
         <v>1161</v>
-      </c>
-    </row>
-    <row r="459" spans="1:2" customFormat="1">
-      <c r="A459" t="s">
-        <v>951</v>
-      </c>
-      <c r="B459" t="s">
-        <v>952</v>
       </c>
     </row>
     <row r="460" spans="1:2" customFormat="1">
       <c r="A460" t="s">
+        <v>951</v>
+      </c>
+      <c r="B460" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="461" spans="1:2" customFormat="1">
+      <c r="A461" t="s">
         <v>953</v>
       </c>
-      <c r="B460" t="s">
+      <c r="B461" t="s">
         <v>1162</v>
-      </c>
-    </row>
-    <row r="462" spans="1:2" customFormat="1">
-      <c r="A462" t="s">
-        <v>954</v>
-      </c>
-      <c r="B462" t="s">
-        <v>955</v>
       </c>
     </row>
     <row r="463" spans="1:2" customFormat="1">
       <c r="A463" t="s">
+        <v>954</v>
+      </c>
+      <c r="B463" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="464" spans="1:2" customFormat="1">
+      <c r="A464" t="s">
         <v>956</v>
       </c>
-      <c r="B463" t="s">
+      <c r="B464" t="s">
         <v>1163</v>
       </c>
     </row>
-    <row r="465" spans="1:2" customFormat="1">
-      <c r="A465" t="s">
-        <v>957</v>
-      </c>
-      <c r="B465" t="s">
-        <v>958</v>
-      </c>
-    </row>
+    <row r="465" spans="1:2" customFormat="1"/>
     <row r="466" spans="1:2" customFormat="1">
       <c r="A466" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="B466" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
     </row>
     <row r="467" spans="1:2" customFormat="1">
       <c r="A467" t="s">
+        <v>959</v>
+      </c>
+      <c r="B467" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="468" spans="1:2" customFormat="1">
+      <c r="A468" t="s">
         <v>961</v>
       </c>
-      <c r="B467" t="s">
+      <c r="B468" t="s">
         <v>1164</v>
-      </c>
-    </row>
-    <row r="469" spans="1:2" customFormat="1">
-      <c r="A469" t="s">
-        <v>962</v>
-      </c>
-      <c r="B469" t="s">
-        <v>963</v>
       </c>
     </row>
     <row r="470" spans="1:2" customFormat="1">
       <c r="A470" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="B470" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
     </row>
     <row r="471" spans="1:2" customFormat="1">
       <c r="A471" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
       <c r="B471" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
     </row>
     <row r="472" spans="1:2" customFormat="1">
       <c r="A472" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
       <c r="B472" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="473" spans="1:2" customFormat="1">
       <c r="A473" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="B473" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
     </row>
     <row r="474" spans="1:2" customFormat="1">
       <c r="A474" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="B474" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
     </row>
     <row r="475" spans="1:2" customFormat="1">
       <c r="A475" t="s">
+        <v>972</v>
+      </c>
+      <c r="B475" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2" customFormat="1">
+      <c r="A476" t="s">
         <v>974</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B476" t="s">
         <v>1129</v>
-      </c>
-    </row>
-    <row r="477" spans="1:2" customFormat="1">
-      <c r="A477" t="s">
-        <v>975</v>
-      </c>
-      <c r="B477" t="s">
-        <v>976</v>
       </c>
     </row>
     <row r="478" spans="1:2" customFormat="1">
       <c r="A478" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="B478" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
     </row>
     <row r="479" spans="1:2" customFormat="1">
       <c r="A479" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="B479" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
     </row>
     <row r="480" spans="1:2" customFormat="1">
       <c r="A480" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="B480" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
     </row>
     <row r="481" spans="1:2" customFormat="1">
       <c r="A481" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="B481" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
     </row>
     <row r="482" spans="1:2" customFormat="1">
       <c r="A482" t="s">
+        <v>983</v>
+      </c>
+      <c r="B482" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="483" spans="1:2" customFormat="1">
+      <c r="A483" t="s">
         <v>985</v>
       </c>
-      <c r="B482" t="s">
+      <c r="B483" t="s">
         <v>1130</v>
-      </c>
-    </row>
-    <row r="484" spans="1:2" customFormat="1">
-      <c r="A484" t="s">
-        <v>986</v>
-      </c>
-      <c r="B484" t="s">
-        <v>987</v>
       </c>
     </row>
     <row r="485" spans="1:2" customFormat="1">
       <c r="A485" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="B485" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
     </row>
     <row r="486" spans="1:2" customFormat="1">
       <c r="A486" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="B486" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
     </row>
     <row r="487" spans="1:2" customFormat="1">
       <c r="A487" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="B487" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
     </row>
     <row r="488" spans="1:2" customFormat="1">
       <c r="A488" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="B488" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
     </row>
     <row r="489" spans="1:2" customFormat="1">
       <c r="A489" t="s">
+        <v>994</v>
+      </c>
+      <c r="B489" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="490" spans="1:2" customFormat="1">
+      <c r="A490" t="s">
         <v>996</v>
       </c>
-      <c r="B489" t="s">
+      <c r="B490" t="s">
         <v>1131</v>
-      </c>
-    </row>
-    <row r="491" spans="1:2" customFormat="1">
-      <c r="A491" t="s">
-        <v>997</v>
-      </c>
-      <c r="B491" t="s">
-        <v>998</v>
       </c>
     </row>
     <row r="492" spans="1:2" customFormat="1">
       <c r="A492" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
       <c r="B492" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
     </row>
     <row r="493" spans="1:2" customFormat="1">
       <c r="A493" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="B493" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="494" spans="1:2" customFormat="1">
       <c r="A494" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="B494" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="495" spans="1:2" customFormat="1">
       <c r="A495" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B495" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="496" spans="1:2" customFormat="1">
+      <c r="A496" t="s">
         <v>1005</v>
       </c>
-      <c r="B495" t="s">
+      <c r="B496" t="s">
         <v>1132</v>
       </c>
     </row>
-    <row r="497" spans="1:2" customFormat="1">
-      <c r="A497" t="s">
-        <v>1047</v>
-      </c>
-      <c r="B497" t="s">
-        <v>1048</v>
-      </c>
-    </row>
+    <row r="497" spans="1:2" customFormat="1"/>
     <row r="498" spans="1:2" customFormat="1">
       <c r="A498" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
       <c r="B498" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="499" spans="1:2" customFormat="1">
       <c r="A499" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
       <c r="B499" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="500" spans="1:2" customFormat="1">
       <c r="A500" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
       <c r="B500" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
     </row>
     <row r="501" spans="1:2" customFormat="1">
       <c r="A501" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
       <c r="B501" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="502" spans="1:2" customFormat="1">
       <c r="A502" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
       <c r="B502" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="503" spans="1:2" customFormat="1">
       <c r="A503" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="B503" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="504" spans="1:2" customFormat="1">
       <c r="A504" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="B504" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="505" spans="1:2" customFormat="1">
       <c r="A505" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
       <c r="B505" t="s">
-        <v>1064</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="506" spans="1:2" customFormat="1">
       <c r="A506" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="B506" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="507" spans="1:2" customFormat="1">
       <c r="A507" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="B507" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="508" spans="1:2" customFormat="1">
       <c r="A508" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
       <c r="B508" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="509" spans="1:2" customFormat="1">
       <c r="A509" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="B509" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="510" spans="1:2" customFormat="1">
       <c r="A510" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B510" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="511" spans="1:2" customFormat="1">
+      <c r="A511" t="s">
         <v>1073</v>
       </c>
-      <c r="B510" t="s">
+      <c r="B511" t="s">
         <v>1133</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A448:A457">
+  <conditionalFormatting sqref="A449:A458">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A465:A466 A462:A463 A459:A460">
+  <conditionalFormatting sqref="A466:A467 A463:A464 A460:A461">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added one findign in config file
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harmandeep.singh\Documents\Git\Application-Review-Process_Performer\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55063BCC-8208-4D71-9060-48F3F79EAC62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D755AE9B-98D3-49DB-BC17-55875275E2C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23160" windowHeight="11010" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="22710" windowHeight="10695" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17784" uniqueCount="1172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17786" uniqueCount="1174">
   <si>
     <t>Name</t>
   </si>
@@ -3556,6 +3556,12 @@
   </si>
   <si>
     <t>Newly added by Harmandeep</t>
+  </si>
+  <si>
+    <t>IAQ_NoSupportingDocument</t>
+  </si>
+  <si>
+    <t>Income listed on IAQ page 2 does not have supporting documentation</t>
   </si>
 </sst>
 </file>
@@ -8442,7 +8448,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:XFD511"/>
+  <dimension ref="A1:XFD513"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -58206,72 +58212,69 @@
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>492</v>
+        <v>652</v>
       </c>
       <c r="B75" t="s">
-        <v>1138</v>
+        <v>651</v>
+      </c>
+      <c r="C75" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>652</v>
+        <v>1172</v>
       </c>
       <c r="B76" t="s">
-        <v>651</v>
-      </c>
-      <c r="C76" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3">
-      <c r="A78" t="s">
-        <v>156</v>
-      </c>
-      <c r="B78" t="s">
-        <v>119</v>
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3">
+      <c r="A77" t="s">
+        <v>492</v>
+      </c>
+      <c r="B77" t="s">
+        <v>1138</v>
       </c>
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>120</v>
+        <v>156</v>
       </c>
       <c r="B79" t="s">
-        <v>535</v>
+        <v>119</v>
       </c>
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B80" t="s">
-        <v>121</v>
+        <v>535</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>574</v>
+        <v>122</v>
       </c>
       <c r="B81" t="s">
-        <v>575</v>
+        <v>121</v>
       </c>
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>662</v>
+        <v>574</v>
       </c>
       <c r="B82" t="s">
-        <v>663</v>
-      </c>
-      <c r="C82" t="s">
-        <v>602</v>
+        <v>575</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>681</v>
+        <v>662</v>
       </c>
       <c r="B83" t="s">
-        <v>682</v>
+        <v>663</v>
       </c>
       <c r="C83" t="s">
         <v>602</v>
@@ -58279,10 +58282,10 @@
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B84" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="C84" t="s">
         <v>602</v>
@@ -58290,10 +58293,10 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="B85" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="C85" t="s">
         <v>602</v>
@@ -58301,37 +58304,37 @@
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
+        <v>679</v>
+      </c>
+      <c r="B86" t="s">
+        <v>684</v>
+      </c>
+      <c r="C86" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3">
+      <c r="A87" t="s">
         <v>491</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B87" t="s">
         <v>1165</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3">
-      <c r="A88" t="s">
-        <v>184</v>
-      </c>
-      <c r="B88" t="s">
-        <v>1018</v>
       </c>
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>661</v>
+        <v>184</v>
       </c>
       <c r="B89" t="s">
-        <v>675</v>
-      </c>
-      <c r="C89" t="s">
-        <v>602</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="B90" t="s">
-        <v>660</v>
+        <v>675</v>
       </c>
       <c r="C90" t="s">
         <v>602</v>
@@ -58339,80 +58342,80 @@
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>123</v>
+        <v>659</v>
       </c>
       <c r="B91" t="s">
-        <v>125</v>
+        <v>660</v>
+      </c>
+      <c r="C91" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B92" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="B93" t="s">
-        <v>536</v>
+        <v>126</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B94" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B95" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B96" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B97" t="s">
-        <v>449</v>
-      </c>
-      <c r="C97" t="s">
-        <v>597</v>
+        <v>539</v>
       </c>
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B98" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C98" t="s">
-        <v>504</v>
+        <v>597</v>
       </c>
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B99" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C99" t="s">
         <v>504</v>
@@ -58420,48 +58423,48 @@
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>576</v>
+        <v>142</v>
       </c>
       <c r="B100" t="s">
-        <v>577</v>
+        <v>452</v>
+      </c>
+      <c r="C100" t="s">
+        <v>504</v>
       </c>
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>626</v>
+        <v>576</v>
       </c>
       <c r="B101" t="s">
-        <v>627</v>
-      </c>
-      <c r="C101" t="s">
-        <v>602</v>
+        <v>577</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>880</v>
+        <v>626</v>
       </c>
       <c r="B102" t="s">
-        <v>881</v>
+        <v>627</v>
+      </c>
+      <c r="C102" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>653</v>
+        <v>880</v>
       </c>
       <c r="B103" t="s">
-        <v>654</v>
-      </c>
-      <c r="C103" t="s">
-        <v>602</v>
+        <v>881</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="B104" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="C104" t="s">
         <v>602</v>
@@ -58469,10 +58472,10 @@
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="B105" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="C105" t="s">
         <v>602</v>
@@ -58480,392 +58483,392 @@
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>490</v>
+        <v>658</v>
       </c>
       <c r="B106" t="s">
-        <v>1139</v>
+        <v>657</v>
+      </c>
+      <c r="C106" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>876</v>
+        <v>490</v>
       </c>
       <c r="B107" t="s">
-        <v>877</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="B108" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="B109" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
+        <v>883</v>
+      </c>
+      <c r="B110" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3">
+      <c r="A111" t="s">
         <v>885</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B111" t="s">
         <v>882</v>
-      </c>
-    </row>
-    <row r="112" spans="1:3">
-      <c r="A112" t="s">
-        <v>145</v>
-      </c>
-      <c r="B112" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B113" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B114" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B115" t="s">
-        <v>523</v>
-      </c>
-      <c r="C115" t="s">
-        <v>601</v>
+        <v>150</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>600</v>
+        <v>143</v>
       </c>
       <c r="B116" t="s">
         <v>523</v>
       </c>
+      <c r="C116" t="s">
+        <v>601</v>
+      </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>144</v>
+        <v>600</v>
       </c>
       <c r="B117" t="s">
-        <v>127</v>
+        <v>523</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="B118" t="s">
-        <v>540</v>
+        <v>127</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B119" t="s">
-        <v>128</v>
+        <v>540</v>
       </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>578</v>
+        <v>130</v>
       </c>
       <c r="B120" t="s">
-        <v>579</v>
+        <v>128</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
+        <v>578</v>
+      </c>
+      <c r="B121" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3">
+      <c r="A122" t="s">
         <v>489</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B122" t="s">
         <v>1140</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3">
-      <c r="A123" t="s">
-        <v>185</v>
-      </c>
-      <c r="B123" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>131</v>
+        <v>185</v>
       </c>
       <c r="B124" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B125" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B126" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>710</v>
+        <v>132</v>
       </c>
       <c r="B127" t="s">
-        <v>709</v>
-      </c>
-      <c r="C127" t="s">
-        <v>602</v>
+        <v>153</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>134</v>
+        <v>710</v>
       </c>
       <c r="B128" t="s">
-        <v>154</v>
+        <v>709</v>
+      </c>
+      <c r="C128" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B129" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>569</v>
+        <v>135</v>
       </c>
       <c r="B130" t="s">
-        <v>605</v>
-      </c>
-      <c r="C130" t="s">
-        <v>609</v>
+        <v>155</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>580</v>
+        <v>569</v>
       </c>
       <c r="B131" t="s">
-        <v>581</v>
+        <v>605</v>
+      </c>
+      <c r="C131" t="s">
+        <v>609</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>628</v>
+        <v>580</v>
       </c>
       <c r="B132" t="s">
-        <v>629</v>
-      </c>
-      <c r="C132" t="s">
-        <v>602</v>
+        <v>581</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
+        <v>628</v>
+      </c>
+      <c r="B133" t="s">
+        <v>629</v>
+      </c>
+      <c r="C133" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3">
+      <c r="A134" t="s">
         <v>488</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B134" t="s">
         <v>1141</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3">
-      <c r="A135" t="s">
-        <v>618</v>
-      </c>
-      <c r="B135" t="s">
-        <v>619</v>
-      </c>
-      <c r="C135" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="B136" t="s">
-        <v>1166</v>
+        <v>619</v>
       </c>
       <c r="C136" t="s">
         <v>620</v>
       </c>
     </row>
-    <row r="138" spans="1:3">
-      <c r="A138" t="s">
-        <v>157</v>
-      </c>
-      <c r="B138" t="s">
-        <v>161</v>
+    <row r="137" spans="1:3">
+      <c r="A137" t="s">
+        <v>621</v>
+      </c>
+      <c r="B137" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C137" t="s">
+        <v>620</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B139" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B140" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B141" t="s">
-        <v>541</v>
+        <v>163</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>505</v>
+        <v>160</v>
       </c>
       <c r="B142" t="s">
-        <v>642</v>
-      </c>
-      <c r="C142" t="s">
-        <v>643</v>
+        <v>541</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>1101</v>
+        <v>505</v>
       </c>
       <c r="B143" t="s">
-        <v>1109</v>
+        <v>642</v>
       </c>
       <c r="C143" t="s">
-        <v>602</v>
+        <v>643</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>586</v>
+        <v>1101</v>
       </c>
       <c r="B144" t="s">
-        <v>587</v>
+        <v>1109</v>
+      </c>
+      <c r="C144" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
+        <v>586</v>
+      </c>
+      <c r="B145" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3">
+      <c r="A146" t="s">
         <v>487</v>
       </c>
-      <c r="B145" t="s">
+      <c r="B146" t="s">
         <v>1167</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3">
-      <c r="A147" t="s">
-        <v>189</v>
-      </c>
-      <c r="B147" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>164</v>
+        <v>189</v>
       </c>
       <c r="B148" t="s">
-        <v>166</v>
+        <v>190</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B149" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>582</v>
+        <v>165</v>
       </c>
       <c r="B150" t="s">
-        <v>583</v>
+        <v>167</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>486</v>
+        <v>582</v>
       </c>
       <c r="B151" t="s">
-        <v>1142</v>
+        <v>583</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
+        <v>486</v>
+      </c>
+      <c r="B152" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3">
+      <c r="A153" t="s">
         <v>630</v>
       </c>
-      <c r="B152" t="s">
+      <c r="B153" t="s">
         <v>631</v>
       </c>
-      <c r="C152" t="s">
+      <c r="C153" t="s">
         <v>602</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3">
-      <c r="A154" t="s">
-        <v>187</v>
-      </c>
-      <c r="B154" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="B155" t="s">
-        <v>170</v>
-      </c>
-      <c r="C155" t="s">
-        <v>531</v>
+        <v>188</v>
       </c>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B156" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C156" t="s">
         <v>531</v>
@@ -58873,10 +58876,10 @@
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B157" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C157" t="s">
         <v>531</v>
@@ -58884,2769 +58887,2777 @@
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="B158" t="s">
-        <v>197</v>
+        <v>172</v>
+      </c>
+      <c r="C158" t="s">
+        <v>531</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B159" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>174</v>
+        <v>195</v>
       </c>
       <c r="B160" t="s">
-        <v>175</v>
-      </c>
-      <c r="C160" t="s">
-        <v>531</v>
+        <v>196</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>584</v>
+        <v>174</v>
       </c>
       <c r="B161" t="s">
-        <v>585</v>
+        <v>175</v>
+      </c>
+      <c r="C161" t="s">
+        <v>531</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
+        <v>584</v>
+      </c>
+      <c r="B162" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3">
+      <c r="A163" t="s">
         <v>475</v>
       </c>
-      <c r="B162" t="s">
+      <c r="B163" t="s">
         <v>1143</v>
       </c>
     </row>
-    <row r="163" spans="1:3" customFormat="1"/>
-    <row r="164" spans="1:3" customFormat="1">
-      <c r="A164" t="s">
+    <row r="165" spans="1:3">
+      <c r="A165" t="s">
         <v>1170</v>
       </c>
-      <c r="B164" t="s">
+      <c r="B165" t="s">
         <v>792</v>
       </c>
-      <c r="C164" t="s">
+      <c r="C165" t="s">
         <v>1171</v>
       </c>
     </row>
-    <row r="165" spans="1:3" customFormat="1">
-      <c r="A165" t="s">
+    <row r="166" spans="1:3">
+      <c r="A166" t="s">
         <v>591</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B166" t="s">
         <v>855</v>
       </c>
-      <c r="C165" t="s">
+      <c r="C166" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="166" spans="1:3" customFormat="1">
-      <c r="A166" t="s">
+    <row r="167" spans="1:3">
+      <c r="A167" t="s">
         <v>633</v>
       </c>
-      <c r="B166" t="s">
+      <c r="B167" t="s">
         <v>634</v>
-      </c>
-      <c r="C166" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" customFormat="1">
-      <c r="A167" t="s">
-        <v>721</v>
-      </c>
-      <c r="B167" t="s">
-        <v>856</v>
       </c>
       <c r="C167" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="168" spans="1:3" customFormat="1">
+    <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="B168" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="C168" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="169" spans="1:3" customFormat="1">
+    <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B169" t="s">
-        <v>706</v>
+        <v>857</v>
       </c>
       <c r="C169" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="170" spans="1:3" customFormat="1">
+    <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>1096</v>
+        <v>723</v>
       </c>
       <c r="B170" t="s">
-        <v>862</v>
+        <v>706</v>
       </c>
       <c r="C170" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="172" spans="1:3" customFormat="1">
-      <c r="A172" t="s">
+    <row r="171" spans="1:3">
+      <c r="A171" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B171" t="s">
+        <v>862</v>
+      </c>
+      <c r="C171" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3">
+      <c r="A173" t="s">
         <v>466</v>
       </c>
-      <c r="B172" t="s">
+      <c r="B173" t="s">
         <v>1113</v>
       </c>
     </row>
-    <row r="173" spans="1:3" customFormat="1">
-      <c r="A173" t="s">
+    <row r="174" spans="1:3">
+      <c r="A174" t="s">
         <v>1110</v>
       </c>
-      <c r="B173" t="s">
+      <c r="B174" t="s">
         <v>1111</v>
       </c>
-      <c r="C173" t="s">
+      <c r="C174" t="s">
         <v>1112</v>
       </c>
     </row>
-    <row r="174" spans="1:3" customFormat="1">
-      <c r="A174" t="s">
+    <row r="175" spans="1:3">
+      <c r="A175" t="s">
         <v>237</v>
       </c>
-      <c r="B174" t="s">
+      <c r="B175" t="s">
         <v>858</v>
       </c>
-      <c r="C174" t="s">
+      <c r="C175" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="175" spans="1:3" customFormat="1">
-      <c r="A175" t="s">
+    <row r="176" spans="1:3">
+      <c r="A176" t="s">
         <v>238</v>
       </c>
-      <c r="B175" t="s">
+      <c r="B176" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="176" spans="1:3" customFormat="1">
-      <c r="A176" t="s">
+    <row r="177" spans="1:3">
+      <c r="A177" t="s">
         <v>246</v>
       </c>
-      <c r="B176" t="s">
+      <c r="B177" t="s">
         <v>860</v>
       </c>
-      <c r="C176" t="s">
+      <c r="C177" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="177" spans="1:3" customFormat="1">
-      <c r="A177" t="s">
+    <row r="178" spans="1:3">
+      <c r="A178" t="s">
         <v>690</v>
       </c>
-      <c r="B177" t="s">
+      <c r="B178" t="s">
         <v>861</v>
       </c>
-      <c r="C177" t="s">
+      <c r="C178" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="178" spans="1:3" customFormat="1">
-      <c r="A178" t="s">
+    <row r="179" spans="1:3">
+      <c r="A179" t="s">
         <v>240</v>
       </c>
-      <c r="B178" t="s">
+      <c r="B179" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="179" spans="1:3" customFormat="1">
-      <c r="A179" t="s">
+    <row r="180" spans="1:3">
+      <c r="A180" t="s">
         <v>456</v>
       </c>
-      <c r="B179" t="s">
+      <c r="B180" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="180" spans="1:3" customFormat="1">
-      <c r="A180" t="s">
+    <row r="181" spans="1:3">
+      <c r="A181" t="s">
         <v>241</v>
       </c>
-      <c r="B180" t="s">
+      <c r="B181" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="181" spans="1:3" customFormat="1">
-      <c r="A181" t="s">
+    <row r="182" spans="1:3">
+      <c r="A182" t="s">
         <v>242</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B182" t="s">
         <v>863</v>
       </c>
     </row>
-    <row r="182" spans="1:3" customFormat="1">
-      <c r="A182" t="s">
+    <row r="183" spans="1:3">
+      <c r="A183" t="s">
         <v>243</v>
       </c>
-      <c r="B182" t="s">
+      <c r="B183" t="s">
         <v>864</v>
       </c>
     </row>
-    <row r="183" spans="1:3" customFormat="1">
-      <c r="A183" t="s">
+    <row r="184" spans="1:3">
+      <c r="A184" t="s">
         <v>244</v>
       </c>
-      <c r="B183" t="s">
+      <c r="B184" t="s">
         <v>865</v>
       </c>
     </row>
-    <row r="184" spans="1:3" customFormat="1">
-      <c r="A184" t="s">
+    <row r="185" spans="1:3">
+      <c r="A185" t="s">
         <v>245</v>
       </c>
-      <c r="B184" t="s">
+      <c r="B185" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="185" spans="1:3" customFormat="1">
-      <c r="A185" t="s">
+    <row r="186" spans="1:3">
+      <c r="A186" t="s">
         <v>277</v>
       </c>
-      <c r="B185" t="s">
+      <c r="B186" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="186" spans="1:3" customFormat="1">
-      <c r="A186" t="s">
+    <row r="187" spans="1:3">
+      <c r="A187" t="s">
         <v>304</v>
       </c>
-      <c r="B186" t="s">
+      <c r="B187" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="187" spans="1:3" customFormat="1">
-      <c r="A187" t="s">
+    <row r="188" spans="1:3">
+      <c r="A188" t="s">
         <v>594</v>
       </c>
-      <c r="B187" t="s">
+      <c r="B188" t="s">
         <v>1094</v>
       </c>
     </row>
-    <row r="188" spans="1:3" customFormat="1">
-      <c r="A188" t="s">
+    <row r="189" spans="1:3">
+      <c r="A189" t="s">
         <v>611</v>
       </c>
-      <c r="B188" t="s">
+      <c r="B189" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="189" spans="1:3" customFormat="1">
-      <c r="A189" t="s">
+    <row r="190" spans="1:3">
+      <c r="A190" t="s">
         <v>676</v>
       </c>
-      <c r="B189" t="s">
+      <c r="B190" t="s">
         <v>677</v>
-      </c>
-      <c r="C189" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3" customFormat="1">
-      <c r="A190" t="s">
-        <v>689</v>
-      </c>
-      <c r="B190" t="s">
-        <v>708</v>
       </c>
       <c r="C190" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="191" spans="1:3" customFormat="1">
+    <row r="191" spans="1:3">
       <c r="A191" t="s">
+        <v>689</v>
+      </c>
+      <c r="B191" t="s">
+        <v>708</v>
+      </c>
+      <c r="C191" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3">
+      <c r="A192" t="s">
         <v>874</v>
       </c>
-      <c r="B191" t="s">
+      <c r="B192" t="s">
         <v>875</v>
       </c>
     </row>
-    <row r="192" spans="1:3" customFormat="1">
-      <c r="A192" t="s">
+    <row r="193" spans="1:3">
+      <c r="A193" t="s">
         <v>474</v>
       </c>
-      <c r="B192" t="s">
+      <c r="B193" t="s">
         <v>1144</v>
       </c>
     </row>
-    <row r="193" spans="1:3" customFormat="1"/>
-    <row r="194" spans="1:3" customFormat="1">
-      <c r="A194" t="s">
+    <row r="195" spans="1:3">
+      <c r="A195" t="s">
         <v>687</v>
       </c>
-      <c r="B194" t="s">
+      <c r="B195" t="s">
         <v>688</v>
       </c>
-      <c r="C194" t="s">
+      <c r="C195" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="195" spans="1:3" customFormat="1">
-      <c r="A195" t="s">
+    <row r="196" spans="1:3">
+      <c r="A196" t="s">
         <v>467</v>
       </c>
-      <c r="B195" t="s">
+      <c r="B196" t="s">
         <v>1118</v>
       </c>
     </row>
-    <row r="196" spans="1:3" customFormat="1">
-      <c r="A196" t="s">
+    <row r="197" spans="1:3">
+      <c r="A197" t="s">
         <v>247</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B197" t="s">
         <v>866</v>
       </c>
-      <c r="C196" t="s">
+      <c r="C197" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="197" spans="1:3" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A197" t="s">
+    <row r="198" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A198" t="s">
         <v>249</v>
       </c>
-      <c r="B197" t="s">
+      <c r="B198" t="s">
         <v>867</v>
       </c>
-      <c r="C197" t="s">
+      <c r="C198" t="s">
         <v>606</v>
       </c>
     </row>
-    <row r="198" spans="1:3" customFormat="1">
-      <c r="A198" t="s">
+    <row r="199" spans="1:3">
+      <c r="A199" t="s">
         <v>248</v>
       </c>
-      <c r="B198" t="s">
+      <c r="B199" t="s">
         <v>828</v>
       </c>
     </row>
-    <row r="199" spans="1:3" customFormat="1">
-      <c r="A199" t="s">
+    <row r="200" spans="1:3">
+      <c r="A200" t="s">
         <v>251</v>
       </c>
-      <c r="B199" t="s">
+      <c r="B200" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="200" spans="1:3" customFormat="1">
-      <c r="A200" t="s">
+    <row r="201" spans="1:3">
+      <c r="A201" t="s">
         <v>252</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B201" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="201" spans="1:3" customFormat="1">
-      <c r="A201" t="s">
+    <row r="202" spans="1:3">
+      <c r="A202" t="s">
         <v>255</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B202" t="s">
         <v>254</v>
       </c>
-      <c r="C201" t="s">
+      <c r="C202" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="202" spans="1:3" customFormat="1">
-      <c r="A202" t="s">
+    <row r="203" spans="1:3">
+      <c r="A203" t="s">
         <v>457</v>
       </c>
-      <c r="B202" t="s">
+      <c r="B203" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="203" spans="1:3" customFormat="1">
-      <c r="A203" t="s">
+    <row r="204" spans="1:3">
+      <c r="A204" t="s">
         <v>256</v>
       </c>
-      <c r="B203" t="s">
+      <c r="B204" t="s">
         <v>830</v>
       </c>
     </row>
-    <row r="204" spans="1:3" customFormat="1">
-      <c r="A204" t="s">
+    <row r="205" spans="1:3">
+      <c r="A205" t="s">
         <v>257</v>
       </c>
-      <c r="B204" t="s">
+      <c r="B205" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="205" spans="1:3" customFormat="1">
-      <c r="A205" t="s">
+    <row r="206" spans="1:3">
+      <c r="A206" t="s">
         <v>262</v>
       </c>
-      <c r="B205" t="s">
+      <c r="B206" t="s">
         <v>831</v>
       </c>
     </row>
-    <row r="206" spans="1:3" customFormat="1">
-      <c r="A206" t="s">
+    <row r="207" spans="1:3">
+      <c r="A207" t="s">
         <v>263</v>
       </c>
-      <c r="B206" t="s">
+      <c r="B207" t="s">
         <v>832</v>
       </c>
     </row>
-    <row r="207" spans="1:3" customFormat="1">
-      <c r="A207" t="s">
+    <row r="208" spans="1:3">
+      <c r="A208" t="s">
         <v>264</v>
       </c>
-      <c r="B207" t="s">
+      <c r="B208" t="s">
         <v>868</v>
       </c>
-      <c r="C207" t="s">
+      <c r="C208" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="208" spans="1:3" customFormat="1">
-      <c r="A208" t="s">
+    <row r="209" spans="1:3">
+      <c r="A209" t="s">
         <v>265</v>
       </c>
-      <c r="B208" t="s">
+      <c r="B209" t="s">
         <v>833</v>
       </c>
     </row>
-    <row r="209" spans="1:3" customFormat="1">
-      <c r="A209" t="s">
+    <row r="210" spans="1:3">
+      <c r="A210" t="s">
         <v>266</v>
       </c>
-      <c r="B209" t="s">
+      <c r="B210" t="s">
         <v>869</v>
       </c>
-      <c r="C209" t="s">
+      <c r="C210" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="210" spans="1:3" customFormat="1">
-      <c r="A210" t="s">
+    <row r="211" spans="1:3">
+      <c r="A211" t="s">
         <v>267</v>
       </c>
-      <c r="B210" t="s">
+      <c r="B211" t="s">
         <v>834</v>
       </c>
     </row>
-    <row r="211" spans="1:3" customFormat="1">
-      <c r="A211" t="s">
+    <row r="212" spans="1:3">
+      <c r="A212" t="s">
         <v>274</v>
       </c>
-      <c r="B211" t="s">
+      <c r="B212" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="212" spans="1:3" customFormat="1">
-      <c r="A212" t="s">
+    <row r="213" spans="1:3">
+      <c r="A213" t="s">
         <v>276</v>
       </c>
-      <c r="B212" t="s">
+      <c r="B213" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="213" spans="1:3" customFormat="1">
-      <c r="A213" t="s">
+    <row r="214" spans="1:3">
+      <c r="A214" t="s">
         <v>278</v>
       </c>
-      <c r="B213" t="s">
+      <c r="B214" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="214" spans="1:3" customFormat="1">
-      <c r="A214" t="s">
+    <row r="215" spans="1:3">
+      <c r="A215" t="s">
         <v>612</v>
       </c>
-      <c r="B214" t="s">
+      <c r="B215" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="215" spans="1:3" customFormat="1">
-      <c r="A215" t="s">
+    <row r="216" spans="1:3">
+      <c r="A216" t="s">
         <v>485</v>
       </c>
-      <c r="B215" t="s">
+      <c r="B216" t="s">
         <v>1145</v>
       </c>
     </row>
-    <row r="216" spans="1:3" customFormat="1">
-      <c r="A216" t="s">
+    <row r="217" spans="1:3">
+      <c r="A217" t="s">
         <v>607</v>
       </c>
-      <c r="B216" t="s">
+      <c r="B217" t="s">
         <v>608</v>
       </c>
-      <c r="C216" t="s">
+      <c r="C217" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="218" spans="1:3" customFormat="1">
-      <c r="A218" t="s">
+    <row r="219" spans="1:3">
+      <c r="A219" t="s">
         <v>468</v>
       </c>
-      <c r="B218" t="s">
+      <c r="B219" t="s">
         <v>1117</v>
       </c>
     </row>
-    <row r="219" spans="1:3" customFormat="1">
-      <c r="A219" t="s">
+    <row r="220" spans="1:3">
+      <c r="A220" t="s">
         <v>458</v>
       </c>
-      <c r="B219" t="s">
+      <c r="B220" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="220" spans="1:3" customFormat="1">
-      <c r="A220" t="s">
+    <row r="221" spans="1:3">
+      <c r="A221" t="s">
         <v>272</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B221" t="s">
         <v>794</v>
       </c>
     </row>
-    <row r="221" spans="1:3" customFormat="1">
-      <c r="A221" t="s">
+    <row r="222" spans="1:3">
+      <c r="A222" t="s">
         <v>273</v>
       </c>
-      <c r="B221" t="s">
+      <c r="B222" t="s">
         <v>795</v>
       </c>
     </row>
-    <row r="222" spans="1:3" customFormat="1">
-      <c r="A222" t="s">
+    <row r="223" spans="1:3">
+      <c r="A223" t="s">
         <v>281</v>
       </c>
-      <c r="B222" t="s">
+      <c r="B223" t="s">
         <v>796</v>
       </c>
     </row>
-    <row r="223" spans="1:3" customFormat="1">
-      <c r="A223" t="s">
+    <row r="224" spans="1:3">
+      <c r="A224" t="s">
         <v>280</v>
       </c>
-      <c r="B223" t="s">
+      <c r="B224" t="s">
         <v>798</v>
       </c>
     </row>
-    <row r="224" spans="1:3" customFormat="1">
-      <c r="A224" t="s">
+    <row r="225" spans="1:2">
+      <c r="A225" t="s">
         <v>282</v>
       </c>
-      <c r="B224" t="s">
+      <c r="B225" t="s">
         <v>797</v>
       </c>
     </row>
-    <row r="225" spans="1:2" customFormat="1">
-      <c r="A225" t="s">
+    <row r="226" spans="1:2">
+      <c r="A226" t="s">
         <v>613</v>
       </c>
-      <c r="B225" t="s">
+      <c r="B226" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="226" spans="1:2" customFormat="1">
-      <c r="A226" t="s">
+    <row r="227" spans="1:2">
+      <c r="A227" t="s">
         <v>484</v>
       </c>
-      <c r="B226" t="s">
+      <c r="B227" t="s">
         <v>1146</v>
       </c>
     </row>
-    <row r="228" spans="1:2" customFormat="1">
-      <c r="A228" t="s">
+    <row r="229" spans="1:2">
+      <c r="A229" t="s">
         <v>469</v>
       </c>
-      <c r="B228" t="s">
+      <c r="B229" t="s">
         <v>1114</v>
       </c>
     </row>
-    <row r="229" spans="1:2" customFormat="1">
-      <c r="A229" t="s">
+    <row r="230" spans="1:2">
+      <c r="A230" t="s">
         <v>459</v>
       </c>
-      <c r="B229" t="s">
+      <c r="B230" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="230" spans="1:2" customFormat="1">
-      <c r="A230" t="s">
+    <row r="231" spans="1:2">
+      <c r="A231" t="s">
         <v>285</v>
       </c>
-      <c r="B230" t="s">
+      <c r="B231" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="231" spans="1:2" customFormat="1">
-      <c r="A231" t="s">
+    <row r="232" spans="1:2">
+      <c r="A232" t="s">
         <v>286</v>
       </c>
-      <c r="B231" t="s">
+      <c r="B232" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="232" spans="1:2" customFormat="1">
-      <c r="A232" t="s">
+    <row r="233" spans="1:2">
+      <c r="A233" t="s">
         <v>287</v>
       </c>
-      <c r="B232" t="s">
+      <c r="B233" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="233" spans="1:2" customFormat="1">
-      <c r="A233" t="s">
+    <row r="234" spans="1:2">
+      <c r="A234" t="s">
         <v>289</v>
       </c>
-      <c r="B233" t="s">
+      <c r="B234" t="s">
         <v>790</v>
       </c>
     </row>
-    <row r="234" spans="1:2" customFormat="1">
-      <c r="A234" t="s">
+    <row r="235" spans="1:2">
+      <c r="A235" t="s">
         <v>290</v>
       </c>
-      <c r="B234" t="s">
+      <c r="B235" t="s">
         <v>789</v>
       </c>
     </row>
-    <row r="235" spans="1:2" customFormat="1">
-      <c r="A235" t="s">
+    <row r="236" spans="1:2">
+      <c r="A236" t="s">
         <v>291</v>
       </c>
-      <c r="B235" t="s">
+      <c r="B236" t="s">
         <v>791</v>
       </c>
     </row>
-    <row r="236" spans="1:2" customFormat="1">
-      <c r="A236" t="s">
+    <row r="237" spans="1:2">
+      <c r="A237" t="s">
         <v>292</v>
       </c>
-      <c r="B236" t="s">
+      <c r="B237" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="237" spans="1:2" customFormat="1">
-      <c r="A237" t="s">
+    <row r="238" spans="1:2">
+      <c r="A238" t="s">
         <v>614</v>
       </c>
-      <c r="B237" t="s">
+      <c r="B238" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="238" spans="1:2" customFormat="1">
-      <c r="A238" t="s">
+    <row r="239" spans="1:2">
+      <c r="A239" t="s">
         <v>483</v>
       </c>
-      <c r="B238" t="s">
+      <c r="B239" t="s">
         <v>1147</v>
       </c>
     </row>
-    <row r="240" spans="1:2" customFormat="1">
-      <c r="A240" t="s">
+    <row r="241" spans="1:3">
+      <c r="A241" t="s">
         <v>470</v>
       </c>
-      <c r="B240" t="s">
+      <c r="B241" t="s">
         <v>1115</v>
       </c>
     </row>
-    <row r="241" spans="1:3" customFormat="1">
-      <c r="A241" t="s">
+    <row r="242" spans="1:3">
+      <c r="A242" t="s">
         <v>454</v>
       </c>
-      <c r="B241" t="s">
+      <c r="B242" t="s">
         <v>298</v>
       </c>
-      <c r="C241" t="s">
+      <c r="C242" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="242" spans="1:3" customFormat="1">
-      <c r="A242" t="s">
+    <row r="243" spans="1:3">
+      <c r="A243" t="s">
         <v>460</v>
       </c>
-      <c r="B242" t="s">
+      <c r="B243" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="243" spans="1:3" customFormat="1">
-      <c r="A243" t="s">
+    <row r="244" spans="1:3">
+      <c r="A244" t="s">
         <v>296</v>
       </c>
-      <c r="B243" t="s">
+      <c r="B244" t="s">
         <v>870</v>
       </c>
-      <c r="C243" t="s">
+      <c r="C244" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="244" spans="1:3" customFormat="1">
-      <c r="A244" t="s">
+    <row r="245" spans="1:3">
+      <c r="A245" t="s">
         <v>297</v>
       </c>
-      <c r="B244" t="s">
+      <c r="B245" t="s">
         <v>853</v>
       </c>
     </row>
-    <row r="245" spans="1:3" customFormat="1">
-      <c r="A245" t="s">
+    <row r="246" spans="1:3">
+      <c r="A246" t="s">
         <v>453</v>
       </c>
-      <c r="B245" t="s">
+      <c r="B246" t="s">
         <v>854</v>
       </c>
     </row>
-    <row r="246" spans="1:3" customFormat="1">
-      <c r="A246" t="s">
+    <row r="247" spans="1:3">
+      <c r="A247" t="s">
         <v>299</v>
       </c>
-      <c r="B246" t="s">
+      <c r="B247" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="247" spans="1:3" customFormat="1">
-      <c r="A247" t="s">
+    <row r="248" spans="1:3">
+      <c r="A248" t="s">
         <v>300</v>
       </c>
-      <c r="B247" t="s">
+      <c r="B248" t="s">
         <v>871</v>
       </c>
     </row>
-    <row r="248" spans="1:3" customFormat="1">
-      <c r="A248" t="s">
+    <row r="249" spans="1:3">
+      <c r="A249" t="s">
         <v>301</v>
       </c>
-      <c r="B248" t="s">
+      <c r="B249" t="s">
         <v>872</v>
       </c>
     </row>
-    <row r="249" spans="1:3" customFormat="1">
-      <c r="A249" t="s">
+    <row r="250" spans="1:3">
+      <c r="A250" t="s">
         <v>302</v>
       </c>
-      <c r="B249" t="s">
+      <c r="B250" t="s">
         <v>873</v>
       </c>
     </row>
-    <row r="250" spans="1:3" customFormat="1">
-      <c r="A250" t="s">
+    <row r="251" spans="1:3">
+      <c r="A251" t="s">
         <v>303</v>
       </c>
-      <c r="B250" t="s">
+      <c r="B251" t="s">
         <v>792</v>
       </c>
     </row>
-    <row r="251" spans="1:3" customFormat="1">
-      <c r="A251" t="s">
+    <row r="252" spans="1:3">
+      <c r="A252" t="s">
         <v>615</v>
       </c>
-      <c r="B251" t="s">
+      <c r="B252" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="252" spans="1:3" customFormat="1">
-      <c r="A252" t="s">
+    <row r="253" spans="1:3">
+      <c r="A253" t="s">
         <v>482</v>
       </c>
-      <c r="B252" t="s">
+      <c r="B253" t="s">
         <v>1148</v>
       </c>
     </row>
-    <row r="254" spans="1:3" customFormat="1">
-      <c r="A254" t="s">
+    <row r="255" spans="1:3">
+      <c r="A255" t="s">
         <v>648</v>
       </c>
-      <c r="B254" t="s">
+      <c r="B255" t="s">
         <v>649</v>
       </c>
-      <c r="C254" t="s">
+      <c r="C255" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="255" spans="1:3" customFormat="1">
-      <c r="A255" t="s">
+    <row r="256" spans="1:3">
+      <c r="A256" t="s">
         <v>499</v>
       </c>
-      <c r="B255" t="s">
+      <c r="B256" t="s">
         <v>502</v>
       </c>
-      <c r="C255" t="s">
+      <c r="C256" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="256" spans="1:3" customFormat="1">
-      <c r="A256" t="s">
+    <row r="257" spans="1:3">
+      <c r="A257" t="s">
         <v>500</v>
       </c>
-      <c r="B256" t="s">
+      <c r="B257" t="s">
         <v>501</v>
       </c>
-      <c r="C256" t="s">
+      <c r="C257" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="257" spans="1:3" customFormat="1">
-      <c r="A257" t="s">
+    <row r="258" spans="1:3">
+      <c r="A258" t="s">
         <v>528</v>
       </c>
-      <c r="B257" t="s">
+      <c r="B258" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="258" spans="1:3" customFormat="1">
-      <c r="A258" t="s">
+    <row r="259" spans="1:3">
+      <c r="A259" t="s">
         <v>320</v>
       </c>
-      <c r="B258" t="s">
+      <c r="B259" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="259" spans="1:3" customFormat="1">
-      <c r="A259" t="s">
+    <row r="260" spans="1:3">
+      <c r="A260" t="s">
         <v>321</v>
       </c>
-      <c r="B259" t="s">
+      <c r="B260" t="s">
         <v>307</v>
       </c>
-      <c r="C259" t="s">
+      <c r="C260" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="260" spans="1:3" customFormat="1">
-      <c r="A260" t="s">
+    <row r="261" spans="1:3">
+      <c r="A261" t="s">
         <v>461</v>
       </c>
-      <c r="B260" t="s">
+      <c r="B261" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="261" spans="1:3" customFormat="1">
-      <c r="A261" t="s">
+    <row r="262" spans="1:3">
+      <c r="A262" t="s">
         <v>322</v>
       </c>
-      <c r="B261" t="s">
+      <c r="B262" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="262" spans="1:3" customFormat="1">
-      <c r="A262" t="s">
+    <row r="263" spans="1:3">
+      <c r="A263" t="s">
         <v>323</v>
       </c>
-      <c r="B262" t="s">
+      <c r="B263" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="263" spans="1:3" customFormat="1">
-      <c r="A263" t="s">
+    <row r="264" spans="1:3">
+      <c r="A264" t="s">
         <v>324</v>
       </c>
-      <c r="B263" t="s">
+      <c r="B264" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="264" spans="1:3" customFormat="1">
-      <c r="A264" t="s">
+    <row r="265" spans="1:3">
+      <c r="A265" t="s">
         <v>325</v>
       </c>
-      <c r="B264" t="s">
+      <c r="B265" t="s">
         <v>311</v>
       </c>
-      <c r="C264" t="s">
+      <c r="C265" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="265" spans="1:3" customFormat="1">
-      <c r="A265" t="s">
+    <row r="266" spans="1:3">
+      <c r="A266" t="s">
         <v>326</v>
       </c>
-      <c r="B265" t="s">
+      <c r="B266" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="266" spans="1:3" customFormat="1">
-      <c r="A266" t="s">
+    <row r="267" spans="1:3">
+      <c r="A267" t="s">
         <v>327</v>
       </c>
-      <c r="B266" t="s">
+      <c r="B267" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="267" spans="1:3" customFormat="1">
-      <c r="A267" t="s">
+    <row r="268" spans="1:3">
+      <c r="A268" t="s">
         <v>328</v>
       </c>
-      <c r="B267" t="s">
+      <c r="B268" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="268" spans="1:3" customFormat="1">
-      <c r="A268" t="s">
+    <row r="269" spans="1:3">
+      <c r="A269" t="s">
         <v>329</v>
       </c>
-      <c r="B268" t="s">
+      <c r="B269" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="269" spans="1:3" customFormat="1">
-      <c r="A269" t="s">
+    <row r="270" spans="1:3">
+      <c r="A270" t="s">
         <v>330</v>
       </c>
-      <c r="B269" t="s">
+      <c r="B270" t="s">
         <v>316</v>
       </c>
-      <c r="C269" t="s">
+      <c r="C270" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="270" spans="1:3" customFormat="1">
-      <c r="A270" t="s">
+    <row r="271" spans="1:3">
+      <c r="A271" t="s">
         <v>331</v>
       </c>
-      <c r="B270" t="s">
+      <c r="B271" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="271" spans="1:3" customFormat="1">
-      <c r="A271" t="s">
+    <row r="272" spans="1:3">
+      <c r="A272" t="s">
         <v>332</v>
       </c>
-      <c r="B271" t="s">
+      <c r="B272" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="272" spans="1:3" customFormat="1">
-      <c r="A272" t="s">
+    <row r="273" spans="1:3">
+      <c r="A273" t="s">
         <v>333</v>
       </c>
-      <c r="B272" t="s">
+      <c r="B273" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="273" spans="1:3" customFormat="1">
-      <c r="A273" t="s">
+    <row r="274" spans="1:3">
+      <c r="A274" t="s">
         <v>481</v>
       </c>
-      <c r="B273" t="s">
+      <c r="B274" t="s">
         <v>1149</v>
       </c>
     </row>
-    <row r="275" spans="1:3" customFormat="1">
-      <c r="A275" t="s">
+    <row r="276" spans="1:3">
+      <c r="A276" t="s">
         <v>546</v>
       </c>
-      <c r="B275" t="s">
+      <c r="B276" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="276" spans="1:3" customFormat="1">
-      <c r="A276" t="s">
+    <row r="277" spans="1:3">
+      <c r="A277" t="s">
         <v>340</v>
       </c>
-      <c r="B276" t="s">
+      <c r="B277" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="277" spans="1:3" customFormat="1">
-      <c r="A277" t="s">
+    <row r="278" spans="1:3">
+      <c r="A278" t="s">
         <v>341</v>
       </c>
-      <c r="B277" t="s">
+      <c r="B278" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="278" spans="1:3" customFormat="1">
-      <c r="A278" t="s">
+    <row r="279" spans="1:3">
+      <c r="A279" t="s">
         <v>342</v>
       </c>
-      <c r="B278" t="s">
+      <c r="B279" t="s">
         <v>356</v>
       </c>
-      <c r="C278" t="s">
+      <c r="C279" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="279" spans="1:3" customFormat="1">
-      <c r="A279" t="s">
+    <row r="280" spans="1:3">
+      <c r="A280" t="s">
         <v>462</v>
       </c>
-      <c r="B279" t="s">
+      <c r="B280" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="280" spans="1:3" customFormat="1">
-      <c r="A280" t="s">
+    <row r="281" spans="1:3">
+      <c r="A281" t="s">
         <v>359</v>
       </c>
-      <c r="B280" t="s">
+      <c r="B281" t="s">
         <v>357</v>
       </c>
-      <c r="C280" t="s">
+      <c r="C281" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="281" spans="1:3" customFormat="1">
-      <c r="A281" t="s">
+    <row r="282" spans="1:3">
+      <c r="A282" t="s">
         <v>343</v>
       </c>
-      <c r="B281" t="s">
+      <c r="B282" t="s">
         <v>349</v>
       </c>
     </row>
-    <row r="282" spans="1:3" customFormat="1">
-      <c r="A282" t="s">
+    <row r="283" spans="1:3">
+      <c r="A283" t="s">
         <v>360</v>
       </c>
-      <c r="B282" t="s">
+      <c r="B283" t="s">
         <v>350</v>
       </c>
-      <c r="C282" t="s">
+      <c r="C283" t="s">
         <v>508</v>
       </c>
     </row>
-    <row r="283" spans="1:3" customFormat="1">
-      <c r="A283" t="s">
+    <row r="284" spans="1:3">
+      <c r="A284" t="s">
         <v>344</v>
       </c>
-      <c r="B283" t="s">
+      <c r="B284" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="284" spans="1:3" customFormat="1">
-      <c r="A284" t="s">
+    <row r="285" spans="1:3">
+      <c r="A285" t="s">
         <v>346</v>
       </c>
-      <c r="B284" t="s">
+      <c r="B285" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="285" spans="1:3" customFormat="1">
-      <c r="A285" t="s">
+    <row r="286" spans="1:3">
+      <c r="A286" t="s">
         <v>345</v>
       </c>
-      <c r="B285" t="s">
+      <c r="B286" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="286" spans="1:3" customFormat="1">
-      <c r="A286" t="s">
+    <row r="287" spans="1:3">
+      <c r="A287" t="s">
         <v>347</v>
       </c>
-      <c r="B286" t="s">
+      <c r="B287" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="287" spans="1:3" customFormat="1">
-      <c r="A287" t="s">
+    <row r="288" spans="1:3">
+      <c r="A288" t="s">
         <v>348</v>
       </c>
-      <c r="B287" t="s">
+      <c r="B288" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="288" spans="1:3" customFormat="1">
-      <c r="A288" t="s">
+    <row r="289" spans="1:3">
+      <c r="A289" t="s">
         <v>1076</v>
       </c>
-      <c r="B288" t="s">
+      <c r="B289" t="s">
         <v>1077</v>
-      </c>
-      <c r="C288" t="s">
-        <v>1078</v>
-      </c>
-    </row>
-    <row r="289" spans="1:3" customFormat="1">
-      <c r="A289" t="s">
-        <v>1079</v>
-      </c>
-      <c r="B289" t="s">
-        <v>1080</v>
       </c>
       <c r="C289" t="s">
         <v>1078</v>
       </c>
     </row>
-    <row r="290" spans="1:3" customFormat="1">
+    <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="B290" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="C290" t="s">
         <v>1078</v>
       </c>
     </row>
-    <row r="291" spans="1:3" customFormat="1">
+    <row r="291" spans="1:3">
       <c r="A291" t="s">
+        <v>1081</v>
+      </c>
+      <c r="B291" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C291" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3">
+      <c r="A292" t="s">
         <v>480</v>
       </c>
-      <c r="B291" t="s">
+      <c r="B292" t="s">
         <v>1150</v>
       </c>
     </row>
-    <row r="293" spans="1:3" customFormat="1">
-      <c r="A293" t="s">
+    <row r="294" spans="1:3">
+      <c r="A294" t="s">
         <v>650</v>
       </c>
-      <c r="B293" t="s">
+      <c r="B294" t="s">
         <v>668</v>
       </c>
-      <c r="C293" t="s">
+      <c r="C294" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="294" spans="1:3" customFormat="1">
-      <c r="A294" t="s">
+    <row r="295" spans="1:3">
+      <c r="A295" t="s">
         <v>1083</v>
       </c>
-      <c r="B294" t="s">
+      <c r="B295" t="s">
         <v>1084</v>
-      </c>
-      <c r="C294" t="s">
-        <v>1078</v>
-      </c>
-    </row>
-    <row r="295" spans="1:3" customFormat="1">
-      <c r="A295" t="s">
-        <v>1085</v>
-      </c>
-      <c r="B295" t="s">
-        <v>1086</v>
       </c>
       <c r="C295" t="s">
         <v>1078</v>
       </c>
     </row>
-    <row r="296" spans="1:3" customFormat="1">
+    <row r="296" spans="1:3">
       <c r="A296" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="B296" t="s">
-        <v>1151</v>
+        <v>1086</v>
       </c>
       <c r="C296" t="s">
         <v>1078</v>
       </c>
     </row>
-    <row r="298" spans="1:3" customFormat="1">
-      <c r="A298" t="s">
+    <row r="297" spans="1:3">
+      <c r="A297" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B297" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C297" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3">
+      <c r="A299" t="s">
         <v>646</v>
       </c>
-      <c r="B298" t="s">
+      <c r="B299" t="s">
         <v>647</v>
       </c>
-      <c r="C298" t="s">
+      <c r="C299" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="299" spans="1:3" customFormat="1">
-      <c r="A299" t="s">
+    <row r="300" spans="1:3">
+      <c r="A300" t="s">
         <v>471</v>
       </c>
-      <c r="B299" t="s">
+      <c r="B300" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="300" spans="1:3" customFormat="1">
-      <c r="A300" t="s">
+    <row r="301" spans="1:3">
+      <c r="A301" t="s">
         <v>366</v>
       </c>
-      <c r="B300" t="s">
+      <c r="B301" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="301" spans="1:3" customFormat="1">
-      <c r="A301" t="s">
+    <row r="302" spans="1:3">
+      <c r="A302" t="s">
         <v>367</v>
       </c>
-      <c r="B301" t="s">
+      <c r="B302" t="s">
         <v>378</v>
       </c>
-      <c r="C301" t="s">
+      <c r="C302" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="302" spans="1:3" customFormat="1">
-      <c r="A302" t="s">
+    <row r="303" spans="1:3">
+      <c r="A303" t="s">
         <v>519</v>
       </c>
-      <c r="B302" t="s">
+      <c r="B303" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="303" spans="1:3" customFormat="1">
-      <c r="A303" t="s">
+    <row r="304" spans="1:3">
+      <c r="A304" t="s">
         <v>368</v>
       </c>
-      <c r="B303" t="s">
+      <c r="B304" t="s">
         <v>379</v>
-      </c>
-      <c r="C303" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="304" spans="1:3" customFormat="1">
-      <c r="A304" t="s">
-        <v>369</v>
-      </c>
-      <c r="B304" t="s">
-        <v>380</v>
       </c>
       <c r="C304" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="305" spans="1:3" customFormat="1">
+    <row r="305" spans="1:3">
       <c r="A305" t="s">
+        <v>369</v>
+      </c>
+      <c r="B305" t="s">
+        <v>380</v>
+      </c>
+      <c r="C305" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3">
+      <c r="A306" t="s">
         <v>370</v>
       </c>
-      <c r="B305" t="s">
+      <c r="B306" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="306" spans="1:3" customFormat="1">
-      <c r="A306" t="s">
+    <row r="307" spans="1:3">
+      <c r="A307" t="s">
         <v>371</v>
       </c>
-      <c r="B306" t="s">
+      <c r="B307" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="307" spans="1:3" customFormat="1">
-      <c r="A307" t="s">
+    <row r="308" spans="1:3">
+      <c r="A308" t="s">
         <v>372</v>
       </c>
-      <c r="B307" t="s">
+      <c r="B308" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="308" spans="1:3" customFormat="1">
-      <c r="A308" t="s">
+    <row r="309" spans="1:3">
+      <c r="A309" t="s">
         <v>373</v>
       </c>
-      <c r="B308" t="s">
+      <c r="B309" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="309" spans="1:3" customFormat="1">
-      <c r="A309" t="s">
+    <row r="310" spans="1:3">
+      <c r="A310" t="s">
         <v>374</v>
       </c>
-      <c r="B309" t="s">
+      <c r="B310" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="310" spans="1:3" customFormat="1">
-      <c r="A310" t="s">
+    <row r="311" spans="1:3">
+      <c r="A311" t="s">
         <v>375</v>
       </c>
-      <c r="B310" t="s">
+      <c r="B311" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="311" spans="1:3" customFormat="1">
-      <c r="A311" t="s">
+    <row r="312" spans="1:3">
+      <c r="A312" t="s">
         <v>376</v>
       </c>
-      <c r="B311" t="s">
+      <c r="B312" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="312" spans="1:3" customFormat="1">
-      <c r="A312" t="s">
+    <row r="313" spans="1:3">
+      <c r="A313" t="s">
         <v>704</v>
       </c>
-      <c r="B312" t="s">
+      <c r="B313" t="s">
         <v>1091</v>
       </c>
-      <c r="C312" t="s">
+      <c r="C313" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="313" spans="1:3" customFormat="1">
-      <c r="A313" t="s">
+    <row r="314" spans="1:3">
+      <c r="A314" t="s">
         <v>1104</v>
       </c>
-      <c r="B313" t="s">
+      <c r="B314" t="s">
         <v>1105</v>
       </c>
     </row>
-    <row r="314" spans="1:3" customFormat="1">
-      <c r="A314" t="s">
+    <row r="315" spans="1:3">
+      <c r="A315" t="s">
         <v>478</v>
       </c>
-      <c r="B314" t="s">
+      <c r="B315" t="s">
         <v>1152</v>
       </c>
     </row>
-    <row r="315" spans="1:3" customFormat="1">
-      <c r="A315" t="s">
+    <row r="316" spans="1:3">
+      <c r="A316" t="s">
         <v>555</v>
       </c>
-      <c r="B315" t="s">
+      <c r="B316" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="317" spans="1:3" customFormat="1">
-      <c r="A317" t="s">
+    <row r="318" spans="1:3">
+      <c r="A318" t="s">
         <v>473</v>
       </c>
-      <c r="B317" t="s">
+      <c r="B318" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="318" spans="1:3" customFormat="1">
-      <c r="A318" t="s">
+    <row r="319" spans="1:3">
+      <c r="A319" t="s">
         <v>393</v>
       </c>
-      <c r="B318" t="s">
+      <c r="B319" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="319" spans="1:3" customFormat="1">
-      <c r="A319" t="s">
+    <row r="320" spans="1:3">
+      <c r="A320" t="s">
         <v>394</v>
       </c>
-      <c r="B319" t="s">
+      <c r="B320" t="s">
         <v>405</v>
       </c>
-      <c r="C319" t="s">
+      <c r="C320" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="320" spans="1:3" customFormat="1">
-      <c r="A320" t="s">
+    <row r="321" spans="1:3">
+      <c r="A321" t="s">
         <v>463</v>
       </c>
-      <c r="B320" t="s">
+      <c r="B321" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="321" spans="1:3" customFormat="1">
-      <c r="A321" t="s">
+    <row r="322" spans="1:3">
+      <c r="A322" t="s">
         <v>395</v>
       </c>
-      <c r="B321" t="s">
+      <c r="B322" t="s">
         <v>406</v>
-      </c>
-      <c r="C321" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="322" spans="1:3" customFormat="1">
-      <c r="A322" t="s">
-        <v>396</v>
-      </c>
-      <c r="B322" t="s">
-        <v>407</v>
       </c>
       <c r="C322" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="323" spans="1:3" customFormat="1">
+    <row r="323" spans="1:3">
       <c r="A323" t="s">
+        <v>396</v>
+      </c>
+      <c r="B323" t="s">
+        <v>407</v>
+      </c>
+      <c r="C323" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3">
+      <c r="A324" t="s">
         <v>397</v>
       </c>
-      <c r="B323" t="s">
+      <c r="B324" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="324" spans="1:3" customFormat="1">
-      <c r="A324" t="s">
+    <row r="325" spans="1:3">
+      <c r="A325" t="s">
         <v>398</v>
       </c>
-      <c r="B324" t="s">
+      <c r="B325" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="325" spans="1:3" customFormat="1">
-      <c r="A325" t="s">
+    <row r="326" spans="1:3">
+      <c r="A326" t="s">
         <v>399</v>
       </c>
-      <c r="B325" t="s">
+      <c r="B326" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="326" spans="1:3" customFormat="1">
-      <c r="A326" t="s">
+    <row r="327" spans="1:3">
+      <c r="A327" t="s">
         <v>400</v>
       </c>
-      <c r="B326" t="s">
+      <c r="B327" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="327" spans="1:3" customFormat="1">
-      <c r="A327" t="s">
+    <row r="328" spans="1:3">
+      <c r="A328" t="s">
         <v>401</v>
       </c>
-      <c r="B327" t="s">
+      <c r="B328" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="328" spans="1:3" customFormat="1">
-      <c r="A328" t="s">
+    <row r="329" spans="1:3">
+      <c r="A329" t="s">
         <v>402</v>
       </c>
-      <c r="B328" t="s">
+      <c r="B329" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="329" spans="1:3" customFormat="1">
-      <c r="A329" t="s">
+    <row r="330" spans="1:3">
+      <c r="A330" t="s">
         <v>403</v>
       </c>
-      <c r="B329" t="s">
+      <c r="B330" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="330" spans="1:3" customFormat="1">
-      <c r="A330" t="s">
+    <row r="331" spans="1:3">
+      <c r="A331" t="s">
         <v>477</v>
       </c>
-      <c r="B330" t="s">
+      <c r="B331" t="s">
         <v>1152</v>
       </c>
     </row>
-    <row r="331" spans="1:3" customFormat="1">
-      <c r="A331" t="s">
+    <row r="332" spans="1:3">
+      <c r="A332" t="s">
         <v>562</v>
       </c>
-      <c r="B331" t="s">
+      <c r="B332" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="333" spans="1:3" customFormat="1">
-      <c r="A333" t="s">
+    <row r="334" spans="1:3">
+      <c r="A334" t="s">
         <v>644</v>
       </c>
-      <c r="B333" t="s">
+      <c r="B334" t="s">
         <v>645</v>
       </c>
-      <c r="C333" t="s">
+      <c r="C334" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="334" spans="1:3" customFormat="1">
-      <c r="A334" t="s">
+    <row r="335" spans="1:3">
+      <c r="A335" t="s">
         <v>387</v>
       </c>
-      <c r="B334" t="s">
+      <c r="B335" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="335" spans="1:3" customFormat="1">
-      <c r="A335" t="s">
+    <row r="336" spans="1:3">
+      <c r="A336" t="s">
         <v>388</v>
       </c>
-      <c r="B335" t="s">
+      <c r="B336" t="s">
         <v>564</v>
       </c>
-      <c r="C335" t="s">
+      <c r="C336" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="336" spans="1:3" customFormat="1">
-      <c r="A336" t="s">
+    <row r="337" spans="1:3">
+      <c r="A337" t="s">
         <v>464</v>
       </c>
-      <c r="B336" t="s">
+      <c r="B337" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="337" spans="1:3" customFormat="1">
-      <c r="A337" t="s">
+    <row r="338" spans="1:3">
+      <c r="A338" t="s">
         <v>389</v>
       </c>
-      <c r="B337" t="s">
+      <c r="B338" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="338" spans="1:3" customFormat="1">
-      <c r="A338" t="s">
+    <row r="339" spans="1:3">
+      <c r="A339" t="s">
         <v>390</v>
       </c>
-      <c r="B338" t="s">
+      <c r="B339" t="s">
         <v>566</v>
       </c>
     </row>
-    <row r="339" spans="1:3" customFormat="1">
-      <c r="A339" t="s">
+    <row r="340" spans="1:3">
+      <c r="A340" t="s">
         <v>391</v>
       </c>
-      <c r="B339" t="s">
+      <c r="B340" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="340" spans="1:3" customFormat="1">
-      <c r="A340" t="s">
+    <row r="341" spans="1:3">
+      <c r="A341" t="s">
         <v>1123</v>
       </c>
-      <c r="B340" t="s">
+      <c r="B341" t="s">
         <v>1124</v>
       </c>
-      <c r="C340" t="s">
+      <c r="C341" t="s">
         <v>1125</v>
       </c>
     </row>
-    <row r="341" spans="1:3" customFormat="1">
-      <c r="A341" t="s">
+    <row r="342" spans="1:3">
+      <c r="A342" t="s">
         <v>476</v>
       </c>
-      <c r="B341" t="s">
+      <c r="B342" t="s">
         <v>1153</v>
       </c>
     </row>
-    <row r="343" spans="1:3" customFormat="1">
-      <c r="A343" t="s">
+    <row r="344" spans="1:3">
+      <c r="A344" t="s">
         <v>718</v>
       </c>
-      <c r="B343" t="s">
+      <c r="B344" t="s">
         <v>719</v>
-      </c>
-      <c r="C343" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="344" spans="1:3" customFormat="1">
-      <c r="A344" t="s">
-        <v>720</v>
-      </c>
-      <c r="B344" t="s">
-        <v>1154</v>
       </c>
       <c r="C344" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="346" spans="1:3" customFormat="1">
-      <c r="A346" t="s">
+    <row r="345" spans="1:3">
+      <c r="A345" t="s">
+        <v>720</v>
+      </c>
+      <c r="B345" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C345" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3">
+      <c r="A347" t="s">
         <v>726</v>
       </c>
-      <c r="B346" t="s">
+      <c r="B347" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="347" spans="1:3" customFormat="1">
-      <c r="A347" t="s">
+    <row r="348" spans="1:3">
+      <c r="A348" t="s">
         <v>728</v>
       </c>
-      <c r="B347" t="s">
+      <c r="B348" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="348" spans="1:3" customFormat="1">
-      <c r="A348" t="s">
+    <row r="349" spans="1:3">
+      <c r="A349" t="s">
         <v>730</v>
       </c>
-      <c r="B348" t="s">
+      <c r="B349" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="349" spans="1:3" customFormat="1">
-      <c r="A349" t="s">
+    <row r="350" spans="1:3">
+      <c r="A350" t="s">
         <v>732</v>
       </c>
-      <c r="B349" t="s">
+      <c r="B350" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="350" spans="1:3" customFormat="1">
-      <c r="A350" t="s">
+    <row r="351" spans="1:3">
+      <c r="A351" t="s">
         <v>734</v>
       </c>
-      <c r="B350" t="s">
+      <c r="B351" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="351" spans="1:3" customFormat="1">
-      <c r="A351" t="s">
+    <row r="352" spans="1:3">
+      <c r="A352" t="s">
         <v>736</v>
       </c>
-      <c r="B351" t="s">
+      <c r="B352" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="352" spans="1:3" customFormat="1">
-      <c r="A352" t="s">
+    <row r="353" spans="1:2">
+      <c r="A353" t="s">
         <v>738</v>
       </c>
-      <c r="B352" t="s">
+      <c r="B353" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="353" spans="1:2" customFormat="1">
-      <c r="A353" t="s">
+    <row r="354" spans="1:2">
+      <c r="A354" t="s">
         <v>740</v>
       </c>
-      <c r="B353" t="s">
+      <c r="B354" t="s">
         <v>741</v>
       </c>
     </row>
-    <row r="354" spans="1:2" customFormat="1">
-      <c r="A354" t="s">
+    <row r="355" spans="1:2">
+      <c r="A355" t="s">
         <v>742</v>
       </c>
-      <c r="B354" t="s">
+      <c r="B355" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="355" spans="1:2" customFormat="1">
-      <c r="A355" t="s">
+    <row r="356" spans="1:2">
+      <c r="A356" t="s">
         <v>744</v>
       </c>
-      <c r="B355" t="s">
+      <c r="B356" t="s">
         <v>745</v>
       </c>
     </row>
-    <row r="356" spans="1:2" customFormat="1">
-      <c r="A356" t="s">
+    <row r="357" spans="1:2">
+      <c r="A357" t="s">
         <v>746</v>
       </c>
-      <c r="B356" t="s">
+      <c r="B357" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="357" spans="1:2" customFormat="1">
-      <c r="A357" t="s">
+    <row r="358" spans="1:2">
+      <c r="A358" t="s">
         <v>748</v>
       </c>
-      <c r="B357" t="s">
+      <c r="B358" t="s">
         <v>749</v>
       </c>
     </row>
-    <row r="358" spans="1:2" customFormat="1">
-      <c r="A358" t="s">
+    <row r="359" spans="1:2">
+      <c r="A359" t="s">
         <v>750</v>
       </c>
-      <c r="B358" t="s">
+      <c r="B359" t="s">
         <v>751</v>
       </c>
     </row>
-    <row r="359" spans="1:2" customFormat="1">
-      <c r="A359" t="s">
+    <row r="360" spans="1:2">
+      <c r="A360" t="s">
         <v>752</v>
       </c>
-      <c r="B359" t="s">
+      <c r="B360" t="s">
         <v>753</v>
       </c>
     </row>
-    <row r="360" spans="1:2" customFormat="1">
-      <c r="A360" t="s">
+    <row r="361" spans="1:2">
+      <c r="A361" t="s">
         <v>754</v>
       </c>
-      <c r="B360" t="s">
+      <c r="B361" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="361" spans="1:2" customFormat="1">
-      <c r="A361" t="s">
+    <row r="362" spans="1:2">
+      <c r="A362" t="s">
         <v>756</v>
       </c>
-      <c r="B361" t="s">
+      <c r="B362" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="362" spans="1:2" customFormat="1">
-      <c r="A362" t="s">
+    <row r="363" spans="1:2">
+      <c r="A363" t="s">
         <v>1119</v>
       </c>
-      <c r="B362" t="s">
+      <c r="B363" t="s">
         <v>1120</v>
       </c>
     </row>
-    <row r="363" spans="1:2" customFormat="1">
-      <c r="A363" t="s">
+    <row r="364" spans="1:2">
+      <c r="A364" t="s">
         <v>758</v>
       </c>
-      <c r="B363" t="s">
+      <c r="B364" t="s">
         <v>759</v>
       </c>
     </row>
-    <row r="364" spans="1:2" customFormat="1">
-      <c r="A364" t="s">
+    <row r="365" spans="1:2">
+      <c r="A365" t="s">
         <v>1122</v>
       </c>
-      <c r="B364" t="s">
+      <c r="B365" t="s">
         <v>1155</v>
       </c>
     </row>
-    <row r="366" spans="1:2" customFormat="1">
-      <c r="A366" t="s">
+    <row r="367" spans="1:2">
+      <c r="A367" t="s">
         <v>760</v>
       </c>
-      <c r="B366" t="s">
+      <c r="B367" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="367" spans="1:2" customFormat="1">
-      <c r="A367" t="s">
+    <row r="368" spans="1:2">
+      <c r="A368" t="s">
         <v>762</v>
       </c>
-      <c r="B367" t="s">
+      <c r="B368" t="s">
         <v>763</v>
       </c>
     </row>
-    <row r="368" spans="1:2" customFormat="1">
-      <c r="A368" t="s">
+    <row r="369" spans="1:2">
+      <c r="A369" t="s">
         <v>764</v>
       </c>
-      <c r="B368" t="s">
+      <c r="B369" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="369" spans="1:2" customFormat="1">
-      <c r="A369" t="s">
+    <row r="370" spans="1:2">
+      <c r="A370" t="s">
         <v>766</v>
       </c>
-      <c r="B369" t="s">
+      <c r="B370" t="s">
         <v>767</v>
       </c>
     </row>
-    <row r="370" spans="1:2" customFormat="1">
-      <c r="A370" t="s">
+    <row r="371" spans="1:2">
+      <c r="A371" t="s">
         <v>768</v>
       </c>
-      <c r="B370" t="s">
+      <c r="B371" t="s">
         <v>769</v>
       </c>
     </row>
-    <row r="371" spans="1:2" customFormat="1">
-      <c r="A371" t="s">
+    <row r="372" spans="1:2">
+      <c r="A372" t="s">
         <v>770</v>
       </c>
-      <c r="B371" t="s">
+      <c r="B372" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="372" spans="1:2" customFormat="1">
-      <c r="A372" t="s">
+    <row r="373" spans="1:2">
+      <c r="A373" t="s">
         <v>772</v>
       </c>
-      <c r="B372" t="s">
+      <c r="B373" t="s">
         <v>773</v>
       </c>
     </row>
-    <row r="373" spans="1:2" customFormat="1">
-      <c r="A373" t="s">
+    <row r="374" spans="1:2">
+      <c r="A374" t="s">
         <v>774</v>
       </c>
-      <c r="B373" t="s">
+      <c r="B374" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="374" spans="1:2" customFormat="1">
-      <c r="A374" t="s">
+    <row r="375" spans="1:2">
+      <c r="A375" t="s">
         <v>775</v>
       </c>
-      <c r="B374" t="s">
+      <c r="B375" t="s">
         <v>776</v>
       </c>
     </row>
-    <row r="375" spans="1:2" customFormat="1">
-      <c r="A375" t="s">
+    <row r="376" spans="1:2">
+      <c r="A376" t="s">
         <v>777</v>
       </c>
-      <c r="B375" t="s">
+      <c r="B376" t="s">
         <v>778</v>
       </c>
     </row>
-    <row r="376" spans="1:2" customFormat="1">
-      <c r="A376" t="s">
+    <row r="377" spans="1:2">
+      <c r="A377" t="s">
         <v>779</v>
       </c>
-      <c r="B376" t="s">
+      <c r="B377" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="377" spans="1:2" customFormat="1">
-      <c r="A377" t="s">
+    <row r="378" spans="1:2">
+      <c r="A378" t="s">
         <v>781</v>
       </c>
-      <c r="B377" t="s">
+      <c r="B378" t="s">
         <v>1156</v>
       </c>
     </row>
-    <row r="379" spans="1:2" customFormat="1">
-      <c r="A379" t="s">
+    <row r="380" spans="1:2">
+      <c r="A380" t="s">
         <v>782</v>
       </c>
-      <c r="B379" t="s">
+      <c r="B380" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="380" spans="1:2" customFormat="1">
-      <c r="A380" t="s">
+    <row r="381" spans="1:2">
+      <c r="A381" t="s">
         <v>783</v>
       </c>
-      <c r="B380" t="s">
+      <c r="B381" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="381" spans="1:2" customFormat="1">
-      <c r="A381" t="s">
+    <row r="382" spans="1:2">
+      <c r="A382" t="s">
         <v>785</v>
       </c>
-      <c r="B381" t="s">
+      <c r="B382" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="382" spans="1:2" customFormat="1">
-      <c r="A382" t="s">
+    <row r="383" spans="1:2">
+      <c r="A383" t="s">
         <v>786</v>
       </c>
-      <c r="B382" t="s">
+      <c r="B383" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="384" spans="1:2" customFormat="1">
-      <c r="A384" t="s">
+    <row r="385" spans="1:2">
+      <c r="A385" t="s">
         <v>808</v>
       </c>
-      <c r="B384" t="s">
+      <c r="B385" t="s">
         <v>809</v>
       </c>
     </row>
-    <row r="385" spans="1:2" customFormat="1">
-      <c r="A385" t="s">
+    <row r="386" spans="1:2">
+      <c r="A386" t="s">
         <v>807</v>
       </c>
-      <c r="B385" t="s">
+      <c r="B386" t="s">
         <v>806</v>
       </c>
     </row>
-    <row r="386" spans="1:2" customFormat="1">
-      <c r="A386" t="s">
+    <row r="387" spans="1:2">
+      <c r="A387" t="s">
         <v>801</v>
       </c>
-      <c r="B386" t="s">
+      <c r="B387" t="s">
         <v>802</v>
       </c>
     </row>
-    <row r="387" spans="1:2" customFormat="1">
-      <c r="A387" t="s">
+    <row r="388" spans="1:2">
+      <c r="A388" t="s">
         <v>799</v>
       </c>
-      <c r="B387" t="s">
+      <c r="B388" t="s">
         <v>803</v>
       </c>
     </row>
-    <row r="388" spans="1:2" customFormat="1">
-      <c r="A388" t="s">
+    <row r="389" spans="1:2">
+      <c r="A389" t="s">
         <v>800</v>
       </c>
-      <c r="B388" t="s">
+      <c r="B389" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="389" spans="1:2" customFormat="1">
-      <c r="A389" t="s">
+    <row r="390" spans="1:2">
+      <c r="A390" t="s">
         <v>805</v>
       </c>
-      <c r="B389" t="s">
+      <c r="B390" t="s">
         <v>1157</v>
       </c>
     </row>
-    <row r="391" spans="1:2" customFormat="1">
-      <c r="A391" t="s">
+    <row r="392" spans="1:2">
+      <c r="A392" t="s">
         <v>812</v>
       </c>
-      <c r="B391" t="s">
+      <c r="B392" t="s">
         <v>817</v>
       </c>
     </row>
-    <row r="392" spans="1:2" customFormat="1">
-      <c r="A392" t="s">
+    <row r="393" spans="1:2">
+      <c r="A393" t="s">
         <v>819</v>
       </c>
-      <c r="B392" t="s">
+      <c r="B393" t="s">
         <v>818</v>
       </c>
     </row>
-    <row r="393" spans="1:2" customFormat="1">
-      <c r="A393" t="s">
+    <row r="394" spans="1:2">
+      <c r="A394" t="s">
         <v>813</v>
       </c>
-      <c r="B393" t="s">
+      <c r="B394" t="s">
         <v>802</v>
       </c>
     </row>
-    <row r="394" spans="1:2" customFormat="1">
-      <c r="A394" t="s">
+    <row r="395" spans="1:2">
+      <c r="A395" t="s">
         <v>814</v>
       </c>
-      <c r="B394" t="s">
+      <c r="B395" t="s">
         <v>803</v>
       </c>
     </row>
-    <row r="395" spans="1:2" customFormat="1">
-      <c r="A395" t="s">
+    <row r="396" spans="1:2">
+      <c r="A396" t="s">
         <v>815</v>
       </c>
-      <c r="B395" t="s">
+      <c r="B396" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="396" spans="1:2" customFormat="1">
-      <c r="A396" t="s">
+    <row r="397" spans="1:2">
+      <c r="A397" t="s">
         <v>816</v>
       </c>
-      <c r="B396" t="s">
+      <c r="B397" t="s">
         <v>1158</v>
       </c>
     </row>
-    <row r="398" spans="1:2" customFormat="1">
-      <c r="A398" t="s">
+    <row r="399" spans="1:2">
+      <c r="A399" t="s">
         <v>824</v>
       </c>
-      <c r="B398" t="s">
+      <c r="B399" t="s">
         <v>825</v>
       </c>
     </row>
-    <row r="399" spans="1:2" customFormat="1">
-      <c r="A399" t="s">
+    <row r="400" spans="1:2">
+      <c r="A400" t="s">
         <v>826</v>
       </c>
-      <c r="B399" t="s">
+      <c r="B400" t="s">
         <v>1116</v>
       </c>
     </row>
-    <row r="400" spans="1:2" customFormat="1">
-      <c r="A400" t="s">
+    <row r="401" spans="1:2">
+      <c r="A401" t="s">
         <v>827</v>
       </c>
-      <c r="B400" t="s">
+      <c r="B401" t="s">
         <v>1020</v>
       </c>
     </row>
-    <row r="401" spans="1:2" customFormat="1">
-      <c r="A401" t="s">
+    <row r="402" spans="1:2">
+      <c r="A402" t="s">
         <v>829</v>
       </c>
-      <c r="B401" t="s">
+      <c r="B402" t="s">
         <v>1021</v>
       </c>
     </row>
-    <row r="402" spans="1:2" customFormat="1">
-      <c r="A402" t="s">
+    <row r="403" spans="1:2">
+      <c r="A403" t="s">
         <v>835</v>
       </c>
-      <c r="B402" t="s">
+      <c r="B403" t="s">
         <v>1022</v>
       </c>
     </row>
-    <row r="403" spans="1:2" customFormat="1">
-      <c r="A403" t="s">
+    <row r="404" spans="1:2">
+      <c r="A404" t="s">
         <v>836</v>
       </c>
-      <c r="B403" t="s">
+      <c r="B404" t="s">
         <v>1023</v>
       </c>
     </row>
-    <row r="404" spans="1:2" customFormat="1">
-      <c r="A404" t="s">
+    <row r="405" spans="1:2">
+      <c r="A405" t="s">
         <v>837</v>
       </c>
-      <c r="B404" t="s">
+      <c r="B405" t="s">
         <v>1024</v>
       </c>
     </row>
-    <row r="405" spans="1:2" customFormat="1">
-      <c r="A405" t="s">
+    <row r="406" spans="1:2">
+      <c r="A406" t="s">
         <v>840</v>
       </c>
-      <c r="B405" t="s">
+      <c r="B406" t="s">
         <v>1025</v>
       </c>
     </row>
-    <row r="406" spans="1:2" customFormat="1">
-      <c r="A406" t="s">
+    <row r="407" spans="1:2">
+      <c r="A407" t="s">
         <v>841</v>
       </c>
-      <c r="B406" t="s">
+      <c r="B407" t="s">
         <v>1026</v>
       </c>
     </row>
-    <row r="407" spans="1:2" customFormat="1">
-      <c r="A407" t="s">
+    <row r="408" spans="1:2">
+      <c r="A408" t="s">
         <v>842</v>
       </c>
-      <c r="B407" t="s">
+      <c r="B408" t="s">
         <v>1027</v>
       </c>
     </row>
-    <row r="408" spans="1:2" customFormat="1">
-      <c r="A408" t="s">
+    <row r="409" spans="1:2">
+      <c r="A409" t="s">
         <v>843</v>
       </c>
-      <c r="B408" t="s">
+      <c r="B409" t="s">
         <v>1028</v>
       </c>
     </row>
-    <row r="409" spans="1:2" customFormat="1">
-      <c r="A409" t="s">
+    <row r="410" spans="1:2">
+      <c r="A410" t="s">
         <v>844</v>
       </c>
-      <c r="B409" t="s">
+      <c r="B410" t="s">
         <v>1029</v>
       </c>
     </row>
-    <row r="410" spans="1:2" customFormat="1">
-      <c r="A410" t="s">
+    <row r="411" spans="1:2">
+      <c r="A411" t="s">
         <v>845</v>
       </c>
-      <c r="B410" t="s">
+      <c r="B411" t="s">
         <v>834</v>
       </c>
     </row>
-    <row r="411" spans="1:2" customFormat="1">
-      <c r="A411" t="s">
+    <row r="412" spans="1:2">
+      <c r="A412" t="s">
         <v>846</v>
       </c>
-      <c r="B411" t="s">
+      <c r="B412" t="s">
         <v>1030</v>
       </c>
     </row>
-    <row r="412" spans="1:2" customFormat="1">
-      <c r="A412" t="s">
+    <row r="413" spans="1:2">
+      <c r="A413" t="s">
         <v>847</v>
       </c>
-      <c r="B412" t="s">
+      <c r="B413" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="413" spans="1:2" customFormat="1">
-      <c r="A413" t="s">
+    <row r="414" spans="1:2">
+      <c r="A414" t="s">
         <v>848</v>
       </c>
-      <c r="B413" t="s">
+      <c r="B414" t="s">
         <v>793</v>
       </c>
     </row>
-    <row r="414" spans="1:2" customFormat="1">
-      <c r="A414" t="s">
+    <row r="415" spans="1:2">
+      <c r="A415" t="s">
         <v>839</v>
       </c>
-      <c r="B414" t="s">
+      <c r="B415" t="s">
         <v>608</v>
       </c>
     </row>
-    <row r="415" spans="1:2" customFormat="1">
-      <c r="A415" t="s">
+    <row r="416" spans="1:2">
+      <c r="A416" t="s">
         <v>838</v>
       </c>
-      <c r="B415" t="s">
+      <c r="B416" t="s">
         <v>1159</v>
       </c>
     </row>
-    <row r="416" spans="1:2" customFormat="1">
-      <c r="A416" t="s">
+    <row r="417" spans="1:2">
+      <c r="A417" t="s">
         <v>1031</v>
       </c>
-      <c r="B416" t="s">
+      <c r="B417" t="s">
         <v>1032</v>
       </c>
     </row>
-    <row r="417" spans="1:2" customFormat="1">
-      <c r="A417" t="s">
+    <row r="418" spans="1:2">
+      <c r="A418" t="s">
         <v>1033</v>
       </c>
-      <c r="B417" t="s">
+      <c r="B418" t="s">
         <v>1034</v>
       </c>
     </row>
-    <row r="418" spans="1:2" customFormat="1">
-      <c r="A418" t="s">
+    <row r="419" spans="1:2">
+      <c r="A419" t="s">
         <v>1035</v>
       </c>
-      <c r="B418" t="s">
+      <c r="B419" t="s">
         <v>1036</v>
       </c>
     </row>
-    <row r="419" spans="1:2" customFormat="1">
-      <c r="A419" t="s">
+    <row r="420" spans="1:2">
+      <c r="A420" t="s">
         <v>1037</v>
       </c>
-      <c r="B419" t="s">
+      <c r="B420" t="s">
         <v>1038</v>
       </c>
     </row>
-    <row r="420" spans="1:2" customFormat="1">
-      <c r="A420" t="s">
+    <row r="421" spans="1:2">
+      <c r="A421" t="s">
         <v>1039</v>
       </c>
-      <c r="B420" t="s">
+      <c r="B421" t="s">
         <v>1040</v>
       </c>
     </row>
-    <row r="421" spans="1:2" customFormat="1">
-      <c r="A421" t="s">
+    <row r="422" spans="1:2">
+      <c r="A422" t="s">
         <v>1041</v>
       </c>
-      <c r="B421" t="s">
+      <c r="B422" t="s">
         <v>1042</v>
       </c>
     </row>
-    <row r="422" spans="1:2" customFormat="1">
-      <c r="A422" t="s">
+    <row r="423" spans="1:2">
+      <c r="A423" t="s">
         <v>1043</v>
       </c>
-      <c r="B422" t="s">
+      <c r="B423" t="s">
         <v>1044</v>
       </c>
     </row>
-    <row r="423" spans="1:2" customFormat="1">
-      <c r="A423" t="s">
+    <row r="424" spans="1:2">
+      <c r="A424" t="s">
         <v>1045</v>
       </c>
-      <c r="B423" t="s">
+      <c r="B424" t="s">
         <v>1046</v>
       </c>
     </row>
-    <row r="424" spans="1:2" customFormat="1">
-      <c r="A424" t="s">
+    <row r="425" spans="1:2">
+      <c r="A425" t="s">
         <v>1168</v>
       </c>
-      <c r="B424" t="s">
+      <c r="B425" t="s">
         <v>1169</v>
       </c>
     </row>
-    <row r="426" spans="1:2" customFormat="1">
-      <c r="A426" t="s">
+    <row r="427" spans="1:2">
+      <c r="A427" t="s">
         <v>888</v>
       </c>
-      <c r="B426" t="s">
+      <c r="B427" t="s">
         <v>889</v>
       </c>
     </row>
-    <row r="427" spans="1:2" customFormat="1">
-      <c r="A427" t="s">
+    <row r="428" spans="1:2">
+      <c r="A428" t="s">
         <v>890</v>
       </c>
-      <c r="B427" t="s">
+      <c r="B428" t="s">
         <v>891</v>
       </c>
     </row>
-    <row r="428" spans="1:2" customFormat="1">
-      <c r="A428" t="s">
+    <row r="429" spans="1:2">
+      <c r="A429" t="s">
         <v>892</v>
       </c>
-      <c r="B428" t="s">
+      <c r="B429" t="s">
         <v>893</v>
       </c>
     </row>
-    <row r="429" spans="1:2" customFormat="1">
-      <c r="A429" t="s">
+    <row r="430" spans="1:2">
+      <c r="A430" t="s">
         <v>894</v>
       </c>
-      <c r="B429" t="s">
+      <c r="B430" t="s">
         <v>895</v>
       </c>
     </row>
-    <row r="430" spans="1:2" customFormat="1">
-      <c r="A430" t="s">
+    <row r="431" spans="1:2">
+      <c r="A431" t="s">
         <v>896</v>
       </c>
-      <c r="B430" t="s">
+      <c r="B431" t="s">
         <v>897</v>
       </c>
     </row>
-    <row r="431" spans="1:2" customFormat="1">
-      <c r="A431" t="s">
+    <row r="432" spans="1:2">
+      <c r="A432" t="s">
         <v>898</v>
       </c>
-      <c r="B431" t="s">
+      <c r="B432" t="s">
         <v>899</v>
       </c>
     </row>
-    <row r="432" spans="1:2" customFormat="1">
-      <c r="A432" t="s">
+    <row r="433" spans="1:2">
+      <c r="A433" t="s">
         <v>900</v>
       </c>
-      <c r="B432" t="s">
+      <c r="B433" t="s">
         <v>901</v>
       </c>
     </row>
-    <row r="433" spans="1:2" customFormat="1">
-      <c r="A433" t="s">
+    <row r="434" spans="1:2">
+      <c r="A434" t="s">
         <v>902</v>
       </c>
-      <c r="B433" t="s">
+      <c r="B434" t="s">
         <v>903</v>
       </c>
     </row>
-    <row r="434" spans="1:2" customFormat="1">
-      <c r="A434" t="s">
+    <row r="435" spans="1:2">
+      <c r="A435" t="s">
         <v>904</v>
       </c>
-      <c r="B434" t="s">
+      <c r="B435" t="s">
         <v>905</v>
       </c>
     </row>
-    <row r="435" spans="1:2" customFormat="1">
-      <c r="A435" t="s">
+    <row r="436" spans="1:2">
+      <c r="A436" t="s">
         <v>906</v>
       </c>
-      <c r="B435" t="s">
+      <c r="B436" t="s">
         <v>907</v>
       </c>
     </row>
-    <row r="436" spans="1:2" customFormat="1">
-      <c r="A436" t="s">
+    <row r="437" spans="1:2">
+      <c r="A437" t="s">
         <v>908</v>
       </c>
-      <c r="B436" t="s">
+      <c r="B437" t="s">
         <v>909</v>
       </c>
     </row>
-    <row r="437" spans="1:2" customFormat="1">
-      <c r="A437" t="s">
+    <row r="438" spans="1:2">
+      <c r="A438" t="s">
         <v>910</v>
       </c>
-      <c r="B437" t="s">
+      <c r="B438" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="438" spans="1:2" customFormat="1">
-      <c r="A438" t="s">
+    <row r="439" spans="1:2">
+      <c r="A439" t="s">
         <v>912</v>
       </c>
-      <c r="B438" t="s">
+      <c r="B439" t="s">
         <v>913</v>
       </c>
     </row>
-    <row r="439" spans="1:2" customFormat="1">
-      <c r="A439" t="s">
+    <row r="440" spans="1:2">
+      <c r="A440" t="s">
         <v>914</v>
       </c>
-      <c r="B439" t="s">
+      <c r="B440" t="s">
         <v>915</v>
       </c>
     </row>
-    <row r="440" spans="1:2" customFormat="1">
-      <c r="A440" t="s">
+    <row r="441" spans="1:2">
+      <c r="A441" t="s">
         <v>916</v>
       </c>
-      <c r="B440" t="s">
+      <c r="B441" t="s">
         <v>917</v>
       </c>
     </row>
-    <row r="441" spans="1:2" customFormat="1">
-      <c r="A441" t="s">
+    <row r="442" spans="1:2">
+      <c r="A442" t="s">
         <v>918</v>
       </c>
-      <c r="B441" t="s">
+      <c r="B442" t="s">
         <v>919</v>
       </c>
     </row>
-    <row r="442" spans="1:2" customFormat="1">
-      <c r="A442" t="s">
+    <row r="443" spans="1:2">
+      <c r="A443" t="s">
         <v>920</v>
       </c>
-      <c r="B442" t="s">
+      <c r="B443" t="s">
         <v>921</v>
       </c>
     </row>
-    <row r="443" spans="1:2" customFormat="1">
-      <c r="A443" t="s">
+    <row r="444" spans="1:2">
+      <c r="A444" t="s">
         <v>922</v>
       </c>
-      <c r="B443" t="s">
+      <c r="B444" t="s">
         <v>923</v>
       </c>
     </row>
-    <row r="444" spans="1:2" customFormat="1">
-      <c r="A444" t="s">
+    <row r="445" spans="1:2">
+      <c r="A445" t="s">
         <v>924</v>
       </c>
-      <c r="B444" t="s">
+      <c r="B445" t="s">
         <v>925</v>
       </c>
     </row>
-    <row r="445" spans="1:2" customFormat="1">
-      <c r="A445" t="s">
+    <row r="446" spans="1:2">
+      <c r="A446" t="s">
         <v>926</v>
       </c>
-      <c r="B445" t="s">
+      <c r="B446" t="s">
         <v>927</v>
       </c>
     </row>
-    <row r="446" spans="1:2" customFormat="1">
-      <c r="A446" t="s">
+    <row r="447" spans="1:2">
+      <c r="A447" t="s">
         <v>928</v>
       </c>
-      <c r="B446" t="s">
+      <c r="B447" t="s">
         <v>1160</v>
       </c>
     </row>
-    <row r="448" spans="1:2" customFormat="1">
-      <c r="A448" t="s">
+    <row r="449" spans="1:2">
+      <c r="A449" t="s">
         <v>1127</v>
       </c>
-      <c r="B448" t="s">
+      <c r="B449" t="s">
         <v>1128</v>
       </c>
     </row>
-    <row r="449" spans="1:2" customFormat="1">
-      <c r="A449" t="s">
+    <row r="450" spans="1:2">
+      <c r="A450" t="s">
         <v>929</v>
       </c>
-      <c r="B449" t="s">
+      <c r="B450" t="s">
         <v>930</v>
       </c>
     </row>
-    <row r="450" spans="1:2" customFormat="1">
-      <c r="A450" t="s">
+    <row r="451" spans="1:2">
+      <c r="A451" t="s">
         <v>931</v>
       </c>
-      <c r="B450" t="s">
+      <c r="B451" t="s">
         <v>932</v>
       </c>
     </row>
-    <row r="451" spans="1:2" customFormat="1">
-      <c r="A451" t="s">
+    <row r="452" spans="1:2">
+      <c r="A452" t="s">
         <v>933</v>
       </c>
-      <c r="B451" t="s">
+      <c r="B452" t="s">
         <v>934</v>
       </c>
     </row>
-    <row r="452" spans="1:2" customFormat="1">
-      <c r="A452" t="s">
+    <row r="453" spans="1:2">
+      <c r="A453" t="s">
         <v>935</v>
       </c>
-      <c r="B452" t="s">
+      <c r="B453" t="s">
         <v>936</v>
       </c>
     </row>
-    <row r="453" spans="1:2" customFormat="1">
-      <c r="A453" t="s">
+    <row r="454" spans="1:2">
+      <c r="A454" t="s">
         <v>937</v>
       </c>
-      <c r="B453" t="s">
+      <c r="B454" t="s">
         <v>1088</v>
       </c>
     </row>
-    <row r="454" spans="1:2" customFormat="1">
-      <c r="A454" t="s">
+    <row r="455" spans="1:2">
+      <c r="A455" t="s">
         <v>938</v>
       </c>
-      <c r="B454" t="s">
+      <c r="B455" t="s">
         <v>1089</v>
       </c>
     </row>
-    <row r="455" spans="1:2" customFormat="1">
-      <c r="A455" t="s">
+    <row r="456" spans="1:2">
+      <c r="A456" t="s">
         <v>939</v>
       </c>
-      <c r="B455" t="s">
+      <c r="B456" t="s">
         <v>1090</v>
       </c>
     </row>
-    <row r="456" spans="1:2" customFormat="1">
-      <c r="A456" t="s">
+    <row r="457" spans="1:2">
+      <c r="A457" t="s">
         <v>940</v>
       </c>
-      <c r="B456" t="s">
+      <c r="B457" t="s">
         <v>941</v>
       </c>
     </row>
-    <row r="457" spans="1:2" customFormat="1">
-      <c r="A457" t="s">
+    <row r="458" spans="1:2">
+      <c r="A458" t="s">
         <v>942</v>
       </c>
-      <c r="B457" t="s">
+      <c r="B458" t="s">
         <v>943</v>
       </c>
     </row>
-    <row r="458" spans="1:2" customFormat="1">
-      <c r="A458" t="s">
+    <row r="459" spans="1:2">
+      <c r="A459" t="s">
         <v>944</v>
       </c>
-      <c r="B458" t="s">
+      <c r="B459" t="s">
         <v>1161</v>
       </c>
     </row>
-    <row r="460" spans="1:2" customFormat="1">
-      <c r="A460" t="s">
+    <row r="461" spans="1:2">
+      <c r="A461" t="s">
         <v>951</v>
       </c>
-      <c r="B460" t="s">
+      <c r="B461" t="s">
         <v>952</v>
       </c>
     </row>
-    <row r="461" spans="1:2" customFormat="1">
-      <c r="A461" t="s">
+    <row r="462" spans="1:2">
+      <c r="A462" t="s">
         <v>953</v>
       </c>
-      <c r="B461" t="s">
+      <c r="B462" t="s">
         <v>1162</v>
       </c>
     </row>
-    <row r="463" spans="1:2" customFormat="1">
-      <c r="A463" t="s">
+    <row r="464" spans="1:2">
+      <c r="A464" t="s">
         <v>954</v>
       </c>
-      <c r="B463" t="s">
+      <c r="B464" t="s">
         <v>955</v>
       </c>
     </row>
-    <row r="464" spans="1:2" customFormat="1">
-      <c r="A464" t="s">
+    <row r="465" spans="1:2">
+      <c r="A465" t="s">
         <v>956</v>
       </c>
-      <c r="B464" t="s">
+      <c r="B465" t="s">
         <v>1163</v>
       </c>
     </row>
-    <row r="465" spans="1:2" customFormat="1"/>
-    <row r="466" spans="1:2" customFormat="1">
-      <c r="A466" t="s">
+    <row r="467" spans="1:2">
+      <c r="A467" t="s">
         <v>957</v>
       </c>
-      <c r="B466" t="s">
+      <c r="B467" t="s">
         <v>958</v>
       </c>
     </row>
-    <row r="467" spans="1:2" customFormat="1">
-      <c r="A467" t="s">
+    <row r="468" spans="1:2">
+      <c r="A468" t="s">
         <v>959</v>
       </c>
-      <c r="B467" t="s">
+      <c r="B468" t="s">
         <v>960</v>
       </c>
     </row>
-    <row r="468" spans="1:2" customFormat="1">
-      <c r="A468" t="s">
+    <row r="469" spans="1:2">
+      <c r="A469" t="s">
         <v>961</v>
       </c>
-      <c r="B468" t="s">
+      <c r="B469" t="s">
         <v>1164</v>
       </c>
     </row>
-    <row r="470" spans="1:2" customFormat="1">
-      <c r="A470" t="s">
+    <row r="471" spans="1:2">
+      <c r="A471" t="s">
         <v>962</v>
       </c>
-      <c r="B470" t="s">
+      <c r="B471" t="s">
         <v>963</v>
       </c>
     </row>
-    <row r="471" spans="1:2" customFormat="1">
-      <c r="A471" t="s">
+    <row r="472" spans="1:2">
+      <c r="A472" t="s">
         <v>964</v>
       </c>
-      <c r="B471" t="s">
+      <c r="B472" t="s">
         <v>965</v>
       </c>
     </row>
-    <row r="472" spans="1:2" customFormat="1">
-      <c r="A472" t="s">
+    <row r="473" spans="1:2">
+      <c r="A473" t="s">
         <v>966</v>
       </c>
-      <c r="B472" t="s">
+      <c r="B473" t="s">
         <v>967</v>
       </c>
     </row>
-    <row r="473" spans="1:2" customFormat="1">
-      <c r="A473" t="s">
+    <row r="474" spans="1:2">
+      <c r="A474" t="s">
         <v>968</v>
       </c>
-      <c r="B473" t="s">
+      <c r="B474" t="s">
         <v>969</v>
       </c>
     </row>
-    <row r="474" spans="1:2" customFormat="1">
-      <c r="A474" t="s">
+    <row r="475" spans="1:2">
+      <c r="A475" t="s">
         <v>970</v>
       </c>
-      <c r="B474" t="s">
+      <c r="B475" t="s">
         <v>971</v>
       </c>
     </row>
-    <row r="475" spans="1:2" customFormat="1">
-      <c r="A475" t="s">
+    <row r="476" spans="1:2">
+      <c r="A476" t="s">
         <v>972</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B476" t="s">
         <v>973</v>
       </c>
     </row>
-    <row r="476" spans="1:2" customFormat="1">
-      <c r="A476" t="s">
+    <row r="477" spans="1:2">
+      <c r="A477" t="s">
         <v>974</v>
       </c>
-      <c r="B476" t="s">
+      <c r="B477" t="s">
         <v>1129</v>
       </c>
     </row>
-    <row r="478" spans="1:2" customFormat="1">
-      <c r="A478" t="s">
+    <row r="479" spans="1:2">
+      <c r="A479" t="s">
         <v>975</v>
       </c>
-      <c r="B478" t="s">
+      <c r="B479" t="s">
         <v>976</v>
       </c>
     </row>
-    <row r="479" spans="1:2" customFormat="1">
-      <c r="A479" t="s">
+    <row r="480" spans="1:2">
+      <c r="A480" t="s">
         <v>977</v>
       </c>
-      <c r="B479" t="s">
+      <c r="B480" t="s">
         <v>978</v>
       </c>
     </row>
-    <row r="480" spans="1:2" customFormat="1">
-      <c r="A480" t="s">
+    <row r="481" spans="1:2">
+      <c r="A481" t="s">
         <v>979</v>
       </c>
-      <c r="B480" t="s">
+      <c r="B481" t="s">
         <v>980</v>
       </c>
     </row>
-    <row r="481" spans="1:2" customFormat="1">
-      <c r="A481" t="s">
+    <row r="482" spans="1:2">
+      <c r="A482" t="s">
         <v>981</v>
       </c>
-      <c r="B481" t="s">
+      <c r="B482" t="s">
         <v>982</v>
       </c>
     </row>
-    <row r="482" spans="1:2" customFormat="1">
-      <c r="A482" t="s">
+    <row r="483" spans="1:2">
+      <c r="A483" t="s">
         <v>983</v>
       </c>
-      <c r="B482" t="s">
+      <c r="B483" t="s">
         <v>984</v>
       </c>
     </row>
-    <row r="483" spans="1:2" customFormat="1">
-      <c r="A483" t="s">
+    <row r="484" spans="1:2">
+      <c r="A484" t="s">
         <v>985</v>
       </c>
-      <c r="B483" t="s">
+      <c r="B484" t="s">
         <v>1130</v>
       </c>
     </row>
-    <row r="485" spans="1:2" customFormat="1">
-      <c r="A485" t="s">
+    <row r="486" spans="1:2">
+      <c r="A486" t="s">
         <v>986</v>
       </c>
-      <c r="B485" t="s">
+      <c r="B486" t="s">
         <v>987</v>
       </c>
     </row>
-    <row r="486" spans="1:2" customFormat="1">
-      <c r="A486" t="s">
+    <row r="487" spans="1:2">
+      <c r="A487" t="s">
         <v>988</v>
       </c>
-      <c r="B486" t="s">
+      <c r="B487" t="s">
         <v>989</v>
       </c>
     </row>
-    <row r="487" spans="1:2" customFormat="1">
-      <c r="A487" t="s">
+    <row r="488" spans="1:2">
+      <c r="A488" t="s">
         <v>990</v>
       </c>
-      <c r="B487" t="s">
+      <c r="B488" t="s">
         <v>991</v>
       </c>
     </row>
-    <row r="488" spans="1:2" customFormat="1">
-      <c r="A488" t="s">
+    <row r="489" spans="1:2">
+      <c r="A489" t="s">
         <v>992</v>
       </c>
-      <c r="B488" t="s">
+      <c r="B489" t="s">
         <v>993</v>
       </c>
     </row>
-    <row r="489" spans="1:2" customFormat="1">
-      <c r="A489" t="s">
+    <row r="490" spans="1:2">
+      <c r="A490" t="s">
         <v>994</v>
       </c>
-      <c r="B489" t="s">
+      <c r="B490" t="s">
         <v>995</v>
       </c>
     </row>
-    <row r="490" spans="1:2" customFormat="1">
-      <c r="A490" t="s">
+    <row r="491" spans="1:2">
+      <c r="A491" t="s">
         <v>996</v>
       </c>
-      <c r="B490" t="s">
+      <c r="B491" t="s">
         <v>1131</v>
       </c>
     </row>
-    <row r="492" spans="1:2" customFormat="1">
-      <c r="A492" t="s">
+    <row r="493" spans="1:2">
+      <c r="A493" t="s">
         <v>997</v>
       </c>
-      <c r="B492" t="s">
+      <c r="B493" t="s">
         <v>998</v>
       </c>
     </row>
-    <row r="493" spans="1:2" customFormat="1">
-      <c r="A493" t="s">
+    <row r="494" spans="1:2">
+      <c r="A494" t="s">
         <v>999</v>
       </c>
-      <c r="B493" t="s">
+      <c r="B494" t="s">
         <v>1000</v>
       </c>
     </row>
-    <row r="494" spans="1:2" customFormat="1">
-      <c r="A494" t="s">
+    <row r="495" spans="1:2">
+      <c r="A495" t="s">
         <v>1001</v>
       </c>
-      <c r="B494" t="s">
+      <c r="B495" t="s">
         <v>1002</v>
       </c>
     </row>
-    <row r="495" spans="1:2" customFormat="1">
-      <c r="A495" t="s">
+    <row r="496" spans="1:2">
+      <c r="A496" t="s">
         <v>1003</v>
       </c>
-      <c r="B495" t="s">
+      <c r="B496" t="s">
         <v>1004</v>
       </c>
     </row>
-    <row r="496" spans="1:2" customFormat="1">
-      <c r="A496" t="s">
+    <row r="497" spans="1:2">
+      <c r="A497" t="s">
         <v>1005</v>
       </c>
-      <c r="B496" t="s">
+      <c r="B497" t="s">
         <v>1132</v>
       </c>
     </row>
-    <row r="497" spans="1:2" customFormat="1"/>
-    <row r="498" spans="1:2" customFormat="1">
-      <c r="A498" t="s">
+    <row r="499" spans="1:2">
+      <c r="A499" t="s">
         <v>1047</v>
       </c>
-      <c r="B498" t="s">
+      <c r="B499" t="s">
         <v>1048</v>
       </c>
     </row>
-    <row r="499" spans="1:2" customFormat="1">
-      <c r="A499" t="s">
+    <row r="500" spans="1:2">
+      <c r="A500" t="s">
         <v>1049</v>
       </c>
-      <c r="B499" t="s">
+      <c r="B500" t="s">
         <v>1050</v>
       </c>
     </row>
-    <row r="500" spans="1:2" customFormat="1">
-      <c r="A500" t="s">
+    <row r="501" spans="1:2">
+      <c r="A501" t="s">
         <v>1051</v>
       </c>
-      <c r="B500" t="s">
+      <c r="B501" t="s">
         <v>1052</v>
       </c>
     </row>
-    <row r="501" spans="1:2" customFormat="1">
-      <c r="A501" t="s">
+    <row r="502" spans="1:2">
+      <c r="A502" t="s">
         <v>1053</v>
       </c>
-      <c r="B501" t="s">
+      <c r="B502" t="s">
         <v>1054</v>
       </c>
     </row>
-    <row r="502" spans="1:2" customFormat="1">
-      <c r="A502" t="s">
+    <row r="503" spans="1:2">
+      <c r="A503" t="s">
         <v>1055</v>
       </c>
-      <c r="B502" t="s">
+      <c r="B503" t="s">
         <v>1056</v>
       </c>
     </row>
-    <row r="503" spans="1:2" customFormat="1">
-      <c r="A503" t="s">
+    <row r="504" spans="1:2">
+      <c r="A504" t="s">
         <v>1057</v>
       </c>
-      <c r="B503" t="s">
+      <c r="B504" t="s">
         <v>1058</v>
       </c>
     </row>
-    <row r="504" spans="1:2" customFormat="1">
-      <c r="A504" t="s">
+    <row r="505" spans="1:2">
+      <c r="A505" t="s">
         <v>1059</v>
       </c>
-      <c r="B504" t="s">
+      <c r="B505" t="s">
         <v>1060</v>
       </c>
     </row>
-    <row r="505" spans="1:2" customFormat="1">
-      <c r="A505" t="s">
+    <row r="506" spans="1:2">
+      <c r="A506" t="s">
         <v>1061</v>
       </c>
-      <c r="B505" t="s">
+      <c r="B506" t="s">
         <v>1062</v>
       </c>
     </row>
-    <row r="506" spans="1:2" customFormat="1">
-      <c r="A506" t="s">
+    <row r="507" spans="1:2">
+      <c r="A507" t="s">
         <v>1063</v>
       </c>
-      <c r="B506" t="s">
+      <c r="B507" t="s">
         <v>1064</v>
       </c>
     </row>
-    <row r="507" spans="1:2" customFormat="1">
-      <c r="A507" t="s">
+    <row r="508" spans="1:2">
+      <c r="A508" t="s">
         <v>1065</v>
       </c>
-      <c r="B507" t="s">
+      <c r="B508" t="s">
         <v>1066</v>
       </c>
     </row>
-    <row r="508" spans="1:2" customFormat="1">
-      <c r="A508" t="s">
+    <row r="509" spans="1:2">
+      <c r="A509" t="s">
         <v>1067</v>
       </c>
-      <c r="B508" t="s">
+      <c r="B509" t="s">
         <v>1068</v>
       </c>
     </row>
-    <row r="509" spans="1:2" customFormat="1">
-      <c r="A509" t="s">
+    <row r="510" spans="1:2">
+      <c r="A510" t="s">
         <v>1069</v>
       </c>
-      <c r="B509" t="s">
+      <c r="B510" t="s">
         <v>1070</v>
       </c>
     </row>
-    <row r="510" spans="1:2" customFormat="1">
-      <c r="A510" t="s">
+    <row r="511" spans="1:2">
+      <c r="A511" t="s">
         <v>1071</v>
       </c>
-      <c r="B510" t="s">
+      <c r="B511" t="s">
         <v>1072</v>
       </c>
     </row>
-    <row r="511" spans="1:2" customFormat="1">
-      <c r="A511" t="s">
+    <row r="512" spans="1:2">
+      <c r="A512" t="s">
         <v>1073</v>
       </c>
-      <c r="B511" t="s">
+      <c r="B512" t="s">
         <v>1133</v>
       </c>
     </row>
+    <row r="513" customFormat="1"/>
   </sheetData>
-  <conditionalFormatting sqref="A449:A458">
+  <conditionalFormatting sqref="A450:A459">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A466:A467 A463:A464 A460:A461">
+  <conditionalFormatting sqref="A467:A468 A464:A465 A461:A462">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added the newly added findings to config file and implemented the approach for files not to be sent to sites
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CEDF37-99FE-4EE8-BAA4-CDCA415BAE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7BD922-12E2-4E1B-BA60-BA14D53F9A66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="37920" windowHeight="18870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1432" uniqueCount="1200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="1203">
   <si>
     <t>Name</t>
   </si>
@@ -3640,6 +3640,15 @@
   </si>
   <si>
     <t>ApplicationReviewProcess</t>
+  </si>
+  <si>
+    <t>BackToSiteStates</t>
+  </si>
+  <si>
+    <t>NotBackToSiteStates</t>
+  </si>
+  <si>
+    <t>YardiReviewer</t>
   </si>
 </sst>
 </file>
@@ -7110,7 +7119,7 @@
   <dimension ref="A1:Z1014"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="1" max="1" width="37.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.140625" customWidth="1"/>
     <col min="3" max="3" width="60.28515625" customWidth="1"/>
     <col min="4" max="26" width="65.42578125" customWidth="1"/>
@@ -7552,9 +7561,30 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="52" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="53" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="54" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="52" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A52" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A53" t="s">
+        <v>1201</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1201</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A54" t="s">
+        <v>1202</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1202</v>
+      </c>
+    </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="56" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="57" spans="1:2" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
updated audit findings and yardi library version
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raluca.ilinca.AzureAI-Jump2\Documents\Git\Application-Review-Process_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB7BD922-12E2-4E1B-BA60-BA14D53F9A66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A7BD996-09F2-4FFC-A8B4-16334B484CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28320" windowHeight="13470" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="1203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1449" uniqueCount="1206">
   <si>
     <t>Name</t>
   </si>
@@ -3649,6 +3649,15 @@
   </si>
   <si>
     <t>YardiReviewer</t>
+  </si>
+  <si>
+    <t>Business asked to remove.</t>
+  </si>
+  <si>
+    <t>ASFAExists</t>
+  </si>
+  <si>
+    <t>Affidavit of Student Financial Assistance is present in the application, manual review required.</t>
   </si>
 </sst>
 </file>
@@ -8553,7 +8562,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB30D651-CF18-42CB-8A58-9F597F965D74}">
-  <dimension ref="A1:C523"/>
+  <dimension ref="A1:C524"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -9509,352 +9518,376 @@
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>141</v>
+        <v>1204</v>
       </c>
       <c r="B115" t="s">
-        <v>144</v>
+        <v>1205</v>
+      </c>
+      <c r="C115" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B116" t="s">
-        <v>145</v>
+        <v>144</v>
+      </c>
+      <c r="C116" t="s">
+        <v>1203</v>
       </c>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B117" t="s">
-        <v>146</v>
+        <v>145</v>
+      </c>
+      <c r="C117" t="s">
+        <v>1203</v>
       </c>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B118" t="s">
-        <v>519</v>
+        <v>146</v>
       </c>
       <c r="C118" t="s">
-        <v>597</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>596</v>
+        <v>139</v>
       </c>
       <c r="B119" t="s">
         <v>519</v>
       </c>
+      <c r="C119" t="s">
+        <v>597</v>
+      </c>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>140</v>
+        <v>596</v>
       </c>
       <c r="B120" t="s">
-        <v>123</v>
+        <v>519</v>
+      </c>
+      <c r="C120" t="s">
+        <v>1203</v>
       </c>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="B121" t="s">
-        <v>536</v>
+        <v>123</v>
+      </c>
+      <c r="C121" t="s">
+        <v>1203</v>
       </c>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B122" t="s">
-        <v>124</v>
+        <v>536</v>
+      </c>
+      <c r="C122" t="s">
+        <v>1203</v>
       </c>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>574</v>
+        <v>126</v>
       </c>
       <c r="B123" t="s">
-        <v>575</v>
+        <v>124</v>
+      </c>
+      <c r="C123" t="s">
+        <v>1203</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
+        <v>574</v>
+      </c>
+      <c r="B124" t="s">
+        <v>575</v>
+      </c>
+      <c r="C124" t="s">
+        <v>1203</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3">
+      <c r="A125" t="s">
         <v>485</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B125" t="s">
         <v>1116</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3">
-      <c r="A126" t="s">
-        <v>181</v>
-      </c>
-      <c r="B126" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>127</v>
+        <v>181</v>
       </c>
       <c r="B127" t="s">
-        <v>147</v>
+        <v>182</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B129" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>705</v>
+        <v>128</v>
       </c>
       <c r="B130" t="s">
-        <v>704</v>
-      </c>
-      <c r="C130" t="s">
-        <v>598</v>
+        <v>149</v>
       </c>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>130</v>
+        <v>705</v>
       </c>
       <c r="B131" t="s">
-        <v>150</v>
+        <v>704</v>
+      </c>
+      <c r="C131" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B132" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>565</v>
+        <v>131</v>
       </c>
       <c r="B133" t="s">
-        <v>601</v>
-      </c>
-      <c r="C133" t="s">
-        <v>605</v>
+        <v>151</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>576</v>
+        <v>565</v>
       </c>
       <c r="B134" t="s">
-        <v>577</v>
+        <v>601</v>
+      </c>
+      <c r="C134" t="s">
+        <v>605</v>
       </c>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>624</v>
+        <v>576</v>
       </c>
       <c r="B135" t="s">
-        <v>625</v>
-      </c>
-      <c r="C135" t="s">
-        <v>598</v>
+        <v>577</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
+        <v>624</v>
+      </c>
+      <c r="B136" t="s">
+        <v>625</v>
+      </c>
+      <c r="C136" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3">
+      <c r="A137" t="s">
         <v>484</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B137" t="s">
         <v>1117</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3">
-      <c r="A138" t="s">
-        <v>614</v>
-      </c>
-      <c r="B138" t="s">
-        <v>615</v>
-      </c>
-      <c r="C138" t="s">
-        <v>616</v>
       </c>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="B139" t="s">
-        <v>1141</v>
+        <v>615</v>
       </c>
       <c r="C139" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="141" spans="1:3">
-      <c r="A141" t="s">
-        <v>153</v>
-      </c>
-      <c r="B141" t="s">
-        <v>157</v>
+    <row r="140" spans="1:3">
+      <c r="A140" t="s">
+        <v>617</v>
+      </c>
+      <c r="B140" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C140" t="s">
+        <v>616</v>
       </c>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B142" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B143" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B144" t="s">
-        <v>537</v>
+        <v>159</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>501</v>
+        <v>156</v>
       </c>
       <c r="B145" t="s">
-        <v>638</v>
-      </c>
-      <c r="C145" t="s">
-        <v>639</v>
+        <v>537</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>1089</v>
+        <v>501</v>
       </c>
       <c r="B146" t="s">
-        <v>1097</v>
+        <v>638</v>
       </c>
       <c r="C146" t="s">
-        <v>598</v>
+        <v>639</v>
       </c>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>582</v>
+        <v>1089</v>
       </c>
       <c r="B147" t="s">
-        <v>583</v>
+        <v>1097</v>
+      </c>
+      <c r="C147" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
+        <v>582</v>
+      </c>
+      <c r="B148" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3">
+      <c r="A149" t="s">
         <v>483</v>
       </c>
-      <c r="B148" t="s">
+      <c r="B149" t="s">
         <v>1142</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3">
-      <c r="A150" t="s">
-        <v>185</v>
-      </c>
-      <c r="B150" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>160</v>
+        <v>185</v>
       </c>
       <c r="B151" t="s">
-        <v>162</v>
+        <v>186</v>
       </c>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B152" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>578</v>
+        <v>161</v>
       </c>
       <c r="B153" t="s">
-        <v>579</v>
+        <v>163</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>482</v>
+        <v>578</v>
       </c>
       <c r="B154" t="s">
-        <v>1118</v>
+        <v>579</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
+        <v>482</v>
+      </c>
+      <c r="B155" t="s">
+        <v>1118</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3">
+      <c r="A156" t="s">
         <v>626</v>
       </c>
-      <c r="B155" t="s">
+      <c r="B156" t="s">
         <v>627</v>
       </c>
-      <c r="C155" t="s">
+      <c r="C156" t="s">
         <v>598</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3">
-      <c r="A157" t="s">
-        <v>183</v>
-      </c>
-      <c r="B157" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="B158" t="s">
-        <v>166</v>
-      </c>
-      <c r="C158" t="s">
-        <v>527</v>
+        <v>184</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B159" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C159" t="s">
         <v>527</v>
@@ -9862,10 +9895,10 @@
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B160" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C160" t="s">
         <v>527</v>
@@ -9873,86 +9906,86 @@
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>194</v>
+        <v>165</v>
       </c>
       <c r="B161" t="s">
-        <v>193</v>
+        <v>168</v>
+      </c>
+      <c r="C161" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B162" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>170</v>
+        <v>191</v>
       </c>
       <c r="B163" t="s">
-        <v>171</v>
-      </c>
-      <c r="C163" t="s">
-        <v>527</v>
+        <v>192</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>580</v>
+        <v>170</v>
       </c>
       <c r="B164" t="s">
-        <v>581</v>
+        <v>171</v>
+      </c>
+      <c r="C164" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
+        <v>580</v>
+      </c>
+      <c r="B165" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3">
+      <c r="A166" t="s">
         <v>471</v>
       </c>
-      <c r="B165" t="s">
+      <c r="B166" t="s">
         <v>1119</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3">
-      <c r="A167" t="s">
-        <v>1144</v>
-      </c>
-      <c r="B167" t="s">
-        <v>785</v>
-      </c>
-      <c r="C167" t="s">
-        <v>1145</v>
       </c>
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>587</v>
+        <v>1144</v>
       </c>
       <c r="B168" t="s">
-        <v>848</v>
+        <v>785</v>
       </c>
       <c r="C168" t="s">
-        <v>588</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>629</v>
+        <v>587</v>
       </c>
       <c r="B169" t="s">
-        <v>630</v>
+        <v>848</v>
       </c>
       <c r="C169" t="s">
-        <v>598</v>
+        <v>588</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>715</v>
+        <v>629</v>
       </c>
       <c r="B170" t="s">
-        <v>849</v>
+        <v>630</v>
       </c>
       <c r="C170" t="s">
         <v>598</v>
@@ -9960,10 +9993,10 @@
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="B171" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="C171" t="s">
         <v>598</v>
@@ -9971,10 +10004,10 @@
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B172" t="s">
-        <v>701</v>
+        <v>850</v>
       </c>
       <c r="C172" t="s">
         <v>598</v>
@@ -9982,186 +10015,186 @@
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
+        <v>717</v>
+      </c>
+      <c r="B173" t="s">
+        <v>701</v>
+      </c>
+      <c r="C173" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3">
+      <c r="A174" t="s">
         <v>1084</v>
       </c>
-      <c r="B173" t="s">
+      <c r="B174" t="s">
         <v>855</v>
       </c>
-      <c r="C173" t="s">
+      <c r="C174" t="s">
         <v>1157</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3">
-      <c r="A175" t="s">
-        <v>462</v>
-      </c>
-      <c r="B175" t="s">
-        <v>1158</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>1098</v>
+        <v>462</v>
       </c>
       <c r="B176" t="s">
-        <v>1099</v>
-      </c>
-      <c r="C176" t="s">
-        <v>1100</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>233</v>
+        <v>1098</v>
       </c>
       <c r="B177" t="s">
-        <v>851</v>
+        <v>1099</v>
       </c>
       <c r="C177" t="s">
-        <v>527</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B178" t="s">
-        <v>852</v>
+        <v>851</v>
+      </c>
+      <c r="C178" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="B179" t="s">
-        <v>853</v>
-      </c>
-      <c r="C179" t="s">
-        <v>585</v>
+        <v>852</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>686</v>
+        <v>242</v>
       </c>
       <c r="B180" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="C180" t="s">
-        <v>598</v>
+        <v>585</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>236</v>
+        <v>686</v>
       </c>
       <c r="B181" t="s">
-        <v>235</v>
+        <v>854</v>
+      </c>
+      <c r="C181" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>452</v>
+        <v>236</v>
       </c>
       <c r="B182" t="s">
-        <v>461</v>
+        <v>235</v>
       </c>
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>237</v>
+        <v>452</v>
       </c>
       <c r="B183" t="s">
-        <v>855</v>
-      </c>
-      <c r="C183" t="s">
-        <v>1159</v>
+        <v>461</v>
       </c>
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B184" t="s">
-        <v>856</v>
+        <v>855</v>
+      </c>
+      <c r="C184" t="s">
+        <v>1159</v>
       </c>
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B185" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B186" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B187" t="s">
-        <v>785</v>
+        <v>858</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>273</v>
+        <v>241</v>
       </c>
       <c r="B188" t="s">
-        <v>855</v>
-      </c>
-      <c r="C188" t="s">
-        <v>1159</v>
+        <v>785</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>300</v>
+        <v>273</v>
       </c>
       <c r="B189" t="s">
-        <v>301</v>
+        <v>855</v>
+      </c>
+      <c r="C189" t="s">
+        <v>1159</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>590</v>
+        <v>300</v>
       </c>
       <c r="B190" t="s">
-        <v>1082</v>
+        <v>301</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>607</v>
+        <v>590</v>
       </c>
       <c r="B191" t="s">
-        <v>786</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>672</v>
+        <v>607</v>
       </c>
       <c r="B192" t="s">
-        <v>673</v>
-      </c>
-      <c r="C192" t="s">
-        <v>598</v>
+        <v>786</v>
       </c>
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>685</v>
+        <v>672</v>
       </c>
       <c r="B193" t="s">
-        <v>703</v>
+        <v>673</v>
       </c>
       <c r="C193" t="s">
         <v>598</v>
@@ -10169,817 +10202,817 @@
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>867</v>
+        <v>685</v>
       </c>
       <c r="B194" t="s">
-        <v>868</v>
+        <v>703</v>
+      </c>
+      <c r="C194" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>470</v>
+        <v>867</v>
       </c>
       <c r="B195" t="s">
-        <v>1120</v>
+        <v>868</v>
       </c>
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
+        <v>470</v>
+      </c>
+      <c r="B196" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3">
+      <c r="A197" t="s">
         <v>1160</v>
       </c>
-      <c r="B196" t="s">
+      <c r="B197" t="s">
         <v>1161</v>
-      </c>
-    </row>
-    <row r="198" spans="1:3">
-      <c r="A198" t="s">
-        <v>683</v>
-      </c>
-      <c r="B198" t="s">
-        <v>684</v>
-      </c>
-      <c r="C198" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>463</v>
+        <v>683</v>
       </c>
       <c r="B199" t="s">
-        <v>1162</v>
+        <v>684</v>
+      </c>
+      <c r="C199" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
+        <v>463</v>
+      </c>
+      <c r="B200" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3">
+      <c r="A201" t="s">
         <v>243</v>
       </c>
-      <c r="B200" t="s">
+      <c r="B201" t="s">
         <v>859</v>
       </c>
-      <c r="C200" t="s">
+      <c r="C201" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="201" spans="1:3" ht="13.5" customHeight="1">
-      <c r="A201" t="s">
+    <row r="202" spans="1:3" ht="13.5" customHeight="1">
+      <c r="A202" t="s">
         <v>245</v>
       </c>
-      <c r="B201" t="s">
+      <c r="B202" t="s">
         <v>860</v>
       </c>
-      <c r="C201" t="s">
+      <c r="C202" t="s">
         <v>602</v>
-      </c>
-    </row>
-    <row r="202" spans="1:3">
-      <c r="A202" t="s">
-        <v>244</v>
-      </c>
-      <c r="B202" t="s">
-        <v>821</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B203" t="s">
-        <v>246</v>
+        <v>821</v>
       </c>
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B204" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B205" t="s">
-        <v>250</v>
-      </c>
-      <c r="C205" t="s">
-        <v>592</v>
+        <v>249</v>
       </c>
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>453</v>
+        <v>251</v>
       </c>
       <c r="B206" t="s">
-        <v>509</v>
+        <v>250</v>
+      </c>
+      <c r="C206" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>252</v>
+        <v>453</v>
       </c>
       <c r="B207" t="s">
-        <v>823</v>
+        <v>509</v>
       </c>
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B208" t="s">
-        <v>254</v>
+        <v>823</v>
       </c>
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="B209" t="s">
-        <v>824</v>
+        <v>254</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B210" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B211" t="s">
-        <v>861</v>
-      </c>
-      <c r="C211" t="s">
-        <v>592</v>
+        <v>825</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B212" t="s">
-        <v>826</v>
+        <v>861</v>
+      </c>
+      <c r="C212" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B213" t="s">
-        <v>862</v>
-      </c>
-      <c r="C213" t="s">
-        <v>592</v>
+        <v>826</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B214" t="s">
-        <v>827</v>
+        <v>862</v>
+      </c>
+      <c r="C214" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="B215" t="s">
-        <v>271</v>
+        <v>827</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B216" t="s">
-        <v>855</v>
-      </c>
-      <c r="C216" t="s">
-        <v>1159</v>
+        <v>271</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B217" t="s">
-        <v>275</v>
+        <v>855</v>
+      </c>
+      <c r="C217" t="s">
+        <v>1159</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>608</v>
+        <v>274</v>
       </c>
       <c r="B218" t="s">
-        <v>786</v>
+        <v>275</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>481</v>
+        <v>608</v>
       </c>
       <c r="B219" t="s">
-        <v>1121</v>
+        <v>786</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
+        <v>481</v>
+      </c>
+      <c r="B220" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3">
+      <c r="A221" t="s">
         <v>603</v>
       </c>
-      <c r="B220" t="s">
+      <c r="B221" t="s">
         <v>604</v>
       </c>
-      <c r="C220" t="s">
+      <c r="C221" t="s">
         <v>598</v>
-      </c>
-    </row>
-    <row r="222" spans="1:3">
-      <c r="A222" t="s">
-        <v>464</v>
-      </c>
-      <c r="B222" t="s">
-        <v>1163</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>454</v>
+        <v>464</v>
       </c>
       <c r="B223" t="s">
-        <v>510</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>268</v>
+        <v>454</v>
       </c>
       <c r="B224" t="s">
-        <v>787</v>
+        <v>510</v>
       </c>
     </row>
     <row r="225" spans="1:2">
       <c r="A225" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B225" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="226" spans="1:2">
       <c r="A226" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="B226" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="227" spans="1:2">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B227" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
     </row>
     <row r="228" spans="1:2">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B228" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
     </row>
     <row r="229" spans="1:2">
       <c r="A229" t="s">
-        <v>609</v>
+        <v>278</v>
       </c>
       <c r="B229" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
     </row>
     <row r="230" spans="1:2">
       <c r="A230" t="s">
+        <v>609</v>
+      </c>
+      <c r="B230" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2">
+      <c r="A231" t="s">
         <v>480</v>
       </c>
-      <c r="B230" t="s">
+      <c r="B231" t="s">
         <v>1122</v>
-      </c>
-    </row>
-    <row r="232" spans="1:2">
-      <c r="A232" t="s">
-        <v>465</v>
-      </c>
-      <c r="B232" t="s">
-        <v>1164</v>
       </c>
     </row>
     <row r="233" spans="1:2">
       <c r="A233" t="s">
-        <v>455</v>
+        <v>465</v>
       </c>
       <c r="B233" t="s">
-        <v>511</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="234" spans="1:2">
       <c r="A234" t="s">
-        <v>281</v>
+        <v>455</v>
       </c>
       <c r="B234" t="s">
-        <v>780</v>
+        <v>511</v>
       </c>
     </row>
     <row r="235" spans="1:2">
       <c r="A235" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B235" t="s">
-        <v>284</v>
+        <v>780</v>
       </c>
     </row>
     <row r="236" spans="1:2">
       <c r="A236" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B236" t="s">
-        <v>781</v>
+        <v>284</v>
       </c>
     </row>
     <row r="237" spans="1:2">
       <c r="A237" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B237" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
     </row>
     <row r="238" spans="1:2">
       <c r="A238" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B238" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
     </row>
     <row r="239" spans="1:2">
       <c r="A239" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B239" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="240" spans="1:2">
       <c r="A240" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B240" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>610</v>
+        <v>288</v>
       </c>
       <c r="B241" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
+        <v>610</v>
+      </c>
+      <c r="B242" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3">
+      <c r="A243" t="s">
         <v>479</v>
       </c>
-      <c r="B242" t="s">
+      <c r="B243" t="s">
         <v>1123</v>
-      </c>
-    </row>
-    <row r="244" spans="1:3">
-      <c r="A244" t="s">
-        <v>466</v>
-      </c>
-      <c r="B244" t="s">
-        <v>1165</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>450</v>
+        <v>466</v>
       </c>
       <c r="B245" t="s">
-        <v>294</v>
-      </c>
-      <c r="C245" t="s">
-        <v>527</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="B246" t="s">
-        <v>512</v>
+        <v>294</v>
+      </c>
+      <c r="C246" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>292</v>
+        <v>456</v>
       </c>
       <c r="B247" t="s">
-        <v>863</v>
-      </c>
-      <c r="C247" t="s">
-        <v>527</v>
+        <v>512</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B248" t="s">
-        <v>846</v>
+        <v>863</v>
+      </c>
+      <c r="C248" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>449</v>
+        <v>293</v>
       </c>
       <c r="B249" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>295</v>
+        <v>449</v>
       </c>
       <c r="B250" t="s">
-        <v>855</v>
-      </c>
-      <c r="C250" t="s">
-        <v>1166</v>
+        <v>847</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B251" t="s">
-        <v>864</v>
+        <v>855</v>
+      </c>
+      <c r="C251" t="s">
+        <v>1166</v>
       </c>
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B252" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B253" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B254" t="s">
-        <v>785</v>
+        <v>866</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>611</v>
+        <v>299</v>
       </c>
       <c r="B255" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
+        <v>611</v>
+      </c>
+      <c r="B256" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3">
+      <c r="A257" t="s">
         <v>478</v>
       </c>
-      <c r="B256" t="s">
+      <c r="B257" t="s">
         <v>1124</v>
-      </c>
-    </row>
-    <row r="258" spans="1:3">
-      <c r="A258" t="s">
-        <v>644</v>
-      </c>
-      <c r="B258" t="s">
-        <v>645</v>
-      </c>
-      <c r="C258" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>495</v>
+        <v>644</v>
       </c>
       <c r="B259" t="s">
-        <v>498</v>
+        <v>645</v>
       </c>
       <c r="C259" t="s">
-        <v>525</v>
+        <v>598</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B260" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C260" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>524</v>
+        <v>496</v>
       </c>
       <c r="B261" t="s">
-        <v>538</v>
+        <v>497</v>
+      </c>
+      <c r="C261" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>316</v>
+        <v>524</v>
       </c>
       <c r="B262" t="s">
-        <v>302</v>
+        <v>538</v>
       </c>
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B263" t="s">
-        <v>303</v>
-      </c>
-      <c r="C263" t="s">
-        <v>527</v>
+        <v>302</v>
       </c>
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>457</v>
+        <v>317</v>
       </c>
       <c r="B264" t="s">
-        <v>513</v>
+        <v>303</v>
+      </c>
+      <c r="C264" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>318</v>
+        <v>457</v>
       </c>
       <c r="B265" t="s">
-        <v>304</v>
+        <v>513</v>
       </c>
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B266" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B267" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B268" t="s">
-        <v>307</v>
-      </c>
-      <c r="C268" t="s">
-        <v>527</v>
+        <v>306</v>
       </c>
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B269" t="s">
-        <v>308</v>
+        <v>307</v>
+      </c>
+      <c r="C269" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B270" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B271" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B272" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B273" t="s">
-        <v>312</v>
-      </c>
-      <c r="C273" t="s">
-        <v>527</v>
+        <v>311</v>
       </c>
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B274" t="s">
-        <v>313</v>
+        <v>312</v>
+      </c>
+      <c r="C274" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B275" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B276" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
+        <v>329</v>
+      </c>
+      <c r="B277" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3">
+      <c r="A278" t="s">
         <v>477</v>
       </c>
-      <c r="B277" t="s">
+      <c r="B278" t="s">
         <v>1125</v>
-      </c>
-    </row>
-    <row r="279" spans="1:3">
-      <c r="A279" t="s">
-        <v>542</v>
-      </c>
-      <c r="B279" t="s">
-        <v>543</v>
       </c>
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>336</v>
+        <v>542</v>
       </c>
       <c r="B280" t="s">
-        <v>354</v>
+        <v>543</v>
       </c>
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B281" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B282" t="s">
-        <v>352</v>
-      </c>
-      <c r="C282" t="s">
-        <v>527</v>
+        <v>351</v>
       </c>
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>458</v>
+        <v>338</v>
       </c>
       <c r="B283" t="s">
-        <v>514</v>
+        <v>352</v>
+      </c>
+      <c r="C283" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
-        <v>355</v>
+        <v>458</v>
       </c>
       <c r="B284" t="s">
-        <v>353</v>
-      </c>
-      <c r="C284" t="s">
-        <v>527</v>
+        <v>514</v>
       </c>
     </row>
     <row r="285" spans="1:3">
       <c r="A285" t="s">
-        <v>339</v>
+        <v>355</v>
       </c>
       <c r="B285" t="s">
-        <v>345</v>
+        <v>353</v>
+      </c>
+      <c r="C285" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="286" spans="1:3">
       <c r="A286" t="s">
-        <v>356</v>
+        <v>339</v>
       </c>
       <c r="B286" t="s">
-        <v>346</v>
-      </c>
-      <c r="C286" t="s">
-        <v>504</v>
+        <v>345</v>
       </c>
     </row>
     <row r="287" spans="1:3">
       <c r="A287" t="s">
-        <v>340</v>
+        <v>356</v>
       </c>
       <c r="B287" t="s">
-        <v>347</v>
+        <v>346</v>
+      </c>
+      <c r="C287" t="s">
+        <v>504</v>
       </c>
     </row>
     <row r="288" spans="1:3">
       <c r="A288" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B288" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="289" spans="1:3">
       <c r="A289" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B289" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="290" spans="1:3">
       <c r="A290" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B290" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="291" spans="1:3">
       <c r="A291" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B291" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="292" spans="1:3">
       <c r="A292" t="s">
-        <v>1067</v>
+        <v>344</v>
       </c>
       <c r="B292" t="s">
-        <v>1068</v>
-      </c>
-      <c r="C292" t="s">
-        <v>1069</v>
+        <v>347</v>
       </c>
     </row>
     <row r="293" spans="1:3">
       <c r="A293" t="s">
-        <v>1070</v>
+        <v>1067</v>
       </c>
       <c r="B293" t="s">
-        <v>1071</v>
+        <v>1068</v>
       </c>
       <c r="C293" t="s">
         <v>1069</v>
@@ -10987,10 +11020,10 @@
     </row>
     <row r="294" spans="1:3">
       <c r="A294" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="B294" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="C294" t="s">
         <v>1069</v>
@@ -10998,48 +11031,48 @@
     </row>
     <row r="295" spans="1:3">
       <c r="A295" t="s">
-        <v>476</v>
+        <v>1072</v>
       </c>
       <c r="B295" t="s">
-        <v>1126</v>
+        <v>1073</v>
+      </c>
+      <c r="C295" t="s">
+        <v>1069</v>
       </c>
     </row>
     <row r="296" spans="1:3">
       <c r="A296" t="s">
+        <v>476</v>
+      </c>
+      <c r="B296" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3">
+      <c r="A297" t="s">
         <v>1167</v>
       </c>
-      <c r="B296" t="s">
+      <c r="B297" t="s">
         <v>1168</v>
-      </c>
-    </row>
-    <row r="298" spans="1:3">
-      <c r="A298" t="s">
-        <v>646</v>
-      </c>
-      <c r="B298" t="s">
-        <v>664</v>
-      </c>
-      <c r="C298" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="299" spans="1:3">
       <c r="A299" t="s">
-        <v>1074</v>
+        <v>646</v>
       </c>
       <c r="B299" t="s">
-        <v>1075</v>
+        <v>664</v>
       </c>
       <c r="C299" t="s">
-        <v>1069</v>
+        <v>598</v>
       </c>
     </row>
     <row r="300" spans="1:3">
       <c r="A300" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="B300" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="C300" t="s">
         <v>1069</v>
@@ -11047,78 +11080,78 @@
     </row>
     <row r="301" spans="1:3">
       <c r="A301" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="B301" t="s">
-        <v>1127</v>
+        <v>1077</v>
       </c>
       <c r="C301" t="s">
         <v>1069</v>
       </c>
     </row>
-    <row r="303" spans="1:3">
-      <c r="A303" t="s">
-        <v>642</v>
-      </c>
-      <c r="B303" t="s">
-        <v>643</v>
-      </c>
-      <c r="C303" t="s">
-        <v>598</v>
+    <row r="302" spans="1:3">
+      <c r="A302" t="s">
+        <v>1078</v>
+      </c>
+      <c r="B302" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C302" t="s">
+        <v>1069</v>
       </c>
     </row>
     <row r="304" spans="1:3">
       <c r="A304" t="s">
-        <v>467</v>
+        <v>642</v>
       </c>
       <c r="B304" t="s">
-        <v>468</v>
+        <v>643</v>
+      </c>
+      <c r="C304" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="305" spans="1:3">
       <c r="A305" t="s">
-        <v>362</v>
+        <v>467</v>
       </c>
       <c r="B305" t="s">
-        <v>373</v>
+        <v>468</v>
       </c>
     </row>
     <row r="306" spans="1:3">
       <c r="A306" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B306" t="s">
-        <v>374</v>
-      </c>
-      <c r="C306" t="s">
-        <v>527</v>
+        <v>373</v>
       </c>
     </row>
     <row r="307" spans="1:3">
       <c r="A307" t="s">
-        <v>515</v>
+        <v>363</v>
       </c>
       <c r="B307" t="s">
-        <v>516</v>
+        <v>374</v>
+      </c>
+      <c r="C307" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="308" spans="1:3">
       <c r="A308" t="s">
-        <v>364</v>
+        <v>515</v>
       </c>
       <c r="B308" t="s">
-        <v>375</v>
-      </c>
-      <c r="C308" t="s">
-        <v>527</v>
+        <v>516</v>
       </c>
     </row>
     <row r="309" spans="1:3">
       <c r="A309" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B309" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C309" t="s">
         <v>527</v>
@@ -11126,155 +11159,155 @@
     </row>
     <row r="310" spans="1:3">
       <c r="A310" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B310" t="s">
-        <v>528</v>
+        <v>376</v>
+      </c>
+      <c r="C310" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="311" spans="1:3">
       <c r="A311" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B311" t="s">
-        <v>377</v>
+        <v>528</v>
       </c>
     </row>
     <row r="312" spans="1:3">
       <c r="A312" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B312" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="313" spans="1:3">
       <c r="A313" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B313" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="314" spans="1:3">
       <c r="A314" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B314" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="315" spans="1:3">
       <c r="A315" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B315" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="316" spans="1:3">
       <c r="A316" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B316" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="317" spans="1:3">
       <c r="A317" t="s">
-        <v>699</v>
+        <v>372</v>
       </c>
       <c r="B317" t="s">
-        <v>1079</v>
-      </c>
-      <c r="C317" t="s">
-        <v>598</v>
+        <v>382</v>
       </c>
     </row>
     <row r="318" spans="1:3">
       <c r="A318" t="s">
-        <v>1092</v>
+        <v>699</v>
       </c>
       <c r="B318" t="s">
-        <v>1093</v>
+        <v>1079</v>
+      </c>
+      <c r="C318" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="319" spans="1:3">
       <c r="A319" t="s">
-        <v>474</v>
+        <v>1092</v>
       </c>
       <c r="B319" t="s">
-        <v>1128</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="320" spans="1:3">
       <c r="A320" t="s">
-        <v>551</v>
+        <v>474</v>
       </c>
       <c r="B320" t="s">
-        <v>552</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="321" spans="1:3">
       <c r="A321" t="s">
+        <v>551</v>
+      </c>
+      <c r="B321" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3">
+      <c r="A322" t="s">
         <v>1169</v>
       </c>
-      <c r="B321" t="s">
+      <c r="B322" t="s">
         <v>1170</v>
-      </c>
-    </row>
-    <row r="323" spans="1:3">
-      <c r="A323" t="s">
-        <v>469</v>
-      </c>
-      <c r="B323" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="324" spans="1:3">
       <c r="A324" t="s">
-        <v>389</v>
+        <v>469</v>
       </c>
       <c r="B324" t="s">
-        <v>400</v>
+        <v>468</v>
       </c>
     </row>
     <row r="325" spans="1:3">
       <c r="A325" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B325" t="s">
-        <v>401</v>
-      </c>
-      <c r="C325" t="s">
-        <v>527</v>
+        <v>400</v>
       </c>
     </row>
     <row r="326" spans="1:3">
       <c r="A326" t="s">
-        <v>459</v>
+        <v>390</v>
       </c>
       <c r="B326" t="s">
-        <v>517</v>
+        <v>401</v>
+      </c>
+      <c r="C326" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="327" spans="1:3">
       <c r="A327" t="s">
-        <v>391</v>
+        <v>459</v>
       </c>
       <c r="B327" t="s">
-        <v>402</v>
-      </c>
-      <c r="C327" t="s">
-        <v>527</v>
+        <v>517</v>
       </c>
     </row>
     <row r="328" spans="1:3">
       <c r="A328" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B328" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C328" t="s">
         <v>527</v>
@@ -11282,1437 +11315,1448 @@
     </row>
     <row r="329" spans="1:3">
       <c r="A329" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B329" t="s">
-        <v>529</v>
+        <v>403</v>
+      </c>
+      <c r="C329" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="330" spans="1:3">
       <c r="A330" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B330" t="s">
-        <v>377</v>
+        <v>529</v>
       </c>
     </row>
     <row r="331" spans="1:3">
       <c r="A331" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B331" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="332" spans="1:3">
       <c r="A332" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B332" t="s">
-        <v>404</v>
+        <v>378</v>
       </c>
     </row>
     <row r="333" spans="1:3">
       <c r="A333" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="B333" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="334" spans="1:3">
       <c r="A334" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B334" t="s">
-        <v>381</v>
+        <v>405</v>
       </c>
     </row>
     <row r="335" spans="1:3">
       <c r="A335" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B335" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="336" spans="1:3">
       <c r="A336" t="s">
-        <v>473</v>
+        <v>399</v>
       </c>
       <c r="B336" t="s">
-        <v>1128</v>
+        <v>382</v>
       </c>
     </row>
     <row r="337" spans="1:3">
       <c r="A337" t="s">
-        <v>558</v>
+        <v>473</v>
       </c>
       <c r="B337" t="s">
-        <v>552</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="338" spans="1:3">
       <c r="A338" t="s">
+        <v>558</v>
+      </c>
+      <c r="B338" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3">
+      <c r="A339" t="s">
         <v>1171</v>
       </c>
-      <c r="B338" t="s">
+      <c r="B339" t="s">
         <v>1172</v>
-      </c>
-    </row>
-    <row r="340" spans="1:3">
-      <c r="A340" t="s">
-        <v>640</v>
-      </c>
-      <c r="B340" t="s">
-        <v>641</v>
-      </c>
-      <c r="C340" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="341" spans="1:3">
       <c r="A341" t="s">
-        <v>383</v>
+        <v>640</v>
       </c>
       <c r="B341" t="s">
-        <v>559</v>
+        <v>641</v>
+      </c>
+      <c r="C341" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="342" spans="1:3">
       <c r="A342" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B342" t="s">
-        <v>560</v>
-      </c>
-      <c r="C342" t="s">
-        <v>527</v>
+        <v>559</v>
       </c>
     </row>
     <row r="343" spans="1:3">
       <c r="A343" t="s">
-        <v>460</v>
+        <v>384</v>
       </c>
       <c r="B343" t="s">
-        <v>561</v>
+        <v>560</v>
+      </c>
+      <c r="C343" t="s">
+        <v>527</v>
       </c>
     </row>
     <row r="344" spans="1:3">
       <c r="A344" t="s">
-        <v>385</v>
+        <v>460</v>
       </c>
       <c r="B344" t="s">
-        <v>586</v>
+        <v>561</v>
       </c>
     </row>
     <row r="345" spans="1:3">
       <c r="A345" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B345" t="s">
-        <v>562</v>
+        <v>586</v>
       </c>
     </row>
     <row r="346" spans="1:3">
       <c r="A346" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B346" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="347" spans="1:3">
       <c r="A347" t="s">
-        <v>1106</v>
+        <v>387</v>
       </c>
       <c r="B347" t="s">
-        <v>1107</v>
-      </c>
-      <c r="C347" t="s">
-        <v>1173</v>
+        <v>563</v>
       </c>
     </row>
     <row r="348" spans="1:3">
       <c r="A348" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B348" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C348" t="s">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3">
+      <c r="A349" t="s">
         <v>472</v>
       </c>
-      <c r="B348" t="s">
+      <c r="B349" t="s">
         <v>1129</v>
-      </c>
-    </row>
-    <row r="350" spans="1:3">
-      <c r="A350" t="s">
-        <v>712</v>
-      </c>
-      <c r="B350" t="s">
-        <v>713</v>
-      </c>
-      <c r="C350" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="351" spans="1:3">
       <c r="A351" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="B351" t="s">
-        <v>1130</v>
+        <v>713</v>
       </c>
       <c r="C351" t="s">
         <v>598</v>
       </c>
     </row>
-    <row r="353" spans="1:2">
-      <c r="A353" t="s">
-        <v>720</v>
-      </c>
-      <c r="B353" t="s">
-        <v>721</v>
+    <row r="352" spans="1:3">
+      <c r="A352" t="s">
+        <v>714</v>
+      </c>
+      <c r="B352" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C352" t="s">
+        <v>598</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="A354" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B354" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
     </row>
     <row r="355" spans="1:2">
       <c r="A355" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="B355" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
     </row>
     <row r="356" spans="1:2">
       <c r="A356" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="B356" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
     </row>
     <row r="357" spans="1:2">
       <c r="A357" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="B357" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
     </row>
     <row r="358" spans="1:2">
       <c r="A358" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="B358" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
     </row>
     <row r="359" spans="1:2">
       <c r="A359" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="B359" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
     </row>
     <row r="360" spans="1:2">
       <c r="A360" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="B360" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
     </row>
     <row r="361" spans="1:2">
       <c r="A361" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="B361" t="s">
-        <v>1174</v>
+        <v>735</v>
       </c>
     </row>
     <row r="362" spans="1:2">
       <c r="A362" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B362" t="s">
-        <v>738</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="363" spans="1:2">
       <c r="A363" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="B363" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
     </row>
     <row r="364" spans="1:2">
       <c r="A364" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="B364" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
     </row>
     <row r="365" spans="1:2">
       <c r="A365" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="B365" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
     </row>
     <row r="366" spans="1:2">
       <c r="A366" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="B366" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
     </row>
     <row r="367" spans="1:2">
       <c r="A367" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="B367" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
     </row>
     <row r="368" spans="1:2">
       <c r="A368" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="B368" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
     </row>
     <row r="369" spans="1:2">
       <c r="A369" t="s">
-        <v>1102</v>
+        <v>749</v>
       </c>
       <c r="B369" t="s">
-        <v>1103</v>
+        <v>750</v>
       </c>
     </row>
     <row r="370" spans="1:2">
       <c r="A370" t="s">
-        <v>751</v>
+        <v>1102</v>
       </c>
       <c r="B370" t="s">
-        <v>752</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="371" spans="1:2">
       <c r="A371" t="s">
-        <v>1105</v>
+        <v>751</v>
       </c>
       <c r="B371" t="s">
-        <v>1131</v>
+        <v>752</v>
       </c>
     </row>
     <row r="372" spans="1:2">
       <c r="A372" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B372" t="s">
+        <v>1131</v>
+      </c>
+    </row>
+    <row r="373" spans="1:2">
+      <c r="A373" t="s">
         <v>1175</v>
       </c>
-      <c r="B372" t="s">
+      <c r="B373" t="s">
         <v>1176</v>
-      </c>
-    </row>
-    <row r="374" spans="1:2">
-      <c r="A374" t="s">
-        <v>753</v>
-      </c>
-      <c r="B374" t="s">
-        <v>754</v>
       </c>
     </row>
     <row r="375" spans="1:2">
       <c r="A375" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="B375" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
     </row>
     <row r="376" spans="1:2">
       <c r="A376" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="B376" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
     </row>
     <row r="377" spans="1:2">
       <c r="A377" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="B377" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
     </row>
     <row r="378" spans="1:2">
       <c r="A378" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="B378" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
     </row>
     <row r="379" spans="1:2">
       <c r="A379" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="B379" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
     </row>
     <row r="380" spans="1:2">
       <c r="A380" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="B380" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
     </row>
     <row r="381" spans="1:2">
       <c r="A381" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B381" t="s">
-        <v>315</v>
+        <v>766</v>
       </c>
     </row>
     <row r="382" spans="1:2">
       <c r="A382" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B382" t="s">
-        <v>769</v>
+        <v>315</v>
       </c>
     </row>
     <row r="383" spans="1:2">
       <c r="A383" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B383" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
     </row>
     <row r="384" spans="1:2">
       <c r="A384" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="B384" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
     </row>
     <row r="385" spans="1:2">
       <c r="A385" t="s">
+        <v>772</v>
+      </c>
+      <c r="B385" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="386" spans="1:2">
+      <c r="A386" t="s">
         <v>774</v>
       </c>
-      <c r="B385" t="s">
+      <c r="B386" t="s">
         <v>1132</v>
-      </c>
-    </row>
-    <row r="387" spans="1:2">
-      <c r="A387" t="s">
-        <v>775</v>
-      </c>
-      <c r="B387" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="388" spans="1:2">
       <c r="A388" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="B388" t="s">
-        <v>777</v>
+        <v>308</v>
       </c>
     </row>
     <row r="389" spans="1:2">
       <c r="A389" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="B389" t="s">
-        <v>310</v>
+        <v>777</v>
       </c>
     </row>
     <row r="390" spans="1:2">
       <c r="A390" t="s">
+        <v>778</v>
+      </c>
+      <c r="B390" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="391" spans="1:2">
+      <c r="A391" t="s">
         <v>779</v>
       </c>
-      <c r="B390" t="s">
+      <c r="B391" t="s">
         <v>1177</v>
-      </c>
-    </row>
-    <row r="392" spans="1:2">
-      <c r="A392" t="s">
-        <v>801</v>
-      </c>
-      <c r="B392" t="s">
-        <v>802</v>
       </c>
     </row>
     <row r="393" spans="1:2">
       <c r="A393" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B393" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
     </row>
     <row r="394" spans="1:2">
       <c r="A394" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="B394" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
     </row>
     <row r="395" spans="1:2">
       <c r="A395" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="B395" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="396" spans="1:2">
       <c r="A396" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="B396" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="397" spans="1:2">
       <c r="A397" t="s">
+        <v>793</v>
+      </c>
+      <c r="B397" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="398" spans="1:2">
+      <c r="A398" t="s">
         <v>798</v>
       </c>
-      <c r="B397" t="s">
+      <c r="B398" t="s">
         <v>1178</v>
-      </c>
-    </row>
-    <row r="399" spans="1:2">
-      <c r="A399" t="s">
-        <v>805</v>
-      </c>
-      <c r="B399" t="s">
-        <v>810</v>
       </c>
     </row>
     <row r="400" spans="1:2">
       <c r="A400" t="s">
-        <v>812</v>
+        <v>805</v>
       </c>
       <c r="B400" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
     </row>
     <row r="401" spans="1:2">
       <c r="A401" t="s">
-        <v>806</v>
+        <v>812</v>
       </c>
       <c r="B401" t="s">
-        <v>795</v>
+        <v>811</v>
       </c>
     </row>
     <row r="402" spans="1:2">
       <c r="A402" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="B402" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
     </row>
     <row r="403" spans="1:2">
       <c r="A403" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="B403" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="404" spans="1:2">
       <c r="A404" t="s">
+        <v>808</v>
+      </c>
+      <c r="B404" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="405" spans="1:2">
+      <c r="A405" t="s">
         <v>809</v>
       </c>
-      <c r="B404" t="s">
+      <c r="B405" t="s">
         <v>1133</v>
-      </c>
-    </row>
-    <row r="406" spans="1:2">
-      <c r="A406" t="s">
-        <v>817</v>
-      </c>
-      <c r="B406" t="s">
-        <v>818</v>
       </c>
     </row>
     <row r="407" spans="1:2">
       <c r="A407" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="B407" t="s">
-        <v>1101</v>
+        <v>818</v>
       </c>
     </row>
     <row r="408" spans="1:2">
       <c r="A408" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="B408" t="s">
-        <v>1011</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="409" spans="1:2">
       <c r="A409" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="B409" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="410" spans="1:2">
       <c r="A410" t="s">
-        <v>828</v>
+        <v>822</v>
       </c>
       <c r="B410" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="411" spans="1:2">
       <c r="A411" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="B411" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="412" spans="1:2">
       <c r="A412" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="B412" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="413" spans="1:2">
       <c r="A413" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="B413" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="414" spans="1:2">
       <c r="A414" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="B414" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="415" spans="1:2">
       <c r="A415" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B415" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="416" spans="1:2">
       <c r="A416" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="B416" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="417" spans="1:2">
       <c r="A417" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B417" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="418" spans="1:2">
       <c r="A418" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B418" t="s">
-        <v>827</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="419" spans="1:2">
       <c r="A419" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B419" t="s">
-        <v>1021</v>
+        <v>827</v>
       </c>
     </row>
     <row r="420" spans="1:2">
       <c r="A420" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B420" t="s">
-        <v>275</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="421" spans="1:2">
       <c r="A421" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="B421" t="s">
-        <v>786</v>
+        <v>275</v>
       </c>
     </row>
     <row r="422" spans="1:2">
       <c r="A422" t="s">
-        <v>832</v>
+        <v>841</v>
       </c>
       <c r="B422" t="s">
-        <v>604</v>
+        <v>786</v>
       </c>
     </row>
     <row r="423" spans="1:2">
       <c r="A423" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="B423" t="s">
-        <v>1134</v>
+        <v>604</v>
       </c>
     </row>
     <row r="424" spans="1:2">
       <c r="A424" t="s">
-        <v>1179</v>
+        <v>831</v>
       </c>
       <c r="B424" t="s">
-        <v>1161</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="425" spans="1:2">
       <c r="A425" t="s">
-        <v>1022</v>
+        <v>1179</v>
       </c>
       <c r="B425" t="s">
-        <v>1023</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="426" spans="1:2">
       <c r="A426" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="B426" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="427" spans="1:2">
       <c r="A427" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="B427" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="428" spans="1:2">
       <c r="A428" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="B428" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="429" spans="1:2">
       <c r="A429" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="B429" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
     </row>
     <row r="430" spans="1:2">
       <c r="A430" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="B430" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="431" spans="1:2">
       <c r="A431" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="B431" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="432" spans="1:2">
       <c r="A432" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="B432" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="433" spans="1:2">
       <c r="A433" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B433" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="434" spans="1:2">
+      <c r="A434" t="s">
         <v>1143</v>
       </c>
-      <c r="B433" t="s">
+      <c r="B434" t="s">
         <v>1180</v>
-      </c>
-    </row>
-    <row r="435" spans="1:2">
-      <c r="A435" t="s">
-        <v>881</v>
-      </c>
-      <c r="B435" t="s">
-        <v>882</v>
       </c>
     </row>
     <row r="436" spans="1:2">
       <c r="A436" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="B436" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
     </row>
     <row r="437" spans="1:2">
       <c r="A437" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="B437" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
     </row>
     <row r="438" spans="1:2">
       <c r="A438" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="B438" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
     </row>
     <row r="439" spans="1:2">
       <c r="A439" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="B439" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
     </row>
     <row r="440" spans="1:2">
       <c r="A440" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="B440" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
     </row>
     <row r="441" spans="1:2">
       <c r="A441" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="B441" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
     </row>
     <row r="442" spans="1:2">
       <c r="A442" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="B442" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
     </row>
     <row r="443" spans="1:2">
       <c r="A443" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="B443" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
     </row>
     <row r="444" spans="1:2">
       <c r="A444" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="B444" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
     </row>
     <row r="445" spans="1:2">
       <c r="A445" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="B445" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
     </row>
     <row r="446" spans="1:2">
       <c r="A446" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="B446" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
     </row>
     <row r="447" spans="1:2">
       <c r="A447" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="B447" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
     </row>
     <row r="448" spans="1:2">
       <c r="A448" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="B448" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
     </row>
     <row r="449" spans="1:2">
       <c r="A449" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="B449" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
     </row>
     <row r="450" spans="1:2">
       <c r="A450" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="B450" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
     </row>
     <row r="451" spans="1:2">
       <c r="A451" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="B451" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
     </row>
     <row r="452" spans="1:2">
       <c r="A452" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
       <c r="B452" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
     </row>
     <row r="453" spans="1:2">
       <c r="A453" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="B453" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
     </row>
     <row r="454" spans="1:2">
       <c r="A454" t="s">
-        <v>919</v>
+        <v>917</v>
       </c>
       <c r="B454" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
     </row>
     <row r="455" spans="1:2">
       <c r="A455" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="B455" t="s">
-        <v>1135</v>
+        <v>920</v>
       </c>
     </row>
     <row r="456" spans="1:2">
       <c r="A456" t="s">
+        <v>921</v>
+      </c>
+      <c r="B456" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="457" spans="1:2">
+      <c r="A457" t="s">
         <v>1181</v>
       </c>
-      <c r="B456" t="s">
+      <c r="B457" t="s">
         <v>1182</v>
-      </c>
-    </row>
-    <row r="458" spans="1:2">
-      <c r="A458" t="s">
-        <v>1108</v>
-      </c>
-      <c r="B458" t="s">
-        <v>1109</v>
       </c>
     </row>
     <row r="459" spans="1:2">
       <c r="A459" t="s">
-        <v>922</v>
+        <v>1108</v>
       </c>
       <c r="B459" t="s">
-        <v>923</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="460" spans="1:2">
       <c r="A460" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="B460" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
     </row>
     <row r="461" spans="1:2">
       <c r="A461" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="B461" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
     </row>
     <row r="462" spans="1:2">
       <c r="A462" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="B462" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
     </row>
     <row r="463" spans="1:2">
       <c r="A463" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="B463" t="s">
-        <v>1183</v>
+        <v>929</v>
       </c>
     </row>
     <row r="464" spans="1:2">
       <c r="A464" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="B464" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="465" spans="1:2">
       <c r="A465" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="B465" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="466" spans="1:2">
       <c r="A466" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="B466" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="467" spans="1:2">
       <c r="A467" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="B467" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="468" spans="1:2">
       <c r="A468" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
       <c r="B468" t="s">
-        <v>1136</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="469" spans="1:2">
       <c r="A469" t="s">
+        <v>935</v>
+      </c>
+      <c r="B469" t="s">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="470" spans="1:2">
+      <c r="A470" t="s">
         <v>1188</v>
       </c>
-      <c r="B469" t="s">
+      <c r="B470" t="s">
         <v>1189</v>
-      </c>
-    </row>
-    <row r="471" spans="1:2">
-      <c r="A471" t="s">
-        <v>942</v>
-      </c>
-      <c r="B471" t="s">
-        <v>943</v>
       </c>
     </row>
     <row r="472" spans="1:2">
       <c r="A472" t="s">
+        <v>942</v>
+      </c>
+      <c r="B472" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="473" spans="1:2">
+      <c r="A473" t="s">
         <v>944</v>
       </c>
-      <c r="B472" t="s">
+      <c r="B473" t="s">
         <v>1137</v>
-      </c>
-    </row>
-    <row r="474" spans="1:2">
-      <c r="A474" t="s">
-        <v>945</v>
-      </c>
-      <c r="B474" t="s">
-        <v>946</v>
       </c>
     </row>
     <row r="475" spans="1:2">
       <c r="A475" t="s">
+        <v>945</v>
+      </c>
+      <c r="B475" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="476" spans="1:2">
+      <c r="A476" t="s">
         <v>947</v>
       </c>
-      <c r="B475" t="s">
+      <c r="B476" t="s">
         <v>1138</v>
-      </c>
-    </row>
-    <row r="477" spans="1:2">
-      <c r="A477" t="s">
-        <v>948</v>
-      </c>
-      <c r="B477" t="s">
-        <v>949</v>
       </c>
     </row>
     <row r="478" spans="1:2">
       <c r="A478" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="B478" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
     </row>
     <row r="479" spans="1:2">
       <c r="A479" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="B479" t="s">
-        <v>1139</v>
+        <v>951</v>
       </c>
     </row>
     <row r="480" spans="1:2">
       <c r="A480" t="s">
+        <v>952</v>
+      </c>
+      <c r="B480" t="s">
+        <v>1139</v>
+      </c>
+    </row>
+    <row r="481" spans="1:2">
+      <c r="A481" t="s">
         <v>1190</v>
       </c>
-      <c r="B480" t="s">
+      <c r="B481" t="s">
         <v>1191</v>
-      </c>
-    </row>
-    <row r="482" spans="1:2">
-      <c r="A482" t="s">
-        <v>953</v>
-      </c>
-      <c r="B482" t="s">
-        <v>954</v>
       </c>
     </row>
     <row r="483" spans="1:2">
       <c r="A483" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="B483" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
     </row>
     <row r="484" spans="1:2">
       <c r="A484" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="B484" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
     </row>
     <row r="485" spans="1:2">
       <c r="A485" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="B485" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
     </row>
     <row r="486" spans="1:2">
       <c r="A486" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="B486" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
     </row>
     <row r="487" spans="1:2">
       <c r="A487" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="B487" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
     </row>
     <row r="488" spans="1:2">
       <c r="A488" t="s">
+        <v>963</v>
+      </c>
+      <c r="B488" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="489" spans="1:2">
+      <c r="A489" t="s">
         <v>965</v>
       </c>
-      <c r="B488" t="s">
+      <c r="B489" t="s">
         <v>1192</v>
-      </c>
-    </row>
-    <row r="490" spans="1:2">
-      <c r="A490" t="s">
-        <v>966</v>
-      </c>
-      <c r="B490" t="s">
-        <v>967</v>
       </c>
     </row>
     <row r="491" spans="1:2">
       <c r="A491" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
       <c r="B491" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
     </row>
     <row r="492" spans="1:2">
       <c r="A492" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="B492" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
     </row>
     <row r="493" spans="1:2">
       <c r="A493" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="B493" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
     </row>
     <row r="494" spans="1:2">
       <c r="A494" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="B494" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
     </row>
     <row r="495" spans="1:2">
       <c r="A495" t="s">
+        <v>974</v>
+      </c>
+      <c r="B495" t="s">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="496" spans="1:2">
+      <c r="A496" t="s">
         <v>976</v>
       </c>
-      <c r="B495" t="s">
+      <c r="B496" t="s">
         <v>1193</v>
-      </c>
-    </row>
-    <row r="497" spans="1:2">
-      <c r="A497" t="s">
-        <v>977</v>
-      </c>
-      <c r="B497" t="s">
-        <v>978</v>
       </c>
     </row>
     <row r="498" spans="1:2">
       <c r="A498" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="B498" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
     </row>
     <row r="499" spans="1:2">
       <c r="A499" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="B499" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
     </row>
     <row r="500" spans="1:2">
       <c r="A500" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="B500" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
     </row>
     <row r="501" spans="1:2">
       <c r="A501" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="B501" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
     </row>
     <row r="502" spans="1:2">
       <c r="A502" t="s">
+        <v>985</v>
+      </c>
+      <c r="B502" t="s">
+        <v>986</v>
+      </c>
+    </row>
+    <row r="503" spans="1:2">
+      <c r="A503" t="s">
         <v>987</v>
       </c>
-      <c r="B502" t="s">
+      <c r="B503" t="s">
         <v>1194</v>
-      </c>
-    </row>
-    <row r="504" spans="1:2">
-      <c r="A504" t="s">
-        <v>988</v>
-      </c>
-      <c r="B504" t="s">
-        <v>989</v>
       </c>
     </row>
     <row r="505" spans="1:2">
       <c r="A505" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="B505" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
     </row>
     <row r="506" spans="1:2">
       <c r="A506" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="B506" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
     </row>
     <row r="507" spans="1:2">
       <c r="A507" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="B507" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
     </row>
     <row r="508" spans="1:2">
       <c r="A508" t="s">
+        <v>994</v>
+      </c>
+      <c r="B508" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="509" spans="1:2">
+      <c r="A509" t="s">
         <v>996</v>
       </c>
-      <c r="B508" t="s">
+      <c r="B509" t="s">
         <v>1195</v>
-      </c>
-    </row>
-    <row r="510" spans="1:2">
-      <c r="A510" t="s">
-        <v>1038</v>
-      </c>
-      <c r="B510" t="s">
-        <v>1039</v>
       </c>
     </row>
     <row r="511" spans="1:2">
       <c r="A511" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="B511" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="512" spans="1:2">
       <c r="A512" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
       <c r="B512" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="513" spans="1:2">
       <c r="A513" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="B513" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="514" spans="1:2">
       <c r="A514" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
       <c r="B514" t="s">
-        <v>1047</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="515" spans="1:2">
       <c r="A515" t="s">
-        <v>1048</v>
+        <v>1046</v>
       </c>
       <c r="B515" t="s">
-        <v>1049</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="516" spans="1:2">
       <c r="A516" t="s">
-        <v>1050</v>
+        <v>1048</v>
       </c>
       <c r="B516" t="s">
-        <v>1051</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="517" spans="1:2">
       <c r="A517" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="B517" t="s">
-        <v>1053</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="518" spans="1:2">
       <c r="A518" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="B518" t="s">
-        <v>1055</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="519" spans="1:2">
       <c r="A519" t="s">
-        <v>1056</v>
+        <v>1054</v>
       </c>
       <c r="B519" t="s">
-        <v>1057</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="520" spans="1:2">
       <c r="A520" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="B520" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="521" spans="1:2">
       <c r="A521" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="B521" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="522" spans="1:2">
       <c r="A522" t="s">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="B522" t="s">
-        <v>1063</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="523" spans="1:2">
       <c r="A523" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B523" t="s">
+        <v>1063</v>
+      </c>
+    </row>
+    <row r="524" spans="1:2">
+      <c r="A524" t="s">
         <v>1064</v>
       </c>
-      <c r="B523" t="s">
+      <c r="B524" t="s">
         <v>1196</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A477:A478 A474:A475 A459:A469 A471:A472 A480">
+  <conditionalFormatting sqref="A478:A479 A475:A476 A460:A470 A472:A473 A481">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>